<commit_message>
update: 2026-04-09 ~ 2026-04-09
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.251</v>
+        <v>3.25</v>
       </c>
       <c r="G2" t="n">
         <v>3.462</v>
       </c>
       <c r="H2" t="n">
-        <v>3.582</v>
+        <v>3.59</v>
       </c>
       <c r="I2" t="n">
-        <v>3.776</v>
+        <v>3.79</v>
       </c>
       <c r="J2" t="n">
-        <v>3.964</v>
+        <v>3.978</v>
       </c>
       <c r="K2" t="n">
-        <v>4.356</v>
+        <v>4.369</v>
       </c>
       <c r="L2" t="n">
-        <v>4.526</v>
+        <v>4.537</v>
       </c>
       <c r="M2" t="n">
-        <v>4.826</v>
+        <v>4.839</v>
       </c>
       <c r="N2" t="n">
-        <v>5.063</v>
+        <v>5.086</v>
       </c>
       <c r="O2" t="n">
-        <v>5.279</v>
+        <v>5.288</v>
       </c>
       <c r="P2" t="n">
-        <v>5.464</v>
+        <v>5.485</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.102</v>
+        <v>6.125</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.275</v>
+        <v>4.273</v>
       </c>
       <c r="G3" t="n">
         <v>4.667</v>
       </c>
       <c r="H3" t="n">
-        <v>4.82</v>
+        <v>4.828</v>
       </c>
       <c r="I3" t="n">
-        <v>5.014</v>
+        <v>5.028</v>
       </c>
       <c r="J3" t="n">
-        <v>5.211</v>
+        <v>5.226</v>
       </c>
       <c r="K3" t="n">
-        <v>5.671</v>
+        <v>5.685</v>
       </c>
       <c r="L3" t="n">
-        <v>5.911</v>
+        <v>5.922</v>
       </c>
       <c r="M3" t="n">
-        <v>6.242</v>
+        <v>6.256</v>
       </c>
       <c r="N3" t="n">
-        <v>6.423</v>
+        <v>6.446</v>
       </c>
       <c r="O3" t="n">
-        <v>6.588</v>
+        <v>6.598</v>
       </c>
       <c r="P3" t="n">
-        <v>6.643</v>
+        <v>6.664</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.17</v>
+        <v>7.193</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.765</v>
+        <v>3.764</v>
       </c>
       <c r="G4" t="n">
         <v>4.047</v>
       </c>
       <c r="H4" t="n">
-        <v>4.229</v>
+        <v>4.237</v>
       </c>
       <c r="I4" t="n">
-        <v>4.454</v>
+        <v>4.468</v>
       </c>
       <c r="J4" t="n">
-        <v>4.658</v>
+        <v>4.672</v>
       </c>
       <c r="K4" t="n">
-        <v>5.111</v>
+        <v>5.125</v>
       </c>
       <c r="L4" t="n">
-        <v>5.282</v>
+        <v>5.292</v>
       </c>
       <c r="M4" t="n">
-        <v>5.6</v>
+        <v>5.614</v>
       </c>
       <c r="N4" t="n">
-        <v>5.751</v>
+        <v>5.774</v>
       </c>
       <c r="O4" t="n">
-        <v>5.94</v>
+        <v>5.95</v>
       </c>
       <c r="P4" t="n">
-        <v>5.992</v>
+        <v>6.013</v>
       </c>
       <c r="Q4" t="n">
-        <v>6.523</v>
+        <v>6.546</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.961</v>
+        <v>2.959</v>
       </c>
       <c r="G5" t="n">
         <v>3.013</v>
       </c>
       <c r="H5" t="n">
-        <v>3.085</v>
+        <v>3.093</v>
       </c>
       <c r="I5" t="n">
-        <v>3.348</v>
+        <v>3.362</v>
       </c>
       <c r="J5" t="n">
-        <v>3.535</v>
+        <v>3.55</v>
       </c>
       <c r="K5" t="n">
-        <v>3.785</v>
+        <v>3.8</v>
       </c>
       <c r="L5" t="n">
-        <v>3.797</v>
+        <v>3.81</v>
       </c>
       <c r="M5" t="n">
-        <v>3.904</v>
+        <v>3.918</v>
       </c>
       <c r="N5" t="n">
-        <v>3.868</v>
+        <v>3.892</v>
       </c>
       <c r="O5" t="n">
-        <v>3.871</v>
+        <v>3.884</v>
       </c>
       <c r="P5" t="n">
-        <v>4.134</v>
+        <v>4.154</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.014</v>
+        <v>5.037</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>3.001</v>
+        <v>3</v>
       </c>
       <c r="G6" t="n">
-        <v>3.065</v>
+        <v>3.066</v>
       </c>
       <c r="H6" t="n">
-        <v>3.154</v>
+        <v>3.162</v>
       </c>
       <c r="I6" t="n">
-        <v>3.422</v>
+        <v>3.436</v>
       </c>
       <c r="J6" t="n">
-        <v>3.62</v>
+        <v>3.633</v>
       </c>
       <c r="K6" t="n">
-        <v>3.887</v>
+        <v>3.901</v>
       </c>
       <c r="L6" t="n">
-        <v>3.912</v>
+        <v>3.923</v>
       </c>
       <c r="M6" t="n">
-        <v>4.051</v>
+        <v>4.064</v>
       </c>
       <c r="N6" t="n">
-        <v>4.038</v>
+        <v>4.061</v>
       </c>
       <c r="O6" t="n">
-        <v>4.147</v>
+        <v>4.156</v>
       </c>
       <c r="P6" t="n">
-        <v>4.566</v>
+        <v>4.587</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.41</v>
+        <v>5.433</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2.981</v>
+        <v>2.98</v>
       </c>
       <c r="G7" t="n">
-        <v>3.031</v>
+        <v>3.032</v>
       </c>
       <c r="H7" t="n">
-        <v>3.101</v>
+        <v>3.109</v>
       </c>
       <c r="I7" t="n">
-        <v>3.363</v>
+        <v>3.377</v>
       </c>
       <c r="J7" t="n">
-        <v>3.56</v>
+        <v>3.575</v>
       </c>
       <c r="K7" t="n">
-        <v>3.81</v>
+        <v>3.825</v>
       </c>
       <c r="L7" t="n">
-        <v>3.823</v>
+        <v>3.835</v>
       </c>
       <c r="M7" t="n">
-        <v>3.961</v>
+        <v>3.976</v>
       </c>
       <c r="N7" t="n">
-        <v>3.928</v>
+        <v>3.952</v>
       </c>
       <c r="O7" t="n">
-        <v>4.046</v>
+        <v>4.056</v>
       </c>
       <c r="P7" t="n">
-        <v>4.35</v>
+        <v>4.371</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.178</v>
+        <v>5.201</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.384</v>
+        <v>5.383</v>
       </c>
       <c r="G8" t="n">
         <v>5.965</v>
       </c>
       <c r="H8" t="n">
-        <v>6.269</v>
+        <v>6.277</v>
       </c>
       <c r="I8" t="n">
-        <v>6.534</v>
+        <v>6.548</v>
       </c>
       <c r="J8" t="n">
-        <v>6.796</v>
+        <v>6.81</v>
       </c>
       <c r="K8" t="n">
-        <v>7.537</v>
+        <v>7.55</v>
       </c>
       <c r="L8" t="n">
-        <v>7.867</v>
+        <v>7.877</v>
       </c>
       <c r="M8" t="n">
-        <v>8.226000000000001</v>
+        <v>8.239000000000001</v>
       </c>
       <c r="N8" t="n">
-        <v>8.343999999999999</v>
+        <v>8.367000000000001</v>
       </c>
       <c r="O8" t="n">
-        <v>8.595000000000001</v>
+        <v>8.605</v>
       </c>
       <c r="P8" t="n">
-        <v>8.749000000000001</v>
+        <v>8.77</v>
       </c>
       <c r="Q8" t="n">
-        <v>9.478999999999999</v>
+        <v>9.502000000000001</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,57 +1063,57 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.614</v>
+        <v>2.618</v>
       </c>
       <c r="G9" t="n">
-        <v>2.701</v>
+        <v>2.689</v>
       </c>
       <c r="H9" t="n">
-        <v>2.775</v>
+        <v>2.777</v>
       </c>
       <c r="I9" t="n">
-        <v>2.907</v>
+        <v>2.908</v>
       </c>
       <c r="J9" t="n">
-        <v>3.072</v>
+        <v>3.074</v>
       </c>
       <c r="K9" t="n">
-        <v>3.201</v>
+        <v>3.2</v>
       </c>
       <c r="L9" t="n">
-        <v>3.25</v>
+        <v>3.252</v>
       </c>
       <c r="M9" t="n">
-        <v>3.319</v>
+        <v>3.329</v>
       </c>
       <c r="N9" t="n">
-        <v>3.451</v>
+        <v>3.472</v>
       </c>
       <c r="O9" t="n">
-        <v>3.479</v>
+        <v>3.483</v>
       </c>
       <c r="P9" t="n">
-        <v>3.555</v>
+        <v>3.575</v>
       </c>
       <c r="Q9" t="n">
-        <v>3.632</v>
+        <v>3.655</v>
       </c>
       <c r="R9" t="n">
-        <v>3.649</v>
+        <v>3.674</v>
       </c>
       <c r="S9" t="n">
-        <v>3.612</v>
+        <v>3.641</v>
       </c>
       <c r="T9" t="n">
-        <v>3.53</v>
+        <v>3.572</v>
       </c>
       <c r="U9" t="n">
-        <v>3.434</v>
+        <v>3.476</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.626</v>
+        <v>2.63</v>
       </c>
       <c r="G10" t="n">
-        <v>2.732</v>
+        <v>2.721</v>
       </c>
       <c r="H10" t="n">
-        <v>2.786</v>
+        <v>2.788</v>
       </c>
       <c r="I10" t="n">
         <v>2.919</v>
       </c>
       <c r="J10" t="n">
-        <v>3.1</v>
+        <v>3.103</v>
       </c>
       <c r="K10" t="n">
-        <v>3.228</v>
+        <v>3.226</v>
       </c>
       <c r="L10" t="n">
-        <v>3.292</v>
+        <v>3.294</v>
       </c>
       <c r="M10" t="n">
-        <v>3.42</v>
+        <v>3.43</v>
       </c>
       <c r="N10" t="n">
-        <v>3.458</v>
+        <v>3.48</v>
       </c>
       <c r="O10" t="n">
-        <v>3.652</v>
+        <v>3.661</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.442</v>
+        <v>2.446</v>
       </c>
       <c r="G11" t="n">
-        <v>2.542</v>
+        <v>2.531</v>
       </c>
       <c r="H11" t="n">
-        <v>2.61</v>
+        <v>2.612</v>
       </c>
       <c r="I11" t="n">
         <v>2.721</v>
       </c>
       <c r="J11" t="n">
-        <v>2.894</v>
+        <v>2.897</v>
       </c>
       <c r="K11" t="n">
-        <v>3.016</v>
+        <v>3.014</v>
       </c>
       <c r="L11" t="n">
-        <v>3.086</v>
+        <v>3.088</v>
       </c>
       <c r="M11" t="n">
-        <v>3.224</v>
+        <v>3.234</v>
       </c>
       <c r="N11" t="n">
-        <v>3.269</v>
+        <v>3.29</v>
       </c>
       <c r="O11" t="n">
-        <v>3.419</v>
+        <v>3.427</v>
       </c>
       <c r="P11" t="n">
-        <v>3.492</v>
+        <v>3.512</v>
       </c>
       <c r="Q11" t="n">
-        <v>3.835</v>
+        <v>3.858</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.218</v>
+        <v>3.221</v>
       </c>
       <c r="G12" t="n">
-        <v>3.367</v>
+        <v>3.371</v>
       </c>
       <c r="H12" t="n">
-        <v>3.458</v>
+        <v>3.469</v>
       </c>
       <c r="I12" t="n">
-        <v>3.664</v>
+        <v>3.681</v>
       </c>
       <c r="J12" t="n">
-        <v>3.949</v>
+        <v>3.962</v>
       </c>
       <c r="K12" t="n">
-        <v>4.15</v>
+        <v>4.159</v>
       </c>
       <c r="L12" t="n">
-        <v>4.199</v>
+        <v>4.208</v>
       </c>
       <c r="M12" t="n">
-        <v>4.335</v>
+        <v>4.346</v>
       </c>
       <c r="N12" t="n">
-        <v>4.338</v>
+        <v>4.361</v>
       </c>
       <c r="O12" t="n">
-        <v>4.488</v>
+        <v>4.494</v>
       </c>
       <c r="P12" t="n">
-        <v>4.598</v>
+        <v>4.62</v>
       </c>
       <c r="Q12" t="n">
-        <v>4.962</v>
+        <v>4.986</v>
       </c>
       <c r="R12" t="n">
-        <v>5.146</v>
+        <v>5.171</v>
       </c>
       <c r="S12" t="n">
-        <v>5.322</v>
+        <v>5.352</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2.972</v>
+        <v>2.975</v>
       </c>
       <c r="G13" t="n">
-        <v>3.057</v>
+        <v>3.061</v>
       </c>
       <c r="H13" t="n">
-        <v>3.125</v>
+        <v>3.137</v>
       </c>
       <c r="I13" t="n">
-        <v>3.312</v>
+        <v>3.329</v>
       </c>
       <c r="J13" t="n">
-        <v>3.586</v>
+        <v>3.599</v>
       </c>
       <c r="K13" t="n">
-        <v>3.784</v>
+        <v>3.793</v>
       </c>
       <c r="L13" t="n">
-        <v>3.839</v>
+        <v>3.847</v>
       </c>
       <c r="M13" t="n">
-        <v>3.962</v>
+        <v>3.974</v>
       </c>
       <c r="N13" t="n">
-        <v>3.966</v>
+        <v>3.989</v>
       </c>
       <c r="O13" t="n">
-        <v>4.114</v>
+        <v>4.12</v>
       </c>
       <c r="P13" t="n">
-        <v>4.19</v>
+        <v>4.212</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.483</v>
+        <v>4.507</v>
       </c>
       <c r="R13" t="n">
-        <v>4.694</v>
+        <v>4.719</v>
       </c>
       <c r="S13" t="n">
-        <v>4.885</v>
+        <v>4.915</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.79</v>
+        <v>2.793</v>
       </c>
       <c r="G14" t="n">
-        <v>2.864</v>
+        <v>2.868</v>
       </c>
       <c r="H14" t="n">
-        <v>2.928</v>
+        <v>2.94</v>
       </c>
       <c r="I14" t="n">
-        <v>3.095</v>
+        <v>3.112</v>
       </c>
       <c r="J14" t="n">
-        <v>3.325</v>
+        <v>3.338</v>
       </c>
       <c r="K14" t="n">
-        <v>3.472</v>
+        <v>3.481</v>
       </c>
       <c r="L14" t="n">
-        <v>3.511</v>
+        <v>3.519</v>
       </c>
       <c r="M14" t="n">
-        <v>3.647</v>
+        <v>3.658</v>
       </c>
       <c r="N14" t="n">
-        <v>3.646</v>
+        <v>3.668</v>
       </c>
       <c r="O14" t="n">
-        <v>3.769</v>
+        <v>3.775</v>
       </c>
       <c r="P14" t="n">
-        <v>3.825</v>
+        <v>3.847</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.072</v>
+        <v>4.096</v>
       </c>
       <c r="R14" t="n">
-        <v>4.209</v>
+        <v>4.234</v>
       </c>
       <c r="S14" t="n">
-        <v>4.338</v>
+        <v>4.367</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.768</v>
+        <v>2.771</v>
       </c>
       <c r="G15" t="n">
-        <v>2.838</v>
+        <v>2.842</v>
       </c>
       <c r="H15" t="n">
-        <v>2.897</v>
+        <v>2.909</v>
       </c>
       <c r="I15" t="n">
-        <v>3.046</v>
+        <v>3.063</v>
       </c>
       <c r="J15" t="n">
-        <v>3.262</v>
+        <v>3.275</v>
       </c>
       <c r="K15" t="n">
-        <v>3.426</v>
+        <v>3.435</v>
       </c>
       <c r="L15" t="n">
-        <v>3.445</v>
+        <v>3.453</v>
       </c>
       <c r="M15" t="n">
-        <v>3.559</v>
+        <v>3.571</v>
       </c>
       <c r="N15" t="n">
-        <v>3.55</v>
+        <v>3.572</v>
       </c>
       <c r="O15" t="n">
-        <v>3.692</v>
+        <v>3.699</v>
       </c>
       <c r="P15" t="n">
-        <v>3.722</v>
+        <v>3.744</v>
       </c>
       <c r="Q15" t="n">
-        <v>3.977</v>
+        <v>4.001</v>
       </c>
       <c r="R15" t="n">
-        <v>4.106</v>
+        <v>4.13</v>
       </c>
       <c r="S15" t="n">
-        <v>4.233</v>
+        <v>4.263</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.768</v>
+        <v>2.771</v>
       </c>
       <c r="G16" t="n">
-        <v>2.838</v>
+        <v>2.842</v>
       </c>
       <c r="H16" t="n">
-        <v>2.897</v>
+        <v>2.909</v>
       </c>
       <c r="I16" t="n">
-        <v>3.046</v>
+        <v>3.063</v>
       </c>
       <c r="J16" t="n">
-        <v>3.262</v>
+        <v>3.275</v>
       </c>
       <c r="K16" t="n">
-        <v>3.426</v>
+        <v>3.435</v>
       </c>
       <c r="L16" t="n">
-        <v>3.445</v>
+        <v>3.453</v>
       </c>
       <c r="M16" t="n">
-        <v>3.559</v>
+        <v>3.571</v>
       </c>
       <c r="N16" t="n">
-        <v>3.553</v>
+        <v>3.575</v>
       </c>
       <c r="O16" t="n">
-        <v>3.698</v>
+        <v>3.706</v>
       </c>
       <c r="P16" t="n">
-        <v>3.745</v>
+        <v>3.767</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.004</v>
+        <v>4.028</v>
       </c>
       <c r="R16" t="n">
-        <v>4.133</v>
+        <v>4.159</v>
       </c>
       <c r="S16" t="n">
-        <v>4.262</v>
+        <v>4.291</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.688</v>
+        <v>2.692</v>
       </c>
       <c r="G17" t="n">
-        <v>2.824</v>
+        <v>2.812</v>
       </c>
       <c r="H17" t="n">
-        <v>2.88</v>
+        <v>2.881</v>
       </c>
       <c r="I17" t="n">
         <v>3.001</v>
       </c>
       <c r="J17" t="n">
-        <v>3.169</v>
+        <v>3.171</v>
       </c>
       <c r="K17" t="n">
-        <v>3.301</v>
+        <v>3.299</v>
       </c>
       <c r="L17" t="n">
-        <v>3.369</v>
+        <v>3.372</v>
       </c>
       <c r="M17" t="n">
-        <v>3.54</v>
+        <v>3.55</v>
       </c>
       <c r="N17" t="n">
-        <v>3.56</v>
+        <v>3.582</v>
       </c>
       <c r="O17" t="n">
-        <v>3.687</v>
+        <v>3.697</v>
       </c>
       <c r="P17" t="n">
-        <v>3.772</v>
+        <v>3.793</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.689</v>
+        <v>2.693</v>
       </c>
       <c r="G18" t="n">
-        <v>2.825</v>
+        <v>2.813</v>
       </c>
       <c r="H18" t="n">
-        <v>2.881</v>
+        <v>2.882</v>
       </c>
       <c r="I18" t="n">
-        <v>3</v>
+        <v>3.001</v>
       </c>
       <c r="J18" t="n">
-        <v>3.169</v>
+        <v>3.171</v>
       </c>
       <c r="K18" t="n">
-        <v>3.303</v>
+        <v>3.301</v>
       </c>
       <c r="L18" t="n">
-        <v>3.369</v>
+        <v>3.371</v>
       </c>
       <c r="M18" t="n">
-        <v>3.54</v>
+        <v>3.55</v>
       </c>
       <c r="N18" t="n">
-        <v>3.559</v>
+        <v>3.581</v>
       </c>
       <c r="O18" t="n">
-        <v>3.685</v>
+        <v>3.695</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.779</v>
+        <v>2.782</v>
       </c>
       <c r="G19" t="n">
-        <v>2.855</v>
+        <v>2.858</v>
       </c>
       <c r="H19" t="n">
-        <v>2.918</v>
+        <v>2.93</v>
       </c>
       <c r="I19" t="n">
-        <v>3.08</v>
+        <v>3.096</v>
       </c>
       <c r="J19" t="n">
-        <v>3.309</v>
+        <v>3.321</v>
       </c>
       <c r="K19" t="n">
-        <v>3.469</v>
+        <v>3.478</v>
       </c>
       <c r="L19" t="n">
-        <v>3.508</v>
+        <v>3.516</v>
       </c>
       <c r="M19" t="n">
-        <v>3.634</v>
+        <v>3.646</v>
       </c>
       <c r="N19" t="n">
-        <v>3.634</v>
+        <v>3.655</v>
       </c>
       <c r="O19" t="n">
-        <v>3.746</v>
+        <v>3.752</v>
       </c>
       <c r="P19" t="n">
-        <v>3.788</v>
+        <v>3.811</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.023</v>
+        <v>4.047</v>
       </c>
       <c r="R19" t="n">
-        <v>4.159</v>
+        <v>4.184</v>
       </c>
       <c r="S19" t="n">
-        <v>4.277</v>
+        <v>4.306</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2.569</v>
+        <v>2.572</v>
       </c>
       <c r="G20" t="n">
-        <v>2.639</v>
+        <v>2.644</v>
       </c>
       <c r="H20" t="n">
-        <v>2.687</v>
+        <v>2.694</v>
       </c>
       <c r="I20" t="n">
-        <v>2.849</v>
+        <v>2.857</v>
       </c>
       <c r="J20" t="n">
-        <v>3.08</v>
+        <v>3.085</v>
       </c>
       <c r="K20" t="n">
-        <v>3.235</v>
+        <v>3.24</v>
       </c>
       <c r="L20" t="n">
-        <v>3.268</v>
+        <v>3.28</v>
       </c>
       <c r="M20" t="n">
-        <v>3.363</v>
+        <v>3.373</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1945,40 +1945,40 @@
         <v>2.956</v>
       </c>
       <c r="H21" t="n">
-        <v>3.067</v>
+        <v>3.072</v>
       </c>
       <c r="I21" t="n">
-        <v>3.224</v>
+        <v>3.238</v>
       </c>
       <c r="J21" t="n">
-        <v>3.44</v>
+        <v>3.45</v>
       </c>
       <c r="K21" t="n">
-        <v>3.704</v>
+        <v>3.713</v>
       </c>
       <c r="L21" t="n">
-        <v>3.774</v>
+        <v>3.78</v>
       </c>
       <c r="M21" t="n">
-        <v>3.891</v>
+        <v>3.904</v>
       </c>
       <c r="N21" t="n">
-        <v>3.899</v>
+        <v>3.921</v>
       </c>
       <c r="O21" t="n">
-        <v>3.984</v>
+        <v>3.992</v>
       </c>
       <c r="P21" t="n">
-        <v>4.053</v>
+        <v>4.076</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.182</v>
+        <v>4.207</v>
       </c>
       <c r="R21" t="n">
-        <v>4.206</v>
+        <v>4.231</v>
       </c>
       <c r="S21" t="n">
-        <v>4.237</v>
+        <v>4.265</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2015,43 +2015,43 @@
         <v>2.822</v>
       </c>
       <c r="G22" t="n">
-        <v>2.903</v>
+        <v>2.902</v>
       </c>
       <c r="H22" t="n">
-        <v>3.001</v>
+        <v>3.007</v>
       </c>
       <c r="I22" t="n">
-        <v>3.142</v>
+        <v>3.157</v>
       </c>
       <c r="J22" t="n">
-        <v>3.324</v>
+        <v>3.335</v>
       </c>
       <c r="K22" t="n">
-        <v>3.585</v>
+        <v>3.593</v>
       </c>
       <c r="L22" t="n">
-        <v>3.643</v>
+        <v>3.649</v>
       </c>
       <c r="M22" t="n">
-        <v>3.763</v>
+        <v>3.775</v>
       </c>
       <c r="N22" t="n">
-        <v>3.771</v>
+        <v>3.794</v>
       </c>
       <c r="O22" t="n">
-        <v>3.853</v>
+        <v>3.86</v>
       </c>
       <c r="P22" t="n">
-        <v>3.915</v>
+        <v>3.938</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.041</v>
+        <v>4.065</v>
       </c>
       <c r="R22" t="n">
-        <v>4.052</v>
+        <v>4.078</v>
       </c>
       <c r="S22" t="n">
-        <v>4.081</v>
+        <v>4.11</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.774</v>
+        <v>2.775</v>
       </c>
       <c r="G23" t="n">
-        <v>2.856</v>
+        <v>2.857</v>
       </c>
       <c r="H23" t="n">
-        <v>2.94</v>
+        <v>2.945</v>
       </c>
       <c r="I23" t="n">
-        <v>3.095</v>
+        <v>3.109</v>
       </c>
       <c r="J23" t="n">
-        <v>3.27</v>
+        <v>3.281</v>
       </c>
       <c r="K23" t="n">
-        <v>3.504</v>
+        <v>3.513</v>
       </c>
       <c r="L23" t="n">
-        <v>3.554</v>
+        <v>3.56</v>
       </c>
       <c r="M23" t="n">
-        <v>3.667</v>
+        <v>3.68</v>
       </c>
       <c r="N23" t="n">
-        <v>3.667</v>
+        <v>3.69</v>
       </c>
       <c r="O23" t="n">
-        <v>3.727</v>
+        <v>3.734</v>
       </c>
       <c r="P23" t="n">
-        <v>3.777</v>
+        <v>3.8</v>
       </c>
       <c r="Q23" t="n">
-        <v>3.851</v>
+        <v>3.875</v>
       </c>
       <c r="R23" t="n">
-        <v>3.835</v>
+        <v>3.862</v>
       </c>
       <c r="S23" t="n">
-        <v>3.835</v>
+        <v>3.864</v>
       </c>
       <c r="T23" t="n">
-        <v>3.742</v>
+        <v>3.784</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2161,43 +2161,43 @@
         <v>2.706</v>
       </c>
       <c r="G24" t="n">
-        <v>2.771</v>
+        <v>2.772</v>
       </c>
       <c r="H24" t="n">
-        <v>2.842</v>
+        <v>2.847</v>
       </c>
       <c r="I24" t="n">
-        <v>3.005</v>
+        <v>3.02</v>
       </c>
       <c r="J24" t="n">
-        <v>3.171</v>
+        <v>3.182</v>
       </c>
       <c r="K24" t="n">
-        <v>3.389</v>
+        <v>3.397</v>
       </c>
       <c r="L24" t="n">
-        <v>3.427</v>
+        <v>3.431</v>
       </c>
       <c r="M24" t="n">
-        <v>3.523</v>
+        <v>3.535</v>
       </c>
       <c r="N24" t="n">
-        <v>3.538</v>
+        <v>3.56</v>
       </c>
       <c r="O24" t="n">
-        <v>3.678</v>
+        <v>3.686</v>
       </c>
       <c r="P24" t="n">
-        <v>3.716</v>
+        <v>3.738</v>
       </c>
       <c r="Q24" t="n">
-        <v>3.771</v>
+        <v>3.795</v>
       </c>
       <c r="R24" t="n">
-        <v>3.755</v>
+        <v>3.781</v>
       </c>
       <c r="S24" t="n">
-        <v>3.751</v>
+        <v>3.78</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.767</v>
+        <v>2.768</v>
       </c>
       <c r="G25" t="n">
-        <v>2.855</v>
+        <v>2.856</v>
       </c>
       <c r="H25" t="n">
-        <v>2.943</v>
+        <v>2.949</v>
       </c>
       <c r="I25" t="n">
-        <v>3.103</v>
+        <v>3.117</v>
       </c>
       <c r="J25" t="n">
-        <v>3.286</v>
+        <v>3.297</v>
       </c>
       <c r="K25" t="n">
-        <v>3.533</v>
+        <v>3.541</v>
       </c>
       <c r="L25" t="n">
-        <v>3.583</v>
+        <v>3.588</v>
       </c>
       <c r="M25" t="n">
-        <v>3.695</v>
+        <v>3.707</v>
       </c>
       <c r="N25" t="n">
-        <v>3.694</v>
+        <v>3.717</v>
       </c>
       <c r="O25" t="n">
-        <v>3.756</v>
+        <v>3.764</v>
       </c>
       <c r="P25" t="n">
-        <v>3.799</v>
+        <v>3.822</v>
       </c>
       <c r="Q25" t="n">
-        <v>3.883</v>
+        <v>3.908</v>
       </c>
       <c r="R25" t="n">
-        <v>3.859</v>
+        <v>3.886</v>
       </c>
       <c r="S25" t="n">
-        <v>3.858</v>
+        <v>3.888</v>
       </c>
       <c r="T25" t="n">
-        <v>3.76</v>
+        <v>3.802</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.085</v>
+        <v>3.086</v>
       </c>
       <c r="G26" t="n">
-        <v>3.213</v>
+        <v>3.216</v>
       </c>
       <c r="H26" t="n">
-        <v>3.386</v>
+        <v>3.395</v>
       </c>
       <c r="I26" t="n">
-        <v>3.627</v>
+        <v>3.641</v>
       </c>
       <c r="J26" t="n">
-        <v>3.93</v>
+        <v>3.944</v>
       </c>
       <c r="K26" t="n">
-        <v>4.31</v>
+        <v>4.323</v>
       </c>
       <c r="L26" t="n">
-        <v>4.41</v>
+        <v>4.422</v>
       </c>
       <c r="M26" t="n">
-        <v>4.6</v>
+        <v>4.614</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>4.814</v>
+        <v>4.823</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.879</v>
+        <v>2.882</v>
       </c>
       <c r="G27" t="n">
-        <v>2.945</v>
+        <v>2.947</v>
       </c>
       <c r="H27" t="n">
-        <v>3.027</v>
+        <v>3.037</v>
       </c>
       <c r="I27" t="n">
-        <v>3.213</v>
+        <v>3.228</v>
       </c>
       <c r="J27" t="n">
-        <v>3.438</v>
+        <v>3.45</v>
       </c>
       <c r="K27" t="n">
-        <v>3.638</v>
+        <v>3.648</v>
       </c>
       <c r="L27" t="n">
-        <v>3.686</v>
+        <v>3.695</v>
       </c>
       <c r="M27" t="n">
-        <v>3.814</v>
+        <v>3.825</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>3.911</v>
+        <v>3.917</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2.978</v>
+        <v>2.983</v>
       </c>
       <c r="G28" t="n">
-        <v>3.05</v>
+        <v>3.054</v>
       </c>
       <c r="H28" t="n">
-        <v>3.15</v>
+        <v>3.16</v>
       </c>
       <c r="I28" t="n">
-        <v>3.349</v>
+        <v>3.364</v>
       </c>
       <c r="J28" t="n">
-        <v>3.611</v>
+        <v>3.624</v>
       </c>
       <c r="K28" t="n">
-        <v>3.831</v>
+        <v>3.841</v>
       </c>
       <c r="L28" t="n">
-        <v>3.889</v>
+        <v>3.898</v>
       </c>
       <c r="M28" t="n">
-        <v>4.026</v>
+        <v>4.038</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.205</v>
+        <v>4.211</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.838</v>
+        <v>2.841</v>
       </c>
       <c r="G29" t="n">
-        <v>2.906</v>
+        <v>2.908</v>
       </c>
       <c r="H29" t="n">
-        <v>2.972</v>
+        <v>2.983</v>
       </c>
       <c r="I29" t="n">
-        <v>3.145</v>
+        <v>3.161</v>
       </c>
       <c r="J29" t="n">
-        <v>3.35</v>
+        <v>3.363</v>
       </c>
       <c r="K29" t="n">
-        <v>3.536</v>
+        <v>3.546</v>
       </c>
       <c r="L29" t="n">
-        <v>3.57</v>
+        <v>3.579</v>
       </c>
       <c r="M29" t="n">
-        <v>3.675</v>
+        <v>3.687</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>3.77</v>
+        <v>3.776</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.103</v>
+        <v>3.106</v>
       </c>
       <c r="G30" t="n">
-        <v>3.17</v>
+        <v>3.175</v>
       </c>
       <c r="H30" t="n">
-        <v>3.309</v>
+        <v>3.319</v>
       </c>
       <c r="I30" t="n">
-        <v>3.545</v>
+        <v>3.56</v>
       </c>
       <c r="J30" t="n">
-        <v>3.791</v>
+        <v>3.804</v>
       </c>
       <c r="K30" t="n">
-        <v>4.102</v>
+        <v>4.114</v>
       </c>
       <c r="L30" t="n">
-        <v>4.178</v>
+        <v>4.189</v>
       </c>
       <c r="M30" t="n">
-        <v>4.359</v>
+        <v>4.372</v>
       </c>
       <c r="N30" t="n">
-        <v>4.489</v>
+        <v>4.515</v>
       </c>
       <c r="O30" t="n">
-        <v>4.773</v>
+        <v>4.779</v>
       </c>
       <c r="P30" t="n">
-        <v>4.944</v>
+        <v>4.963</v>
       </c>
       <c r="Q30" t="n">
-        <v>5.706</v>
+        <v>5.73</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.429</v>
+        <v>3.432</v>
       </c>
       <c r="G31" t="n">
-        <v>3.53</v>
+        <v>3.535</v>
       </c>
       <c r="H31" t="n">
-        <v>3.721</v>
+        <v>3.731</v>
       </c>
       <c r="I31" t="n">
-        <v>3.973</v>
+        <v>3.987</v>
       </c>
       <c r="J31" t="n">
-        <v>4.279</v>
+        <v>4.292</v>
       </c>
       <c r="K31" t="n">
-        <v>4.634</v>
+        <v>4.646</v>
       </c>
       <c r="L31" t="n">
-        <v>4.788</v>
+        <v>4.799</v>
       </c>
       <c r="M31" t="n">
-        <v>5.088</v>
+        <v>5.101</v>
       </c>
       <c r="N31" t="n">
-        <v>5.345</v>
+        <v>5.372</v>
       </c>
       <c r="O31" t="n">
-        <v>5.804</v>
+        <v>5.81</v>
       </c>
       <c r="P31" t="n">
-        <v>5.93</v>
+        <v>5.95</v>
       </c>
       <c r="Q31" t="n">
-        <v>6.68</v>
+        <v>6.703</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.2</v>
+        <v>3.203</v>
       </c>
       <c r="G32" t="n">
-        <v>3.286</v>
+        <v>3.291</v>
       </c>
       <c r="H32" t="n">
-        <v>3.452</v>
+        <v>3.462</v>
       </c>
       <c r="I32" t="n">
-        <v>3.704</v>
+        <v>3.719</v>
       </c>
       <c r="J32" t="n">
-        <v>3.968</v>
+        <v>3.981</v>
       </c>
       <c r="K32" t="n">
-        <v>4.287</v>
+        <v>4.299</v>
       </c>
       <c r="L32" t="n">
-        <v>4.381</v>
+        <v>4.392</v>
       </c>
       <c r="M32" t="n">
-        <v>4.631</v>
+        <v>4.644</v>
       </c>
       <c r="N32" t="n">
-        <v>4.849</v>
+        <v>4.875</v>
       </c>
       <c r="O32" t="n">
-        <v>5.216</v>
+        <v>5.223</v>
       </c>
       <c r="P32" t="n">
-        <v>5.401</v>
+        <v>5.422</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.168</v>
+        <v>6.191</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2.992</v>
+        <v>2.991</v>
       </c>
       <c r="G33" t="n">
-        <v>3.055</v>
+        <v>3.054</v>
       </c>
       <c r="H33" t="n">
-        <v>3.135</v>
+        <v>3.145</v>
       </c>
       <c r="I33" t="n">
-        <v>3.335</v>
+        <v>3.349</v>
       </c>
       <c r="J33" t="n">
-        <v>3.502</v>
+        <v>3.515</v>
       </c>
       <c r="K33" t="n">
-        <v>3.744</v>
+        <v>3.756</v>
       </c>
       <c r="L33" t="n">
-        <v>3.784</v>
+        <v>3.795</v>
       </c>
       <c r="M33" t="n">
-        <v>3.89</v>
+        <v>3.903</v>
       </c>
       <c r="N33" t="n">
-        <v>3.87</v>
+        <v>3.899</v>
       </c>
       <c r="O33" t="n">
-        <v>3.925</v>
+        <v>3.932</v>
       </c>
       <c r="P33" t="n">
-        <v>3.972</v>
+        <v>3.993</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.423</v>
+        <v>4.447</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.051</v>
+        <v>3.05</v>
       </c>
       <c r="G34" t="n">
         <v>3.107</v>
       </c>
       <c r="H34" t="n">
-        <v>3.195</v>
+        <v>3.205</v>
       </c>
       <c r="I34" t="n">
-        <v>3.403</v>
+        <v>3.418</v>
       </c>
       <c r="J34" t="n">
-        <v>3.574</v>
+        <v>3.587</v>
       </c>
       <c r="K34" t="n">
-        <v>3.821</v>
+        <v>3.832</v>
       </c>
       <c r="L34" t="n">
-        <v>3.863</v>
+        <v>3.874</v>
       </c>
       <c r="M34" t="n">
-        <v>3.98</v>
+        <v>3.993</v>
       </c>
       <c r="N34" t="n">
-        <v>3.975</v>
+        <v>4.004</v>
       </c>
       <c r="O34" t="n">
-        <v>4.093</v>
+        <v>4.101</v>
       </c>
       <c r="P34" t="n">
-        <v>4.267</v>
+        <v>4.287</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.124</v>
+        <v>5.148</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.025</v>
+        <v>3.024</v>
       </c>
       <c r="G35" t="n">
-        <v>3.081</v>
+        <v>3.08</v>
       </c>
       <c r="H35" t="n">
-        <v>3.162</v>
+        <v>3.172</v>
       </c>
       <c r="I35" t="n">
-        <v>3.37</v>
+        <v>3.384</v>
       </c>
       <c r="J35" t="n">
-        <v>3.541</v>
+        <v>3.555</v>
       </c>
       <c r="K35" t="n">
-        <v>3.775</v>
+        <v>3.787</v>
       </c>
       <c r="L35" t="n">
-        <v>3.818</v>
+        <v>3.829</v>
       </c>
       <c r="M35" t="n">
-        <v>3.927</v>
+        <v>3.94</v>
       </c>
       <c r="N35" t="n">
-        <v>3.911</v>
+        <v>3.94</v>
       </c>
       <c r="O35" t="n">
-        <v>3.991</v>
+        <v>3.999</v>
       </c>
       <c r="P35" t="n">
-        <v>4.069</v>
+        <v>4.09</v>
       </c>
       <c r="Q35" t="n">
-        <v>4.76</v>
+        <v>4.783</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.936</v>
+        <v>2.935</v>
       </c>
       <c r="G36" t="n">
-        <v>2.999</v>
+        <v>2.998</v>
       </c>
       <c r="H36" t="n">
-        <v>3.064</v>
+        <v>3.074</v>
       </c>
       <c r="I36" t="n">
-        <v>3.264</v>
+        <v>3.278</v>
       </c>
       <c r="J36" t="n">
-        <v>3.439</v>
+        <v>3.452</v>
       </c>
       <c r="K36" t="n">
-        <v>3.667</v>
+        <v>3.679</v>
       </c>
       <c r="L36" t="n">
-        <v>3.708</v>
+        <v>3.719</v>
       </c>
       <c r="M36" t="n">
-        <v>3.79</v>
+        <v>3.803</v>
       </c>
       <c r="N36" t="n">
-        <v>3.775</v>
+        <v>3.804</v>
       </c>
       <c r="O36" t="n">
-        <v>3.835</v>
+        <v>3.842</v>
       </c>
       <c r="P36" t="n">
-        <v>3.871</v>
+        <v>3.891</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.14</v>
+        <v>4.164</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.774</v>
+        <v>3.777</v>
       </c>
       <c r="G37" t="n">
-        <v>4.225</v>
+        <v>4.23</v>
       </c>
       <c r="H37" t="n">
-        <v>4.699</v>
+        <v>4.709</v>
       </c>
       <c r="I37" t="n">
-        <v>5.045</v>
+        <v>5.059</v>
       </c>
       <c r="J37" t="n">
-        <v>5.77</v>
+        <v>5.783</v>
       </c>
       <c r="K37" t="n">
-        <v>6.672</v>
+        <v>6.684</v>
       </c>
       <c r="L37" t="n">
-        <v>6.987</v>
+        <v>6.999</v>
       </c>
       <c r="M37" t="n">
-        <v>7.361</v>
+        <v>7.374</v>
       </c>
       <c r="N37" t="n">
-        <v>7.498</v>
+        <v>7.524</v>
       </c>
       <c r="O37" t="n">
-        <v>7.684</v>
+        <v>7.691</v>
       </c>
       <c r="P37" t="n">
-        <v>7.727</v>
+        <v>7.748</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.170999999999999</v>
+        <v>8.195</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.83</v>
+        <v>4.833</v>
       </c>
       <c r="G38" t="n">
-        <v>5.535</v>
+        <v>5.54</v>
       </c>
       <c r="H38" t="n">
-        <v>6.223</v>
+        <v>6.233</v>
       </c>
       <c r="I38" t="n">
-        <v>6.725</v>
+        <v>6.739</v>
       </c>
       <c r="J38" t="n">
-        <v>7.71</v>
+        <v>7.723</v>
       </c>
       <c r="K38" t="n">
-        <v>8.787000000000001</v>
+        <v>8.798999999999999</v>
       </c>
       <c r="L38" t="n">
-        <v>9.263</v>
+        <v>9.273999999999999</v>
       </c>
       <c r="M38" t="n">
-        <v>9.768000000000001</v>
+        <v>9.781000000000001</v>
       </c>
       <c r="N38" t="n">
-        <v>9.914999999999999</v>
+        <v>9.942</v>
       </c>
       <c r="O38" t="n">
-        <v>10.083</v>
+        <v>10.09</v>
       </c>
       <c r="P38" t="n">
-        <v>10.126</v>
+        <v>10.146</v>
       </c>
       <c r="Q38" t="n">
-        <v>10.623</v>
+        <v>10.646</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.151</v>
+        <v>4.154</v>
       </c>
       <c r="G39" t="n">
-        <v>4.733</v>
+        <v>4.738</v>
       </c>
       <c r="H39" t="n">
-        <v>5.287</v>
+        <v>5.297</v>
       </c>
       <c r="I39" t="n">
-        <v>5.729</v>
+        <v>5.743</v>
       </c>
       <c r="J39" t="n">
-        <v>6.583</v>
+        <v>6.596</v>
       </c>
       <c r="K39" t="n">
-        <v>7.62</v>
+        <v>7.632</v>
       </c>
       <c r="L39" t="n">
-        <v>8.022</v>
+        <v>8.032999999999999</v>
       </c>
       <c r="M39" t="n">
-        <v>8.406000000000001</v>
+        <v>8.419</v>
       </c>
       <c r="N39" t="n">
-        <v>8.542999999999999</v>
+        <v>8.569000000000001</v>
       </c>
       <c r="O39" t="n">
-        <v>8.733000000000001</v>
+        <v>8.74</v>
       </c>
       <c r="P39" t="n">
-        <v>8.781000000000001</v>
+        <v>8.801</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.266999999999999</v>
+        <v>9.291</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.296</v>
+        <v>3.299</v>
       </c>
       <c r="G40" t="n">
-        <v>3.409</v>
+        <v>3.414</v>
       </c>
       <c r="H40" t="n">
-        <v>3.569</v>
+        <v>3.579</v>
       </c>
       <c r="I40" t="n">
-        <v>3.82</v>
+        <v>3.834</v>
       </c>
       <c r="J40" t="n">
-        <v>4.084</v>
+        <v>4.097</v>
       </c>
       <c r="K40" t="n">
-        <v>4.407</v>
+        <v>4.419</v>
       </c>
       <c r="L40" t="n">
-        <v>4.502</v>
+        <v>4.513</v>
       </c>
       <c r="M40" t="n">
-        <v>4.7</v>
+        <v>4.713</v>
       </c>
       <c r="N40" t="n">
-        <v>4.847</v>
+        <v>4.873</v>
       </c>
       <c r="O40" t="n">
-        <v>5.151</v>
+        <v>5.158</v>
       </c>
       <c r="P40" t="n">
-        <v>5.365</v>
+        <v>5.384</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.157</v>
+        <v>6.181</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.679</v>
+        <v>3.682</v>
       </c>
       <c r="G41" t="n">
-        <v>3.833</v>
+        <v>3.838</v>
       </c>
       <c r="H41" t="n">
-        <v>4.052</v>
+        <v>4.062</v>
       </c>
       <c r="I41" t="n">
-        <v>4.322</v>
+        <v>4.336</v>
       </c>
       <c r="J41" t="n">
-        <v>4.636</v>
+        <v>4.649</v>
       </c>
       <c r="K41" t="n">
-        <v>5.006</v>
+        <v>5.018</v>
       </c>
       <c r="L41" t="n">
-        <v>5.178</v>
+        <v>5.189</v>
       </c>
       <c r="M41" t="n">
-        <v>5.502</v>
+        <v>5.515</v>
       </c>
       <c r="N41" t="n">
-        <v>5.775</v>
+        <v>5.801</v>
       </c>
       <c r="O41" t="n">
-        <v>6.261</v>
+        <v>6.268</v>
       </c>
       <c r="P41" t="n">
-        <v>6.422</v>
+        <v>6.443</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.205</v>
+        <v>7.228</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.416</v>
+        <v>3.419</v>
       </c>
       <c r="G42" t="n">
-        <v>3.557</v>
+        <v>3.562</v>
       </c>
       <c r="H42" t="n">
-        <v>3.744</v>
+        <v>3.754</v>
       </c>
       <c r="I42" t="n">
-        <v>4.009</v>
+        <v>4.023</v>
       </c>
       <c r="J42" t="n">
-        <v>4.285</v>
+        <v>4.298</v>
       </c>
       <c r="K42" t="n">
-        <v>4.628</v>
+        <v>4.64</v>
       </c>
       <c r="L42" t="n">
-        <v>4.737</v>
+        <v>4.748</v>
       </c>
       <c r="M42" t="n">
-        <v>5.007</v>
+        <v>5.02</v>
       </c>
       <c r="N42" t="n">
-        <v>5.261</v>
+        <v>5.287</v>
       </c>
       <c r="O42" t="n">
-        <v>5.64</v>
+        <v>5.647</v>
       </c>
       <c r="P42" t="n">
-        <v>5.865</v>
+        <v>5.885</v>
       </c>
       <c r="Q42" t="n">
-        <v>6.67</v>
+        <v>6.693</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.14</v>
+        <v>3.139</v>
       </c>
       <c r="G43" t="n">
-        <v>3.237</v>
+        <v>3.236</v>
       </c>
       <c r="H43" t="n">
-        <v>3.334</v>
+        <v>3.344</v>
       </c>
       <c r="I43" t="n">
-        <v>3.545</v>
+        <v>3.559</v>
       </c>
       <c r="J43" t="n">
-        <v>3.729</v>
+        <v>3.744</v>
       </c>
       <c r="K43" t="n">
-        <v>3.975</v>
+        <v>3.987</v>
       </c>
       <c r="L43" t="n">
-        <v>4.025</v>
+        <v>4.036</v>
       </c>
       <c r="M43" t="n">
-        <v>4.143</v>
+        <v>4.156</v>
       </c>
       <c r="N43" t="n">
-        <v>4.139</v>
+        <v>4.169</v>
       </c>
       <c r="O43" t="n">
-        <v>4.237</v>
+        <v>4.245</v>
       </c>
       <c r="P43" t="n">
-        <v>4.338</v>
+        <v>4.358</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.033</v>
+        <v>5.057</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46120</v>
+        <v>46121</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>3.014</v>
+        <v>3.013</v>
       </c>
       <c r="G44" t="n">
-        <v>3.109</v>
+        <v>3.108</v>
       </c>
       <c r="H44" t="n">
-        <v>3.189</v>
+        <v>3.199</v>
       </c>
       <c r="I44" t="n">
-        <v>3.392</v>
+        <v>3.406</v>
       </c>
       <c r="J44" t="n">
-        <v>3.581</v>
+        <v>3.594</v>
       </c>
       <c r="K44" t="n">
-        <v>3.818</v>
+        <v>3.829</v>
       </c>
       <c r="L44" t="n">
-        <v>3.868</v>
+        <v>3.879</v>
       </c>
       <c r="M44" t="n">
-        <v>3.958</v>
+        <v>3.971</v>
       </c>
       <c r="N44" t="n">
-        <v>3.957</v>
+        <v>3.986</v>
       </c>
       <c r="O44" t="n">
-        <v>4.034</v>
+        <v>4.042</v>
       </c>
       <c r="P44" t="n">
-        <v>4.101</v>
+        <v>4.121</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.404</v>
+        <v>4.427</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-04-10 ~ 2026-04-10
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.25</v>
+        <v>3.248</v>
       </c>
       <c r="G2" t="n">
-        <v>3.462</v>
+        <v>3.461</v>
       </c>
       <c r="H2" t="n">
-        <v>3.59</v>
+        <v>3.594</v>
       </c>
       <c r="I2" t="n">
-        <v>3.79</v>
+        <v>3.804</v>
       </c>
       <c r="J2" t="n">
-        <v>3.978</v>
+        <v>4.002</v>
       </c>
       <c r="K2" t="n">
-        <v>4.369</v>
+        <v>4.392</v>
       </c>
       <c r="L2" t="n">
-        <v>4.537</v>
+        <v>4.562</v>
       </c>
       <c r="M2" t="n">
-        <v>4.839</v>
+        <v>4.867</v>
       </c>
       <c r="N2" t="n">
-        <v>5.086</v>
+        <v>5.116</v>
       </c>
       <c r="O2" t="n">
-        <v>5.288</v>
+        <v>5.321</v>
       </c>
       <c r="P2" t="n">
-        <v>5.485</v>
+        <v>5.517</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.125</v>
+        <v>6.155</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.273</v>
+        <v>4.271</v>
       </c>
       <c r="G3" t="n">
-        <v>4.667</v>
+        <v>4.665</v>
       </c>
       <c r="H3" t="n">
-        <v>4.828</v>
+        <v>4.832</v>
       </c>
       <c r="I3" t="n">
-        <v>5.028</v>
+        <v>5.042</v>
       </c>
       <c r="J3" t="n">
-        <v>5.226</v>
+        <v>5.25</v>
       </c>
       <c r="K3" t="n">
-        <v>5.685</v>
+        <v>5.708</v>
       </c>
       <c r="L3" t="n">
-        <v>5.922</v>
+        <v>5.948</v>
       </c>
       <c r="M3" t="n">
-        <v>6.256</v>
+        <v>6.284</v>
       </c>
       <c r="N3" t="n">
-        <v>6.446</v>
+        <v>6.476</v>
       </c>
       <c r="O3" t="n">
-        <v>6.598</v>
+        <v>6.63</v>
       </c>
       <c r="P3" t="n">
-        <v>6.664</v>
+        <v>6.696</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.193</v>
+        <v>7.223</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.764</v>
+        <v>3.762</v>
       </c>
       <c r="G4" t="n">
-        <v>4.047</v>
+        <v>4.045</v>
       </c>
       <c r="H4" t="n">
-        <v>4.237</v>
+        <v>4.24</v>
       </c>
       <c r="I4" t="n">
-        <v>4.468</v>
+        <v>4.482</v>
       </c>
       <c r="J4" t="n">
-        <v>4.672</v>
+        <v>4.696</v>
       </c>
       <c r="K4" t="n">
-        <v>5.125</v>
+        <v>5.148</v>
       </c>
       <c r="L4" t="n">
-        <v>5.292</v>
+        <v>5.318</v>
       </c>
       <c r="M4" t="n">
-        <v>5.614</v>
+        <v>5.642</v>
       </c>
       <c r="N4" t="n">
-        <v>5.774</v>
+        <v>5.804</v>
       </c>
       <c r="O4" t="n">
-        <v>5.95</v>
+        <v>5.982</v>
       </c>
       <c r="P4" t="n">
-        <v>6.013</v>
+        <v>6.046</v>
       </c>
       <c r="Q4" t="n">
-        <v>6.546</v>
+        <v>6.576</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.959</v>
+        <v>2.955</v>
       </c>
       <c r="G5" t="n">
-        <v>3.013</v>
+        <v>3.009</v>
       </c>
       <c r="H5" t="n">
-        <v>3.093</v>
+        <v>3.097</v>
       </c>
       <c r="I5" t="n">
-        <v>3.362</v>
+        <v>3.379</v>
       </c>
       <c r="J5" t="n">
-        <v>3.55</v>
+        <v>3.574</v>
       </c>
       <c r="K5" t="n">
-        <v>3.8</v>
+        <v>3.823</v>
       </c>
       <c r="L5" t="n">
-        <v>3.81</v>
+        <v>3.836</v>
       </c>
       <c r="M5" t="n">
-        <v>3.918</v>
+        <v>3.946</v>
       </c>
       <c r="N5" t="n">
-        <v>3.892</v>
+        <v>3.924</v>
       </c>
       <c r="O5" t="n">
-        <v>3.884</v>
+        <v>3.917</v>
       </c>
       <c r="P5" t="n">
-        <v>4.154</v>
+        <v>4.186</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.037</v>
+        <v>5.067</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>3</v>
+        <v>2.996</v>
       </c>
       <c r="G6" t="n">
-        <v>3.066</v>
+        <v>3.065</v>
       </c>
       <c r="H6" t="n">
-        <v>3.162</v>
+        <v>3.167</v>
       </c>
       <c r="I6" t="n">
-        <v>3.436</v>
+        <v>3.453</v>
       </c>
       <c r="J6" t="n">
-        <v>3.633</v>
+        <v>3.658</v>
       </c>
       <c r="K6" t="n">
-        <v>3.901</v>
+        <v>3.924</v>
       </c>
       <c r="L6" t="n">
-        <v>3.923</v>
+        <v>3.949</v>
       </c>
       <c r="M6" t="n">
-        <v>4.064</v>
+        <v>4.093</v>
       </c>
       <c r="N6" t="n">
-        <v>4.061</v>
+        <v>4.093</v>
       </c>
       <c r="O6" t="n">
-        <v>4.156</v>
+        <v>4.189</v>
       </c>
       <c r="P6" t="n">
-        <v>4.587</v>
+        <v>4.619</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.433</v>
+        <v>5.463</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2.98</v>
+        <v>2.976</v>
       </c>
       <c r="G7" t="n">
-        <v>3.032</v>
+        <v>3.028</v>
       </c>
       <c r="H7" t="n">
-        <v>3.109</v>
+        <v>3.113</v>
       </c>
       <c r="I7" t="n">
-        <v>3.377</v>
+        <v>3.394</v>
       </c>
       <c r="J7" t="n">
-        <v>3.575</v>
+        <v>3.599</v>
       </c>
       <c r="K7" t="n">
-        <v>3.825</v>
+        <v>3.849</v>
       </c>
       <c r="L7" t="n">
-        <v>3.835</v>
+        <v>3.86</v>
       </c>
       <c r="M7" t="n">
-        <v>3.976</v>
+        <v>4.004</v>
       </c>
       <c r="N7" t="n">
-        <v>3.952</v>
+        <v>3.984</v>
       </c>
       <c r="O7" t="n">
-        <v>4.056</v>
+        <v>4.088</v>
       </c>
       <c r="P7" t="n">
-        <v>4.371</v>
+        <v>4.402</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.201</v>
+        <v>5.231</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.383</v>
+        <v>5.381</v>
       </c>
       <c r="G8" t="n">
-        <v>5.965</v>
+        <v>5.963</v>
       </c>
       <c r="H8" t="n">
-        <v>6.277</v>
+        <v>6.281</v>
       </c>
       <c r="I8" t="n">
-        <v>6.548</v>
+        <v>6.562</v>
       </c>
       <c r="J8" t="n">
-        <v>6.81</v>
+        <v>6.834</v>
       </c>
       <c r="K8" t="n">
-        <v>7.55</v>
+        <v>7.573</v>
       </c>
       <c r="L8" t="n">
-        <v>7.877</v>
+        <v>7.903</v>
       </c>
       <c r="M8" t="n">
-        <v>8.239000000000001</v>
+        <v>8.266999999999999</v>
       </c>
       <c r="N8" t="n">
-        <v>8.367000000000001</v>
+        <v>8.397</v>
       </c>
       <c r="O8" t="n">
-        <v>8.605</v>
+        <v>8.637</v>
       </c>
       <c r="P8" t="n">
-        <v>8.77</v>
+        <v>8.803000000000001</v>
       </c>
       <c r="Q8" t="n">
-        <v>9.502000000000001</v>
+        <v>9.532</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1066,54 +1066,54 @@
         <v>2.618</v>
       </c>
       <c r="G9" t="n">
-        <v>2.689</v>
+        <v>2.686</v>
       </c>
       <c r="H9" t="n">
         <v>2.777</v>
       </c>
       <c r="I9" t="n">
-        <v>2.908</v>
+        <v>2.917</v>
       </c>
       <c r="J9" t="n">
-        <v>3.074</v>
+        <v>3.098</v>
       </c>
       <c r="K9" t="n">
-        <v>3.2</v>
+        <v>3.225</v>
       </c>
       <c r="L9" t="n">
-        <v>3.252</v>
+        <v>3.274</v>
       </c>
       <c r="M9" t="n">
-        <v>3.329</v>
+        <v>3.357</v>
       </c>
       <c r="N9" t="n">
-        <v>3.472</v>
+        <v>3.5</v>
       </c>
       <c r="O9" t="n">
-        <v>3.483</v>
+        <v>3.514</v>
       </c>
       <c r="P9" t="n">
-        <v>3.575</v>
+        <v>3.607</v>
       </c>
       <c r="Q9" t="n">
-        <v>3.655</v>
+        <v>3.685</v>
       </c>
       <c r="R9" t="n">
-        <v>3.674</v>
+        <v>3.69</v>
       </c>
       <c r="S9" t="n">
-        <v>3.641</v>
+        <v>3.645</v>
       </c>
       <c r="T9" t="n">
-        <v>3.572</v>
+        <v>3.569</v>
       </c>
       <c r="U9" t="n">
-        <v>3.476</v>
+        <v>3.442</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1139,31 +1139,31 @@
         <v>2.63</v>
       </c>
       <c r="G10" t="n">
-        <v>2.721</v>
+        <v>2.718</v>
       </c>
       <c r="H10" t="n">
-        <v>2.788</v>
+        <v>2.789</v>
       </c>
       <c r="I10" t="n">
-        <v>2.919</v>
+        <v>2.926</v>
       </c>
       <c r="J10" t="n">
-        <v>3.103</v>
+        <v>3.127</v>
       </c>
       <c r="K10" t="n">
-        <v>3.226</v>
+        <v>3.252</v>
       </c>
       <c r="L10" t="n">
-        <v>3.294</v>
+        <v>3.316</v>
       </c>
       <c r="M10" t="n">
-        <v>3.43</v>
+        <v>3.457</v>
       </c>
       <c r="N10" t="n">
-        <v>3.48</v>
+        <v>3.508</v>
       </c>
       <c r="O10" t="n">
-        <v>3.661</v>
+        <v>3.677</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1212,37 +1212,37 @@
         <v>2.446</v>
       </c>
       <c r="G11" t="n">
-        <v>2.531</v>
+        <v>2.528</v>
       </c>
       <c r="H11" t="n">
-        <v>2.612</v>
+        <v>2.613</v>
       </c>
       <c r="I11" t="n">
-        <v>2.721</v>
+        <v>2.728</v>
       </c>
       <c r="J11" t="n">
-        <v>2.897</v>
+        <v>2.921</v>
       </c>
       <c r="K11" t="n">
-        <v>3.014</v>
+        <v>3.039</v>
       </c>
       <c r="L11" t="n">
-        <v>3.088</v>
+        <v>3.11</v>
       </c>
       <c r="M11" t="n">
-        <v>3.234</v>
+        <v>3.262</v>
       </c>
       <c r="N11" t="n">
-        <v>3.29</v>
+        <v>3.318</v>
       </c>
       <c r="O11" t="n">
-        <v>3.427</v>
+        <v>3.443</v>
       </c>
       <c r="P11" t="n">
-        <v>3.512</v>
+        <v>3.544</v>
       </c>
       <c r="Q11" t="n">
-        <v>3.858</v>
+        <v>3.888</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.221</v>
+        <v>3.216</v>
       </c>
       <c r="G12" t="n">
-        <v>3.371</v>
+        <v>3.369</v>
       </c>
       <c r="H12" t="n">
-        <v>3.469</v>
+        <v>3.468</v>
       </c>
       <c r="I12" t="n">
-        <v>3.681</v>
+        <v>3.685</v>
       </c>
       <c r="J12" t="n">
-        <v>3.962</v>
+        <v>3.982</v>
       </c>
       <c r="K12" t="n">
-        <v>4.159</v>
+        <v>4.177</v>
       </c>
       <c r="L12" t="n">
-        <v>4.208</v>
+        <v>4.228</v>
       </c>
       <c r="M12" t="n">
-        <v>4.346</v>
+        <v>4.373</v>
       </c>
       <c r="N12" t="n">
-        <v>4.361</v>
+        <v>4.392</v>
       </c>
       <c r="O12" t="n">
-        <v>4.494</v>
+        <v>4.525</v>
       </c>
       <c r="P12" t="n">
-        <v>4.62</v>
+        <v>4.653</v>
       </c>
       <c r="Q12" t="n">
-        <v>4.986</v>
+        <v>5.016</v>
       </c>
       <c r="R12" t="n">
-        <v>5.171</v>
+        <v>5.187</v>
       </c>
       <c r="S12" t="n">
-        <v>5.352</v>
+        <v>5.356</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2.975</v>
+        <v>2.97</v>
       </c>
       <c r="G13" t="n">
-        <v>3.061</v>
+        <v>3.059</v>
       </c>
       <c r="H13" t="n">
-        <v>3.137</v>
+        <v>3.136</v>
       </c>
       <c r="I13" t="n">
-        <v>3.329</v>
+        <v>3.332</v>
       </c>
       <c r="J13" t="n">
-        <v>3.599</v>
+        <v>3.619</v>
       </c>
       <c r="K13" t="n">
-        <v>3.793</v>
+        <v>3.81</v>
       </c>
       <c r="L13" t="n">
-        <v>3.847</v>
+        <v>3.867</v>
       </c>
       <c r="M13" t="n">
-        <v>3.974</v>
+        <v>4</v>
       </c>
       <c r="N13" t="n">
-        <v>3.989</v>
+        <v>4.02</v>
       </c>
       <c r="O13" t="n">
-        <v>4.12</v>
+        <v>4.151</v>
       </c>
       <c r="P13" t="n">
-        <v>4.212</v>
+        <v>4.244</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.507</v>
+        <v>4.537</v>
       </c>
       <c r="R13" t="n">
-        <v>4.719</v>
+        <v>4.735</v>
       </c>
       <c r="S13" t="n">
-        <v>4.915</v>
+        <v>4.918</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.793</v>
+        <v>2.788</v>
       </c>
       <c r="G14" t="n">
-        <v>2.868</v>
+        <v>2.865</v>
       </c>
       <c r="H14" t="n">
-        <v>2.94</v>
+        <v>2.939</v>
       </c>
       <c r="I14" t="n">
-        <v>3.112</v>
+        <v>3.115</v>
       </c>
       <c r="J14" t="n">
-        <v>3.338</v>
+        <v>3.359</v>
       </c>
       <c r="K14" t="n">
-        <v>3.481</v>
+        <v>3.498</v>
       </c>
       <c r="L14" t="n">
-        <v>3.519</v>
+        <v>3.539</v>
       </c>
       <c r="M14" t="n">
-        <v>3.658</v>
+        <v>3.685</v>
       </c>
       <c r="N14" t="n">
-        <v>3.668</v>
+        <v>3.699</v>
       </c>
       <c r="O14" t="n">
-        <v>3.775</v>
+        <v>3.806</v>
       </c>
       <c r="P14" t="n">
-        <v>3.847</v>
+        <v>3.88</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.096</v>
+        <v>4.126</v>
       </c>
       <c r="R14" t="n">
-        <v>4.234</v>
+        <v>4.25</v>
       </c>
       <c r="S14" t="n">
-        <v>4.367</v>
+        <v>4.371</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.771</v>
+        <v>2.766</v>
       </c>
       <c r="G15" t="n">
-        <v>2.842</v>
+        <v>2.84</v>
       </c>
       <c r="H15" t="n">
-        <v>2.909</v>
+        <v>2.908</v>
       </c>
       <c r="I15" t="n">
-        <v>3.063</v>
+        <v>3.066</v>
       </c>
       <c r="J15" t="n">
-        <v>3.275</v>
+        <v>3.296</v>
       </c>
       <c r="K15" t="n">
-        <v>3.435</v>
+        <v>3.451</v>
       </c>
       <c r="L15" t="n">
-        <v>3.453</v>
+        <v>3.474</v>
       </c>
       <c r="M15" t="n">
-        <v>3.571</v>
+        <v>3.598</v>
       </c>
       <c r="N15" t="n">
-        <v>3.572</v>
+        <v>3.603</v>
       </c>
       <c r="O15" t="n">
-        <v>3.699</v>
+        <v>3.73</v>
       </c>
       <c r="P15" t="n">
-        <v>3.744</v>
+        <v>3.777</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.001</v>
+        <v>4.031</v>
       </c>
       <c r="R15" t="n">
-        <v>4.13</v>
+        <v>4.146</v>
       </c>
       <c r="S15" t="n">
-        <v>4.263</v>
+        <v>4.266</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.771</v>
+        <v>2.766</v>
       </c>
       <c r="G16" t="n">
-        <v>2.842</v>
+        <v>2.84</v>
       </c>
       <c r="H16" t="n">
-        <v>2.909</v>
+        <v>2.908</v>
       </c>
       <c r="I16" t="n">
-        <v>3.063</v>
+        <v>3.066</v>
       </c>
       <c r="J16" t="n">
-        <v>3.275</v>
+        <v>3.296</v>
       </c>
       <c r="K16" t="n">
-        <v>3.435</v>
+        <v>3.451</v>
       </c>
       <c r="L16" t="n">
-        <v>3.453</v>
+        <v>3.474</v>
       </c>
       <c r="M16" t="n">
-        <v>3.571</v>
+        <v>3.598</v>
       </c>
       <c r="N16" t="n">
-        <v>3.575</v>
+        <v>3.606</v>
       </c>
       <c r="O16" t="n">
-        <v>3.706</v>
+        <v>3.737</v>
       </c>
       <c r="P16" t="n">
-        <v>3.767</v>
+        <v>3.8</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.028</v>
+        <v>4.058</v>
       </c>
       <c r="R16" t="n">
-        <v>4.159</v>
+        <v>4.174</v>
       </c>
       <c r="S16" t="n">
-        <v>4.291</v>
+        <v>4.295</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1650,34 +1650,34 @@
         <v>2.692</v>
       </c>
       <c r="G17" t="n">
-        <v>2.812</v>
+        <v>2.809</v>
       </c>
       <c r="H17" t="n">
-        <v>2.881</v>
+        <v>2.882</v>
       </c>
       <c r="I17" t="n">
-        <v>3.001</v>
+        <v>3.008</v>
       </c>
       <c r="J17" t="n">
-        <v>3.171</v>
+        <v>3.195</v>
       </c>
       <c r="K17" t="n">
-        <v>3.299</v>
+        <v>3.324</v>
       </c>
       <c r="L17" t="n">
-        <v>3.372</v>
+        <v>3.394</v>
       </c>
       <c r="M17" t="n">
-        <v>3.55</v>
+        <v>3.577</v>
       </c>
       <c r="N17" t="n">
-        <v>3.582</v>
+        <v>3.609</v>
       </c>
       <c r="O17" t="n">
-        <v>3.697</v>
+        <v>3.713</v>
       </c>
       <c r="P17" t="n">
-        <v>3.793</v>
+        <v>3.824</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1723,31 +1723,31 @@
         <v>2.693</v>
       </c>
       <c r="G18" t="n">
-        <v>2.813</v>
+        <v>2.81</v>
       </c>
       <c r="H18" t="n">
-        <v>2.882</v>
+        <v>2.883</v>
       </c>
       <c r="I18" t="n">
-        <v>3.001</v>
+        <v>3.009</v>
       </c>
       <c r="J18" t="n">
-        <v>3.171</v>
+        <v>3.195</v>
       </c>
       <c r="K18" t="n">
-        <v>3.301</v>
+        <v>3.325</v>
       </c>
       <c r="L18" t="n">
-        <v>3.371</v>
+        <v>3.394</v>
       </c>
       <c r="M18" t="n">
-        <v>3.55</v>
+        <v>3.577</v>
       </c>
       <c r="N18" t="n">
-        <v>3.581</v>
+        <v>3.608</v>
       </c>
       <c r="O18" t="n">
-        <v>3.695</v>
+        <v>3.711</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.782</v>
+        <v>2.777</v>
       </c>
       <c r="G19" t="n">
-        <v>2.858</v>
+        <v>2.856</v>
       </c>
       <c r="H19" t="n">
-        <v>2.93</v>
+        <v>2.929</v>
       </c>
       <c r="I19" t="n">
-        <v>3.096</v>
+        <v>3.1</v>
       </c>
       <c r="J19" t="n">
-        <v>3.321</v>
+        <v>3.342</v>
       </c>
       <c r="K19" t="n">
-        <v>3.478</v>
+        <v>3.495</v>
       </c>
       <c r="L19" t="n">
-        <v>3.516</v>
+        <v>3.536</v>
       </c>
       <c r="M19" t="n">
-        <v>3.646</v>
+        <v>3.673</v>
       </c>
       <c r="N19" t="n">
-        <v>3.655</v>
+        <v>3.686</v>
       </c>
       <c r="O19" t="n">
-        <v>3.752</v>
+        <v>3.784</v>
       </c>
       <c r="P19" t="n">
-        <v>3.811</v>
+        <v>3.843</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.047</v>
+        <v>4.076</v>
       </c>
       <c r="R19" t="n">
-        <v>4.184</v>
+        <v>4.199</v>
       </c>
       <c r="S19" t="n">
-        <v>4.306</v>
+        <v>4.309</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2.572</v>
+        <v>2.573</v>
       </c>
       <c r="G20" t="n">
-        <v>2.644</v>
+        <v>2.645</v>
       </c>
       <c r="H20" t="n">
-        <v>2.694</v>
+        <v>2.695</v>
       </c>
       <c r="I20" t="n">
-        <v>2.857</v>
+        <v>2.858</v>
       </c>
       <c r="J20" t="n">
-        <v>3.085</v>
+        <v>3.105</v>
       </c>
       <c r="K20" t="n">
-        <v>3.24</v>
+        <v>3.261</v>
       </c>
       <c r="L20" t="n">
-        <v>3.28</v>
+        <v>3.3</v>
       </c>
       <c r="M20" t="n">
-        <v>3.373</v>
+        <v>3.394</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1942,43 +1942,43 @@
         <v>2.874</v>
       </c>
       <c r="G21" t="n">
-        <v>2.956</v>
+        <v>2.955</v>
       </c>
       <c r="H21" t="n">
-        <v>3.072</v>
+        <v>3.07</v>
       </c>
       <c r="I21" t="n">
-        <v>3.238</v>
+        <v>3.239</v>
       </c>
       <c r="J21" t="n">
-        <v>3.45</v>
+        <v>3.471</v>
       </c>
       <c r="K21" t="n">
-        <v>3.713</v>
+        <v>3.732</v>
       </c>
       <c r="L21" t="n">
-        <v>3.78</v>
+        <v>3.8</v>
       </c>
       <c r="M21" t="n">
-        <v>3.904</v>
+        <v>3.931</v>
       </c>
       <c r="N21" t="n">
-        <v>3.921</v>
+        <v>3.953</v>
       </c>
       <c r="O21" t="n">
-        <v>3.992</v>
+        <v>4.023</v>
       </c>
       <c r="P21" t="n">
-        <v>4.076</v>
+        <v>4.108</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.207</v>
+        <v>4.237</v>
       </c>
       <c r="R21" t="n">
-        <v>4.231</v>
+        <v>4.246</v>
       </c>
       <c r="S21" t="n">
-        <v>4.265</v>
+        <v>4.269</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2018,40 +2018,40 @@
         <v>2.902</v>
       </c>
       <c r="H22" t="n">
-        <v>3.007</v>
+        <v>3.004</v>
       </c>
       <c r="I22" t="n">
-        <v>3.157</v>
+        <v>3.158</v>
       </c>
       <c r="J22" t="n">
-        <v>3.335</v>
+        <v>3.355</v>
       </c>
       <c r="K22" t="n">
-        <v>3.593</v>
+        <v>3.613</v>
       </c>
       <c r="L22" t="n">
-        <v>3.649</v>
+        <v>3.67</v>
       </c>
       <c r="M22" t="n">
-        <v>3.775</v>
+        <v>3.802</v>
       </c>
       <c r="N22" t="n">
-        <v>3.794</v>
+        <v>3.826</v>
       </c>
       <c r="O22" t="n">
-        <v>3.86</v>
+        <v>3.891</v>
       </c>
       <c r="P22" t="n">
-        <v>3.938</v>
+        <v>3.97</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.065</v>
+        <v>4.095</v>
       </c>
       <c r="R22" t="n">
-        <v>4.078</v>
+        <v>4.094</v>
       </c>
       <c r="S22" t="n">
-        <v>4.11</v>
+        <v>4.114</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.775</v>
+        <v>2.774</v>
       </c>
       <c r="G23" t="n">
         <v>2.857</v>
       </c>
       <c r="H23" t="n">
-        <v>2.945</v>
+        <v>2.943</v>
       </c>
       <c r="I23" t="n">
-        <v>3.109</v>
+        <v>3.11</v>
       </c>
       <c r="J23" t="n">
-        <v>3.281</v>
+        <v>3.301</v>
       </c>
       <c r="K23" t="n">
-        <v>3.513</v>
+        <v>3.532</v>
       </c>
       <c r="L23" t="n">
-        <v>3.56</v>
+        <v>3.581</v>
       </c>
       <c r="M23" t="n">
-        <v>3.68</v>
+        <v>3.707</v>
       </c>
       <c r="N23" t="n">
-        <v>3.69</v>
+        <v>3.722</v>
       </c>
       <c r="O23" t="n">
-        <v>3.734</v>
+        <v>3.765</v>
       </c>
       <c r="P23" t="n">
-        <v>3.8</v>
+        <v>3.831</v>
       </c>
       <c r="Q23" t="n">
-        <v>3.875</v>
+        <v>3.903</v>
       </c>
       <c r="R23" t="n">
-        <v>3.862</v>
+        <v>3.878</v>
       </c>
       <c r="S23" t="n">
-        <v>3.864</v>
+        <v>3.869</v>
       </c>
       <c r="T23" t="n">
-        <v>3.784</v>
+        <v>3.783</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2161,43 +2161,43 @@
         <v>2.706</v>
       </c>
       <c r="G24" t="n">
-        <v>2.772</v>
+        <v>2.771</v>
       </c>
       <c r="H24" t="n">
-        <v>2.847</v>
+        <v>2.844</v>
       </c>
       <c r="I24" t="n">
-        <v>3.02</v>
+        <v>3.021</v>
       </c>
       <c r="J24" t="n">
-        <v>3.182</v>
+        <v>3.202</v>
       </c>
       <c r="K24" t="n">
-        <v>3.397</v>
+        <v>3.415</v>
       </c>
       <c r="L24" t="n">
-        <v>3.431</v>
+        <v>3.452</v>
       </c>
       <c r="M24" t="n">
-        <v>3.535</v>
+        <v>3.562</v>
       </c>
       <c r="N24" t="n">
-        <v>3.56</v>
+        <v>3.592</v>
       </c>
       <c r="O24" t="n">
-        <v>3.686</v>
+        <v>3.717</v>
       </c>
       <c r="P24" t="n">
-        <v>3.738</v>
+        <v>3.77</v>
       </c>
       <c r="Q24" t="n">
-        <v>3.795</v>
+        <v>3.825</v>
       </c>
       <c r="R24" t="n">
-        <v>3.781</v>
+        <v>3.799</v>
       </c>
       <c r="S24" t="n">
-        <v>3.78</v>
+        <v>3.784</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.768</v>
+        <v>2.767</v>
       </c>
       <c r="G25" t="n">
         <v>2.856</v>
       </c>
       <c r="H25" t="n">
-        <v>2.949</v>
+        <v>2.946</v>
       </c>
       <c r="I25" t="n">
-        <v>3.117</v>
+        <v>3.118</v>
       </c>
       <c r="J25" t="n">
-        <v>3.297</v>
+        <v>3.317</v>
       </c>
       <c r="K25" t="n">
-        <v>3.541</v>
+        <v>3.561</v>
       </c>
       <c r="L25" t="n">
-        <v>3.588</v>
+        <v>3.609</v>
       </c>
       <c r="M25" t="n">
-        <v>3.707</v>
+        <v>3.735</v>
       </c>
       <c r="N25" t="n">
-        <v>3.717</v>
+        <v>3.749</v>
       </c>
       <c r="O25" t="n">
-        <v>3.764</v>
+        <v>3.795</v>
       </c>
       <c r="P25" t="n">
-        <v>3.822</v>
+        <v>3.853</v>
       </c>
       <c r="Q25" t="n">
-        <v>3.908</v>
+        <v>3.936</v>
       </c>
       <c r="R25" t="n">
-        <v>3.886</v>
+        <v>3.901</v>
       </c>
       <c r="S25" t="n">
-        <v>3.888</v>
+        <v>3.892</v>
       </c>
       <c r="T25" t="n">
-        <v>3.802</v>
+        <v>3.801</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2307,31 +2307,31 @@
         <v>3.086</v>
       </c>
       <c r="G26" t="n">
-        <v>3.216</v>
+        <v>3.215</v>
       </c>
       <c r="H26" t="n">
-        <v>3.395</v>
+        <v>3.398</v>
       </c>
       <c r="I26" t="n">
-        <v>3.641</v>
+        <v>3.651</v>
       </c>
       <c r="J26" t="n">
-        <v>3.944</v>
+        <v>3.969</v>
       </c>
       <c r="K26" t="n">
-        <v>4.323</v>
+        <v>4.345</v>
       </c>
       <c r="L26" t="n">
-        <v>4.422</v>
+        <v>4.445</v>
       </c>
       <c r="M26" t="n">
-        <v>4.614</v>
+        <v>4.641</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>4.823</v>
+        <v>4.856</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.882</v>
+        <v>2.88</v>
       </c>
       <c r="G27" t="n">
-        <v>2.947</v>
+        <v>2.948</v>
       </c>
       <c r="H27" t="n">
         <v>3.037</v>
       </c>
       <c r="I27" t="n">
-        <v>3.228</v>
+        <v>3.232</v>
       </c>
       <c r="J27" t="n">
-        <v>3.45</v>
+        <v>3.472</v>
       </c>
       <c r="K27" t="n">
-        <v>3.648</v>
+        <v>3.668</v>
       </c>
       <c r="L27" t="n">
-        <v>3.695</v>
+        <v>3.716</v>
       </c>
       <c r="M27" t="n">
-        <v>3.825</v>
+        <v>3.852</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>3.917</v>
+        <v>3.949</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2.983</v>
+        <v>2.981</v>
       </c>
       <c r="G28" t="n">
         <v>3.054</v>
       </c>
       <c r="H28" t="n">
-        <v>3.16</v>
+        <v>3.161</v>
       </c>
       <c r="I28" t="n">
-        <v>3.364</v>
+        <v>3.369</v>
       </c>
       <c r="J28" t="n">
-        <v>3.624</v>
+        <v>3.646</v>
       </c>
       <c r="K28" t="n">
-        <v>3.841</v>
+        <v>3.861</v>
       </c>
       <c r="L28" t="n">
-        <v>3.898</v>
+        <v>3.919</v>
       </c>
       <c r="M28" t="n">
-        <v>4.038</v>
+        <v>4.064</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.211</v>
+        <v>4.242</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,7 +2523,7 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.841</v>
+        <v>2.839</v>
       </c>
       <c r="G29" t="n">
         <v>2.908</v>
@@ -2532,25 +2532,25 @@
         <v>2.983</v>
       </c>
       <c r="I29" t="n">
-        <v>3.161</v>
+        <v>3.165</v>
       </c>
       <c r="J29" t="n">
-        <v>3.363</v>
+        <v>3.385</v>
       </c>
       <c r="K29" t="n">
-        <v>3.546</v>
+        <v>3.565</v>
       </c>
       <c r="L29" t="n">
-        <v>3.579</v>
+        <v>3.6</v>
       </c>
       <c r="M29" t="n">
-        <v>3.687</v>
+        <v>3.714</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>3.776</v>
+        <v>3.808</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.106</v>
+        <v>3.107</v>
       </c>
       <c r="G30" t="n">
         <v>3.175</v>
       </c>
       <c r="H30" t="n">
-        <v>3.319</v>
+        <v>3.322</v>
       </c>
       <c r="I30" t="n">
-        <v>3.56</v>
+        <v>3.569</v>
       </c>
       <c r="J30" t="n">
-        <v>3.804</v>
+        <v>3.827</v>
       </c>
       <c r="K30" t="n">
-        <v>4.114</v>
+        <v>4.137</v>
       </c>
       <c r="L30" t="n">
-        <v>4.189</v>
+        <v>4.214</v>
       </c>
       <c r="M30" t="n">
-        <v>4.372</v>
+        <v>4.4</v>
       </c>
       <c r="N30" t="n">
-        <v>4.515</v>
+        <v>4.545</v>
       </c>
       <c r="O30" t="n">
-        <v>4.779</v>
+        <v>4.81</v>
       </c>
       <c r="P30" t="n">
-        <v>4.963</v>
+        <v>4.995</v>
       </c>
       <c r="Q30" t="n">
-        <v>5.73</v>
+        <v>5.76</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.432</v>
+        <v>3.433</v>
       </c>
       <c r="G31" t="n">
         <v>3.535</v>
       </c>
       <c r="H31" t="n">
-        <v>3.731</v>
+        <v>3.734</v>
       </c>
       <c r="I31" t="n">
-        <v>3.987</v>
+        <v>3.996</v>
       </c>
       <c r="J31" t="n">
-        <v>4.292</v>
+        <v>4.317</v>
       </c>
       <c r="K31" t="n">
-        <v>4.646</v>
+        <v>4.669</v>
       </c>
       <c r="L31" t="n">
-        <v>4.799</v>
+        <v>4.824</v>
       </c>
       <c r="M31" t="n">
-        <v>5.101</v>
+        <v>5.129</v>
       </c>
       <c r="N31" t="n">
-        <v>5.372</v>
+        <v>5.401</v>
       </c>
       <c r="O31" t="n">
-        <v>5.81</v>
+        <v>5.842</v>
       </c>
       <c r="P31" t="n">
-        <v>5.95</v>
+        <v>5.982</v>
       </c>
       <c r="Q31" t="n">
-        <v>6.703</v>
+        <v>6.733</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.203</v>
+        <v>3.204</v>
       </c>
       <c r="G32" t="n">
         <v>3.291</v>
       </c>
       <c r="H32" t="n">
-        <v>3.462</v>
+        <v>3.464</v>
       </c>
       <c r="I32" t="n">
-        <v>3.719</v>
+        <v>3.728</v>
       </c>
       <c r="J32" t="n">
-        <v>3.981</v>
+        <v>4.006</v>
       </c>
       <c r="K32" t="n">
-        <v>4.299</v>
+        <v>4.322</v>
       </c>
       <c r="L32" t="n">
-        <v>4.392</v>
+        <v>4.417</v>
       </c>
       <c r="M32" t="n">
-        <v>4.644</v>
+        <v>4.672</v>
       </c>
       <c r="N32" t="n">
-        <v>4.875</v>
+        <v>4.905</v>
       </c>
       <c r="O32" t="n">
-        <v>5.223</v>
+        <v>5.254</v>
       </c>
       <c r="P32" t="n">
-        <v>5.422</v>
+        <v>5.454</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.191</v>
+        <v>6.221</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2.991</v>
+        <v>2.992</v>
       </c>
       <c r="G33" t="n">
-        <v>3.054</v>
+        <v>3.053</v>
       </c>
       <c r="H33" t="n">
-        <v>3.145</v>
+        <v>3.148</v>
       </c>
       <c r="I33" t="n">
-        <v>3.349</v>
+        <v>3.358</v>
       </c>
       <c r="J33" t="n">
-        <v>3.515</v>
+        <v>3.54</v>
       </c>
       <c r="K33" t="n">
-        <v>3.756</v>
+        <v>3.779</v>
       </c>
       <c r="L33" t="n">
-        <v>3.795</v>
+        <v>3.82</v>
       </c>
       <c r="M33" t="n">
-        <v>3.903</v>
+        <v>3.932</v>
       </c>
       <c r="N33" t="n">
-        <v>3.899</v>
+        <v>3.931</v>
       </c>
       <c r="O33" t="n">
-        <v>3.932</v>
+        <v>3.964</v>
       </c>
       <c r="P33" t="n">
-        <v>3.993</v>
+        <v>4.024</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.447</v>
+        <v>4.476</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.05</v>
+        <v>3.051</v>
       </c>
       <c r="G34" t="n">
-        <v>3.107</v>
+        <v>3.106</v>
       </c>
       <c r="H34" t="n">
-        <v>3.205</v>
+        <v>3.207</v>
       </c>
       <c r="I34" t="n">
-        <v>3.418</v>
+        <v>3.427</v>
       </c>
       <c r="J34" t="n">
-        <v>3.587</v>
+        <v>3.612</v>
       </c>
       <c r="K34" t="n">
-        <v>3.832</v>
+        <v>3.856</v>
       </c>
       <c r="L34" t="n">
-        <v>3.874</v>
+        <v>3.899</v>
       </c>
       <c r="M34" t="n">
-        <v>3.993</v>
+        <v>4.022</v>
       </c>
       <c r="N34" t="n">
-        <v>4.004</v>
+        <v>4.036</v>
       </c>
       <c r="O34" t="n">
-        <v>4.101</v>
+        <v>4.132</v>
       </c>
       <c r="P34" t="n">
-        <v>4.287</v>
+        <v>4.319</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.148</v>
+        <v>5.178</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.024</v>
+        <v>3.025</v>
       </c>
       <c r="G35" t="n">
-        <v>3.08</v>
+        <v>3.079</v>
       </c>
       <c r="H35" t="n">
-        <v>3.172</v>
+        <v>3.175</v>
       </c>
       <c r="I35" t="n">
-        <v>3.384</v>
+        <v>3.393</v>
       </c>
       <c r="J35" t="n">
-        <v>3.555</v>
+        <v>3.58</v>
       </c>
       <c r="K35" t="n">
-        <v>3.787</v>
+        <v>3.81</v>
       </c>
       <c r="L35" t="n">
-        <v>3.829</v>
+        <v>3.854</v>
       </c>
       <c r="M35" t="n">
-        <v>3.94</v>
+        <v>3.968</v>
       </c>
       <c r="N35" t="n">
-        <v>3.94</v>
+        <v>3.972</v>
       </c>
       <c r="O35" t="n">
-        <v>3.999</v>
+        <v>4.03</v>
       </c>
       <c r="P35" t="n">
-        <v>4.09</v>
+        <v>4.121</v>
       </c>
       <c r="Q35" t="n">
-        <v>4.783</v>
+        <v>4.813</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.935</v>
+        <v>2.936</v>
       </c>
       <c r="G36" t="n">
-        <v>2.998</v>
+        <v>2.997</v>
       </c>
       <c r="H36" t="n">
-        <v>3.074</v>
+        <v>3.077</v>
       </c>
       <c r="I36" t="n">
-        <v>3.278</v>
+        <v>3.287</v>
       </c>
       <c r="J36" t="n">
-        <v>3.452</v>
+        <v>3.477</v>
       </c>
       <c r="K36" t="n">
-        <v>3.679</v>
+        <v>3.702</v>
       </c>
       <c r="L36" t="n">
-        <v>3.719</v>
+        <v>3.742</v>
       </c>
       <c r="M36" t="n">
-        <v>3.803</v>
+        <v>3.83</v>
       </c>
       <c r="N36" t="n">
-        <v>3.804</v>
+        <v>3.835</v>
       </c>
       <c r="O36" t="n">
-        <v>3.842</v>
+        <v>3.874</v>
       </c>
       <c r="P36" t="n">
-        <v>3.891</v>
+        <v>3.923</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.164</v>
+        <v>4.194</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.777</v>
+        <v>3.778</v>
       </c>
       <c r="G37" t="n">
         <v>4.23</v>
       </c>
       <c r="H37" t="n">
-        <v>4.709</v>
+        <v>4.711</v>
       </c>
       <c r="I37" t="n">
-        <v>5.059</v>
+        <v>5.068</v>
       </c>
       <c r="J37" t="n">
-        <v>5.783</v>
+        <v>5.808</v>
       </c>
       <c r="K37" t="n">
-        <v>6.684</v>
+        <v>6.706</v>
       </c>
       <c r="L37" t="n">
-        <v>6.999</v>
+        <v>7.023</v>
       </c>
       <c r="M37" t="n">
-        <v>7.374</v>
+        <v>7.402</v>
       </c>
       <c r="N37" t="n">
-        <v>7.524</v>
+        <v>7.554</v>
       </c>
       <c r="O37" t="n">
-        <v>7.691</v>
+        <v>7.722</v>
       </c>
       <c r="P37" t="n">
-        <v>7.748</v>
+        <v>7.779</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.195</v>
+        <v>8.225</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.833</v>
+        <v>4.834</v>
       </c>
       <c r="G38" t="n">
         <v>5.54</v>
       </c>
       <c r="H38" t="n">
-        <v>6.233</v>
+        <v>6.235</v>
       </c>
       <c r="I38" t="n">
-        <v>6.739</v>
+        <v>6.748</v>
       </c>
       <c r="J38" t="n">
-        <v>7.723</v>
+        <v>7.748</v>
       </c>
       <c r="K38" t="n">
-        <v>8.798999999999999</v>
+        <v>8.821</v>
       </c>
       <c r="L38" t="n">
-        <v>9.273999999999999</v>
+        <v>9.298999999999999</v>
       </c>
       <c r="M38" t="n">
-        <v>9.781000000000001</v>
+        <v>9.808999999999999</v>
       </c>
       <c r="N38" t="n">
-        <v>9.942</v>
+        <v>9.971</v>
       </c>
       <c r="O38" t="n">
-        <v>10.09</v>
+        <v>10.121</v>
       </c>
       <c r="P38" t="n">
-        <v>10.146</v>
+        <v>10.178</v>
       </c>
       <c r="Q38" t="n">
-        <v>10.646</v>
+        <v>10.676</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.154</v>
+        <v>4.155</v>
       </c>
       <c r="G39" t="n">
         <v>4.738</v>
       </c>
       <c r="H39" t="n">
-        <v>5.297</v>
+        <v>5.3</v>
       </c>
       <c r="I39" t="n">
-        <v>5.743</v>
+        <v>5.752</v>
       </c>
       <c r="J39" t="n">
-        <v>6.596</v>
+        <v>6.621</v>
       </c>
       <c r="K39" t="n">
-        <v>7.632</v>
+        <v>7.655</v>
       </c>
       <c r="L39" t="n">
-        <v>8.032999999999999</v>
+        <v>8.058</v>
       </c>
       <c r="M39" t="n">
-        <v>8.419</v>
+        <v>8.446999999999999</v>
       </c>
       <c r="N39" t="n">
-        <v>8.569000000000001</v>
+        <v>8.599</v>
       </c>
       <c r="O39" t="n">
-        <v>8.74</v>
+        <v>8.771000000000001</v>
       </c>
       <c r="P39" t="n">
-        <v>8.801</v>
+        <v>8.833</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.291</v>
+        <v>9.321</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.299</v>
+        <v>3.3</v>
       </c>
       <c r="G40" t="n">
         <v>3.414</v>
       </c>
       <c r="H40" t="n">
-        <v>3.579</v>
+        <v>3.582</v>
       </c>
       <c r="I40" t="n">
-        <v>3.834</v>
+        <v>3.843</v>
       </c>
       <c r="J40" t="n">
-        <v>4.097</v>
+        <v>4.12</v>
       </c>
       <c r="K40" t="n">
-        <v>4.419</v>
+        <v>4.441</v>
       </c>
       <c r="L40" t="n">
-        <v>4.513</v>
+        <v>4.537</v>
       </c>
       <c r="M40" t="n">
-        <v>4.713</v>
+        <v>4.741</v>
       </c>
       <c r="N40" t="n">
-        <v>4.873</v>
+        <v>4.903</v>
       </c>
       <c r="O40" t="n">
-        <v>5.158</v>
+        <v>5.188</v>
       </c>
       <c r="P40" t="n">
-        <v>5.384</v>
+        <v>5.416</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.181</v>
+        <v>6.211</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.682</v>
+        <v>3.683</v>
       </c>
       <c r="G41" t="n">
         <v>3.838</v>
       </c>
       <c r="H41" t="n">
-        <v>4.062</v>
+        <v>4.064</v>
       </c>
       <c r="I41" t="n">
-        <v>4.336</v>
+        <v>4.345</v>
       </c>
       <c r="J41" t="n">
-        <v>4.649</v>
+        <v>4.674</v>
       </c>
       <c r="K41" t="n">
-        <v>5.018</v>
+        <v>5.041</v>
       </c>
       <c r="L41" t="n">
-        <v>5.189</v>
+        <v>5.214</v>
       </c>
       <c r="M41" t="n">
-        <v>5.515</v>
+        <v>5.542</v>
       </c>
       <c r="N41" t="n">
-        <v>5.801</v>
+        <v>5.831</v>
       </c>
       <c r="O41" t="n">
-        <v>6.268</v>
+        <v>6.299</v>
       </c>
       <c r="P41" t="n">
-        <v>6.443</v>
+        <v>6.474</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.228</v>
+        <v>7.258</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.419</v>
+        <v>3.42</v>
       </c>
       <c r="G42" t="n">
         <v>3.562</v>
       </c>
       <c r="H42" t="n">
-        <v>3.754</v>
+        <v>3.756</v>
       </c>
       <c r="I42" t="n">
-        <v>4.023</v>
+        <v>4.032</v>
       </c>
       <c r="J42" t="n">
-        <v>4.298</v>
+        <v>4.323</v>
       </c>
       <c r="K42" t="n">
-        <v>4.64</v>
+        <v>4.662</v>
       </c>
       <c r="L42" t="n">
-        <v>4.748</v>
+        <v>4.773</v>
       </c>
       <c r="M42" t="n">
-        <v>5.02</v>
+        <v>5.048</v>
       </c>
       <c r="N42" t="n">
-        <v>5.287</v>
+        <v>5.317</v>
       </c>
       <c r="O42" t="n">
-        <v>5.647</v>
+        <v>5.678</v>
       </c>
       <c r="P42" t="n">
-        <v>5.885</v>
+        <v>5.917</v>
       </c>
       <c r="Q42" t="n">
-        <v>6.693</v>
+        <v>6.723</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.139</v>
+        <v>3.14</v>
       </c>
       <c r="G43" t="n">
-        <v>3.236</v>
+        <v>3.235</v>
       </c>
       <c r="H43" t="n">
-        <v>3.344</v>
+        <v>3.347</v>
       </c>
       <c r="I43" t="n">
-        <v>3.559</v>
+        <v>3.568</v>
       </c>
       <c r="J43" t="n">
-        <v>3.744</v>
+        <v>3.768</v>
       </c>
       <c r="K43" t="n">
-        <v>3.987</v>
+        <v>4.01</v>
       </c>
       <c r="L43" t="n">
-        <v>4.036</v>
+        <v>4.061</v>
       </c>
       <c r="M43" t="n">
-        <v>4.156</v>
+        <v>4.185</v>
       </c>
       <c r="N43" t="n">
-        <v>4.169</v>
+        <v>4.2</v>
       </c>
       <c r="O43" t="n">
-        <v>4.245</v>
+        <v>4.276</v>
       </c>
       <c r="P43" t="n">
-        <v>4.358</v>
+        <v>4.39</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.057</v>
+        <v>5.087</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46121</v>
+        <v>46122</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>3.013</v>
+        <v>3.014</v>
       </c>
       <c r="G44" t="n">
-        <v>3.108</v>
+        <v>3.107</v>
       </c>
       <c r="H44" t="n">
-        <v>3.199</v>
+        <v>3.201</v>
       </c>
       <c r="I44" t="n">
-        <v>3.406</v>
+        <v>3.415</v>
       </c>
       <c r="J44" t="n">
-        <v>3.594</v>
+        <v>3.619</v>
       </c>
       <c r="K44" t="n">
-        <v>3.829</v>
+        <v>3.852</v>
       </c>
       <c r="L44" t="n">
-        <v>3.879</v>
+        <v>3.902</v>
       </c>
       <c r="M44" t="n">
-        <v>3.971</v>
+        <v>3.999</v>
       </c>
       <c r="N44" t="n">
-        <v>3.986</v>
+        <v>4.017</v>
       </c>
       <c r="O44" t="n">
-        <v>4.042</v>
+        <v>4.073</v>
       </c>
       <c r="P44" t="n">
-        <v>4.121</v>
+        <v>4.153</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.427</v>
+        <v>4.457</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-04-13 ~ 2026-04-13
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.248</v>
+        <v>3.244</v>
       </c>
       <c r="G2" t="n">
-        <v>3.461</v>
+        <v>3.456</v>
       </c>
       <c r="H2" t="n">
-        <v>3.594</v>
+        <v>3.593</v>
       </c>
       <c r="I2" t="n">
-        <v>3.804</v>
+        <v>3.819</v>
       </c>
       <c r="J2" t="n">
-        <v>4.002</v>
+        <v>4.029</v>
       </c>
       <c r="K2" t="n">
-        <v>4.392</v>
+        <v>4.416</v>
       </c>
       <c r="L2" t="n">
-        <v>4.562</v>
+        <v>4.583</v>
       </c>
       <c r="M2" t="n">
-        <v>4.867</v>
+        <v>4.891</v>
       </c>
       <c r="N2" t="n">
-        <v>5.116</v>
+        <v>5.147</v>
       </c>
       <c r="O2" t="n">
-        <v>5.321</v>
+        <v>5.356</v>
       </c>
       <c r="P2" t="n">
-        <v>5.517</v>
+        <v>5.547</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.155</v>
+        <v>6.182</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.271</v>
+        <v>4.267</v>
       </c>
       <c r="G3" t="n">
-        <v>4.665</v>
+        <v>4.66</v>
       </c>
       <c r="H3" t="n">
-        <v>4.832</v>
+        <v>4.831</v>
       </c>
       <c r="I3" t="n">
-        <v>5.042</v>
+        <v>5.057</v>
       </c>
       <c r="J3" t="n">
-        <v>5.25</v>
+        <v>5.276</v>
       </c>
       <c r="K3" t="n">
-        <v>5.708</v>
+        <v>5.731</v>
       </c>
       <c r="L3" t="n">
-        <v>5.948</v>
+        <v>5.968</v>
       </c>
       <c r="M3" t="n">
-        <v>6.284</v>
+        <v>6.307</v>
       </c>
       <c r="N3" t="n">
-        <v>6.476</v>
+        <v>6.507</v>
       </c>
       <c r="O3" t="n">
-        <v>6.63</v>
+        <v>6.665</v>
       </c>
       <c r="P3" t="n">
-        <v>6.696</v>
+        <v>6.727</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.223</v>
+        <v>7.25</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.762</v>
+        <v>3.758</v>
       </c>
       <c r="G4" t="n">
-        <v>4.045</v>
+        <v>4.04</v>
       </c>
       <c r="H4" t="n">
         <v>4.24</v>
       </c>
       <c r="I4" t="n">
-        <v>4.482</v>
+        <v>4.497</v>
       </c>
       <c r="J4" t="n">
-        <v>4.696</v>
+        <v>4.723</v>
       </c>
       <c r="K4" t="n">
-        <v>5.148</v>
+        <v>5.171</v>
       </c>
       <c r="L4" t="n">
-        <v>5.318</v>
+        <v>5.338</v>
       </c>
       <c r="M4" t="n">
-        <v>5.642</v>
+        <v>5.665</v>
       </c>
       <c r="N4" t="n">
-        <v>5.804</v>
+        <v>5.835</v>
       </c>
       <c r="O4" t="n">
-        <v>5.982</v>
+        <v>6.017</v>
       </c>
       <c r="P4" t="n">
-        <v>6.046</v>
+        <v>6.077</v>
       </c>
       <c r="Q4" t="n">
-        <v>6.576</v>
+        <v>6.603</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.955</v>
+        <v>2.951</v>
       </c>
       <c r="G5" t="n">
-        <v>3.009</v>
+        <v>3.004</v>
       </c>
       <c r="H5" t="n">
-        <v>3.097</v>
+        <v>3.096</v>
       </c>
       <c r="I5" t="n">
-        <v>3.379</v>
+        <v>3.394</v>
       </c>
       <c r="J5" t="n">
-        <v>3.574</v>
+        <v>3.601</v>
       </c>
       <c r="K5" t="n">
-        <v>3.823</v>
+        <v>3.846</v>
       </c>
       <c r="L5" t="n">
-        <v>3.836</v>
+        <v>3.856</v>
       </c>
       <c r="M5" t="n">
-        <v>3.946</v>
+        <v>3.969</v>
       </c>
       <c r="N5" t="n">
-        <v>3.924</v>
+        <v>3.957</v>
       </c>
       <c r="O5" t="n">
-        <v>3.917</v>
+        <v>3.957</v>
       </c>
       <c r="P5" t="n">
-        <v>4.186</v>
+        <v>4.217</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.067</v>
+        <v>5.094</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2.996</v>
+        <v>2.992</v>
       </c>
       <c r="G6" t="n">
-        <v>3.065</v>
+        <v>3.06</v>
       </c>
       <c r="H6" t="n">
-        <v>3.167</v>
+        <v>3.166</v>
       </c>
       <c r="I6" t="n">
-        <v>3.453</v>
+        <v>3.469</v>
       </c>
       <c r="J6" t="n">
-        <v>3.658</v>
+        <v>3.684</v>
       </c>
       <c r="K6" t="n">
-        <v>3.924</v>
+        <v>3.947</v>
       </c>
       <c r="L6" t="n">
-        <v>3.949</v>
+        <v>3.969</v>
       </c>
       <c r="M6" t="n">
-        <v>4.093</v>
+        <v>4.116</v>
       </c>
       <c r="N6" t="n">
-        <v>4.093</v>
+        <v>4.127</v>
       </c>
       <c r="O6" t="n">
-        <v>4.189</v>
+        <v>4.223</v>
       </c>
       <c r="P6" t="n">
-        <v>4.619</v>
+        <v>4.649</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.463</v>
+        <v>5.49</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2.976</v>
+        <v>2.972</v>
       </c>
       <c r="G7" t="n">
-        <v>3.028</v>
+        <v>3.023</v>
       </c>
       <c r="H7" t="n">
-        <v>3.113</v>
+        <v>3.112</v>
       </c>
       <c r="I7" t="n">
-        <v>3.394</v>
+        <v>3.409</v>
       </c>
       <c r="J7" t="n">
-        <v>3.599</v>
+        <v>3.626</v>
       </c>
       <c r="K7" t="n">
-        <v>3.849</v>
+        <v>3.872</v>
       </c>
       <c r="L7" t="n">
-        <v>3.86</v>
+        <v>3.881</v>
       </c>
       <c r="M7" t="n">
-        <v>4.004</v>
+        <v>4.027</v>
       </c>
       <c r="N7" t="n">
-        <v>3.984</v>
+        <v>4.017</v>
       </c>
       <c r="O7" t="n">
-        <v>4.088</v>
+        <v>4.122</v>
       </c>
       <c r="P7" t="n">
-        <v>4.402</v>
+        <v>4.433</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.231</v>
+        <v>5.258</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.381</v>
+        <v>5.377</v>
       </c>
       <c r="G8" t="n">
-        <v>5.963</v>
+        <v>5.958</v>
       </c>
       <c r="H8" t="n">
-        <v>6.281</v>
+        <v>6.28</v>
       </c>
       <c r="I8" t="n">
-        <v>6.562</v>
+        <v>6.577</v>
       </c>
       <c r="J8" t="n">
-        <v>6.834</v>
+        <v>6.861</v>
       </c>
       <c r="K8" t="n">
-        <v>7.573</v>
+        <v>7.596</v>
       </c>
       <c r="L8" t="n">
-        <v>7.903</v>
+        <v>7.923</v>
       </c>
       <c r="M8" t="n">
-        <v>8.266999999999999</v>
+        <v>8.291</v>
       </c>
       <c r="N8" t="n">
-        <v>8.397</v>
+        <v>8.428000000000001</v>
       </c>
       <c r="O8" t="n">
-        <v>8.637</v>
+        <v>8.672000000000001</v>
       </c>
       <c r="P8" t="n">
-        <v>8.803000000000001</v>
+        <v>8.834</v>
       </c>
       <c r="Q8" t="n">
-        <v>9.532</v>
+        <v>9.558999999999999</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1066,54 +1066,54 @@
         <v>2.618</v>
       </c>
       <c r="G9" t="n">
-        <v>2.686</v>
+        <v>2.687</v>
       </c>
       <c r="H9" t="n">
-        <v>2.777</v>
+        <v>2.782</v>
       </c>
       <c r="I9" t="n">
-        <v>2.917</v>
+        <v>2.921</v>
       </c>
       <c r="J9" t="n">
-        <v>3.098</v>
+        <v>3.119</v>
       </c>
       <c r="K9" t="n">
-        <v>3.225</v>
+        <v>3.242</v>
       </c>
       <c r="L9" t="n">
-        <v>3.274</v>
+        <v>3.29</v>
       </c>
       <c r="M9" t="n">
-        <v>3.357</v>
+        <v>3.38</v>
       </c>
       <c r="N9" t="n">
-        <v>3.5</v>
+        <v>3.532</v>
       </c>
       <c r="O9" t="n">
-        <v>3.514</v>
+        <v>3.55</v>
       </c>
       <c r="P9" t="n">
-        <v>3.607</v>
+        <v>3.638</v>
       </c>
       <c r="Q9" t="n">
-        <v>3.685</v>
+        <v>3.712</v>
       </c>
       <c r="R9" t="n">
-        <v>3.69</v>
+        <v>3.72</v>
       </c>
       <c r="S9" t="n">
-        <v>3.645</v>
+        <v>3.677</v>
       </c>
       <c r="T9" t="n">
-        <v>3.569</v>
+        <v>3.601</v>
       </c>
       <c r="U9" t="n">
-        <v>3.442</v>
+        <v>3.475</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1139,31 +1139,31 @@
         <v>2.63</v>
       </c>
       <c r="G10" t="n">
-        <v>2.718</v>
+        <v>2.72</v>
       </c>
       <c r="H10" t="n">
-        <v>2.789</v>
+        <v>2.792</v>
       </c>
       <c r="I10" t="n">
-        <v>2.926</v>
+        <v>2.93</v>
       </c>
       <c r="J10" t="n">
-        <v>3.127</v>
+        <v>3.146</v>
       </c>
       <c r="K10" t="n">
-        <v>3.252</v>
+        <v>3.27</v>
       </c>
       <c r="L10" t="n">
-        <v>3.316</v>
+        <v>3.332</v>
       </c>
       <c r="M10" t="n">
-        <v>3.457</v>
+        <v>3.479</v>
       </c>
       <c r="N10" t="n">
-        <v>3.508</v>
+        <v>3.54</v>
       </c>
       <c r="O10" t="n">
-        <v>3.677</v>
+        <v>3.727</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1212,37 +1212,37 @@
         <v>2.446</v>
       </c>
       <c r="G11" t="n">
-        <v>2.528</v>
+        <v>2.53</v>
       </c>
       <c r="H11" t="n">
-        <v>2.613</v>
+        <v>2.616</v>
       </c>
       <c r="I11" t="n">
-        <v>2.728</v>
+        <v>2.732</v>
       </c>
       <c r="J11" t="n">
-        <v>2.921</v>
+        <v>2.94</v>
       </c>
       <c r="K11" t="n">
-        <v>3.039</v>
+        <v>3.057</v>
       </c>
       <c r="L11" t="n">
-        <v>3.11</v>
+        <v>3.126</v>
       </c>
       <c r="M11" t="n">
-        <v>3.262</v>
+        <v>3.284</v>
       </c>
       <c r="N11" t="n">
-        <v>3.318</v>
+        <v>3.35</v>
       </c>
       <c r="O11" t="n">
-        <v>3.443</v>
+        <v>3.494</v>
       </c>
       <c r="P11" t="n">
-        <v>3.544</v>
+        <v>3.574</v>
       </c>
       <c r="Q11" t="n">
-        <v>3.888</v>
+        <v>3.915</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.216</v>
+        <v>3.213</v>
       </c>
       <c r="G12" t="n">
-        <v>3.369</v>
+        <v>3.364</v>
       </c>
       <c r="H12" t="n">
-        <v>3.468</v>
+        <v>3.466</v>
       </c>
       <c r="I12" t="n">
-        <v>3.685</v>
+        <v>3.695</v>
       </c>
       <c r="J12" t="n">
-        <v>3.982</v>
+        <v>4.003</v>
       </c>
       <c r="K12" t="n">
-        <v>4.177</v>
+        <v>4.196</v>
       </c>
       <c r="L12" t="n">
-        <v>4.228</v>
+        <v>4.248</v>
       </c>
       <c r="M12" t="n">
-        <v>4.373</v>
+        <v>4.396</v>
       </c>
       <c r="N12" t="n">
-        <v>4.392</v>
+        <v>4.424</v>
       </c>
       <c r="O12" t="n">
-        <v>4.525</v>
+        <v>4.559</v>
       </c>
       <c r="P12" t="n">
-        <v>4.653</v>
+        <v>4.684</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.016</v>
+        <v>5.043</v>
       </c>
       <c r="R12" t="n">
-        <v>5.187</v>
+        <v>5.217</v>
       </c>
       <c r="S12" t="n">
-        <v>5.356</v>
+        <v>5.388</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2.97</v>
+        <v>2.966</v>
       </c>
       <c r="G13" t="n">
-        <v>3.059</v>
+        <v>3.054</v>
       </c>
       <c r="H13" t="n">
-        <v>3.136</v>
+        <v>3.133</v>
       </c>
       <c r="I13" t="n">
-        <v>3.332</v>
+        <v>3.343</v>
       </c>
       <c r="J13" t="n">
-        <v>3.619</v>
+        <v>3.639</v>
       </c>
       <c r="K13" t="n">
-        <v>3.81</v>
+        <v>3.829</v>
       </c>
       <c r="L13" t="n">
-        <v>3.867</v>
+        <v>3.888</v>
       </c>
       <c r="M13" t="n">
-        <v>4</v>
+        <v>4.023</v>
       </c>
       <c r="N13" t="n">
-        <v>4.02</v>
+        <v>4.052</v>
       </c>
       <c r="O13" t="n">
-        <v>4.151</v>
+        <v>4.185</v>
       </c>
       <c r="P13" t="n">
-        <v>4.244</v>
+        <v>4.275</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.537</v>
+        <v>4.564</v>
       </c>
       <c r="R13" t="n">
-        <v>4.735</v>
+        <v>4.765</v>
       </c>
       <c r="S13" t="n">
-        <v>4.918</v>
+        <v>4.95</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.788</v>
+        <v>2.784</v>
       </c>
       <c r="G14" t="n">
-        <v>2.865</v>
+        <v>2.861</v>
       </c>
       <c r="H14" t="n">
-        <v>2.939</v>
+        <v>2.937</v>
       </c>
       <c r="I14" t="n">
-        <v>3.115</v>
+        <v>3.126</v>
       </c>
       <c r="J14" t="n">
-        <v>3.359</v>
+        <v>3.379</v>
       </c>
       <c r="K14" t="n">
-        <v>3.498</v>
+        <v>3.517</v>
       </c>
       <c r="L14" t="n">
-        <v>3.539</v>
+        <v>3.56</v>
       </c>
       <c r="M14" t="n">
-        <v>3.685</v>
+        <v>3.708</v>
       </c>
       <c r="N14" t="n">
-        <v>3.699</v>
+        <v>3.731</v>
       </c>
       <c r="O14" t="n">
-        <v>3.806</v>
+        <v>3.84</v>
       </c>
       <c r="P14" t="n">
-        <v>3.88</v>
+        <v>3.91</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.126</v>
+        <v>4.153</v>
       </c>
       <c r="R14" t="n">
-        <v>4.25</v>
+        <v>4.28</v>
       </c>
       <c r="S14" t="n">
-        <v>4.371</v>
+        <v>4.403</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.766</v>
+        <v>2.763</v>
       </c>
       <c r="G15" t="n">
-        <v>2.84</v>
+        <v>2.835</v>
       </c>
       <c r="H15" t="n">
-        <v>2.908</v>
+        <v>2.905</v>
       </c>
       <c r="I15" t="n">
-        <v>3.066</v>
+        <v>3.077</v>
       </c>
       <c r="J15" t="n">
-        <v>3.296</v>
+        <v>3.316</v>
       </c>
       <c r="K15" t="n">
-        <v>3.451</v>
+        <v>3.47</v>
       </c>
       <c r="L15" t="n">
-        <v>3.474</v>
+        <v>3.495</v>
       </c>
       <c r="M15" t="n">
-        <v>3.598</v>
+        <v>3.621</v>
       </c>
       <c r="N15" t="n">
-        <v>3.603</v>
+        <v>3.635</v>
       </c>
       <c r="O15" t="n">
-        <v>3.73</v>
+        <v>3.765</v>
       </c>
       <c r="P15" t="n">
-        <v>3.777</v>
+        <v>3.807</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.031</v>
+        <v>4.058</v>
       </c>
       <c r="R15" t="n">
-        <v>4.146</v>
+        <v>4.176</v>
       </c>
       <c r="S15" t="n">
-        <v>4.266</v>
+        <v>4.298</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.766</v>
+        <v>2.763</v>
       </c>
       <c r="G16" t="n">
-        <v>2.84</v>
+        <v>2.835</v>
       </c>
       <c r="H16" t="n">
-        <v>2.908</v>
+        <v>2.905</v>
       </c>
       <c r="I16" t="n">
-        <v>3.066</v>
+        <v>3.077</v>
       </c>
       <c r="J16" t="n">
-        <v>3.296</v>
+        <v>3.316</v>
       </c>
       <c r="K16" t="n">
-        <v>3.451</v>
+        <v>3.47</v>
       </c>
       <c r="L16" t="n">
-        <v>3.474</v>
+        <v>3.495</v>
       </c>
       <c r="M16" t="n">
-        <v>3.598</v>
+        <v>3.621</v>
       </c>
       <c r="N16" t="n">
-        <v>3.606</v>
+        <v>3.638</v>
       </c>
       <c r="O16" t="n">
-        <v>3.737</v>
+        <v>3.772</v>
       </c>
       <c r="P16" t="n">
-        <v>3.8</v>
+        <v>3.831</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.058</v>
+        <v>4.085</v>
       </c>
       <c r="R16" t="n">
-        <v>4.174</v>
+        <v>4.204</v>
       </c>
       <c r="S16" t="n">
-        <v>4.295</v>
+        <v>4.327</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.692</v>
+        <v>2.693</v>
       </c>
       <c r="G17" t="n">
-        <v>2.809</v>
+        <v>2.811</v>
       </c>
       <c r="H17" t="n">
-        <v>2.882</v>
+        <v>2.886</v>
       </c>
       <c r="I17" t="n">
-        <v>3.008</v>
+        <v>3.012</v>
       </c>
       <c r="J17" t="n">
-        <v>3.195</v>
+        <v>3.215</v>
       </c>
       <c r="K17" t="n">
-        <v>3.324</v>
+        <v>3.342</v>
       </c>
       <c r="L17" t="n">
-        <v>3.394</v>
+        <v>3.409</v>
       </c>
       <c r="M17" t="n">
-        <v>3.577</v>
+        <v>3.599</v>
       </c>
       <c r="N17" t="n">
-        <v>3.609</v>
+        <v>3.641</v>
       </c>
       <c r="O17" t="n">
-        <v>3.713</v>
+        <v>3.762</v>
       </c>
       <c r="P17" t="n">
-        <v>3.824</v>
+        <v>3.853</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.693</v>
+        <v>2.694</v>
       </c>
       <c r="G18" t="n">
-        <v>2.81</v>
+        <v>2.812</v>
       </c>
       <c r="H18" t="n">
-        <v>2.883</v>
+        <v>2.886</v>
       </c>
       <c r="I18" t="n">
-        <v>3.009</v>
+        <v>3.013</v>
       </c>
       <c r="J18" t="n">
-        <v>3.195</v>
+        <v>3.215</v>
       </c>
       <c r="K18" t="n">
-        <v>3.325</v>
+        <v>3.343</v>
       </c>
       <c r="L18" t="n">
-        <v>3.394</v>
+        <v>3.409</v>
       </c>
       <c r="M18" t="n">
-        <v>3.577</v>
+        <v>3.599</v>
       </c>
       <c r="N18" t="n">
-        <v>3.608</v>
+        <v>3.641</v>
       </c>
       <c r="O18" t="n">
-        <v>3.711</v>
+        <v>3.76</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.777</v>
+        <v>2.773</v>
       </c>
       <c r="G19" t="n">
-        <v>2.856</v>
+        <v>2.851</v>
       </c>
       <c r="H19" t="n">
-        <v>2.929</v>
+        <v>2.926</v>
       </c>
       <c r="I19" t="n">
-        <v>3.1</v>
+        <v>3.11</v>
       </c>
       <c r="J19" t="n">
-        <v>3.342</v>
+        <v>3.362</v>
       </c>
       <c r="K19" t="n">
-        <v>3.495</v>
+        <v>3.513</v>
       </c>
       <c r="L19" t="n">
-        <v>3.536</v>
+        <v>3.557</v>
       </c>
       <c r="M19" t="n">
-        <v>3.673</v>
+        <v>3.697</v>
       </c>
       <c r="N19" t="n">
-        <v>3.686</v>
+        <v>3.719</v>
       </c>
       <c r="O19" t="n">
-        <v>3.784</v>
+        <v>3.819</v>
       </c>
       <c r="P19" t="n">
-        <v>3.843</v>
+        <v>3.873</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.076</v>
+        <v>4.103</v>
       </c>
       <c r="R19" t="n">
-        <v>4.199</v>
+        <v>4.229</v>
       </c>
       <c r="S19" t="n">
-        <v>4.309</v>
+        <v>4.341</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2.573</v>
+        <v>2.574</v>
       </c>
       <c r="G20" t="n">
-        <v>2.645</v>
+        <v>2.646</v>
       </c>
       <c r="H20" t="n">
         <v>2.695</v>
       </c>
       <c r="I20" t="n">
-        <v>2.858</v>
+        <v>2.862</v>
       </c>
       <c r="J20" t="n">
-        <v>3.105</v>
+        <v>3.123</v>
       </c>
       <c r="K20" t="n">
-        <v>3.261</v>
+        <v>3.278</v>
       </c>
       <c r="L20" t="n">
-        <v>3.3</v>
+        <v>3.324</v>
       </c>
       <c r="M20" t="n">
-        <v>3.394</v>
+        <v>3.42</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1945,40 +1945,40 @@
         <v>2.955</v>
       </c>
       <c r="H21" t="n">
-        <v>3.07</v>
+        <v>3.068</v>
       </c>
       <c r="I21" t="n">
-        <v>3.239</v>
+        <v>3.248</v>
       </c>
       <c r="J21" t="n">
-        <v>3.471</v>
+        <v>3.492</v>
       </c>
       <c r="K21" t="n">
-        <v>3.732</v>
+        <v>3.75</v>
       </c>
       <c r="L21" t="n">
-        <v>3.8</v>
+        <v>3.817</v>
       </c>
       <c r="M21" t="n">
-        <v>3.931</v>
+        <v>3.953</v>
       </c>
       <c r="N21" t="n">
-        <v>3.953</v>
+        <v>3.985</v>
       </c>
       <c r="O21" t="n">
-        <v>4.023</v>
+        <v>4.057</v>
       </c>
       <c r="P21" t="n">
-        <v>4.108</v>
+        <v>4.137</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.237</v>
+        <v>4.264</v>
       </c>
       <c r="R21" t="n">
-        <v>4.246</v>
+        <v>4.276</v>
       </c>
       <c r="S21" t="n">
-        <v>4.269</v>
+        <v>4.301</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2018,40 +2018,40 @@
         <v>2.902</v>
       </c>
       <c r="H22" t="n">
-        <v>3.004</v>
+        <v>3.002</v>
       </c>
       <c r="I22" t="n">
-        <v>3.158</v>
+        <v>3.166</v>
       </c>
       <c r="J22" t="n">
-        <v>3.355</v>
+        <v>3.376</v>
       </c>
       <c r="K22" t="n">
-        <v>3.613</v>
+        <v>3.63</v>
       </c>
       <c r="L22" t="n">
-        <v>3.67</v>
+        <v>3.686</v>
       </c>
       <c r="M22" t="n">
-        <v>3.802</v>
+        <v>3.825</v>
       </c>
       <c r="N22" t="n">
-        <v>3.826</v>
+        <v>3.858</v>
       </c>
       <c r="O22" t="n">
-        <v>3.891</v>
+        <v>3.925</v>
       </c>
       <c r="P22" t="n">
-        <v>3.97</v>
+        <v>3.999</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.095</v>
+        <v>4.122</v>
       </c>
       <c r="R22" t="n">
-        <v>4.094</v>
+        <v>4.124</v>
       </c>
       <c r="S22" t="n">
-        <v>4.114</v>
+        <v>4.146</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.774</v>
+        <v>2.775</v>
       </c>
       <c r="G23" t="n">
         <v>2.857</v>
       </c>
       <c r="H23" t="n">
-        <v>2.943</v>
+        <v>2.941</v>
       </c>
       <c r="I23" t="n">
-        <v>3.11</v>
+        <v>3.119</v>
       </c>
       <c r="J23" t="n">
-        <v>3.301</v>
+        <v>3.322</v>
       </c>
       <c r="K23" t="n">
-        <v>3.532</v>
+        <v>3.55</v>
       </c>
       <c r="L23" t="n">
-        <v>3.581</v>
+        <v>3.597</v>
       </c>
       <c r="M23" t="n">
-        <v>3.707</v>
+        <v>3.73</v>
       </c>
       <c r="N23" t="n">
-        <v>3.722</v>
+        <v>3.754</v>
       </c>
       <c r="O23" t="n">
-        <v>3.765</v>
+        <v>3.8</v>
       </c>
       <c r="P23" t="n">
-        <v>3.831</v>
+        <v>3.861</v>
       </c>
       <c r="Q23" t="n">
-        <v>3.903</v>
+        <v>3.93</v>
       </c>
       <c r="R23" t="n">
-        <v>3.878</v>
+        <v>3.908</v>
       </c>
       <c r="S23" t="n">
-        <v>3.869</v>
+        <v>3.901</v>
       </c>
       <c r="T23" t="n">
-        <v>3.783</v>
+        <v>3.815</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2164,40 +2164,40 @@
         <v>2.771</v>
       </c>
       <c r="H24" t="n">
-        <v>2.844</v>
+        <v>2.842</v>
       </c>
       <c r="I24" t="n">
-        <v>3.021</v>
+        <v>3.029</v>
       </c>
       <c r="J24" t="n">
-        <v>3.202</v>
+        <v>3.223</v>
       </c>
       <c r="K24" t="n">
-        <v>3.415</v>
+        <v>3.434</v>
       </c>
       <c r="L24" t="n">
-        <v>3.452</v>
+        <v>3.469</v>
       </c>
       <c r="M24" t="n">
-        <v>3.562</v>
+        <v>3.585</v>
       </c>
       <c r="N24" t="n">
-        <v>3.592</v>
+        <v>3.624</v>
       </c>
       <c r="O24" t="n">
-        <v>3.717</v>
+        <v>3.751</v>
       </c>
       <c r="P24" t="n">
-        <v>3.77</v>
+        <v>3.8</v>
       </c>
       <c r="Q24" t="n">
-        <v>3.825</v>
+        <v>3.853</v>
       </c>
       <c r="R24" t="n">
-        <v>3.799</v>
+        <v>3.829</v>
       </c>
       <c r="S24" t="n">
-        <v>3.784</v>
+        <v>3.816</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.767</v>
+        <v>2.768</v>
       </c>
       <c r="G25" t="n">
         <v>2.856</v>
       </c>
       <c r="H25" t="n">
-        <v>2.946</v>
+        <v>2.944</v>
       </c>
       <c r="I25" t="n">
-        <v>3.118</v>
+        <v>3.127</v>
       </c>
       <c r="J25" t="n">
-        <v>3.317</v>
+        <v>3.338</v>
       </c>
       <c r="K25" t="n">
-        <v>3.561</v>
+        <v>3.579</v>
       </c>
       <c r="L25" t="n">
-        <v>3.609</v>
+        <v>3.626</v>
       </c>
       <c r="M25" t="n">
-        <v>3.735</v>
+        <v>3.758</v>
       </c>
       <c r="N25" t="n">
-        <v>3.749</v>
+        <v>3.781</v>
       </c>
       <c r="O25" t="n">
-        <v>3.795</v>
+        <v>3.829</v>
       </c>
       <c r="P25" t="n">
-        <v>3.853</v>
+        <v>3.883</v>
       </c>
       <c r="Q25" t="n">
-        <v>3.936</v>
+        <v>3.963</v>
       </c>
       <c r="R25" t="n">
-        <v>3.901</v>
+        <v>3.931</v>
       </c>
       <c r="S25" t="n">
-        <v>3.892</v>
+        <v>3.924</v>
       </c>
       <c r="T25" t="n">
-        <v>3.801</v>
+        <v>3.833</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.086</v>
+        <v>3.082</v>
       </c>
       <c r="G26" t="n">
-        <v>3.215</v>
+        <v>3.209</v>
       </c>
       <c r="H26" t="n">
-        <v>3.398</v>
+        <v>3.4</v>
       </c>
       <c r="I26" t="n">
-        <v>3.651</v>
+        <v>3.66</v>
       </c>
       <c r="J26" t="n">
-        <v>3.969</v>
+        <v>3.989</v>
       </c>
       <c r="K26" t="n">
-        <v>4.345</v>
+        <v>4.368</v>
       </c>
       <c r="L26" t="n">
-        <v>4.445</v>
+        <v>4.464</v>
       </c>
       <c r="M26" t="n">
-        <v>4.641</v>
+        <v>4.664</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>4.856</v>
+        <v>4.891</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.88</v>
+        <v>2.876</v>
       </c>
       <c r="G27" t="n">
-        <v>2.948</v>
+        <v>2.942</v>
       </c>
       <c r="H27" t="n">
-        <v>3.037</v>
+        <v>3.039</v>
       </c>
       <c r="I27" t="n">
-        <v>3.232</v>
+        <v>3.242</v>
       </c>
       <c r="J27" t="n">
-        <v>3.472</v>
+        <v>3.493</v>
       </c>
       <c r="K27" t="n">
-        <v>3.668</v>
+        <v>3.688</v>
       </c>
       <c r="L27" t="n">
-        <v>3.716</v>
+        <v>3.735</v>
       </c>
       <c r="M27" t="n">
-        <v>3.852</v>
+        <v>3.875</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>3.949</v>
+        <v>3.982</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2.981</v>
+        <v>2.977</v>
       </c>
       <c r="G28" t="n">
-        <v>3.054</v>
+        <v>3.048</v>
       </c>
       <c r="H28" t="n">
-        <v>3.161</v>
+        <v>3.162</v>
       </c>
       <c r="I28" t="n">
-        <v>3.369</v>
+        <v>3.379</v>
       </c>
       <c r="J28" t="n">
-        <v>3.646</v>
+        <v>3.667</v>
       </c>
       <c r="K28" t="n">
-        <v>3.861</v>
+        <v>3.881</v>
       </c>
       <c r="L28" t="n">
-        <v>3.919</v>
+        <v>3.939</v>
       </c>
       <c r="M28" t="n">
-        <v>4.064</v>
+        <v>4.088</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.242</v>
+        <v>4.276</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.839</v>
+        <v>2.835</v>
       </c>
       <c r="G29" t="n">
-        <v>2.908</v>
+        <v>2.902</v>
       </c>
       <c r="H29" t="n">
-        <v>2.983</v>
+        <v>2.984</v>
       </c>
       <c r="I29" t="n">
-        <v>3.165</v>
+        <v>3.176</v>
       </c>
       <c r="J29" t="n">
-        <v>3.385</v>
+        <v>3.406</v>
       </c>
       <c r="K29" t="n">
-        <v>3.565</v>
+        <v>3.584</v>
       </c>
       <c r="L29" t="n">
-        <v>3.6</v>
+        <v>3.62</v>
       </c>
       <c r="M29" t="n">
-        <v>3.714</v>
+        <v>3.737</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>3.808</v>
+        <v>3.842</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.107</v>
+        <v>3.105</v>
       </c>
       <c r="G30" t="n">
-        <v>3.175</v>
+        <v>3.17</v>
       </c>
       <c r="H30" t="n">
-        <v>3.322</v>
+        <v>3.324</v>
       </c>
       <c r="I30" t="n">
-        <v>3.569</v>
+        <v>3.575</v>
       </c>
       <c r="J30" t="n">
-        <v>3.827</v>
+        <v>3.847</v>
       </c>
       <c r="K30" t="n">
-        <v>4.137</v>
+        <v>4.158</v>
       </c>
       <c r="L30" t="n">
-        <v>4.214</v>
+        <v>4.231</v>
       </c>
       <c r="M30" t="n">
-        <v>4.4</v>
+        <v>4.423</v>
       </c>
       <c r="N30" t="n">
-        <v>4.545</v>
+        <v>4.577</v>
       </c>
       <c r="O30" t="n">
-        <v>4.81</v>
+        <v>4.844</v>
       </c>
       <c r="P30" t="n">
-        <v>4.995</v>
+        <v>5.025</v>
       </c>
       <c r="Q30" t="n">
-        <v>5.76</v>
+        <v>5.787</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.433</v>
+        <v>3.431</v>
       </c>
       <c r="G31" t="n">
-        <v>3.535</v>
+        <v>3.53</v>
       </c>
       <c r="H31" t="n">
-        <v>3.734</v>
+        <v>3.736</v>
       </c>
       <c r="I31" t="n">
-        <v>3.996</v>
+        <v>4.003</v>
       </c>
       <c r="J31" t="n">
-        <v>4.317</v>
+        <v>4.338</v>
       </c>
       <c r="K31" t="n">
-        <v>4.669</v>
+        <v>4.691</v>
       </c>
       <c r="L31" t="n">
-        <v>4.824</v>
+        <v>4.842</v>
       </c>
       <c r="M31" t="n">
-        <v>5.129</v>
+        <v>5.152</v>
       </c>
       <c r="N31" t="n">
-        <v>5.401</v>
+        <v>5.433</v>
       </c>
       <c r="O31" t="n">
-        <v>5.842</v>
+        <v>5.876</v>
       </c>
       <c r="P31" t="n">
-        <v>5.982</v>
+        <v>6.012</v>
       </c>
       <c r="Q31" t="n">
-        <v>6.733</v>
+        <v>6.76</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.204</v>
+        <v>3.203</v>
       </c>
       <c r="G32" t="n">
-        <v>3.291</v>
+        <v>3.286</v>
       </c>
       <c r="H32" t="n">
-        <v>3.464</v>
+        <v>3.466</v>
       </c>
       <c r="I32" t="n">
-        <v>3.728</v>
+        <v>3.735</v>
       </c>
       <c r="J32" t="n">
-        <v>4.006</v>
+        <v>4.026</v>
       </c>
       <c r="K32" t="n">
-        <v>4.322</v>
+        <v>4.343</v>
       </c>
       <c r="L32" t="n">
-        <v>4.417</v>
+        <v>4.434</v>
       </c>
       <c r="M32" t="n">
-        <v>4.672</v>
+        <v>4.695</v>
       </c>
       <c r="N32" t="n">
-        <v>4.905</v>
+        <v>4.937</v>
       </c>
       <c r="O32" t="n">
-        <v>5.254</v>
+        <v>5.288</v>
       </c>
       <c r="P32" t="n">
-        <v>5.454</v>
+        <v>5.484</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.221</v>
+        <v>6.248</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2.992</v>
+        <v>2.989</v>
       </c>
       <c r="G33" t="n">
-        <v>3.053</v>
+        <v>3.047</v>
       </c>
       <c r="H33" t="n">
-        <v>3.148</v>
+        <v>3.149</v>
       </c>
       <c r="I33" t="n">
-        <v>3.358</v>
+        <v>3.365</v>
       </c>
       <c r="J33" t="n">
-        <v>3.54</v>
+        <v>3.561</v>
       </c>
       <c r="K33" t="n">
-        <v>3.779</v>
+        <v>3.8</v>
       </c>
       <c r="L33" t="n">
-        <v>3.82</v>
+        <v>3.837</v>
       </c>
       <c r="M33" t="n">
-        <v>3.932</v>
+        <v>3.955</v>
       </c>
       <c r="N33" t="n">
-        <v>3.931</v>
+        <v>3.965</v>
       </c>
       <c r="O33" t="n">
-        <v>3.964</v>
+        <v>3.998</v>
       </c>
       <c r="P33" t="n">
-        <v>4.024</v>
+        <v>4.055</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.476</v>
+        <v>4.504</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.051</v>
+        <v>3.048</v>
       </c>
       <c r="G34" t="n">
-        <v>3.106</v>
+        <v>3.1</v>
       </c>
       <c r="H34" t="n">
-        <v>3.207</v>
+        <v>3.208</v>
       </c>
       <c r="I34" t="n">
-        <v>3.427</v>
+        <v>3.434</v>
       </c>
       <c r="J34" t="n">
-        <v>3.612</v>
+        <v>3.632</v>
       </c>
       <c r="K34" t="n">
-        <v>3.856</v>
+        <v>3.877</v>
       </c>
       <c r="L34" t="n">
-        <v>3.899</v>
+        <v>3.916</v>
       </c>
       <c r="M34" t="n">
-        <v>4.022</v>
+        <v>4.045</v>
       </c>
       <c r="N34" t="n">
-        <v>4.036</v>
+        <v>4.069</v>
       </c>
       <c r="O34" t="n">
-        <v>4.132</v>
+        <v>4.166</v>
       </c>
       <c r="P34" t="n">
-        <v>4.319</v>
+        <v>4.349</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.178</v>
+        <v>5.205</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.025</v>
+        <v>3.022</v>
       </c>
       <c r="G35" t="n">
-        <v>3.079</v>
+        <v>3.073</v>
       </c>
       <c r="H35" t="n">
-        <v>3.175</v>
+        <v>3.176</v>
       </c>
       <c r="I35" t="n">
-        <v>3.393</v>
+        <v>3.4</v>
       </c>
       <c r="J35" t="n">
-        <v>3.58</v>
+        <v>3.601</v>
       </c>
       <c r="K35" t="n">
-        <v>3.81</v>
+        <v>3.832</v>
       </c>
       <c r="L35" t="n">
-        <v>3.854</v>
+        <v>3.871</v>
       </c>
       <c r="M35" t="n">
-        <v>3.968</v>
+        <v>3.991</v>
       </c>
       <c r="N35" t="n">
-        <v>3.972</v>
+        <v>4.006</v>
       </c>
       <c r="O35" t="n">
-        <v>4.03</v>
+        <v>4.064</v>
       </c>
       <c r="P35" t="n">
-        <v>4.121</v>
+        <v>4.152</v>
       </c>
       <c r="Q35" t="n">
-        <v>4.813</v>
+        <v>4.84</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.936</v>
+        <v>2.934</v>
       </c>
       <c r="G36" t="n">
-        <v>2.997</v>
+        <v>2.992</v>
       </c>
       <c r="H36" t="n">
-        <v>3.077</v>
+        <v>3.079</v>
       </c>
       <c r="I36" t="n">
-        <v>3.287</v>
+        <v>3.296</v>
       </c>
       <c r="J36" t="n">
-        <v>3.477</v>
+        <v>3.497</v>
       </c>
       <c r="K36" t="n">
-        <v>3.702</v>
+        <v>3.723</v>
       </c>
       <c r="L36" t="n">
-        <v>3.742</v>
+        <v>3.76</v>
       </c>
       <c r="M36" t="n">
-        <v>3.83</v>
+        <v>3.854</v>
       </c>
       <c r="N36" t="n">
-        <v>3.835</v>
+        <v>3.869</v>
       </c>
       <c r="O36" t="n">
-        <v>3.874</v>
+        <v>3.908</v>
       </c>
       <c r="P36" t="n">
-        <v>3.923</v>
+        <v>3.953</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.194</v>
+        <v>4.221</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.778</v>
+        <v>3.776</v>
       </c>
       <c r="G37" t="n">
-        <v>4.23</v>
+        <v>4.225</v>
       </c>
       <c r="H37" t="n">
-        <v>4.711</v>
+        <v>4.713</v>
       </c>
       <c r="I37" t="n">
-        <v>5.068</v>
+        <v>5.075</v>
       </c>
       <c r="J37" t="n">
-        <v>5.808</v>
+        <v>5.828</v>
       </c>
       <c r="K37" t="n">
-        <v>6.706</v>
+        <v>6.728</v>
       </c>
       <c r="L37" t="n">
-        <v>7.023</v>
+        <v>7.041</v>
       </c>
       <c r="M37" t="n">
-        <v>7.402</v>
+        <v>7.425</v>
       </c>
       <c r="N37" t="n">
-        <v>7.554</v>
+        <v>7.586</v>
       </c>
       <c r="O37" t="n">
-        <v>7.722</v>
+        <v>7.756</v>
       </c>
       <c r="P37" t="n">
-        <v>7.779</v>
+        <v>7.81</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.225</v>
+        <v>8.252000000000001</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.834</v>
+        <v>4.832</v>
       </c>
       <c r="G38" t="n">
-        <v>5.54</v>
+        <v>5.535</v>
       </c>
       <c r="H38" t="n">
-        <v>6.235</v>
+        <v>6.237</v>
       </c>
       <c r="I38" t="n">
-        <v>6.748</v>
+        <v>6.755</v>
       </c>
       <c r="J38" t="n">
-        <v>7.748</v>
+        <v>7.769</v>
       </c>
       <c r="K38" t="n">
-        <v>8.821</v>
+        <v>8.843</v>
       </c>
       <c r="L38" t="n">
-        <v>9.298999999999999</v>
+        <v>9.317</v>
       </c>
       <c r="M38" t="n">
-        <v>9.808999999999999</v>
+        <v>9.832000000000001</v>
       </c>
       <c r="N38" t="n">
-        <v>9.971</v>
+        <v>10.003</v>
       </c>
       <c r="O38" t="n">
-        <v>10.121</v>
+        <v>10.155</v>
       </c>
       <c r="P38" t="n">
-        <v>10.178</v>
+        <v>10.208</v>
       </c>
       <c r="Q38" t="n">
-        <v>10.676</v>
+        <v>10.703</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.155</v>
+        <v>4.153</v>
       </c>
       <c r="G39" t="n">
-        <v>4.738</v>
+        <v>4.733</v>
       </c>
       <c r="H39" t="n">
-        <v>5.3</v>
+        <v>5.302</v>
       </c>
       <c r="I39" t="n">
-        <v>5.752</v>
+        <v>5.759</v>
       </c>
       <c r="J39" t="n">
-        <v>6.621</v>
+        <v>6.641</v>
       </c>
       <c r="K39" t="n">
-        <v>7.655</v>
+        <v>7.677</v>
       </c>
       <c r="L39" t="n">
-        <v>8.058</v>
+        <v>8.074999999999999</v>
       </c>
       <c r="M39" t="n">
-        <v>8.446999999999999</v>
+        <v>8.470000000000001</v>
       </c>
       <c r="N39" t="n">
-        <v>8.599</v>
+        <v>8.631</v>
       </c>
       <c r="O39" t="n">
-        <v>8.771000000000001</v>
+        <v>8.805</v>
       </c>
       <c r="P39" t="n">
-        <v>8.833</v>
+        <v>8.863</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.321</v>
+        <v>9.347</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.3</v>
+        <v>3.298</v>
       </c>
       <c r="G40" t="n">
-        <v>3.414</v>
+        <v>3.409</v>
       </c>
       <c r="H40" t="n">
-        <v>3.582</v>
+        <v>3.584</v>
       </c>
       <c r="I40" t="n">
-        <v>3.843</v>
+        <v>3.85</v>
       </c>
       <c r="J40" t="n">
-        <v>4.12</v>
+        <v>4.14</v>
       </c>
       <c r="K40" t="n">
-        <v>4.441</v>
+        <v>4.463</v>
       </c>
       <c r="L40" t="n">
-        <v>4.537</v>
+        <v>4.555</v>
       </c>
       <c r="M40" t="n">
-        <v>4.741</v>
+        <v>4.764</v>
       </c>
       <c r="N40" t="n">
-        <v>4.903</v>
+        <v>4.935</v>
       </c>
       <c r="O40" t="n">
-        <v>5.188</v>
+        <v>5.222</v>
       </c>
       <c r="P40" t="n">
-        <v>5.416</v>
+        <v>5.446</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.211</v>
+        <v>6.238</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.683</v>
+        <v>3.681</v>
       </c>
       <c r="G41" t="n">
-        <v>3.838</v>
+        <v>3.833</v>
       </c>
       <c r="H41" t="n">
-        <v>4.064</v>
+        <v>4.066</v>
       </c>
       <c r="I41" t="n">
-        <v>4.345</v>
+        <v>4.352</v>
       </c>
       <c r="J41" t="n">
-        <v>4.674</v>
+        <v>4.694</v>
       </c>
       <c r="K41" t="n">
-        <v>5.041</v>
+        <v>5.063</v>
       </c>
       <c r="L41" t="n">
-        <v>5.214</v>
+        <v>5.232</v>
       </c>
       <c r="M41" t="n">
-        <v>5.542</v>
+        <v>5.565</v>
       </c>
       <c r="N41" t="n">
-        <v>5.831</v>
+        <v>5.863</v>
       </c>
       <c r="O41" t="n">
-        <v>6.299</v>
+        <v>6.333</v>
       </c>
       <c r="P41" t="n">
-        <v>6.474</v>
+        <v>6.505</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.258</v>
+        <v>7.285</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.42</v>
+        <v>3.418</v>
       </c>
       <c r="G42" t="n">
-        <v>3.562</v>
+        <v>3.557</v>
       </c>
       <c r="H42" t="n">
-        <v>3.756</v>
+        <v>3.758</v>
       </c>
       <c r="I42" t="n">
-        <v>4.032</v>
+        <v>4.039</v>
       </c>
       <c r="J42" t="n">
-        <v>4.323</v>
+        <v>4.343</v>
       </c>
       <c r="K42" t="n">
-        <v>4.662</v>
+        <v>4.684</v>
       </c>
       <c r="L42" t="n">
-        <v>4.773</v>
+        <v>4.79</v>
       </c>
       <c r="M42" t="n">
-        <v>5.048</v>
+        <v>5.071</v>
       </c>
       <c r="N42" t="n">
-        <v>5.317</v>
+        <v>5.349</v>
       </c>
       <c r="O42" t="n">
-        <v>5.678</v>
+        <v>5.712</v>
       </c>
       <c r="P42" t="n">
-        <v>5.917</v>
+        <v>5.947</v>
       </c>
       <c r="Q42" t="n">
-        <v>6.723</v>
+        <v>6.75</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.14</v>
+        <v>3.137</v>
       </c>
       <c r="G43" t="n">
-        <v>3.235</v>
+        <v>3.229</v>
       </c>
       <c r="H43" t="n">
-        <v>3.347</v>
+        <v>3.348</v>
       </c>
       <c r="I43" t="n">
-        <v>3.568</v>
+        <v>3.575</v>
       </c>
       <c r="J43" t="n">
-        <v>3.768</v>
+        <v>3.789</v>
       </c>
       <c r="K43" t="n">
-        <v>4.01</v>
+        <v>4.032</v>
       </c>
       <c r="L43" t="n">
-        <v>4.061</v>
+        <v>4.078</v>
       </c>
       <c r="M43" t="n">
-        <v>4.185</v>
+        <v>4.208</v>
       </c>
       <c r="N43" t="n">
-        <v>4.2</v>
+        <v>4.234</v>
       </c>
       <c r="O43" t="n">
-        <v>4.276</v>
+        <v>4.31</v>
       </c>
       <c r="P43" t="n">
-        <v>4.39</v>
+        <v>4.42</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.087</v>
+        <v>5.114</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46122</v>
+        <v>46125</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>3.014</v>
+        <v>3.012</v>
       </c>
       <c r="G44" t="n">
-        <v>3.107</v>
+        <v>3.102</v>
       </c>
       <c r="H44" t="n">
-        <v>3.201</v>
+        <v>3.203</v>
       </c>
       <c r="I44" t="n">
-        <v>3.415</v>
+        <v>3.424</v>
       </c>
       <c r="J44" t="n">
-        <v>3.619</v>
+        <v>3.639</v>
       </c>
       <c r="K44" t="n">
-        <v>3.852</v>
+        <v>3.874</v>
       </c>
       <c r="L44" t="n">
-        <v>3.902</v>
+        <v>3.92</v>
       </c>
       <c r="M44" t="n">
-        <v>3.999</v>
+        <v>4.023</v>
       </c>
       <c r="N44" t="n">
-        <v>4.017</v>
+        <v>4.05</v>
       </c>
       <c r="O44" t="n">
-        <v>4.073</v>
+        <v>4.107</v>
       </c>
       <c r="P44" t="n">
-        <v>4.153</v>
+        <v>4.184</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.457</v>
+        <v>4.484</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-04-14 ~ 2026-04-14
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.244</v>
+        <v>3.239</v>
       </c>
       <c r="G2" t="n">
-        <v>3.456</v>
+        <v>3.449</v>
       </c>
       <c r="H2" t="n">
-        <v>3.593</v>
+        <v>3.586</v>
       </c>
       <c r="I2" t="n">
-        <v>3.819</v>
+        <v>3.809</v>
       </c>
       <c r="J2" t="n">
-        <v>4.029</v>
+        <v>4.001</v>
       </c>
       <c r="K2" t="n">
-        <v>4.416</v>
+        <v>4.379</v>
       </c>
       <c r="L2" t="n">
-        <v>4.583</v>
+        <v>4.545</v>
       </c>
       <c r="M2" t="n">
-        <v>4.891</v>
+        <v>4.851</v>
       </c>
       <c r="N2" t="n">
-        <v>5.147</v>
+        <v>5.108</v>
       </c>
       <c r="O2" t="n">
-        <v>5.356</v>
+        <v>5.323</v>
       </c>
       <c r="P2" t="n">
-        <v>5.547</v>
+        <v>5.491</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.182</v>
+        <v>6.122</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.267</v>
+        <v>4.262</v>
       </c>
       <c r="G3" t="n">
-        <v>4.66</v>
+        <v>4.653</v>
       </c>
       <c r="H3" t="n">
-        <v>4.831</v>
+        <v>4.824</v>
       </c>
       <c r="I3" t="n">
-        <v>5.057</v>
+        <v>5.047</v>
       </c>
       <c r="J3" t="n">
-        <v>5.276</v>
+        <v>5.248</v>
       </c>
       <c r="K3" t="n">
-        <v>5.731</v>
+        <v>5.694</v>
       </c>
       <c r="L3" t="n">
-        <v>5.968</v>
+        <v>5.93</v>
       </c>
       <c r="M3" t="n">
-        <v>6.307</v>
+        <v>6.267</v>
       </c>
       <c r="N3" t="n">
-        <v>6.507</v>
+        <v>6.468</v>
       </c>
       <c r="O3" t="n">
-        <v>6.665</v>
+        <v>6.633</v>
       </c>
       <c r="P3" t="n">
-        <v>6.727</v>
+        <v>6.671</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.25</v>
+        <v>7.19</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.758</v>
+        <v>3.753</v>
       </c>
       <c r="G4" t="n">
-        <v>4.04</v>
+        <v>4.033</v>
       </c>
       <c r="H4" t="n">
-        <v>4.24</v>
+        <v>4.233</v>
       </c>
       <c r="I4" t="n">
-        <v>4.497</v>
+        <v>4.486</v>
       </c>
       <c r="J4" t="n">
-        <v>4.723</v>
+        <v>4.694</v>
       </c>
       <c r="K4" t="n">
-        <v>5.171</v>
+        <v>5.134</v>
       </c>
       <c r="L4" t="n">
-        <v>5.338</v>
+        <v>5.3</v>
       </c>
       <c r="M4" t="n">
-        <v>5.665</v>
+        <v>5.625</v>
       </c>
       <c r="N4" t="n">
-        <v>5.835</v>
+        <v>5.797</v>
       </c>
       <c r="O4" t="n">
-        <v>6.017</v>
+        <v>5.985</v>
       </c>
       <c r="P4" t="n">
-        <v>6.077</v>
+        <v>6.021</v>
       </c>
       <c r="Q4" t="n">
-        <v>6.603</v>
+        <v>6.543</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.951</v>
+        <v>2.946</v>
       </c>
       <c r="G5" t="n">
-        <v>3.004</v>
+        <v>2.997</v>
       </c>
       <c r="H5" t="n">
-        <v>3.096</v>
+        <v>3.089</v>
       </c>
       <c r="I5" t="n">
-        <v>3.394</v>
+        <v>3.383</v>
       </c>
       <c r="J5" t="n">
-        <v>3.601</v>
+        <v>3.571</v>
       </c>
       <c r="K5" t="n">
-        <v>3.846</v>
+        <v>3.806</v>
       </c>
       <c r="L5" t="n">
-        <v>3.856</v>
+        <v>3.816</v>
       </c>
       <c r="M5" t="n">
-        <v>3.969</v>
+        <v>3.927</v>
       </c>
       <c r="N5" t="n">
-        <v>3.957</v>
+        <v>3.923</v>
       </c>
       <c r="O5" t="n">
-        <v>3.957</v>
+        <v>3.925</v>
       </c>
       <c r="P5" t="n">
-        <v>4.217</v>
+        <v>4.159</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.094</v>
+        <v>5.034</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2.992</v>
+        <v>2.987</v>
       </c>
       <c r="G6" t="n">
-        <v>3.06</v>
+        <v>3.053</v>
       </c>
       <c r="H6" t="n">
-        <v>3.166</v>
+        <v>3.159</v>
       </c>
       <c r="I6" t="n">
-        <v>3.469</v>
+        <v>3.46</v>
       </c>
       <c r="J6" t="n">
-        <v>3.684</v>
+        <v>3.657</v>
       </c>
       <c r="K6" t="n">
-        <v>3.947</v>
+        <v>3.91</v>
       </c>
       <c r="L6" t="n">
-        <v>3.969</v>
+        <v>3.931</v>
       </c>
       <c r="M6" t="n">
-        <v>4.116</v>
+        <v>4.076</v>
       </c>
       <c r="N6" t="n">
-        <v>4.127</v>
+        <v>4.091</v>
       </c>
       <c r="O6" t="n">
-        <v>4.223</v>
+        <v>4.191</v>
       </c>
       <c r="P6" t="n">
-        <v>4.649</v>
+        <v>4.592</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.49</v>
+        <v>5.43</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2.972</v>
+        <v>2.967</v>
       </c>
       <c r="G7" t="n">
-        <v>3.023</v>
+        <v>3.016</v>
       </c>
       <c r="H7" t="n">
-        <v>3.112</v>
+        <v>3.105</v>
       </c>
       <c r="I7" t="n">
-        <v>3.409</v>
+        <v>3.398</v>
       </c>
       <c r="J7" t="n">
-        <v>3.626</v>
+        <v>3.596</v>
       </c>
       <c r="K7" t="n">
-        <v>3.872</v>
+        <v>3.832</v>
       </c>
       <c r="L7" t="n">
-        <v>3.881</v>
+        <v>3.841</v>
       </c>
       <c r="M7" t="n">
-        <v>4.027</v>
+        <v>3.985</v>
       </c>
       <c r="N7" t="n">
-        <v>4.017</v>
+        <v>3.983</v>
       </c>
       <c r="O7" t="n">
-        <v>4.122</v>
+        <v>4.089</v>
       </c>
       <c r="P7" t="n">
-        <v>4.433</v>
+        <v>4.375</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.258</v>
+        <v>5.198</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.377</v>
+        <v>5.372</v>
       </c>
       <c r="G8" t="n">
-        <v>5.958</v>
+        <v>5.951</v>
       </c>
       <c r="H8" t="n">
-        <v>6.28</v>
+        <v>6.274</v>
       </c>
       <c r="I8" t="n">
-        <v>6.577</v>
+        <v>6.567</v>
       </c>
       <c r="J8" t="n">
-        <v>6.861</v>
+        <v>6.832</v>
       </c>
       <c r="K8" t="n">
-        <v>7.596</v>
+        <v>7.56</v>
       </c>
       <c r="L8" t="n">
-        <v>7.923</v>
+        <v>7.885</v>
       </c>
       <c r="M8" t="n">
-        <v>8.291</v>
+        <v>8.250999999999999</v>
       </c>
       <c r="N8" t="n">
-        <v>8.428000000000001</v>
+        <v>8.388999999999999</v>
       </c>
       <c r="O8" t="n">
-        <v>8.672000000000001</v>
+        <v>8.640000000000001</v>
       </c>
       <c r="P8" t="n">
-        <v>8.834</v>
+        <v>8.779</v>
       </c>
       <c r="Q8" t="n">
-        <v>9.558999999999999</v>
+        <v>9.499000000000001</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,57 +1063,57 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.618</v>
+        <v>2.616</v>
       </c>
       <c r="G9" t="n">
-        <v>2.687</v>
+        <v>2.678</v>
       </c>
       <c r="H9" t="n">
-        <v>2.782</v>
+        <v>2.774</v>
       </c>
       <c r="I9" t="n">
-        <v>2.921</v>
+        <v>2.916</v>
       </c>
       <c r="J9" t="n">
-        <v>3.119</v>
+        <v>3.098</v>
       </c>
       <c r="K9" t="n">
-        <v>3.242</v>
+        <v>3.203</v>
       </c>
       <c r="L9" t="n">
-        <v>3.29</v>
+        <v>3.25</v>
       </c>
       <c r="M9" t="n">
-        <v>3.38</v>
+        <v>3.337</v>
       </c>
       <c r="N9" t="n">
-        <v>3.532</v>
+        <v>3.491</v>
       </c>
       <c r="O9" t="n">
-        <v>3.55</v>
+        <v>3.516</v>
       </c>
       <c r="P9" t="n">
-        <v>3.638</v>
+        <v>3.579</v>
       </c>
       <c r="Q9" t="n">
-        <v>3.712</v>
+        <v>3.652</v>
       </c>
       <c r="R9" t="n">
-        <v>3.72</v>
+        <v>3.665</v>
       </c>
       <c r="S9" t="n">
-        <v>3.677</v>
+        <v>3.63</v>
       </c>
       <c r="T9" t="n">
-        <v>3.601</v>
+        <v>3.537</v>
       </c>
       <c r="U9" t="n">
-        <v>3.475</v>
+        <v>3.41</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.63</v>
+        <v>2.628</v>
       </c>
       <c r="G10" t="n">
-        <v>2.72</v>
+        <v>2.71</v>
       </c>
       <c r="H10" t="n">
-        <v>2.792</v>
+        <v>2.786</v>
       </c>
       <c r="I10" t="n">
-        <v>2.93</v>
+        <v>2.927</v>
       </c>
       <c r="J10" t="n">
-        <v>3.146</v>
+        <v>3.123</v>
       </c>
       <c r="K10" t="n">
-        <v>3.27</v>
+        <v>3.232</v>
       </c>
       <c r="L10" t="n">
-        <v>3.332</v>
+        <v>3.293</v>
       </c>
       <c r="M10" t="n">
-        <v>3.479</v>
+        <v>3.436</v>
       </c>
       <c r="N10" t="n">
-        <v>3.54</v>
+        <v>3.501</v>
       </c>
       <c r="O10" t="n">
-        <v>3.727</v>
+        <v>3.686</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.446</v>
+        <v>2.444</v>
       </c>
       <c r="G11" t="n">
-        <v>2.53</v>
+        <v>2.52</v>
       </c>
       <c r="H11" t="n">
-        <v>2.616</v>
+        <v>2.61</v>
       </c>
       <c r="I11" t="n">
-        <v>2.732</v>
+        <v>2.729</v>
       </c>
       <c r="J11" t="n">
-        <v>2.94</v>
+        <v>2.917</v>
       </c>
       <c r="K11" t="n">
-        <v>3.057</v>
+        <v>3.019</v>
       </c>
       <c r="L11" t="n">
-        <v>3.126</v>
+        <v>3.086</v>
       </c>
       <c r="M11" t="n">
-        <v>3.284</v>
+        <v>3.24</v>
       </c>
       <c r="N11" t="n">
-        <v>3.35</v>
+        <v>3.311</v>
       </c>
       <c r="O11" t="n">
-        <v>3.494</v>
+        <v>3.452</v>
       </c>
       <c r="P11" t="n">
-        <v>3.574</v>
+        <v>3.516</v>
       </c>
       <c r="Q11" t="n">
-        <v>3.915</v>
+        <v>3.855</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.213</v>
+        <v>3.207</v>
       </c>
       <c r="G12" t="n">
-        <v>3.364</v>
+        <v>3.358</v>
       </c>
       <c r="H12" t="n">
-        <v>3.466</v>
+        <v>3.459</v>
       </c>
       <c r="I12" t="n">
-        <v>3.695</v>
+        <v>3.682</v>
       </c>
       <c r="J12" t="n">
-        <v>4.003</v>
+        <v>3.971</v>
       </c>
       <c r="K12" t="n">
-        <v>4.196</v>
+        <v>4.155</v>
       </c>
       <c r="L12" t="n">
-        <v>4.248</v>
+        <v>4.207</v>
       </c>
       <c r="M12" t="n">
-        <v>4.396</v>
+        <v>4.352</v>
       </c>
       <c r="N12" t="n">
-        <v>4.424</v>
+        <v>4.384</v>
       </c>
       <c r="O12" t="n">
-        <v>4.559</v>
+        <v>4.522</v>
       </c>
       <c r="P12" t="n">
-        <v>4.684</v>
+        <v>4.627</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.043</v>
+        <v>4.983</v>
       </c>
       <c r="R12" t="n">
-        <v>5.217</v>
+        <v>5.162</v>
       </c>
       <c r="S12" t="n">
-        <v>5.388</v>
+        <v>5.34</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2.966</v>
+        <v>2.96</v>
       </c>
       <c r="G13" t="n">
-        <v>3.054</v>
+        <v>3.048</v>
       </c>
       <c r="H13" t="n">
-        <v>3.133</v>
+        <v>3.127</v>
       </c>
       <c r="I13" t="n">
-        <v>3.343</v>
+        <v>3.329</v>
       </c>
       <c r="J13" t="n">
-        <v>3.639</v>
+        <v>3.607</v>
       </c>
       <c r="K13" t="n">
-        <v>3.829</v>
+        <v>3.788</v>
       </c>
       <c r="L13" t="n">
-        <v>3.888</v>
+        <v>3.846</v>
       </c>
       <c r="M13" t="n">
-        <v>4.023</v>
+        <v>3.979</v>
       </c>
       <c r="N13" t="n">
-        <v>4.052</v>
+        <v>4.012</v>
       </c>
       <c r="O13" t="n">
-        <v>4.185</v>
+        <v>4.151</v>
       </c>
       <c r="P13" t="n">
-        <v>4.275</v>
+        <v>4.218</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.564</v>
+        <v>4.503</v>
       </c>
       <c r="R13" t="n">
-        <v>4.765</v>
+        <v>4.71</v>
       </c>
       <c r="S13" t="n">
-        <v>4.95</v>
+        <v>4.903</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.784</v>
+        <v>2.778</v>
       </c>
       <c r="G14" t="n">
-        <v>2.861</v>
+        <v>2.855</v>
       </c>
       <c r="H14" t="n">
-        <v>2.937</v>
+        <v>2.93</v>
       </c>
       <c r="I14" t="n">
-        <v>3.126</v>
+        <v>3.112</v>
       </c>
       <c r="J14" t="n">
-        <v>3.379</v>
+        <v>3.347</v>
       </c>
       <c r="K14" t="n">
-        <v>3.517</v>
+        <v>3.476</v>
       </c>
       <c r="L14" t="n">
-        <v>3.56</v>
+        <v>3.518</v>
       </c>
       <c r="M14" t="n">
-        <v>3.708</v>
+        <v>3.664</v>
       </c>
       <c r="N14" t="n">
-        <v>3.731</v>
+        <v>3.691</v>
       </c>
       <c r="O14" t="n">
-        <v>3.84</v>
+        <v>3.806</v>
       </c>
       <c r="P14" t="n">
-        <v>3.91</v>
+        <v>3.853</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.153</v>
+        <v>4.093</v>
       </c>
       <c r="R14" t="n">
-        <v>4.28</v>
+        <v>4.225</v>
       </c>
       <c r="S14" t="n">
-        <v>4.403</v>
+        <v>4.356</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.763</v>
+        <v>2.757</v>
       </c>
       <c r="G15" t="n">
-        <v>2.835</v>
+        <v>2.829</v>
       </c>
       <c r="H15" t="n">
-        <v>2.905</v>
+        <v>2.898</v>
       </c>
       <c r="I15" t="n">
-        <v>3.077</v>
+        <v>3.063</v>
       </c>
       <c r="J15" t="n">
-        <v>3.316</v>
+        <v>3.284</v>
       </c>
       <c r="K15" t="n">
-        <v>3.47</v>
+        <v>3.429</v>
       </c>
       <c r="L15" t="n">
-        <v>3.495</v>
+        <v>3.453</v>
       </c>
       <c r="M15" t="n">
-        <v>3.621</v>
+        <v>3.577</v>
       </c>
       <c r="N15" t="n">
-        <v>3.635</v>
+        <v>3.595</v>
       </c>
       <c r="O15" t="n">
-        <v>3.765</v>
+        <v>3.73</v>
       </c>
       <c r="P15" t="n">
-        <v>3.807</v>
+        <v>3.751</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.058</v>
+        <v>3.997</v>
       </c>
       <c r="R15" t="n">
-        <v>4.176</v>
+        <v>4.122</v>
       </c>
       <c r="S15" t="n">
-        <v>4.298</v>
+        <v>4.251</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.763</v>
+        <v>2.757</v>
       </c>
       <c r="G16" t="n">
-        <v>2.835</v>
+        <v>2.829</v>
       </c>
       <c r="H16" t="n">
-        <v>2.905</v>
+        <v>2.898</v>
       </c>
       <c r="I16" t="n">
-        <v>3.077</v>
+        <v>3.063</v>
       </c>
       <c r="J16" t="n">
-        <v>3.316</v>
+        <v>3.284</v>
       </c>
       <c r="K16" t="n">
-        <v>3.47</v>
+        <v>3.429</v>
       </c>
       <c r="L16" t="n">
-        <v>3.495</v>
+        <v>3.453</v>
       </c>
       <c r="M16" t="n">
-        <v>3.621</v>
+        <v>3.577</v>
       </c>
       <c r="N16" t="n">
-        <v>3.638</v>
+        <v>3.598</v>
       </c>
       <c r="O16" t="n">
-        <v>3.772</v>
+        <v>3.737</v>
       </c>
       <c r="P16" t="n">
-        <v>3.831</v>
+        <v>3.775</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.085</v>
+        <v>4.024</v>
       </c>
       <c r="R16" t="n">
-        <v>4.204</v>
+        <v>4.15</v>
       </c>
       <c r="S16" t="n">
-        <v>4.327</v>
+        <v>4.28</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1650,34 +1650,34 @@
         <v>2.693</v>
       </c>
       <c r="G17" t="n">
-        <v>2.811</v>
+        <v>2.801</v>
       </c>
       <c r="H17" t="n">
-        <v>2.886</v>
+        <v>2.881</v>
       </c>
       <c r="I17" t="n">
-        <v>3.012</v>
+        <v>3.009</v>
       </c>
       <c r="J17" t="n">
-        <v>3.215</v>
+        <v>3.194</v>
       </c>
       <c r="K17" t="n">
-        <v>3.342</v>
+        <v>3.306</v>
       </c>
       <c r="L17" t="n">
-        <v>3.409</v>
+        <v>3.371</v>
       </c>
       <c r="M17" t="n">
-        <v>3.599</v>
+        <v>3.556</v>
       </c>
       <c r="N17" t="n">
-        <v>3.641</v>
+        <v>3.603</v>
       </c>
       <c r="O17" t="n">
-        <v>3.762</v>
+        <v>3.721</v>
       </c>
       <c r="P17" t="n">
-        <v>3.853</v>
+        <v>3.794</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1723,31 +1723,31 @@
         <v>2.694</v>
       </c>
       <c r="G18" t="n">
-        <v>2.812</v>
+        <v>2.802</v>
       </c>
       <c r="H18" t="n">
-        <v>2.886</v>
+        <v>2.881</v>
       </c>
       <c r="I18" t="n">
-        <v>3.013</v>
+        <v>3.01</v>
       </c>
       <c r="J18" t="n">
-        <v>3.215</v>
+        <v>3.194</v>
       </c>
       <c r="K18" t="n">
-        <v>3.343</v>
+        <v>3.307</v>
       </c>
       <c r="L18" t="n">
-        <v>3.409</v>
+        <v>3.371</v>
       </c>
       <c r="M18" t="n">
-        <v>3.599</v>
+        <v>3.556</v>
       </c>
       <c r="N18" t="n">
-        <v>3.641</v>
+        <v>3.603</v>
       </c>
       <c r="O18" t="n">
-        <v>3.76</v>
+        <v>3.72</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.773</v>
+        <v>2.767</v>
       </c>
       <c r="G19" t="n">
-        <v>2.851</v>
+        <v>2.845</v>
       </c>
       <c r="H19" t="n">
-        <v>2.926</v>
+        <v>2.919</v>
       </c>
       <c r="I19" t="n">
-        <v>3.11</v>
+        <v>3.097</v>
       </c>
       <c r="J19" t="n">
-        <v>3.362</v>
+        <v>3.33</v>
       </c>
       <c r="K19" t="n">
-        <v>3.513</v>
+        <v>3.472</v>
       </c>
       <c r="L19" t="n">
-        <v>3.557</v>
+        <v>3.515</v>
       </c>
       <c r="M19" t="n">
-        <v>3.697</v>
+        <v>3.654</v>
       </c>
       <c r="N19" t="n">
-        <v>3.719</v>
+        <v>3.679</v>
       </c>
       <c r="O19" t="n">
-        <v>3.819</v>
+        <v>3.784</v>
       </c>
       <c r="P19" t="n">
-        <v>3.873</v>
+        <v>3.816</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.103</v>
+        <v>4.041</v>
       </c>
       <c r="R19" t="n">
-        <v>4.229</v>
+        <v>4.174</v>
       </c>
       <c r="S19" t="n">
-        <v>4.341</v>
+        <v>4.294</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1869,25 +1869,25 @@
         <v>2.574</v>
       </c>
       <c r="G20" t="n">
-        <v>2.646</v>
+        <v>2.644</v>
       </c>
       <c r="H20" t="n">
-        <v>2.695</v>
+        <v>2.692</v>
       </c>
       <c r="I20" t="n">
-        <v>2.862</v>
+        <v>2.851</v>
       </c>
       <c r="J20" t="n">
-        <v>3.123</v>
+        <v>3.09</v>
       </c>
       <c r="K20" t="n">
-        <v>3.278</v>
+        <v>3.238</v>
       </c>
       <c r="L20" t="n">
-        <v>3.324</v>
+        <v>3.285</v>
       </c>
       <c r="M20" t="n">
-        <v>3.42</v>
+        <v>3.382</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2.874</v>
+        <v>2.871</v>
       </c>
       <c r="G21" t="n">
-        <v>2.955</v>
+        <v>2.949</v>
       </c>
       <c r="H21" t="n">
-        <v>3.068</v>
+        <v>3.061</v>
       </c>
       <c r="I21" t="n">
-        <v>3.248</v>
+        <v>3.235</v>
       </c>
       <c r="J21" t="n">
-        <v>3.492</v>
+        <v>3.46</v>
       </c>
       <c r="K21" t="n">
-        <v>3.75</v>
+        <v>3.711</v>
       </c>
       <c r="L21" t="n">
-        <v>3.817</v>
+        <v>3.776</v>
       </c>
       <c r="M21" t="n">
-        <v>3.953</v>
+        <v>3.911</v>
       </c>
       <c r="N21" t="n">
-        <v>3.985</v>
+        <v>3.945</v>
       </c>
       <c r="O21" t="n">
-        <v>4.057</v>
+        <v>4.024</v>
       </c>
       <c r="P21" t="n">
-        <v>4.137</v>
+        <v>4.08</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.264</v>
+        <v>4.204</v>
       </c>
       <c r="R21" t="n">
-        <v>4.276</v>
+        <v>4.222</v>
       </c>
       <c r="S21" t="n">
-        <v>4.301</v>
+        <v>4.255</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.822</v>
+        <v>2.819</v>
       </c>
       <c r="G22" t="n">
-        <v>2.902</v>
+        <v>2.896</v>
       </c>
       <c r="H22" t="n">
-        <v>3.002</v>
+        <v>2.996</v>
       </c>
       <c r="I22" t="n">
-        <v>3.166</v>
+        <v>3.154</v>
       </c>
       <c r="J22" t="n">
-        <v>3.376</v>
+        <v>3.343</v>
       </c>
       <c r="K22" t="n">
-        <v>3.63</v>
+        <v>3.591</v>
       </c>
       <c r="L22" t="n">
-        <v>3.686</v>
+        <v>3.645</v>
       </c>
       <c r="M22" t="n">
-        <v>3.825</v>
+        <v>3.782</v>
       </c>
       <c r="N22" t="n">
-        <v>3.858</v>
+        <v>3.818</v>
       </c>
       <c r="O22" t="n">
-        <v>3.925</v>
+        <v>3.892</v>
       </c>
       <c r="P22" t="n">
-        <v>3.999</v>
+        <v>3.942</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.122</v>
+        <v>4.062</v>
       </c>
       <c r="R22" t="n">
-        <v>4.124</v>
+        <v>4.07</v>
       </c>
       <c r="S22" t="n">
-        <v>4.146</v>
+        <v>4.1</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.775</v>
+        <v>2.771</v>
       </c>
       <c r="G23" t="n">
-        <v>2.857</v>
+        <v>2.851</v>
       </c>
       <c r="H23" t="n">
-        <v>2.941</v>
+        <v>2.934</v>
       </c>
       <c r="I23" t="n">
-        <v>3.119</v>
+        <v>3.107</v>
       </c>
       <c r="J23" t="n">
-        <v>3.322</v>
+        <v>3.289</v>
       </c>
       <c r="K23" t="n">
-        <v>3.55</v>
+        <v>3.511</v>
       </c>
       <c r="L23" t="n">
-        <v>3.597</v>
+        <v>3.556</v>
       </c>
       <c r="M23" t="n">
-        <v>3.73</v>
+        <v>3.686</v>
       </c>
       <c r="N23" t="n">
-        <v>3.754</v>
+        <v>3.714</v>
       </c>
       <c r="O23" t="n">
-        <v>3.8</v>
+        <v>3.767</v>
       </c>
       <c r="P23" t="n">
-        <v>3.861</v>
+        <v>3.803</v>
       </c>
       <c r="Q23" t="n">
-        <v>3.93</v>
+        <v>3.87</v>
       </c>
       <c r="R23" t="n">
-        <v>3.908</v>
+        <v>3.854</v>
       </c>
       <c r="S23" t="n">
-        <v>3.901</v>
+        <v>3.854</v>
       </c>
       <c r="T23" t="n">
-        <v>3.815</v>
+        <v>3.75</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.706</v>
+        <v>2.703</v>
       </c>
       <c r="G24" t="n">
-        <v>2.771</v>
+        <v>2.764</v>
       </c>
       <c r="H24" t="n">
-        <v>2.842</v>
+        <v>2.835</v>
       </c>
       <c r="I24" t="n">
-        <v>3.029</v>
+        <v>3.017</v>
       </c>
       <c r="J24" t="n">
-        <v>3.223</v>
+        <v>3.19</v>
       </c>
       <c r="K24" t="n">
-        <v>3.434</v>
+        <v>3.395</v>
       </c>
       <c r="L24" t="n">
-        <v>3.469</v>
+        <v>3.428</v>
       </c>
       <c r="M24" t="n">
+        <v>3.542</v>
+      </c>
+      <c r="N24" t="n">
         <v>3.585</v>
       </c>
-      <c r="N24" t="n">
-        <v>3.624</v>
-      </c>
       <c r="O24" t="n">
-        <v>3.751</v>
+        <v>3.715</v>
       </c>
       <c r="P24" t="n">
-        <v>3.8</v>
+        <v>3.742</v>
       </c>
       <c r="Q24" t="n">
-        <v>3.853</v>
+        <v>3.793</v>
       </c>
       <c r="R24" t="n">
-        <v>3.829</v>
+        <v>3.774</v>
       </c>
       <c r="S24" t="n">
-        <v>3.816</v>
+        <v>3.769</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.768</v>
+        <v>2.764</v>
       </c>
       <c r="G25" t="n">
-        <v>2.856</v>
+        <v>2.85</v>
       </c>
       <c r="H25" t="n">
-        <v>2.944</v>
+        <v>2.938</v>
       </c>
       <c r="I25" t="n">
-        <v>3.127</v>
+        <v>3.114</v>
       </c>
       <c r="J25" t="n">
-        <v>3.338</v>
+        <v>3.305</v>
       </c>
       <c r="K25" t="n">
-        <v>3.579</v>
+        <v>3.54</v>
       </c>
       <c r="L25" t="n">
-        <v>3.626</v>
+        <v>3.585</v>
       </c>
       <c r="M25" t="n">
-        <v>3.758</v>
+        <v>3.715</v>
       </c>
       <c r="N25" t="n">
-        <v>3.781</v>
+        <v>3.741</v>
       </c>
       <c r="O25" t="n">
-        <v>3.829</v>
+        <v>3.796</v>
       </c>
       <c r="P25" t="n">
-        <v>3.883</v>
+        <v>3.825</v>
       </c>
       <c r="Q25" t="n">
-        <v>3.963</v>
+        <v>3.903</v>
       </c>
       <c r="R25" t="n">
-        <v>3.931</v>
+        <v>3.877</v>
       </c>
       <c r="S25" t="n">
-        <v>3.924</v>
+        <v>3.877</v>
       </c>
       <c r="T25" t="n">
-        <v>3.833</v>
+        <v>3.768</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.082</v>
+        <v>3.077</v>
       </c>
       <c r="G26" t="n">
-        <v>3.209</v>
+        <v>3.204</v>
       </c>
       <c r="H26" t="n">
-        <v>3.4</v>
+        <v>3.396</v>
       </c>
       <c r="I26" t="n">
-        <v>3.66</v>
+        <v>3.648</v>
       </c>
       <c r="J26" t="n">
-        <v>3.989</v>
+        <v>3.959</v>
       </c>
       <c r="K26" t="n">
-        <v>4.368</v>
+        <v>4.328</v>
       </c>
       <c r="L26" t="n">
-        <v>4.464</v>
+        <v>4.425</v>
       </c>
       <c r="M26" t="n">
-        <v>4.664</v>
+        <v>4.622</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>4.891</v>
+        <v>4.856</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.876</v>
+        <v>2.869</v>
       </c>
       <c r="G27" t="n">
-        <v>2.942</v>
+        <v>2.936</v>
       </c>
       <c r="H27" t="n">
-        <v>3.039</v>
+        <v>3.032</v>
       </c>
       <c r="I27" t="n">
-        <v>3.242</v>
+        <v>3.23</v>
       </c>
       <c r="J27" t="n">
-        <v>3.493</v>
+        <v>3.461</v>
       </c>
       <c r="K27" t="n">
-        <v>3.688</v>
+        <v>3.648</v>
       </c>
       <c r="L27" t="n">
-        <v>3.735</v>
+        <v>3.695</v>
       </c>
       <c r="M27" t="n">
-        <v>3.875</v>
+        <v>3.832</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>3.982</v>
+        <v>3.948</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2.977</v>
+        <v>2.97</v>
       </c>
       <c r="G28" t="n">
-        <v>3.048</v>
+        <v>3.042</v>
       </c>
       <c r="H28" t="n">
-        <v>3.162</v>
+        <v>3.155</v>
       </c>
       <c r="I28" t="n">
-        <v>3.379</v>
+        <v>3.366</v>
       </c>
       <c r="J28" t="n">
-        <v>3.667</v>
+        <v>3.634</v>
       </c>
       <c r="K28" t="n">
-        <v>3.881</v>
+        <v>3.84</v>
       </c>
       <c r="L28" t="n">
-        <v>3.939</v>
+        <v>3.898</v>
       </c>
       <c r="M28" t="n">
-        <v>4.088</v>
+        <v>4.045</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.276</v>
+        <v>4.242</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.835</v>
+        <v>2.828</v>
       </c>
       <c r="G29" t="n">
-        <v>2.902</v>
+        <v>2.896</v>
       </c>
       <c r="H29" t="n">
-        <v>2.984</v>
+        <v>2.977</v>
       </c>
       <c r="I29" t="n">
-        <v>3.176</v>
+        <v>3.164</v>
       </c>
       <c r="J29" t="n">
-        <v>3.406</v>
+        <v>3.373</v>
       </c>
       <c r="K29" t="n">
-        <v>3.584</v>
+        <v>3.544</v>
       </c>
       <c r="L29" t="n">
-        <v>3.62</v>
+        <v>3.579</v>
       </c>
       <c r="M29" t="n">
-        <v>3.737</v>
+        <v>3.694</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>3.842</v>
+        <v>3.808</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.105</v>
+        <v>3.101</v>
       </c>
       <c r="G30" t="n">
-        <v>3.17</v>
+        <v>3.167</v>
       </c>
       <c r="H30" t="n">
-        <v>3.324</v>
+        <v>3.321</v>
       </c>
       <c r="I30" t="n">
-        <v>3.575</v>
+        <v>3.565</v>
       </c>
       <c r="J30" t="n">
-        <v>3.847</v>
+        <v>3.817</v>
       </c>
       <c r="K30" t="n">
-        <v>4.158</v>
+        <v>4.119</v>
       </c>
       <c r="L30" t="n">
-        <v>4.231</v>
+        <v>4.193</v>
       </c>
       <c r="M30" t="n">
-        <v>4.423</v>
+        <v>4.38</v>
       </c>
       <c r="N30" t="n">
-        <v>4.577</v>
+        <v>4.537</v>
       </c>
       <c r="O30" t="n">
-        <v>4.844</v>
+        <v>4.809</v>
       </c>
       <c r="P30" t="n">
-        <v>5.025</v>
+        <v>4.967</v>
       </c>
       <c r="Q30" t="n">
-        <v>5.787</v>
+        <v>5.727</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.431</v>
+        <v>3.427</v>
       </c>
       <c r="G31" t="n">
-        <v>3.53</v>
+        <v>3.527</v>
       </c>
       <c r="H31" t="n">
-        <v>3.736</v>
+        <v>3.733</v>
       </c>
       <c r="I31" t="n">
-        <v>4.003</v>
+        <v>3.993</v>
       </c>
       <c r="J31" t="n">
-        <v>4.338</v>
+        <v>4.307</v>
       </c>
       <c r="K31" t="n">
-        <v>4.691</v>
+        <v>4.651</v>
       </c>
       <c r="L31" t="n">
-        <v>4.842</v>
+        <v>4.803</v>
       </c>
       <c r="M31" t="n">
-        <v>5.152</v>
+        <v>5.109</v>
       </c>
       <c r="N31" t="n">
-        <v>5.433</v>
+        <v>5.394</v>
       </c>
       <c r="O31" t="n">
-        <v>5.876</v>
+        <v>5.841</v>
       </c>
       <c r="P31" t="n">
-        <v>6.012</v>
+        <v>5.954</v>
       </c>
       <c r="Q31" t="n">
-        <v>6.76</v>
+        <v>6.7</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.203</v>
+        <v>3.199</v>
       </c>
       <c r="G32" t="n">
-        <v>3.286</v>
+        <v>3.283</v>
       </c>
       <c r="H32" t="n">
-        <v>3.466</v>
+        <v>3.463</v>
       </c>
       <c r="I32" t="n">
-        <v>3.735</v>
+        <v>3.724</v>
       </c>
       <c r="J32" t="n">
-        <v>4.026</v>
+        <v>3.996</v>
       </c>
       <c r="K32" t="n">
-        <v>4.343</v>
+        <v>4.305</v>
       </c>
       <c r="L32" t="n">
-        <v>4.434</v>
+        <v>4.396</v>
       </c>
       <c r="M32" t="n">
-        <v>4.695</v>
+        <v>4.652</v>
       </c>
       <c r="N32" t="n">
-        <v>4.937</v>
+        <v>4.897</v>
       </c>
       <c r="O32" t="n">
-        <v>5.288</v>
+        <v>5.253</v>
       </c>
       <c r="P32" t="n">
-        <v>5.484</v>
+        <v>5.426</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.248</v>
+        <v>6.188</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2.989</v>
+        <v>2.983</v>
       </c>
       <c r="G33" t="n">
-        <v>3.047</v>
+        <v>3.041</v>
       </c>
       <c r="H33" t="n">
-        <v>3.149</v>
+        <v>3.145</v>
       </c>
       <c r="I33" t="n">
-        <v>3.365</v>
+        <v>3.355</v>
       </c>
       <c r="J33" t="n">
-        <v>3.561</v>
+        <v>3.529</v>
       </c>
       <c r="K33" t="n">
-        <v>3.8</v>
+        <v>3.761</v>
       </c>
       <c r="L33" t="n">
-        <v>3.837</v>
+        <v>3.799</v>
       </c>
       <c r="M33" t="n">
-        <v>3.955</v>
+        <v>3.913</v>
       </c>
       <c r="N33" t="n">
-        <v>3.965</v>
+        <v>3.926</v>
       </c>
       <c r="O33" t="n">
-        <v>3.998</v>
+        <v>3.963</v>
       </c>
       <c r="P33" t="n">
-        <v>4.055</v>
+        <v>3.997</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.504</v>
+        <v>4.444</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.048</v>
+        <v>3.042</v>
       </c>
       <c r="G34" t="n">
-        <v>3.1</v>
+        <v>3.094</v>
       </c>
       <c r="H34" t="n">
-        <v>3.208</v>
+        <v>3.204</v>
       </c>
       <c r="I34" t="n">
-        <v>3.434</v>
+        <v>3.423</v>
       </c>
       <c r="J34" t="n">
-        <v>3.632</v>
+        <v>3.601</v>
       </c>
       <c r="K34" t="n">
-        <v>3.877</v>
+        <v>3.838</v>
       </c>
       <c r="L34" t="n">
-        <v>3.916</v>
+        <v>3.878</v>
       </c>
       <c r="M34" t="n">
-        <v>4.045</v>
+        <v>4.003</v>
       </c>
       <c r="N34" t="n">
-        <v>4.069</v>
+        <v>4.03</v>
       </c>
       <c r="O34" t="n">
-        <v>4.166</v>
+        <v>4.131</v>
       </c>
       <c r="P34" t="n">
-        <v>4.349</v>
+        <v>4.291</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.205</v>
+        <v>5.145</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.022</v>
+        <v>3.016</v>
       </c>
       <c r="G35" t="n">
-        <v>3.073</v>
+        <v>3.067</v>
       </c>
       <c r="H35" t="n">
-        <v>3.176</v>
+        <v>3.172</v>
       </c>
       <c r="I35" t="n">
-        <v>3.4</v>
+        <v>3.39</v>
       </c>
       <c r="J35" t="n">
-        <v>3.601</v>
+        <v>3.569</v>
       </c>
       <c r="K35" t="n">
-        <v>3.832</v>
+        <v>3.793</v>
       </c>
       <c r="L35" t="n">
-        <v>3.871</v>
+        <v>3.833</v>
       </c>
       <c r="M35" t="n">
-        <v>3.991</v>
+        <v>3.95</v>
       </c>
       <c r="N35" t="n">
-        <v>4.006</v>
+        <v>3.967</v>
       </c>
       <c r="O35" t="n">
-        <v>4.064</v>
+        <v>4.029</v>
       </c>
       <c r="P35" t="n">
-        <v>4.152</v>
+        <v>4.094</v>
       </c>
       <c r="Q35" t="n">
-        <v>4.84</v>
+        <v>4.78</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.934</v>
+        <v>2.928</v>
       </c>
       <c r="G36" t="n">
-        <v>2.992</v>
+        <v>2.986</v>
       </c>
       <c r="H36" t="n">
-        <v>3.079</v>
+        <v>3.075</v>
       </c>
       <c r="I36" t="n">
-        <v>3.296</v>
+        <v>3.286</v>
       </c>
       <c r="J36" t="n">
-        <v>3.497</v>
+        <v>3.467</v>
       </c>
       <c r="K36" t="n">
-        <v>3.723</v>
+        <v>3.684</v>
       </c>
       <c r="L36" t="n">
-        <v>3.76</v>
+        <v>3.722</v>
       </c>
       <c r="M36" t="n">
-        <v>3.854</v>
+        <v>3.812</v>
       </c>
       <c r="N36" t="n">
-        <v>3.869</v>
+        <v>3.829</v>
       </c>
       <c r="O36" t="n">
-        <v>3.908</v>
+        <v>3.873</v>
       </c>
       <c r="P36" t="n">
-        <v>3.953</v>
+        <v>3.896</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.221</v>
+        <v>4.161</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.776</v>
+        <v>3.771</v>
       </c>
       <c r="G37" t="n">
-        <v>4.225</v>
+        <v>4.221</v>
       </c>
       <c r="H37" t="n">
-        <v>4.713</v>
+        <v>4.71</v>
       </c>
       <c r="I37" t="n">
-        <v>5.075</v>
+        <v>5.065</v>
       </c>
       <c r="J37" t="n">
-        <v>5.828</v>
+        <v>5.798</v>
       </c>
       <c r="K37" t="n">
-        <v>6.728</v>
+        <v>6.689</v>
       </c>
       <c r="L37" t="n">
-        <v>7.041</v>
+        <v>7.003</v>
       </c>
       <c r="M37" t="n">
-        <v>7.425</v>
+        <v>7.382</v>
       </c>
       <c r="N37" t="n">
-        <v>7.586</v>
+        <v>7.546</v>
       </c>
       <c r="O37" t="n">
-        <v>7.756</v>
+        <v>7.721</v>
       </c>
       <c r="P37" t="n">
-        <v>7.81</v>
+        <v>7.752</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.252000000000001</v>
+        <v>8.192</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.832</v>
+        <v>4.827</v>
       </c>
       <c r="G38" t="n">
-        <v>5.535</v>
+        <v>5.531</v>
       </c>
       <c r="H38" t="n">
-        <v>6.237</v>
+        <v>6.234</v>
       </c>
       <c r="I38" t="n">
-        <v>6.755</v>
+        <v>6.745</v>
       </c>
       <c r="J38" t="n">
-        <v>7.769</v>
+        <v>7.738</v>
       </c>
       <c r="K38" t="n">
-        <v>8.843</v>
+        <v>8.804</v>
       </c>
       <c r="L38" t="n">
-        <v>9.317</v>
+        <v>9.278</v>
       </c>
       <c r="M38" t="n">
-        <v>9.832000000000001</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="N38" t="n">
-        <v>10.003</v>
+        <v>9.964</v>
       </c>
       <c r="O38" t="n">
-        <v>10.155</v>
+        <v>10.12</v>
       </c>
       <c r="P38" t="n">
-        <v>10.208</v>
+        <v>10.15</v>
       </c>
       <c r="Q38" t="n">
-        <v>10.703</v>
+        <v>10.643</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.153</v>
+        <v>4.148</v>
       </c>
       <c r="G39" t="n">
-        <v>4.733</v>
+        <v>4.729</v>
       </c>
       <c r="H39" t="n">
-        <v>5.302</v>
+        <v>5.299</v>
       </c>
       <c r="I39" t="n">
-        <v>5.759</v>
+        <v>5.749</v>
       </c>
       <c r="J39" t="n">
-        <v>6.641</v>
+        <v>6.611</v>
       </c>
       <c r="K39" t="n">
-        <v>7.677</v>
+        <v>7.638</v>
       </c>
       <c r="L39" t="n">
-        <v>8.074999999999999</v>
+        <v>8.037000000000001</v>
       </c>
       <c r="M39" t="n">
-        <v>8.470000000000001</v>
+        <v>8.427</v>
       </c>
       <c r="N39" t="n">
-        <v>8.631</v>
+        <v>8.590999999999999</v>
       </c>
       <c r="O39" t="n">
+        <v>8.771000000000001</v>
+      </c>
+      <c r="P39" t="n">
         <v>8.805</v>
       </c>
-      <c r="P39" t="n">
-        <v>8.863</v>
-      </c>
       <c r="Q39" t="n">
-        <v>9.347</v>
+        <v>9.288</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.298</v>
+        <v>3.293</v>
       </c>
       <c r="G40" t="n">
-        <v>3.409</v>
+        <v>3.406</v>
       </c>
       <c r="H40" t="n">
-        <v>3.584</v>
+        <v>3.581</v>
       </c>
       <c r="I40" t="n">
-        <v>3.85</v>
+        <v>3.84</v>
       </c>
       <c r="J40" t="n">
-        <v>4.14</v>
+        <v>4.11</v>
       </c>
       <c r="K40" t="n">
-        <v>4.463</v>
+        <v>4.424</v>
       </c>
       <c r="L40" t="n">
-        <v>4.555</v>
+        <v>4.517</v>
       </c>
       <c r="M40" t="n">
-        <v>4.764</v>
+        <v>4.721</v>
       </c>
       <c r="N40" t="n">
-        <v>4.935</v>
+        <v>4.895</v>
       </c>
       <c r="O40" t="n">
-        <v>5.222</v>
+        <v>5.188</v>
       </c>
       <c r="P40" t="n">
-        <v>5.446</v>
+        <v>5.388</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.238</v>
+        <v>6.178</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.681</v>
+        <v>3.677</v>
       </c>
       <c r="G41" t="n">
-        <v>3.833</v>
+        <v>3.83</v>
       </c>
       <c r="H41" t="n">
-        <v>4.066</v>
+        <v>4.063</v>
       </c>
       <c r="I41" t="n">
-        <v>4.352</v>
+        <v>4.342</v>
       </c>
       <c r="J41" t="n">
-        <v>4.694</v>
+        <v>4.664</v>
       </c>
       <c r="K41" t="n">
-        <v>5.063</v>
+        <v>5.024</v>
       </c>
       <c r="L41" t="n">
-        <v>5.232</v>
+        <v>5.193</v>
       </c>
       <c r="M41" t="n">
-        <v>5.565</v>
+        <v>5.523</v>
       </c>
       <c r="N41" t="n">
-        <v>5.863</v>
+        <v>5.823</v>
       </c>
       <c r="O41" t="n">
-        <v>6.333</v>
+        <v>6.298</v>
       </c>
       <c r="P41" t="n">
-        <v>6.505</v>
+        <v>6.447</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.285</v>
+        <v>7.225</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.418</v>
+        <v>3.414</v>
       </c>
       <c r="G42" t="n">
-        <v>3.557</v>
+        <v>3.554</v>
       </c>
       <c r="H42" t="n">
-        <v>3.758</v>
+        <v>3.755</v>
       </c>
       <c r="I42" t="n">
-        <v>4.039</v>
+        <v>4.028</v>
       </c>
       <c r="J42" t="n">
-        <v>4.343</v>
+        <v>4.313</v>
       </c>
       <c r="K42" t="n">
-        <v>4.684</v>
+        <v>4.645</v>
       </c>
       <c r="L42" t="n">
-        <v>4.79</v>
+        <v>4.752</v>
       </c>
       <c r="M42" t="n">
-        <v>5.071</v>
+        <v>5.028</v>
       </c>
       <c r="N42" t="n">
-        <v>5.349</v>
+        <v>5.309</v>
       </c>
       <c r="O42" t="n">
-        <v>5.712</v>
+        <v>5.677</v>
       </c>
       <c r="P42" t="n">
-        <v>5.947</v>
+        <v>5.889</v>
       </c>
       <c r="Q42" t="n">
-        <v>6.75</v>
+        <v>6.69</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.137</v>
+        <v>3.131</v>
       </c>
       <c r="G43" t="n">
-        <v>3.229</v>
+        <v>3.223</v>
       </c>
       <c r="H43" t="n">
-        <v>3.348</v>
+        <v>3.344</v>
       </c>
       <c r="I43" t="n">
-        <v>3.575</v>
+        <v>3.565</v>
       </c>
       <c r="J43" t="n">
-        <v>3.789</v>
+        <v>3.758</v>
       </c>
       <c r="K43" t="n">
-        <v>4.032</v>
+        <v>3.993</v>
       </c>
       <c r="L43" t="n">
-        <v>4.078</v>
+        <v>4.04</v>
       </c>
       <c r="M43" t="n">
-        <v>4.208</v>
+        <v>4.166</v>
       </c>
       <c r="N43" t="n">
-        <v>4.234</v>
+        <v>4.196</v>
       </c>
       <c r="O43" t="n">
-        <v>4.31</v>
+        <v>4.275</v>
       </c>
       <c r="P43" t="n">
-        <v>4.42</v>
+        <v>4.362</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.114</v>
+        <v>5.054</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46125</v>
+        <v>46126</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>3.012</v>
+        <v>3.006</v>
       </c>
       <c r="G44" t="n">
-        <v>3.102</v>
+        <v>3.096</v>
       </c>
       <c r="H44" t="n">
-        <v>3.203</v>
+        <v>3.199</v>
       </c>
       <c r="I44" t="n">
-        <v>3.424</v>
+        <v>3.414</v>
       </c>
       <c r="J44" t="n">
-        <v>3.639</v>
+        <v>3.608</v>
       </c>
       <c r="K44" t="n">
-        <v>3.874</v>
+        <v>3.835</v>
       </c>
       <c r="L44" t="n">
-        <v>3.92</v>
+        <v>3.882</v>
       </c>
       <c r="M44" t="n">
-        <v>4.023</v>
+        <v>3.981</v>
       </c>
       <c r="N44" t="n">
-        <v>4.05</v>
+        <v>4.011</v>
       </c>
       <c r="O44" t="n">
-        <v>4.107</v>
+        <v>4.072</v>
       </c>
       <c r="P44" t="n">
-        <v>4.184</v>
+        <v>4.126</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.484</v>
+        <v>4.424</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-04-21 ~ 2026-04-21
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.219</v>
+        <v>3.218</v>
       </c>
       <c r="G2" t="n">
-        <v>3.429</v>
+        <v>3.426</v>
       </c>
       <c r="H2" t="n">
-        <v>3.579</v>
+        <v>3.582</v>
       </c>
       <c r="I2" t="n">
-        <v>3.792</v>
+        <v>3.786</v>
       </c>
       <c r="J2" t="n">
-        <v>4.011</v>
+        <v>4.005</v>
       </c>
       <c r="K2" t="n">
-        <v>4.381</v>
+        <v>4.375</v>
       </c>
       <c r="L2" t="n">
-        <v>4.559</v>
+        <v>4.549</v>
       </c>
       <c r="M2" t="n">
-        <v>4.863</v>
+        <v>4.851</v>
       </c>
       <c r="N2" t="n">
-        <v>5.125</v>
+        <v>5.108</v>
       </c>
       <c r="O2" t="n">
-        <v>5.374</v>
+        <v>5.347</v>
       </c>
       <c r="P2" t="n">
-        <v>5.531</v>
+        <v>5.504</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.155</v>
+        <v>6.126</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.242</v>
+        <v>4.241</v>
       </c>
       <c r="G3" t="n">
-        <v>4.634</v>
+        <v>4.631</v>
       </c>
       <c r="H3" t="n">
-        <v>4.817</v>
+        <v>4.82</v>
       </c>
       <c r="I3" t="n">
-        <v>5.029</v>
+        <v>5.024</v>
       </c>
       <c r="J3" t="n">
-        <v>5.258</v>
+        <v>5.252</v>
       </c>
       <c r="K3" t="n">
-        <v>5.697</v>
+        <v>5.691</v>
       </c>
       <c r="L3" t="n">
-        <v>5.945</v>
+        <v>5.934</v>
       </c>
       <c r="M3" t="n">
-        <v>6.28</v>
+        <v>6.268</v>
       </c>
       <c r="N3" t="n">
-        <v>6.486</v>
+        <v>6.468</v>
       </c>
       <c r="O3" t="n">
+        <v>6.657</v>
+      </c>
+      <c r="P3" t="n">
         <v>6.684</v>
       </c>
-      <c r="P3" t="n">
-        <v>6.711</v>
-      </c>
       <c r="Q3" t="n">
-        <v>7.223</v>
+        <v>7.195</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.734</v>
+        <v>3.732</v>
       </c>
       <c r="G4" t="n">
-        <v>4.015</v>
+        <v>4.012</v>
       </c>
       <c r="H4" t="n">
-        <v>4.227</v>
+        <v>4.229</v>
       </c>
       <c r="I4" t="n">
-        <v>4.47</v>
+        <v>4.465</v>
       </c>
       <c r="J4" t="n">
-        <v>4.704</v>
+        <v>4.698</v>
       </c>
       <c r="K4" t="n">
-        <v>5.137</v>
+        <v>5.131</v>
       </c>
       <c r="L4" t="n">
-        <v>5.314</v>
+        <v>5.304</v>
       </c>
       <c r="M4" t="n">
-        <v>5.638</v>
+        <v>5.626</v>
       </c>
       <c r="N4" t="n">
-        <v>5.814</v>
+        <v>5.796</v>
       </c>
       <c r="O4" t="n">
-        <v>6.036</v>
+        <v>6.009</v>
       </c>
       <c r="P4" t="n">
-        <v>6.061</v>
+        <v>6.034</v>
       </c>
       <c r="Q4" t="n">
-        <v>6.576</v>
+        <v>6.547</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.92</v>
+        <v>2.915</v>
       </c>
       <c r="G5" t="n">
-        <v>2.975</v>
+        <v>2.969</v>
       </c>
       <c r="H5" t="n">
-        <v>3.078</v>
+        <v>3.081</v>
       </c>
       <c r="I5" t="n">
-        <v>3.36</v>
+        <v>3.355</v>
       </c>
       <c r="J5" t="n">
-        <v>3.575</v>
+        <v>3.568</v>
       </c>
       <c r="K5" t="n">
-        <v>3.802</v>
+        <v>3.796</v>
       </c>
       <c r="L5" t="n">
-        <v>3.824</v>
+        <v>3.813</v>
       </c>
       <c r="M5" t="n">
-        <v>3.935</v>
+        <v>3.918</v>
       </c>
       <c r="N5" t="n">
-        <v>3.943</v>
+        <v>3.925</v>
       </c>
       <c r="O5" t="n">
-        <v>3.975</v>
+        <v>3.948</v>
       </c>
       <c r="P5" t="n">
-        <v>4.199</v>
+        <v>4.173</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.067</v>
+        <v>5.038</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2.959</v>
+        <v>2.954</v>
       </c>
       <c r="G6" t="n">
-        <v>3.028</v>
+        <v>3.022</v>
       </c>
       <c r="H6" t="n">
-        <v>3.149</v>
+        <v>3.151</v>
       </c>
       <c r="I6" t="n">
-        <v>3.44</v>
+        <v>3.436</v>
       </c>
       <c r="J6" t="n">
-        <v>3.663</v>
+        <v>3.656</v>
       </c>
       <c r="K6" t="n">
-        <v>3.91</v>
+        <v>3.904</v>
       </c>
       <c r="L6" t="n">
-        <v>3.942</v>
+        <v>3.931</v>
       </c>
       <c r="M6" t="n">
-        <v>4.087</v>
+        <v>4.075</v>
       </c>
       <c r="N6" t="n">
-        <v>4.11</v>
+        <v>4.092</v>
       </c>
       <c r="O6" t="n">
-        <v>4.242</v>
+        <v>4.215</v>
       </c>
       <c r="P6" t="n">
-        <v>4.632</v>
+        <v>4.605</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.463</v>
+        <v>5.434</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2.94</v>
+        <v>2.935</v>
       </c>
       <c r="G7" t="n">
-        <v>2.992</v>
+        <v>2.986</v>
       </c>
       <c r="H7" t="n">
-        <v>3.093</v>
+        <v>3.096</v>
       </c>
       <c r="I7" t="n">
-        <v>3.375</v>
+        <v>3.37</v>
       </c>
       <c r="J7" t="n">
-        <v>3.601</v>
+        <v>3.593</v>
       </c>
       <c r="K7" t="n">
-        <v>3.829</v>
+        <v>3.823</v>
       </c>
       <c r="L7" t="n">
-        <v>3.849</v>
+        <v>3.838</v>
       </c>
       <c r="M7" t="n">
-        <v>3.993</v>
+        <v>3.979</v>
       </c>
       <c r="N7" t="n">
-        <v>4.003</v>
+        <v>3.985</v>
       </c>
       <c r="O7" t="n">
-        <v>4.14</v>
+        <v>4.113</v>
       </c>
       <c r="P7" t="n">
-        <v>4.415</v>
+        <v>4.389</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.231</v>
+        <v>5.202</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.352</v>
+        <v>5.35</v>
       </c>
       <c r="G8" t="n">
-        <v>5.932</v>
+        <v>5.929</v>
       </c>
       <c r="H8" t="n">
-        <v>6.267</v>
+        <v>6.269</v>
       </c>
       <c r="I8" t="n">
-        <v>6.55</v>
+        <v>6.544</v>
       </c>
       <c r="J8" t="n">
-        <v>6.842</v>
+        <v>6.836</v>
       </c>
       <c r="K8" t="n">
-        <v>7.562</v>
+        <v>7.556</v>
       </c>
       <c r="L8" t="n">
-        <v>7.9</v>
+        <v>7.889</v>
       </c>
       <c r="M8" t="n">
-        <v>8.263</v>
+        <v>8.250999999999999</v>
       </c>
       <c r="N8" t="n">
-        <v>8.407</v>
+        <v>8.388999999999999</v>
       </c>
       <c r="O8" t="n">
-        <v>8.69</v>
+        <v>8.664</v>
       </c>
       <c r="P8" t="n">
-        <v>8.819000000000001</v>
+        <v>8.792</v>
       </c>
       <c r="Q8" t="n">
-        <v>9.532</v>
+        <v>9.503</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,57 +1063,57 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.62</v>
+        <v>2.619</v>
       </c>
       <c r="G9" t="n">
-        <v>2.679</v>
+        <v>2.677</v>
       </c>
       <c r="H9" t="n">
-        <v>2.764</v>
+        <v>2.767</v>
       </c>
       <c r="I9" t="n">
         <v>2.925</v>
       </c>
       <c r="J9" t="n">
-        <v>3.113</v>
+        <v>3.107</v>
       </c>
       <c r="K9" t="n">
-        <v>3.215</v>
+        <v>3.206</v>
       </c>
       <c r="L9" t="n">
-        <v>3.259</v>
+        <v>3.25</v>
       </c>
       <c r="M9" t="n">
-        <v>3.347</v>
+        <v>3.335</v>
       </c>
       <c r="N9" t="n">
-        <v>3.509</v>
+        <v>3.492</v>
       </c>
       <c r="O9" t="n">
-        <v>3.567</v>
+        <v>3.54</v>
       </c>
       <c r="P9" t="n">
+        <v>3.593</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>3.656</v>
+      </c>
+      <c r="R9" t="n">
+        <v>3.657</v>
+      </c>
+      <c r="S9" t="n">
         <v>3.62</v>
       </c>
-      <c r="Q9" t="n">
-        <v>3.685</v>
-      </c>
-      <c r="R9" t="n">
-        <v>3.687</v>
-      </c>
-      <c r="S9" t="n">
-        <v>3.65</v>
-      </c>
       <c r="T9" t="n">
-        <v>3.567</v>
+        <v>3.535</v>
       </c>
       <c r="U9" t="n">
-        <v>3.44</v>
+        <v>3.406</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1139,28 +1139,28 @@
         <v>2.633</v>
       </c>
       <c r="G10" t="n">
-        <v>2.717</v>
+        <v>2.715</v>
       </c>
       <c r="H10" t="n">
-        <v>2.779</v>
+        <v>2.782</v>
       </c>
       <c r="I10" t="n">
         <v>2.938</v>
       </c>
       <c r="J10" t="n">
-        <v>3.139</v>
+        <v>3.133</v>
       </c>
       <c r="K10" t="n">
-        <v>3.247</v>
+        <v>3.238</v>
       </c>
       <c r="L10" t="n">
-        <v>3.306</v>
+        <v>3.297</v>
       </c>
       <c r="M10" t="n">
-        <v>3.445</v>
+        <v>3.433</v>
       </c>
       <c r="N10" t="n">
-        <v>3.522</v>
+        <v>3.505</v>
       </c>
       <c r="O10" t="n">
         <v>3.732</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1212,37 +1212,37 @@
         <v>2.448</v>
       </c>
       <c r="G11" t="n">
-        <v>2.527</v>
+        <v>2.525</v>
       </c>
       <c r="H11" t="n">
-        <v>2.604</v>
+        <v>2.606</v>
       </c>
       <c r="I11" t="n">
         <v>2.741</v>
       </c>
       <c r="J11" t="n">
-        <v>2.934</v>
+        <v>2.928</v>
       </c>
       <c r="K11" t="n">
-        <v>3.034</v>
+        <v>3.025</v>
       </c>
       <c r="L11" t="n">
-        <v>3.1</v>
+        <v>3.091</v>
       </c>
       <c r="M11" t="n">
-        <v>3.25</v>
+        <v>3.238</v>
       </c>
       <c r="N11" t="n">
-        <v>3.331</v>
+        <v>3.314</v>
       </c>
       <c r="O11" t="n">
         <v>3.499</v>
       </c>
       <c r="P11" t="n">
-        <v>3.56</v>
+        <v>3.535</v>
       </c>
       <c r="Q11" t="n">
-        <v>3.888</v>
+        <v>3.859</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.198</v>
+        <v>3.195</v>
       </c>
       <c r="G12" t="n">
-        <v>3.351</v>
+        <v>3.347</v>
       </c>
       <c r="H12" t="n">
-        <v>3.457</v>
+        <v>3.458</v>
       </c>
       <c r="I12" t="n">
-        <v>3.673</v>
+        <v>3.67</v>
       </c>
       <c r="J12" t="n">
-        <v>3.977</v>
+        <v>3.973</v>
       </c>
       <c r="K12" t="n">
-        <v>4.152</v>
+        <v>4.145</v>
       </c>
       <c r="L12" t="n">
-        <v>4.215</v>
+        <v>4.204</v>
       </c>
       <c r="M12" t="n">
-        <v>4.362</v>
+        <v>4.347</v>
       </c>
       <c r="N12" t="n">
-        <v>4.403</v>
+        <v>4.385</v>
       </c>
       <c r="O12" t="n">
-        <v>4.571</v>
+        <v>4.544</v>
       </c>
       <c r="P12" t="n">
-        <v>4.667</v>
+        <v>4.64</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.015</v>
+        <v>4.986</v>
       </c>
       <c r="R12" t="n">
-        <v>5.186</v>
+        <v>5.156</v>
       </c>
       <c r="S12" t="n">
-        <v>5.361</v>
+        <v>5.331</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2.951</v>
+        <v>2.949</v>
       </c>
       <c r="G13" t="n">
-        <v>3.041</v>
+        <v>3.038</v>
       </c>
       <c r="H13" t="n">
         <v>3.125</v>
       </c>
       <c r="I13" t="n">
-        <v>3.321</v>
+        <v>3.318</v>
       </c>
       <c r="J13" t="n">
-        <v>3.614</v>
+        <v>3.61</v>
       </c>
       <c r="K13" t="n">
-        <v>3.786</v>
+        <v>3.778</v>
       </c>
       <c r="L13" t="n">
-        <v>3.855</v>
+        <v>3.843</v>
       </c>
       <c r="M13" t="n">
-        <v>3.989</v>
+        <v>3.975</v>
       </c>
       <c r="N13" t="n">
-        <v>4.031</v>
+        <v>4.013</v>
       </c>
       <c r="O13" t="n">
-        <v>4.2</v>
+        <v>4.172</v>
       </c>
       <c r="P13" t="n">
-        <v>4.258</v>
+        <v>4.231</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.536</v>
+        <v>4.507</v>
       </c>
       <c r="R13" t="n">
-        <v>4.734</v>
+        <v>4.704</v>
       </c>
       <c r="S13" t="n">
-        <v>4.923</v>
+        <v>4.893</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.77</v>
+        <v>2.767</v>
       </c>
       <c r="G14" t="n">
-        <v>2.847</v>
+        <v>2.843</v>
       </c>
       <c r="H14" t="n">
-        <v>2.928</v>
+        <v>2.929</v>
       </c>
       <c r="I14" t="n">
-        <v>3.104</v>
+        <v>3.102</v>
       </c>
       <c r="J14" t="n">
-        <v>3.354</v>
+        <v>3.35</v>
       </c>
       <c r="K14" t="n">
-        <v>3.474</v>
+        <v>3.466</v>
       </c>
       <c r="L14" t="n">
-        <v>3.527</v>
+        <v>3.515</v>
       </c>
       <c r="M14" t="n">
-        <v>3.674</v>
+        <v>3.66</v>
       </c>
       <c r="N14" t="n">
-        <v>3.711</v>
+        <v>3.693</v>
       </c>
       <c r="O14" t="n">
-        <v>3.855</v>
+        <v>3.827</v>
       </c>
       <c r="P14" t="n">
-        <v>3.893</v>
+        <v>3.866</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.125</v>
+        <v>4.096</v>
       </c>
       <c r="R14" t="n">
-        <v>4.249</v>
+        <v>4.219</v>
       </c>
       <c r="S14" t="n">
-        <v>4.375</v>
+        <v>4.346</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.749</v>
+        <v>2.746</v>
       </c>
       <c r="G15" t="n">
-        <v>2.821</v>
+        <v>2.817</v>
       </c>
       <c r="H15" t="n">
         <v>2.897</v>
       </c>
       <c r="I15" t="n">
-        <v>3.057</v>
+        <v>3.054</v>
       </c>
       <c r="J15" t="n">
-        <v>3.293</v>
+        <v>3.289</v>
       </c>
       <c r="K15" t="n">
-        <v>3.426</v>
+        <v>3.419</v>
       </c>
       <c r="L15" t="n">
-        <v>3.462</v>
+        <v>3.451</v>
       </c>
       <c r="M15" t="n">
-        <v>3.588</v>
+        <v>3.573</v>
       </c>
       <c r="N15" t="n">
-        <v>3.614</v>
+        <v>3.596</v>
       </c>
       <c r="O15" t="n">
-        <v>3.78</v>
+        <v>3.753</v>
       </c>
       <c r="P15" t="n">
-        <v>3.792</v>
+        <v>3.765</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.029</v>
+        <v>4.001</v>
       </c>
       <c r="R15" t="n">
-        <v>4.145</v>
+        <v>4.115</v>
       </c>
       <c r="S15" t="n">
-        <v>4.271</v>
+        <v>4.241</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.749</v>
+        <v>2.746</v>
       </c>
       <c r="G16" t="n">
-        <v>2.821</v>
+        <v>2.817</v>
       </c>
       <c r="H16" t="n">
         <v>2.897</v>
       </c>
       <c r="I16" t="n">
-        <v>3.057</v>
+        <v>3.054</v>
       </c>
       <c r="J16" t="n">
-        <v>3.293</v>
+        <v>3.289</v>
       </c>
       <c r="K16" t="n">
-        <v>3.426</v>
+        <v>3.419</v>
       </c>
       <c r="L16" t="n">
-        <v>3.462</v>
+        <v>3.451</v>
       </c>
       <c r="M16" t="n">
-        <v>3.588</v>
+        <v>3.573</v>
       </c>
       <c r="N16" t="n">
-        <v>3.617</v>
+        <v>3.599</v>
       </c>
       <c r="O16" t="n">
-        <v>3.787</v>
+        <v>3.76</v>
       </c>
       <c r="P16" t="n">
-        <v>3.815</v>
+        <v>3.789</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.057</v>
+        <v>4.028</v>
       </c>
       <c r="R16" t="n">
-        <v>4.173</v>
+        <v>4.143</v>
       </c>
       <c r="S16" t="n">
-        <v>4.3</v>
+        <v>4.27</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.698</v>
+        <v>2.697</v>
       </c>
       <c r="G17" t="n">
-        <v>2.807</v>
+        <v>2.805</v>
       </c>
       <c r="H17" t="n">
-        <v>2.874</v>
+        <v>2.876</v>
       </c>
       <c r="I17" t="n">
         <v>3.02</v>
       </c>
       <c r="J17" t="n">
-        <v>3.21</v>
+        <v>3.204</v>
       </c>
       <c r="K17" t="n">
-        <v>3.322</v>
+        <v>3.314</v>
       </c>
       <c r="L17" t="n">
-        <v>3.385</v>
+        <v>3.376</v>
       </c>
       <c r="M17" t="n">
-        <v>3.563</v>
+        <v>3.551</v>
       </c>
       <c r="N17" t="n">
-        <v>3.624</v>
+        <v>3.606</v>
       </c>
       <c r="O17" t="n">
-        <v>3.767</v>
+        <v>3.763</v>
       </c>
       <c r="P17" t="n">
-        <v>3.832</v>
+        <v>3.807</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.699</v>
+        <v>2.698</v>
       </c>
       <c r="G18" t="n">
-        <v>2.808</v>
+        <v>2.806</v>
       </c>
       <c r="H18" t="n">
-        <v>2.874</v>
+        <v>2.876</v>
       </c>
       <c r="I18" t="n">
         <v>3.02</v>
       </c>
       <c r="J18" t="n">
-        <v>3.21</v>
+        <v>3.204</v>
       </c>
       <c r="K18" t="n">
-        <v>3.323</v>
+        <v>3.314</v>
       </c>
       <c r="L18" t="n">
-        <v>3.385</v>
+        <v>3.376</v>
       </c>
       <c r="M18" t="n">
-        <v>3.563</v>
+        <v>3.551</v>
       </c>
       <c r="N18" t="n">
-        <v>3.624</v>
+        <v>3.607</v>
       </c>
       <c r="O18" t="n">
-        <v>3.765</v>
+        <v>3.761</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.761</v>
+        <v>2.759</v>
       </c>
       <c r="G19" t="n">
-        <v>2.838</v>
+        <v>2.834</v>
       </c>
       <c r="H19" t="n">
         <v>2.918</v>
       </c>
       <c r="I19" t="n">
-        <v>3.091</v>
+        <v>3.088</v>
       </c>
       <c r="J19" t="n">
-        <v>3.338</v>
+        <v>3.334</v>
       </c>
       <c r="K19" t="n">
-        <v>3.47</v>
+        <v>3.462</v>
       </c>
       <c r="L19" t="n">
-        <v>3.524</v>
+        <v>3.512</v>
       </c>
       <c r="M19" t="n">
-        <v>3.665</v>
+        <v>3.651</v>
       </c>
       <c r="N19" t="n">
-        <v>3.698</v>
+        <v>3.68</v>
       </c>
       <c r="O19" t="n">
-        <v>3.834</v>
+        <v>3.806</v>
       </c>
       <c r="P19" t="n">
-        <v>3.854</v>
+        <v>3.828</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.072</v>
+        <v>4.043</v>
       </c>
       <c r="R19" t="n">
-        <v>4.195</v>
+        <v>4.165</v>
       </c>
       <c r="S19" t="n">
-        <v>4.314</v>
+        <v>4.284</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1869,25 +1869,25 @@
         <v>2.573</v>
       </c>
       <c r="G20" t="n">
-        <v>2.644</v>
+        <v>2.643</v>
       </c>
       <c r="H20" t="n">
-        <v>2.691</v>
+        <v>2.69</v>
       </c>
       <c r="I20" t="n">
-        <v>2.84</v>
+        <v>2.832</v>
       </c>
       <c r="J20" t="n">
-        <v>3.103</v>
+        <v>3.099</v>
       </c>
       <c r="K20" t="n">
-        <v>3.242</v>
+        <v>3.237</v>
       </c>
       <c r="L20" t="n">
-        <v>3.291</v>
+        <v>3.28</v>
       </c>
       <c r="M20" t="n">
-        <v>3.394</v>
+        <v>3.381</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2.869</v>
+        <v>2.867</v>
       </c>
       <c r="G21" t="n">
-        <v>2.947</v>
+        <v>2.946</v>
       </c>
       <c r="H21" t="n">
-        <v>3.061</v>
+        <v>3.06</v>
       </c>
       <c r="I21" t="n">
-        <v>3.225</v>
+        <v>3.22</v>
       </c>
       <c r="J21" t="n">
-        <v>3.47</v>
+        <v>3.464</v>
       </c>
       <c r="K21" t="n">
-        <v>3.712</v>
+        <v>3.705</v>
       </c>
       <c r="L21" t="n">
-        <v>3.775</v>
+        <v>3.761</v>
       </c>
       <c r="M21" t="n">
-        <v>3.913</v>
+        <v>3.898</v>
       </c>
       <c r="N21" t="n">
-        <v>3.96</v>
+        <v>3.943</v>
       </c>
       <c r="O21" t="n">
-        <v>4.064</v>
+        <v>4.036</v>
       </c>
       <c r="P21" t="n">
-        <v>4.119</v>
+        <v>4.092</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.237</v>
+        <v>4.208</v>
       </c>
       <c r="R21" t="n">
+        <v>4.215</v>
+      </c>
+      <c r="S21" t="n">
         <v>4.245</v>
-      </c>
-      <c r="S21" t="n">
-        <v>4.275</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.817</v>
+        <v>2.814</v>
       </c>
       <c r="G22" t="n">
-        <v>2.894</v>
+        <v>2.892</v>
       </c>
       <c r="H22" t="n">
-        <v>2.993</v>
+        <v>2.992</v>
       </c>
       <c r="I22" t="n">
-        <v>3.145</v>
+        <v>3.14</v>
       </c>
       <c r="J22" t="n">
-        <v>3.353</v>
+        <v>3.348</v>
       </c>
       <c r="K22" t="n">
-        <v>3.592</v>
+        <v>3.584</v>
       </c>
       <c r="L22" t="n">
-        <v>3.643</v>
+        <v>3.63</v>
       </c>
       <c r="M22" t="n">
-        <v>3.783</v>
+        <v>3.768</v>
       </c>
       <c r="N22" t="n">
-        <v>3.833</v>
+        <v>3.815</v>
       </c>
       <c r="O22" t="n">
-        <v>3.932</v>
+        <v>3.904</v>
       </c>
       <c r="P22" t="n">
-        <v>3.981</v>
+        <v>3.954</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.095</v>
+        <v>4.067</v>
       </c>
       <c r="R22" t="n">
-        <v>4.093</v>
+        <v>4.063</v>
       </c>
       <c r="S22" t="n">
-        <v>4.12</v>
+        <v>4.09</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.769</v>
+        <v>2.766</v>
       </c>
       <c r="G23" t="n">
-        <v>2.849</v>
+        <v>2.847</v>
       </c>
       <c r="H23" t="n">
-        <v>2.933</v>
+        <v>2.932</v>
       </c>
       <c r="I23" t="n">
-        <v>3.098</v>
+        <v>3.093</v>
       </c>
       <c r="J23" t="n">
-        <v>3.299</v>
+        <v>3.294</v>
       </c>
       <c r="K23" t="n">
-        <v>3.511</v>
+        <v>3.503</v>
       </c>
       <c r="L23" t="n">
-        <v>3.554</v>
+        <v>3.541</v>
       </c>
       <c r="M23" t="n">
-        <v>3.687</v>
+        <v>3.672</v>
       </c>
       <c r="N23" t="n">
-        <v>3.729</v>
+        <v>3.712</v>
       </c>
       <c r="O23" t="n">
-        <v>3.806</v>
+        <v>3.779</v>
       </c>
       <c r="P23" t="n">
-        <v>3.842</v>
+        <v>3.816</v>
       </c>
       <c r="Q23" t="n">
-        <v>3.903</v>
+        <v>3.874</v>
       </c>
       <c r="R23" t="n">
-        <v>3.877</v>
+        <v>3.847</v>
       </c>
       <c r="S23" t="n">
-        <v>3.875</v>
+        <v>3.845</v>
       </c>
       <c r="T23" t="n">
-        <v>3.782</v>
+        <v>3.75</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.703</v>
+        <v>2.701</v>
       </c>
       <c r="G24" t="n">
-        <v>2.763</v>
+        <v>2.761</v>
       </c>
       <c r="H24" t="n">
-        <v>2.834</v>
+        <v>2.833</v>
       </c>
       <c r="I24" t="n">
-        <v>3.008</v>
+        <v>3.003</v>
       </c>
       <c r="J24" t="n">
-        <v>3.198</v>
+        <v>3.193</v>
       </c>
       <c r="K24" t="n">
-        <v>3.395</v>
+        <v>3.386</v>
       </c>
       <c r="L24" t="n">
-        <v>3.426</v>
+        <v>3.413</v>
       </c>
       <c r="M24" t="n">
-        <v>3.545</v>
+        <v>3.53</v>
       </c>
       <c r="N24" t="n">
-        <v>3.599</v>
+        <v>3.582</v>
       </c>
       <c r="O24" t="n">
-        <v>3.757</v>
+        <v>3.731</v>
       </c>
       <c r="P24" t="n">
-        <v>3.781</v>
+        <v>3.755</v>
       </c>
       <c r="Q24" t="n">
-        <v>3.825</v>
+        <v>3.796</v>
       </c>
       <c r="R24" t="n">
-        <v>3.798</v>
+        <v>3.768</v>
       </c>
       <c r="S24" t="n">
-        <v>3.79</v>
+        <v>3.76</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.763</v>
+        <v>2.76</v>
       </c>
       <c r="G25" t="n">
-        <v>2.848</v>
+        <v>2.846</v>
       </c>
       <c r="H25" t="n">
-        <v>2.936</v>
+        <v>2.935</v>
       </c>
       <c r="I25" t="n">
-        <v>3.106</v>
+        <v>3.101</v>
       </c>
       <c r="J25" t="n">
-        <v>3.315</v>
+        <v>3.309</v>
       </c>
       <c r="K25" t="n">
-        <v>3.541</v>
+        <v>3.533</v>
       </c>
       <c r="L25" t="n">
-        <v>3.583</v>
+        <v>3.57</v>
       </c>
       <c r="M25" t="n">
-        <v>3.717</v>
+        <v>3.702</v>
       </c>
       <c r="N25" t="n">
-        <v>3.756</v>
+        <v>3.739</v>
       </c>
       <c r="O25" t="n">
-        <v>3.835</v>
+        <v>3.808</v>
       </c>
       <c r="P25" t="n">
-        <v>3.864</v>
+        <v>3.838</v>
       </c>
       <c r="Q25" t="n">
-        <v>3.936</v>
+        <v>3.907</v>
       </c>
       <c r="R25" t="n">
-        <v>3.9</v>
+        <v>3.87</v>
       </c>
       <c r="S25" t="n">
-        <v>3.898</v>
+        <v>3.868</v>
       </c>
       <c r="T25" t="n">
-        <v>3.8</v>
+        <v>3.768</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.067</v>
+        <v>3.066</v>
       </c>
       <c r="G26" t="n">
-        <v>3.199</v>
+        <v>3.198</v>
       </c>
       <c r="H26" t="n">
-        <v>3.397</v>
+        <v>3.399</v>
       </c>
       <c r="I26" t="n">
-        <v>3.636</v>
+        <v>3.631</v>
       </c>
       <c r="J26" t="n">
-        <v>3.974</v>
+        <v>3.969</v>
       </c>
       <c r="K26" t="n">
-        <v>4.332</v>
+        <v>4.327</v>
       </c>
       <c r="L26" t="n">
-        <v>4.438</v>
+        <v>4.428</v>
       </c>
       <c r="M26" t="n">
-        <v>4.631</v>
+        <v>4.618</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>4.907</v>
+        <v>4.88</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.86</v>
+        <v>2.859</v>
       </c>
       <c r="G27" t="n">
-        <v>2.929</v>
+        <v>2.926</v>
       </c>
       <c r="H27" t="n">
-        <v>3.032</v>
+        <v>3.033</v>
       </c>
       <c r="I27" t="n">
-        <v>3.219</v>
+        <v>3.215</v>
       </c>
       <c r="J27" t="n">
-        <v>3.473</v>
+        <v>3.468</v>
       </c>
       <c r="K27" t="n">
-        <v>3.647</v>
+        <v>3.642</v>
       </c>
       <c r="L27" t="n">
-        <v>3.706</v>
+        <v>3.695</v>
       </c>
       <c r="M27" t="n">
-        <v>3.841</v>
+        <v>3.828</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>3.997</v>
+        <v>3.969</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2.964</v>
+        <v>2.962</v>
       </c>
       <c r="G28" t="n">
-        <v>3.039</v>
+        <v>3.036</v>
       </c>
       <c r="H28" t="n">
-        <v>3.156</v>
+        <v>3.157</v>
       </c>
       <c r="I28" t="n">
-        <v>3.357</v>
+        <v>3.353</v>
       </c>
       <c r="J28" t="n">
-        <v>3.646</v>
+        <v>3.641</v>
       </c>
       <c r="K28" t="n">
-        <v>3.84</v>
+        <v>3.834</v>
       </c>
       <c r="L28" t="n">
-        <v>3.909</v>
+        <v>3.899</v>
       </c>
       <c r="M28" t="n">
-        <v>4.053</v>
+        <v>4.04</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.291</v>
+        <v>4.263</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.819</v>
+        <v>2.817</v>
       </c>
       <c r="G29" t="n">
-        <v>2.886</v>
+        <v>2.884</v>
       </c>
       <c r="H29" t="n">
-        <v>2.975</v>
+        <v>2.976</v>
       </c>
       <c r="I29" t="n">
-        <v>3.153</v>
+        <v>3.149</v>
       </c>
       <c r="J29" t="n">
-        <v>3.385</v>
+        <v>3.381</v>
       </c>
       <c r="K29" t="n">
-        <v>3.543</v>
+        <v>3.538</v>
       </c>
       <c r="L29" t="n">
-        <v>3.59</v>
+        <v>3.58</v>
       </c>
       <c r="M29" t="n">
-        <v>3.703</v>
+        <v>3.69</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>3.857</v>
+        <v>3.83</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2602,34 +2602,34 @@
         <v>3.166</v>
       </c>
       <c r="H30" t="n">
-        <v>3.328</v>
+        <v>3.329</v>
       </c>
       <c r="I30" t="n">
-        <v>3.561</v>
+        <v>3.553</v>
       </c>
       <c r="J30" t="n">
-        <v>3.835</v>
+        <v>3.831</v>
       </c>
       <c r="K30" t="n">
-        <v>4.123</v>
+        <v>4.118</v>
       </c>
       <c r="L30" t="n">
-        <v>4.206</v>
+        <v>4.196</v>
       </c>
       <c r="M30" t="n">
-        <v>4.39</v>
+        <v>4.377</v>
       </c>
       <c r="N30" t="n">
-        <v>4.555</v>
+        <v>4.537</v>
       </c>
       <c r="O30" t="n">
-        <v>4.858</v>
+        <v>4.831</v>
       </c>
       <c r="P30" t="n">
-        <v>5.008</v>
+        <v>4.981</v>
       </c>
       <c r="Q30" t="n">
-        <v>5.759</v>
+        <v>5.73</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2675,34 +2675,34 @@
         <v>3.526</v>
       </c>
       <c r="H31" t="n">
-        <v>3.74</v>
+        <v>3.742</v>
       </c>
       <c r="I31" t="n">
-        <v>3.988</v>
+        <v>3.981</v>
       </c>
       <c r="J31" t="n">
-        <v>4.325</v>
+        <v>4.321</v>
       </c>
       <c r="K31" t="n">
-        <v>4.655</v>
+        <v>4.65</v>
       </c>
       <c r="L31" t="n">
-        <v>4.818</v>
+        <v>4.808</v>
       </c>
       <c r="M31" t="n">
-        <v>5.119</v>
+        <v>5.107</v>
       </c>
       <c r="N31" t="n">
-        <v>5.412</v>
+        <v>5.394</v>
       </c>
       <c r="O31" t="n">
-        <v>5.89</v>
+        <v>5.863</v>
       </c>
       <c r="P31" t="n">
-        <v>5.995</v>
+        <v>5.968</v>
       </c>
       <c r="Q31" t="n">
-        <v>6.733</v>
+        <v>6.704</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2748,34 +2748,34 @@
         <v>3.282</v>
       </c>
       <c r="H32" t="n">
-        <v>3.471</v>
+        <v>3.472</v>
       </c>
       <c r="I32" t="n">
-        <v>3.72</v>
+        <v>3.712</v>
       </c>
       <c r="J32" t="n">
-        <v>4.014</v>
+        <v>4.01</v>
       </c>
       <c r="K32" t="n">
-        <v>4.308</v>
+        <v>4.303</v>
       </c>
       <c r="L32" t="n">
-        <v>4.41</v>
+        <v>4.4</v>
       </c>
       <c r="M32" t="n">
-        <v>4.662</v>
+        <v>4.65</v>
       </c>
       <c r="N32" t="n">
-        <v>4.916</v>
+        <v>4.898</v>
       </c>
       <c r="O32" t="n">
-        <v>5.302</v>
+        <v>5.275</v>
       </c>
       <c r="P32" t="n">
-        <v>5.467</v>
+        <v>5.44</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.22</v>
+        <v>6.192</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2821,34 +2821,34 @@
         <v>3.036</v>
       </c>
       <c r="H33" t="n">
-        <v>3.15</v>
+        <v>3.152</v>
       </c>
       <c r="I33" t="n">
-        <v>3.347</v>
+        <v>3.34</v>
       </c>
       <c r="J33" t="n">
-        <v>3.549</v>
+        <v>3.545</v>
       </c>
       <c r="K33" t="n">
-        <v>3.766</v>
+        <v>3.761</v>
       </c>
       <c r="L33" t="n">
-        <v>3.812</v>
+        <v>3.802</v>
       </c>
       <c r="M33" t="n">
-        <v>3.923</v>
+        <v>3.911</v>
       </c>
       <c r="N33" t="n">
-        <v>3.946</v>
+        <v>3.928</v>
       </c>
       <c r="O33" t="n">
-        <v>4.012</v>
+        <v>3.985</v>
       </c>
       <c r="P33" t="n">
-        <v>4.039</v>
+        <v>4.013</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.476</v>
+        <v>4.447</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2894,34 +2894,34 @@
         <v>3.089</v>
       </c>
       <c r="H34" t="n">
-        <v>3.21</v>
+        <v>3.211</v>
       </c>
       <c r="I34" t="n">
-        <v>3.415</v>
+        <v>3.409</v>
       </c>
       <c r="J34" t="n">
-        <v>3.621</v>
+        <v>3.617</v>
       </c>
       <c r="K34" t="n">
-        <v>3.843</v>
+        <v>3.838</v>
       </c>
       <c r="L34" t="n">
-        <v>3.891</v>
+        <v>3.881</v>
       </c>
       <c r="M34" t="n">
-        <v>4.014</v>
+        <v>4.001</v>
       </c>
       <c r="N34" t="n">
-        <v>4.05</v>
+        <v>4.032</v>
       </c>
       <c r="O34" t="n">
-        <v>4.18</v>
+        <v>4.153</v>
       </c>
       <c r="P34" t="n">
-        <v>4.334</v>
+        <v>4.307</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.177</v>
+        <v>5.148</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2967,34 +2967,34 @@
         <v>3.062</v>
       </c>
       <c r="H35" t="n">
-        <v>3.177</v>
+        <v>3.179</v>
       </c>
       <c r="I35" t="n">
-        <v>3.382</v>
+        <v>3.375</v>
       </c>
       <c r="J35" t="n">
-        <v>3.589</v>
+        <v>3.585</v>
       </c>
       <c r="K35" t="n">
-        <v>3.797</v>
+        <v>3.793</v>
       </c>
       <c r="L35" t="n">
-        <v>3.846</v>
+        <v>3.836</v>
       </c>
       <c r="M35" t="n">
-        <v>3.961</v>
+        <v>3.948</v>
       </c>
       <c r="N35" t="n">
-        <v>3.987</v>
+        <v>3.969</v>
       </c>
       <c r="O35" t="n">
-        <v>4.078</v>
+        <v>4.051</v>
       </c>
       <c r="P35" t="n">
-        <v>4.136</v>
+        <v>4.11</v>
       </c>
       <c r="Q35" t="n">
-        <v>4.813</v>
+        <v>4.784</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3040,34 +3040,34 @@
         <v>2.978</v>
       </c>
       <c r="H36" t="n">
-        <v>3.076</v>
+        <v>3.078</v>
       </c>
       <c r="I36" t="n">
-        <v>3.275</v>
+        <v>3.268</v>
       </c>
       <c r="J36" t="n">
-        <v>3.485</v>
+        <v>3.481</v>
       </c>
       <c r="K36" t="n">
-        <v>3.689</v>
+        <v>3.685</v>
       </c>
       <c r="L36" t="n">
-        <v>3.735</v>
+        <v>3.726</v>
       </c>
       <c r="M36" t="n">
-        <v>3.821</v>
+        <v>3.81</v>
       </c>
       <c r="N36" t="n">
-        <v>3.848</v>
+        <v>3.831</v>
       </c>
       <c r="O36" t="n">
-        <v>3.923</v>
+        <v>3.896</v>
       </c>
       <c r="P36" t="n">
-        <v>3.938</v>
+        <v>3.911</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.193</v>
+        <v>4.164</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3113,34 +3113,34 @@
         <v>4.221</v>
       </c>
       <c r="H37" t="n">
-        <v>4.717</v>
+        <v>4.718</v>
       </c>
       <c r="I37" t="n">
-        <v>5.059</v>
+        <v>5.052</v>
       </c>
       <c r="J37" t="n">
-        <v>5.816</v>
+        <v>5.812</v>
       </c>
       <c r="K37" t="n">
-        <v>6.694</v>
+        <v>6.689</v>
       </c>
       <c r="L37" t="n">
-        <v>7.017</v>
+        <v>7.007</v>
       </c>
       <c r="M37" t="n">
-        <v>7.393</v>
+        <v>7.381</v>
       </c>
       <c r="N37" t="n">
-        <v>7.564</v>
+        <v>7.546</v>
       </c>
       <c r="O37" t="n">
-        <v>7.77</v>
+        <v>7.742</v>
       </c>
       <c r="P37" t="n">
-        <v>7.794</v>
+        <v>7.768</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.224</v>
+        <v>8.195</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3186,34 +3186,34 @@
         <v>5.531</v>
       </c>
       <c r="H38" t="n">
-        <v>6.241</v>
+        <v>6.242</v>
       </c>
       <c r="I38" t="n">
-        <v>6.739</v>
+        <v>6.732</v>
       </c>
       <c r="J38" t="n">
-        <v>7.756</v>
+        <v>7.752</v>
       </c>
       <c r="K38" t="n">
-        <v>8.808999999999999</v>
+        <v>8.804</v>
       </c>
       <c r="L38" t="n">
-        <v>9.292999999999999</v>
+        <v>9.282999999999999</v>
       </c>
       <c r="M38" t="n">
-        <v>9.801</v>
+        <v>9.788</v>
       </c>
       <c r="N38" t="n">
-        <v>9.981999999999999</v>
+        <v>9.964</v>
       </c>
       <c r="O38" t="n">
-        <v>10.17</v>
+        <v>10.142</v>
       </c>
       <c r="P38" t="n">
-        <v>10.192</v>
+        <v>10.166</v>
       </c>
       <c r="Q38" t="n">
-        <v>10.675</v>
+        <v>10.647</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3259,34 +3259,34 @@
         <v>4.729</v>
       </c>
       <c r="H39" t="n">
-        <v>5.305</v>
+        <v>5.307</v>
       </c>
       <c r="I39" t="n">
-        <v>5.743</v>
+        <v>5.736</v>
       </c>
       <c r="J39" t="n">
-        <v>6.629</v>
+        <v>6.624</v>
       </c>
       <c r="K39" t="n">
-        <v>7.643</v>
+        <v>7.638</v>
       </c>
       <c r="L39" t="n">
-        <v>8.051</v>
+        <v>8.041</v>
       </c>
       <c r="M39" t="n">
-        <v>8.438000000000001</v>
+        <v>8.425000000000001</v>
       </c>
       <c r="N39" t="n">
-        <v>8.609999999999999</v>
+        <v>8.592000000000001</v>
       </c>
       <c r="O39" t="n">
+        <v>8.792</v>
+      </c>
+      <c r="P39" t="n">
         <v>8.82</v>
       </c>
-      <c r="P39" t="n">
-        <v>8.846</v>
-      </c>
       <c r="Q39" t="n">
-        <v>9.32</v>
+        <v>9.291</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3332,34 +3332,34 @@
         <v>3.405</v>
       </c>
       <c r="H40" t="n">
-        <v>3.588</v>
+        <v>3.59</v>
       </c>
       <c r="I40" t="n">
-        <v>3.836</v>
+        <v>3.828</v>
       </c>
       <c r="J40" t="n">
-        <v>4.128</v>
+        <v>4.123</v>
       </c>
       <c r="K40" t="n">
-        <v>4.428</v>
+        <v>4.423</v>
       </c>
       <c r="L40" t="n">
-        <v>4.53</v>
+        <v>4.52</v>
       </c>
       <c r="M40" t="n">
-        <v>4.731</v>
+        <v>4.718</v>
       </c>
       <c r="N40" t="n">
-        <v>4.913</v>
+        <v>4.895</v>
       </c>
       <c r="O40" t="n">
-        <v>5.236</v>
+        <v>5.209</v>
       </c>
       <c r="P40" t="n">
-        <v>5.429</v>
+        <v>5.402</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.21</v>
+        <v>6.182</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3405,34 +3405,34 @@
         <v>3.829</v>
       </c>
       <c r="H41" t="n">
-        <v>4.071</v>
+        <v>4.072</v>
       </c>
       <c r="I41" t="n">
-        <v>4.337</v>
+        <v>4.33</v>
       </c>
       <c r="J41" t="n">
-        <v>4.682</v>
+        <v>4.677</v>
       </c>
       <c r="K41" t="n">
-        <v>5.028</v>
+        <v>5.023</v>
       </c>
       <c r="L41" t="n">
-        <v>5.208</v>
+        <v>5.198</v>
       </c>
       <c r="M41" t="n">
-        <v>5.533</v>
+        <v>5.52</v>
       </c>
       <c r="N41" t="n">
-        <v>5.842</v>
+        <v>5.824</v>
       </c>
       <c r="O41" t="n">
-        <v>6.348</v>
+        <v>6.321</v>
       </c>
       <c r="P41" t="n">
-        <v>6.487</v>
+        <v>6.461</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.257</v>
+        <v>7.228</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3478,34 +3478,34 @@
         <v>3.553</v>
       </c>
       <c r="H42" t="n">
-        <v>3.763</v>
+        <v>3.764</v>
       </c>
       <c r="I42" t="n">
-        <v>4.024</v>
+        <v>4.017</v>
       </c>
       <c r="J42" t="n">
-        <v>4.331</v>
+        <v>4.327</v>
       </c>
       <c r="K42" t="n">
-        <v>4.649</v>
+        <v>4.644</v>
       </c>
       <c r="L42" t="n">
-        <v>4.766</v>
+        <v>4.756</v>
       </c>
       <c r="M42" t="n">
-        <v>5.038</v>
+        <v>5.026</v>
       </c>
       <c r="N42" t="n">
-        <v>5.327</v>
+        <v>5.309</v>
       </c>
       <c r="O42" t="n">
-        <v>5.727</v>
+        <v>5.7</v>
       </c>
       <c r="P42" t="n">
-        <v>5.93</v>
+        <v>5.903</v>
       </c>
       <c r="Q42" t="n">
-        <v>6.723</v>
+        <v>6.694</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3551,34 +3551,34 @@
         <v>3.218</v>
       </c>
       <c r="H43" t="n">
-        <v>3.349</v>
+        <v>3.351</v>
       </c>
       <c r="I43" t="n">
-        <v>3.557</v>
+        <v>3.55</v>
       </c>
       <c r="J43" t="n">
-        <v>3.778</v>
+        <v>3.773</v>
       </c>
       <c r="K43" t="n">
-        <v>3.998</v>
+        <v>3.993</v>
       </c>
       <c r="L43" t="n">
-        <v>4.053</v>
+        <v>4.043</v>
       </c>
       <c r="M43" t="n">
-        <v>4.177</v>
+        <v>4.164</v>
       </c>
       <c r="N43" t="n">
-        <v>4.215</v>
+        <v>4.197</v>
       </c>
       <c r="O43" t="n">
-        <v>4.325</v>
+        <v>4.298</v>
       </c>
       <c r="P43" t="n">
-        <v>4.405</v>
+        <v>4.378</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.086</v>
+        <v>5.057</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3624,34 +3624,34 @@
         <v>3.088</v>
       </c>
       <c r="H44" t="n">
-        <v>3.201</v>
+        <v>3.202</v>
       </c>
       <c r="I44" t="n">
-        <v>3.403</v>
+        <v>3.396</v>
       </c>
       <c r="J44" t="n">
-        <v>3.627</v>
+        <v>3.622</v>
       </c>
       <c r="K44" t="n">
-        <v>3.839</v>
+        <v>3.835</v>
       </c>
       <c r="L44" t="n">
-        <v>3.895</v>
+        <v>3.886</v>
       </c>
       <c r="M44" t="n">
-        <v>3.99</v>
+        <v>3.979</v>
       </c>
       <c r="N44" t="n">
-        <v>4.029</v>
+        <v>4.013</v>
       </c>
       <c r="O44" t="n">
-        <v>4.122</v>
+        <v>4.096</v>
       </c>
       <c r="P44" t="n">
-        <v>4.168</v>
+        <v>4.141</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.457</v>
+        <v>4.428</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-04-23 ~ 2026-04-23
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.212</v>
+        <v>3.211</v>
       </c>
       <c r="G2" t="n">
         <v>3.418</v>
       </c>
       <c r="H2" t="n">
-        <v>3.575</v>
+        <v>3.584</v>
       </c>
       <c r="I2" t="n">
-        <v>3.777</v>
+        <v>3.787</v>
       </c>
       <c r="J2" t="n">
-        <v>4.027</v>
+        <v>4.084</v>
       </c>
       <c r="K2" t="n">
-        <v>4.401</v>
+        <v>4.482</v>
       </c>
       <c r="L2" t="n">
-        <v>4.572</v>
+        <v>4.653</v>
       </c>
       <c r="M2" t="n">
-        <v>4.877</v>
+        <v>4.958</v>
       </c>
       <c r="N2" t="n">
-        <v>5.133</v>
+        <v>5.225</v>
       </c>
       <c r="O2" t="n">
-        <v>5.369</v>
+        <v>5.454</v>
       </c>
       <c r="P2" t="n">
-        <v>5.534</v>
+        <v>5.627</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.167</v>
+        <v>6.257</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.235</v>
+        <v>4.234</v>
       </c>
       <c r="G3" t="n">
         <v>4.623</v>
       </c>
       <c r="H3" t="n">
-        <v>4.813</v>
+        <v>4.822</v>
       </c>
       <c r="I3" t="n">
-        <v>5.015</v>
+        <v>5.021</v>
       </c>
       <c r="J3" t="n">
-        <v>5.274</v>
+        <v>5.33</v>
       </c>
       <c r="K3" t="n">
-        <v>5.716</v>
+        <v>5.798</v>
       </c>
       <c r="L3" t="n">
-        <v>5.958</v>
+        <v>6.039</v>
       </c>
       <c r="M3" t="n">
-        <v>6.294</v>
+        <v>6.375</v>
       </c>
       <c r="N3" t="n">
-        <v>6.493</v>
+        <v>6.585</v>
       </c>
       <c r="O3" t="n">
-        <v>6.679</v>
+        <v>6.764</v>
       </c>
       <c r="P3" t="n">
-        <v>6.714</v>
+        <v>6.807</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.235</v>
+        <v>7.325</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -704,34 +704,34 @@
         <v>4.004</v>
       </c>
       <c r="H4" t="n">
-        <v>4.223</v>
+        <v>4.232</v>
       </c>
       <c r="I4" t="n">
-        <v>4.456</v>
+        <v>4.464</v>
       </c>
       <c r="J4" t="n">
-        <v>4.721</v>
+        <v>4.778</v>
       </c>
       <c r="K4" t="n">
-        <v>5.156</v>
+        <v>5.238</v>
       </c>
       <c r="L4" t="n">
-        <v>5.327</v>
+        <v>5.409</v>
       </c>
       <c r="M4" t="n">
-        <v>5.652</v>
+        <v>5.733</v>
       </c>
       <c r="N4" t="n">
-        <v>5.821</v>
+        <v>5.913</v>
       </c>
       <c r="O4" t="n">
-        <v>6.031</v>
+        <v>6.116</v>
       </c>
       <c r="P4" t="n">
-        <v>6.064</v>
+        <v>6.157</v>
       </c>
       <c r="Q4" t="n">
-        <v>6.588</v>
+        <v>6.678</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.907</v>
+        <v>2.906</v>
       </c>
       <c r="G5" t="n">
         <v>2.959</v>
       </c>
       <c r="H5" t="n">
-        <v>3.073</v>
+        <v>3.082</v>
       </c>
       <c r="I5" t="n">
-        <v>3.345</v>
+        <v>3.357</v>
       </c>
       <c r="J5" t="n">
-        <v>3.589</v>
+        <v>3.645</v>
       </c>
       <c r="K5" t="n">
-        <v>3.821</v>
+        <v>3.902</v>
       </c>
       <c r="L5" t="n">
-        <v>3.835</v>
+        <v>3.916</v>
       </c>
       <c r="M5" t="n">
-        <v>3.943</v>
+        <v>4.022</v>
       </c>
       <c r="N5" t="n">
-        <v>3.949</v>
+        <v>4.042</v>
       </c>
       <c r="O5" t="n">
-        <v>3.968</v>
+        <v>4.053</v>
       </c>
       <c r="P5" t="n">
-        <v>4.203</v>
+        <v>4.296</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.079</v>
+        <v>5.169</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2.946</v>
+        <v>2.945</v>
       </c>
       <c r="G6" t="n">
         <v>3.012</v>
       </c>
       <c r="H6" t="n">
-        <v>3.143</v>
+        <v>3.152</v>
       </c>
       <c r="I6" t="n">
-        <v>3.427</v>
+        <v>3.439</v>
       </c>
       <c r="J6" t="n">
-        <v>3.678</v>
+        <v>3.734</v>
       </c>
       <c r="K6" t="n">
-        <v>3.93</v>
+        <v>4.012</v>
       </c>
       <c r="L6" t="n">
-        <v>3.953</v>
+        <v>4.035</v>
       </c>
       <c r="M6" t="n">
-        <v>4.1</v>
+        <v>4.181</v>
       </c>
       <c r="N6" t="n">
-        <v>4.117</v>
+        <v>4.209</v>
       </c>
       <c r="O6" t="n">
-        <v>4.236</v>
+        <v>4.321</v>
       </c>
       <c r="P6" t="n">
-        <v>4.635</v>
+        <v>4.728</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.475</v>
+        <v>5.565</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2.927</v>
+        <v>2.926</v>
       </c>
       <c r="G7" t="n">
         <v>2.976</v>
       </c>
       <c r="H7" t="n">
-        <v>3.088</v>
+        <v>3.097</v>
       </c>
       <c r="I7" t="n">
-        <v>3.36</v>
+        <v>3.372</v>
       </c>
       <c r="J7" t="n">
-        <v>3.614</v>
+        <v>3.671</v>
       </c>
       <c r="K7" t="n">
-        <v>3.848</v>
+        <v>3.929</v>
       </c>
       <c r="L7" t="n">
-        <v>3.86</v>
+        <v>3.941</v>
       </c>
       <c r="M7" t="n">
-        <v>4.003</v>
+        <v>4.085</v>
       </c>
       <c r="N7" t="n">
-        <v>4.01</v>
+        <v>4.102</v>
       </c>
       <c r="O7" t="n">
-        <v>4.134</v>
+        <v>4.218</v>
       </c>
       <c r="P7" t="n">
-        <v>4.419</v>
+        <v>4.512</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.243</v>
+        <v>5.333</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.345</v>
+        <v>5.343</v>
       </c>
       <c r="G8" t="n">
         <v>5.921</v>
       </c>
       <c r="H8" t="n">
-        <v>6.262</v>
+        <v>6.271</v>
       </c>
       <c r="I8" t="n">
-        <v>6.535</v>
+        <v>6.546</v>
       </c>
       <c r="J8" t="n">
-        <v>6.859</v>
+        <v>6.919</v>
       </c>
       <c r="K8" t="n">
-        <v>7.583</v>
+        <v>7.666</v>
       </c>
       <c r="L8" t="n">
-        <v>7.913</v>
+        <v>7.996</v>
       </c>
       <c r="M8" t="n">
-        <v>8.278</v>
+        <v>8.363</v>
       </c>
       <c r="N8" t="n">
-        <v>8.414</v>
+        <v>8.507999999999999</v>
       </c>
       <c r="O8" t="n">
-        <v>8.686</v>
+        <v>8.773</v>
       </c>
       <c r="P8" t="n">
-        <v>8.823</v>
+        <v>8.917999999999999</v>
       </c>
       <c r="Q8" t="n">
-        <v>9.544</v>
+        <v>9.634</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,57 +1063,57 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.619</v>
+        <v>2.623</v>
       </c>
       <c r="G9" t="n">
-        <v>2.682</v>
+        <v>2.694</v>
       </c>
       <c r="H9" t="n">
-        <v>2.774</v>
+        <v>2.801</v>
       </c>
       <c r="I9" t="n">
-        <v>2.936</v>
+        <v>2.963</v>
       </c>
       <c r="J9" t="n">
-        <v>3.125</v>
+        <v>3.194</v>
       </c>
       <c r="K9" t="n">
-        <v>3.24</v>
+        <v>3.331</v>
       </c>
       <c r="L9" t="n">
-        <v>3.276</v>
+        <v>3.365</v>
       </c>
       <c r="M9" t="n">
-        <v>3.364</v>
+        <v>3.453</v>
       </c>
       <c r="N9" t="n">
-        <v>3.517</v>
+        <v>3.615</v>
       </c>
       <c r="O9" t="n">
-        <v>3.562</v>
+        <v>3.65</v>
       </c>
       <c r="P9" t="n">
-        <v>3.623</v>
+        <v>3.718</v>
       </c>
       <c r="Q9" t="n">
-        <v>3.697</v>
+        <v>3.787</v>
       </c>
       <c r="R9" t="n">
-        <v>3.691</v>
+        <v>3.759</v>
       </c>
       <c r="S9" t="n">
-        <v>3.645</v>
+        <v>3.729</v>
       </c>
       <c r="T9" t="n">
-        <v>3.569</v>
+        <v>3.65</v>
       </c>
       <c r="U9" t="n">
-        <v>3.441</v>
+        <v>3.522</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.633</v>
+        <v>2.636</v>
       </c>
       <c r="G10" t="n">
-        <v>2.72</v>
+        <v>2.728</v>
       </c>
       <c r="H10" t="n">
-        <v>2.789</v>
+        <v>2.816</v>
       </c>
       <c r="I10" t="n">
-        <v>2.949</v>
+        <v>2.976</v>
       </c>
       <c r="J10" t="n">
-        <v>3.151</v>
+        <v>3.219</v>
       </c>
       <c r="K10" t="n">
-        <v>3.273</v>
+        <v>3.364</v>
       </c>
       <c r="L10" t="n">
-        <v>3.324</v>
+        <v>3.415</v>
       </c>
       <c r="M10" t="n">
-        <v>3.463</v>
+        <v>3.55</v>
       </c>
       <c r="N10" t="n">
-        <v>3.531</v>
+        <v>3.628</v>
       </c>
       <c r="O10" t="n">
-        <v>3.774</v>
+        <v>3.864</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.448</v>
+        <v>2.452</v>
       </c>
       <c r="G11" t="n">
-        <v>2.53</v>
+        <v>2.538</v>
       </c>
       <c r="H11" t="n">
-        <v>2.613</v>
+        <v>2.64</v>
       </c>
       <c r="I11" t="n">
-        <v>2.752</v>
+        <v>2.779</v>
       </c>
       <c r="J11" t="n">
-        <v>2.946</v>
+        <v>3.014</v>
       </c>
       <c r="K11" t="n">
-        <v>3.06</v>
+        <v>3.152</v>
       </c>
       <c r="L11" t="n">
-        <v>3.118</v>
+        <v>3.209</v>
       </c>
       <c r="M11" t="n">
-        <v>3.267</v>
+        <v>3.356</v>
       </c>
       <c r="N11" t="n">
-        <v>3.339</v>
+        <v>3.437</v>
       </c>
       <c r="O11" t="n">
-        <v>3.54</v>
+        <v>3.631</v>
       </c>
       <c r="P11" t="n">
-        <v>3.567</v>
+        <v>3.664</v>
       </c>
       <c r="Q11" t="n">
-        <v>3.899</v>
+        <v>3.988</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1285,43 +1285,43 @@
         <v>3.193</v>
       </c>
       <c r="G12" t="n">
-        <v>3.341</v>
+        <v>3.349</v>
       </c>
       <c r="H12" t="n">
-        <v>3.45</v>
+        <v>3.458</v>
       </c>
       <c r="I12" t="n">
-        <v>3.668</v>
+        <v>3.696</v>
       </c>
       <c r="J12" t="n">
-        <v>3.995</v>
+        <v>4.051</v>
       </c>
       <c r="K12" t="n">
-        <v>4.169</v>
+        <v>4.249</v>
       </c>
       <c r="L12" t="n">
-        <v>4.229</v>
+        <v>4.309</v>
       </c>
       <c r="M12" t="n">
-        <v>4.375</v>
+        <v>4.454</v>
       </c>
       <c r="N12" t="n">
-        <v>4.411</v>
+        <v>4.501</v>
       </c>
       <c r="O12" t="n">
-        <v>4.566</v>
+        <v>4.651</v>
       </c>
       <c r="P12" t="n">
-        <v>4.67</v>
+        <v>4.763</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.027</v>
+        <v>5.116</v>
       </c>
       <c r="R12" t="n">
-        <v>5.189</v>
+        <v>5.26</v>
       </c>
       <c r="S12" t="n">
-        <v>5.356</v>
+        <v>5.44</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2.946</v>
+        <v>2.947</v>
       </c>
       <c r="G13" t="n">
-        <v>3.031</v>
+        <v>3.039</v>
       </c>
       <c r="H13" t="n">
-        <v>3.117</v>
+        <v>3.126</v>
       </c>
       <c r="I13" t="n">
-        <v>3.316</v>
+        <v>3.344</v>
       </c>
       <c r="J13" t="n">
-        <v>3.632</v>
+        <v>3.688</v>
       </c>
       <c r="K13" t="n">
-        <v>3.802</v>
+        <v>3.882</v>
       </c>
       <c r="L13" t="n">
-        <v>3.869</v>
+        <v>3.949</v>
       </c>
       <c r="M13" t="n">
-        <v>4.002</v>
+        <v>4.081</v>
       </c>
       <c r="N13" t="n">
-        <v>4.039</v>
+        <v>4.13</v>
       </c>
       <c r="O13" t="n">
-        <v>4.195</v>
+        <v>4.279</v>
       </c>
       <c r="P13" t="n">
-        <v>4.261</v>
+        <v>4.354</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.548</v>
+        <v>4.636</v>
       </c>
       <c r="R13" t="n">
-        <v>4.738</v>
+        <v>4.808</v>
       </c>
       <c r="S13" t="n">
-        <v>4.919</v>
+        <v>5.003</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.765</v>
+        <v>2.766</v>
       </c>
       <c r="G14" t="n">
-        <v>2.837</v>
+        <v>2.844</v>
       </c>
       <c r="H14" t="n">
-        <v>2.921</v>
+        <v>2.929</v>
       </c>
       <c r="I14" t="n">
-        <v>3.1</v>
+        <v>3.127</v>
       </c>
       <c r="J14" t="n">
-        <v>3.372</v>
+        <v>3.428</v>
       </c>
       <c r="K14" t="n">
-        <v>3.49</v>
+        <v>3.57</v>
       </c>
       <c r="L14" t="n">
-        <v>3.541</v>
+        <v>3.621</v>
       </c>
       <c r="M14" t="n">
-        <v>3.687</v>
+        <v>3.767</v>
       </c>
       <c r="N14" t="n">
-        <v>3.718</v>
+        <v>3.809</v>
       </c>
       <c r="O14" t="n">
-        <v>3.85</v>
+        <v>3.935</v>
       </c>
       <c r="P14" t="n">
-        <v>3.896</v>
+        <v>3.989</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.137</v>
+        <v>4.225</v>
       </c>
       <c r="R14" t="n">
-        <v>4.253</v>
+        <v>4.323</v>
       </c>
       <c r="S14" t="n">
-        <v>4.371</v>
+        <v>4.455</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1504,43 +1504,43 @@
         <v>2.744</v>
       </c>
       <c r="G15" t="n">
-        <v>2.811</v>
+        <v>2.819</v>
       </c>
       <c r="H15" t="n">
-        <v>2.889</v>
+        <v>2.898</v>
       </c>
       <c r="I15" t="n">
-        <v>3.052</v>
+        <v>3.08</v>
       </c>
       <c r="J15" t="n">
-        <v>3.311</v>
+        <v>3.367</v>
       </c>
       <c r="K15" t="n">
-        <v>3.443</v>
+        <v>3.523</v>
       </c>
       <c r="L15" t="n">
-        <v>3.476</v>
+        <v>3.556</v>
       </c>
       <c r="M15" t="n">
-        <v>3.601</v>
+        <v>3.68</v>
       </c>
       <c r="N15" t="n">
-        <v>3.622</v>
+        <v>3.713</v>
       </c>
       <c r="O15" t="n">
-        <v>3.776</v>
+        <v>3.864</v>
       </c>
       <c r="P15" t="n">
-        <v>3.795</v>
+        <v>3.888</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.042</v>
+        <v>4.13</v>
       </c>
       <c r="R15" t="n">
-        <v>4.149</v>
+        <v>4.219</v>
       </c>
       <c r="S15" t="n">
-        <v>4.267</v>
+        <v>4.351</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1577,43 +1577,43 @@
         <v>2.744</v>
       </c>
       <c r="G16" t="n">
-        <v>2.811</v>
+        <v>2.819</v>
       </c>
       <c r="H16" t="n">
-        <v>2.889</v>
+        <v>2.898</v>
       </c>
       <c r="I16" t="n">
-        <v>3.052</v>
+        <v>3.08</v>
       </c>
       <c r="J16" t="n">
-        <v>3.311</v>
+        <v>3.367</v>
       </c>
       <c r="K16" t="n">
-        <v>3.443</v>
+        <v>3.523</v>
       </c>
       <c r="L16" t="n">
-        <v>3.476</v>
+        <v>3.556</v>
       </c>
       <c r="M16" t="n">
-        <v>3.601</v>
+        <v>3.68</v>
       </c>
       <c r="N16" t="n">
-        <v>3.625</v>
+        <v>3.716</v>
       </c>
       <c r="O16" t="n">
-        <v>3.783</v>
+        <v>3.871</v>
       </c>
       <c r="P16" t="n">
-        <v>3.819</v>
+        <v>3.912</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.069</v>
+        <v>4.157</v>
       </c>
       <c r="R16" t="n">
-        <v>4.177</v>
+        <v>4.247</v>
       </c>
       <c r="S16" t="n">
-        <v>4.296</v>
+        <v>4.38</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.696</v>
+        <v>2.699</v>
       </c>
       <c r="G17" t="n">
-        <v>2.809</v>
+        <v>2.817</v>
       </c>
       <c r="H17" t="n">
-        <v>2.883</v>
+        <v>2.91</v>
       </c>
       <c r="I17" t="n">
-        <v>3.031</v>
+        <v>3.058</v>
       </c>
       <c r="J17" t="n">
-        <v>3.222</v>
+        <v>3.29</v>
       </c>
       <c r="K17" t="n">
-        <v>3.348</v>
+        <v>3.439</v>
       </c>
       <c r="L17" t="n">
-        <v>3.403</v>
+        <v>3.493</v>
       </c>
       <c r="M17" t="n">
-        <v>3.58</v>
+        <v>3.67</v>
       </c>
       <c r="N17" t="n">
-        <v>3.631</v>
+        <v>3.729</v>
       </c>
       <c r="O17" t="n">
-        <v>3.8</v>
+        <v>3.892</v>
       </c>
       <c r="P17" t="n">
-        <v>3.839</v>
+        <v>3.936</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.697</v>
+        <v>2.7</v>
       </c>
       <c r="G18" t="n">
-        <v>2.81</v>
+        <v>2.818</v>
       </c>
       <c r="H18" t="n">
-        <v>2.883</v>
+        <v>2.91</v>
       </c>
       <c r="I18" t="n">
-        <v>3.031</v>
+        <v>3.058</v>
       </c>
       <c r="J18" t="n">
-        <v>3.222</v>
+        <v>3.29</v>
       </c>
       <c r="K18" t="n">
-        <v>3.349</v>
+        <v>3.44</v>
       </c>
       <c r="L18" t="n">
-        <v>3.403</v>
+        <v>3.493</v>
       </c>
       <c r="M18" t="n">
-        <v>3.58</v>
+        <v>3.67</v>
       </c>
       <c r="N18" t="n">
-        <v>3.632</v>
+        <v>3.73</v>
       </c>
       <c r="O18" t="n">
-        <v>3.8</v>
+        <v>3.89</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.756</v>
+        <v>2.757</v>
       </c>
       <c r="G19" t="n">
-        <v>2.828</v>
+        <v>2.836</v>
       </c>
       <c r="H19" t="n">
-        <v>2.91</v>
+        <v>2.919</v>
       </c>
       <c r="I19" t="n">
-        <v>3.087</v>
+        <v>3.114</v>
       </c>
       <c r="J19" t="n">
-        <v>3.356</v>
+        <v>3.412</v>
       </c>
       <c r="K19" t="n">
-        <v>3.486</v>
+        <v>3.567</v>
       </c>
       <c r="L19" t="n">
-        <v>3.538</v>
+        <v>3.618</v>
       </c>
       <c r="M19" t="n">
-        <v>3.679</v>
+        <v>3.758</v>
       </c>
       <c r="N19" t="n">
-        <v>3.705</v>
+        <v>3.796</v>
       </c>
       <c r="O19" t="n">
-        <v>3.828</v>
+        <v>3.915</v>
       </c>
       <c r="P19" t="n">
-        <v>3.857</v>
+        <v>3.95</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.084</v>
+        <v>4.173</v>
       </c>
       <c r="R19" t="n">
-        <v>4.199</v>
+        <v>4.271</v>
       </c>
       <c r="S19" t="n">
-        <v>4.31</v>
+        <v>4.394</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2.573</v>
+        <v>2.578</v>
       </c>
       <c r="G20" t="n">
-        <v>2.64</v>
+        <v>2.648</v>
       </c>
       <c r="H20" t="n">
-        <v>2.685</v>
+        <v>2.693</v>
       </c>
       <c r="I20" t="n">
-        <v>2.821</v>
+        <v>2.834</v>
       </c>
       <c r="J20" t="n">
-        <v>3.125</v>
+        <v>3.19</v>
       </c>
       <c r="K20" t="n">
-        <v>3.266</v>
+        <v>3.354</v>
       </c>
       <c r="L20" t="n">
-        <v>3.309</v>
+        <v>3.397</v>
       </c>
       <c r="M20" t="n">
-        <v>3.409</v>
+        <v>3.498</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2.863</v>
+        <v>2.866</v>
       </c>
       <c r="G21" t="n">
-        <v>2.939</v>
+        <v>2.943</v>
       </c>
       <c r="H21" t="n">
-        <v>3.056</v>
+        <v>3.065</v>
       </c>
       <c r="I21" t="n">
-        <v>3.213</v>
+        <v>3.237</v>
       </c>
       <c r="J21" t="n">
-        <v>3.488</v>
+        <v>3.547</v>
       </c>
       <c r="K21" t="n">
-        <v>3.727</v>
+        <v>3.807</v>
       </c>
       <c r="L21" t="n">
-        <v>3.786</v>
+        <v>3.864</v>
       </c>
       <c r="M21" t="n">
-        <v>3.925</v>
+        <v>4.003</v>
       </c>
       <c r="N21" t="n">
-        <v>3.968</v>
+        <v>4.058</v>
       </c>
       <c r="O21" t="n">
-        <v>4.058</v>
+        <v>4.138</v>
       </c>
       <c r="P21" t="n">
-        <v>4.122</v>
+        <v>4.215</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.249</v>
+        <v>4.338</v>
       </c>
       <c r="R21" t="n">
-        <v>4.249</v>
+        <v>4.321</v>
       </c>
       <c r="S21" t="n">
-        <v>4.271</v>
+        <v>4.354</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.81</v>
+        <v>2.813</v>
       </c>
       <c r="G22" t="n">
-        <v>2.886</v>
+        <v>2.89</v>
       </c>
       <c r="H22" t="n">
-        <v>2.988</v>
+        <v>2.997</v>
       </c>
       <c r="I22" t="n">
-        <v>3.133</v>
+        <v>3.157</v>
       </c>
       <c r="J22" t="n">
-        <v>3.372</v>
+        <v>3.431</v>
       </c>
       <c r="K22" t="n">
-        <v>3.607</v>
+        <v>3.687</v>
       </c>
       <c r="L22" t="n">
-        <v>3.654</v>
+        <v>3.732</v>
       </c>
       <c r="M22" t="n">
-        <v>3.795</v>
+        <v>3.872</v>
       </c>
       <c r="N22" t="n">
-        <v>3.84</v>
+        <v>3.93</v>
       </c>
       <c r="O22" t="n">
-        <v>3.926</v>
+        <v>4.006</v>
       </c>
       <c r="P22" t="n">
-        <v>3.985</v>
+        <v>4.078</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.107</v>
+        <v>4.196</v>
       </c>
       <c r="R22" t="n">
-        <v>4.096</v>
+        <v>4.169</v>
       </c>
       <c r="S22" t="n">
-        <v>4.116</v>
+        <v>4.2</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.763</v>
+        <v>2.766</v>
       </c>
       <c r="G23" t="n">
-        <v>2.841</v>
+        <v>2.844</v>
       </c>
       <c r="H23" t="n">
-        <v>2.928</v>
+        <v>2.937</v>
       </c>
       <c r="I23" t="n">
-        <v>3.086</v>
+        <v>3.11</v>
       </c>
       <c r="J23" t="n">
-        <v>3.318</v>
+        <v>3.376</v>
       </c>
       <c r="K23" t="n">
-        <v>3.524</v>
+        <v>3.6</v>
       </c>
       <c r="L23" t="n">
-        <v>3.565</v>
+        <v>3.643</v>
       </c>
       <c r="M23" t="n">
-        <v>3.699</v>
+        <v>3.776</v>
       </c>
       <c r="N23" t="n">
-        <v>3.737</v>
+        <v>3.827</v>
       </c>
       <c r="O23" t="n">
-        <v>3.8</v>
+        <v>3.881</v>
       </c>
       <c r="P23" t="n">
-        <v>3.846</v>
+        <v>3.939</v>
       </c>
       <c r="Q23" t="n">
-        <v>3.915</v>
+        <v>4.004</v>
       </c>
       <c r="R23" t="n">
-        <v>3.88</v>
+        <v>3.953</v>
       </c>
       <c r="S23" t="n">
-        <v>3.87</v>
+        <v>3.954</v>
       </c>
       <c r="T23" t="n">
-        <v>3.785</v>
+        <v>3.865</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.698</v>
+        <v>2.701</v>
       </c>
       <c r="G24" t="n">
-        <v>2.755</v>
+        <v>2.759</v>
       </c>
       <c r="H24" t="n">
-        <v>2.829</v>
+        <v>2.838</v>
       </c>
       <c r="I24" t="n">
-        <v>2.996</v>
+        <v>3.02</v>
       </c>
       <c r="J24" t="n">
-        <v>3.217</v>
+        <v>3.275</v>
       </c>
       <c r="K24" t="n">
-        <v>3.409</v>
+        <v>3.484</v>
       </c>
       <c r="L24" t="n">
-        <v>3.438</v>
+        <v>3.517</v>
       </c>
       <c r="M24" t="n">
-        <v>3.556</v>
+        <v>3.636</v>
       </c>
       <c r="N24" t="n">
-        <v>3.608</v>
+        <v>3.7</v>
       </c>
       <c r="O24" t="n">
-        <v>3.766</v>
+        <v>3.859</v>
       </c>
       <c r="P24" t="n">
-        <v>3.787</v>
+        <v>3.88</v>
       </c>
       <c r="Q24" t="n">
-        <v>3.837</v>
+        <v>3.926</v>
       </c>
       <c r="R24" t="n">
-        <v>3.802</v>
+        <v>3.874</v>
       </c>
       <c r="S24" t="n">
-        <v>3.785</v>
+        <v>3.869</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.756</v>
+        <v>2.759</v>
       </c>
       <c r="G25" t="n">
-        <v>2.84</v>
+        <v>2.844</v>
       </c>
       <c r="H25" t="n">
-        <v>2.931</v>
+        <v>2.94</v>
       </c>
       <c r="I25" t="n">
-        <v>3.093</v>
+        <v>3.118</v>
       </c>
       <c r="J25" t="n">
-        <v>3.333</v>
+        <v>3.392</v>
       </c>
       <c r="K25" t="n">
-        <v>3.556</v>
+        <v>3.633</v>
       </c>
       <c r="L25" t="n">
-        <v>3.594</v>
+        <v>3.672</v>
       </c>
       <c r="M25" t="n">
-        <v>3.729</v>
+        <v>3.807</v>
       </c>
       <c r="N25" t="n">
-        <v>3.764</v>
+        <v>3.854</v>
       </c>
       <c r="O25" t="n">
-        <v>3.83</v>
+        <v>3.91</v>
       </c>
       <c r="P25" t="n">
-        <v>3.868</v>
+        <v>3.961</v>
       </c>
       <c r="Q25" t="n">
-        <v>3.948</v>
+        <v>4.037</v>
       </c>
       <c r="R25" t="n">
-        <v>3.904</v>
+        <v>3.976</v>
       </c>
       <c r="S25" t="n">
-        <v>3.893</v>
+        <v>3.977</v>
       </c>
       <c r="T25" t="n">
-        <v>3.803</v>
+        <v>3.884</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.062</v>
+        <v>3.064</v>
       </c>
       <c r="G26" t="n">
-        <v>3.19</v>
+        <v>3.195</v>
       </c>
       <c r="H26" t="n">
-        <v>3.394</v>
+        <v>3.405</v>
       </c>
       <c r="I26" t="n">
-        <v>3.627</v>
+        <v>3.647</v>
       </c>
       <c r="J26" t="n">
-        <v>3.993</v>
+        <v>4.055</v>
       </c>
       <c r="K26" t="n">
-        <v>4.354</v>
+        <v>4.438</v>
       </c>
       <c r="L26" t="n">
-        <v>4.454</v>
+        <v>4.539</v>
       </c>
       <c r="M26" t="n">
-        <v>4.646</v>
+        <v>4.731</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>4.901</v>
+        <v>4.987</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.856</v>
+        <v>2.857</v>
       </c>
       <c r="G27" t="n">
-        <v>2.919</v>
+        <v>2.926</v>
       </c>
       <c r="H27" t="n">
-        <v>3.026</v>
+        <v>3.036</v>
       </c>
       <c r="I27" t="n">
-        <v>3.213</v>
+        <v>3.239</v>
       </c>
       <c r="J27" t="n">
-        <v>3.493</v>
+        <v>3.552</v>
       </c>
       <c r="K27" t="n">
-        <v>3.667</v>
+        <v>3.75</v>
       </c>
       <c r="L27" t="n">
-        <v>3.721</v>
+        <v>3.804</v>
       </c>
       <c r="M27" t="n">
-        <v>3.855</v>
+        <v>3.937</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>3.992</v>
+        <v>4.078</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2453,31 +2453,31 @@
         <v>2.96</v>
       </c>
       <c r="G28" t="n">
-        <v>3.029</v>
+        <v>3.037</v>
       </c>
       <c r="H28" t="n">
-        <v>3.15</v>
+        <v>3.162</v>
       </c>
       <c r="I28" t="n">
-        <v>3.351</v>
+        <v>3.377</v>
       </c>
       <c r="J28" t="n">
-        <v>3.666</v>
+        <v>3.725</v>
       </c>
       <c r="K28" t="n">
-        <v>3.859</v>
+        <v>3.942</v>
       </c>
       <c r="L28" t="n">
-        <v>3.925</v>
+        <v>4.008</v>
       </c>
       <c r="M28" t="n">
-        <v>4.067</v>
+        <v>4.149</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.286</v>
+        <v>4.372</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.812</v>
+        <v>2.813</v>
       </c>
       <c r="G29" t="n">
-        <v>2.876</v>
+        <v>2.883</v>
       </c>
       <c r="H29" t="n">
-        <v>2.969</v>
+        <v>2.98</v>
       </c>
       <c r="I29" t="n">
-        <v>3.147</v>
+        <v>3.173</v>
       </c>
       <c r="J29" t="n">
-        <v>3.405</v>
+        <v>3.464</v>
       </c>
       <c r="K29" t="n">
-        <v>3.563</v>
+        <v>3.646</v>
       </c>
       <c r="L29" t="n">
-        <v>3.606</v>
+        <v>3.689</v>
       </c>
       <c r="M29" t="n">
-        <v>3.717</v>
+        <v>3.799</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>3.853</v>
+        <v>3.941</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.095</v>
+        <v>3.097</v>
       </c>
       <c r="G30" t="n">
-        <v>3.16</v>
+        <v>3.165</v>
       </c>
       <c r="H30" t="n">
-        <v>3.325</v>
+        <v>3.338</v>
       </c>
       <c r="I30" t="n">
-        <v>3.552</v>
+        <v>3.574</v>
       </c>
       <c r="J30" t="n">
-        <v>3.859</v>
+        <v>3.923</v>
       </c>
       <c r="K30" t="n">
-        <v>4.147</v>
+        <v>4.229</v>
       </c>
       <c r="L30" t="n">
-        <v>4.223</v>
+        <v>4.307</v>
       </c>
       <c r="M30" t="n">
-        <v>4.407</v>
+        <v>4.492</v>
       </c>
       <c r="N30" t="n">
-        <v>4.562</v>
+        <v>4.658</v>
       </c>
       <c r="O30" t="n">
-        <v>4.853</v>
+        <v>4.938</v>
       </c>
       <c r="P30" t="n">
-        <v>5.011</v>
+        <v>5.104</v>
       </c>
       <c r="Q30" t="n">
-        <v>5.771</v>
+        <v>5.861</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.421</v>
+        <v>3.423</v>
       </c>
       <c r="G31" t="n">
-        <v>3.52</v>
+        <v>3.525</v>
       </c>
       <c r="H31" t="n">
-        <v>3.738</v>
+        <v>3.75</v>
       </c>
       <c r="I31" t="n">
-        <v>3.98</v>
+        <v>4.002</v>
       </c>
       <c r="J31" t="n">
-        <v>4.349</v>
+        <v>4.413</v>
       </c>
       <c r="K31" t="n">
-        <v>4.679</v>
+        <v>4.762</v>
       </c>
       <c r="L31" t="n">
-        <v>4.835</v>
+        <v>4.919</v>
       </c>
       <c r="M31" t="n">
-        <v>5.136</v>
+        <v>5.222</v>
       </c>
       <c r="N31" t="n">
-        <v>5.419</v>
+        <v>5.515</v>
       </c>
       <c r="O31" t="n">
-        <v>5.885</v>
+        <v>5.971</v>
       </c>
       <c r="P31" t="n">
-        <v>5.998</v>
+        <v>6.091</v>
       </c>
       <c r="Q31" t="n">
-        <v>6.745</v>
+        <v>6.834</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.193</v>
+        <v>3.195</v>
       </c>
       <c r="G32" t="n">
-        <v>3.276</v>
+        <v>3.281</v>
       </c>
       <c r="H32" t="n">
-        <v>3.468</v>
+        <v>3.48</v>
       </c>
       <c r="I32" t="n">
-        <v>3.711</v>
+        <v>3.733</v>
       </c>
       <c r="J32" t="n">
-        <v>4.038</v>
+        <v>4.102</v>
       </c>
       <c r="K32" t="n">
-        <v>4.332</v>
+        <v>4.415</v>
       </c>
       <c r="L32" t="n">
-        <v>4.427</v>
+        <v>4.512</v>
       </c>
       <c r="M32" t="n">
-        <v>4.679</v>
+        <v>4.765</v>
       </c>
       <c r="N32" t="n">
-        <v>4.923</v>
+        <v>5.019</v>
       </c>
       <c r="O32" t="n">
-        <v>5.297</v>
+        <v>5.382</v>
       </c>
       <c r="P32" t="n">
-        <v>5.47</v>
+        <v>5.563</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.232</v>
+        <v>6.322</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2.97</v>
+        <v>2.972</v>
       </c>
       <c r="G33" t="n">
-        <v>3.03</v>
+        <v>3.034</v>
       </c>
       <c r="H33" t="n">
-        <v>3.148</v>
+        <v>3.158</v>
       </c>
       <c r="I33" t="n">
-        <v>3.336</v>
+        <v>3.357</v>
       </c>
       <c r="J33" t="n">
-        <v>3.57</v>
+        <v>3.632</v>
       </c>
       <c r="K33" t="n">
-        <v>3.789</v>
+        <v>3.873</v>
       </c>
       <c r="L33" t="n">
-        <v>3.829</v>
+        <v>3.914</v>
       </c>
       <c r="M33" t="n">
-        <v>3.94</v>
+        <v>4.027</v>
       </c>
       <c r="N33" t="n">
-        <v>3.953</v>
+        <v>4.049</v>
       </c>
       <c r="O33" t="n">
-        <v>4.007</v>
+        <v>4.093</v>
       </c>
       <c r="P33" t="n">
-        <v>4.043</v>
+        <v>4.136</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.488</v>
+        <v>4.578</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.029</v>
+        <v>3.031</v>
       </c>
       <c r="G34" t="n">
-        <v>3.082</v>
+        <v>3.088</v>
       </c>
       <c r="H34" t="n">
-        <v>3.207</v>
+        <v>3.218</v>
       </c>
       <c r="I34" t="n">
-        <v>3.405</v>
+        <v>3.425</v>
       </c>
       <c r="J34" t="n">
-        <v>3.642</v>
+        <v>3.704</v>
       </c>
       <c r="K34" t="n">
-        <v>3.866</v>
+        <v>3.95</v>
       </c>
       <c r="L34" t="n">
-        <v>3.908</v>
+        <v>3.994</v>
       </c>
       <c r="M34" t="n">
-        <v>4.031</v>
+        <v>4.117</v>
       </c>
       <c r="N34" t="n">
-        <v>4.058</v>
+        <v>4.154</v>
       </c>
       <c r="O34" t="n">
-        <v>4.175</v>
+        <v>4.261</v>
       </c>
       <c r="P34" t="n">
-        <v>4.337</v>
+        <v>4.43</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.189</v>
+        <v>5.279</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.004</v>
+        <v>3.006</v>
       </c>
       <c r="G35" t="n">
-        <v>3.056</v>
+        <v>3.061</v>
       </c>
       <c r="H35" t="n">
-        <v>3.175</v>
+        <v>3.186</v>
       </c>
       <c r="I35" t="n">
-        <v>3.371</v>
+        <v>3.391</v>
       </c>
       <c r="J35" t="n">
-        <v>3.61</v>
+        <v>3.672</v>
       </c>
       <c r="K35" t="n">
-        <v>3.82</v>
+        <v>3.904</v>
       </c>
       <c r="L35" t="n">
-        <v>3.863</v>
+        <v>3.948</v>
       </c>
       <c r="M35" t="n">
-        <v>3.978</v>
+        <v>4.064</v>
       </c>
       <c r="N35" t="n">
-        <v>3.994</v>
+        <v>4.09</v>
       </c>
       <c r="O35" t="n">
-        <v>4.073</v>
+        <v>4.159</v>
       </c>
       <c r="P35" t="n">
-        <v>4.14</v>
+        <v>4.233</v>
       </c>
       <c r="Q35" t="n">
-        <v>4.825</v>
+        <v>4.915</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.912</v>
+        <v>2.914</v>
       </c>
       <c r="G36" t="n">
-        <v>2.97</v>
+        <v>2.974</v>
       </c>
       <c r="H36" t="n">
-        <v>3.074</v>
+        <v>3.083</v>
       </c>
       <c r="I36" t="n">
-        <v>3.264</v>
+        <v>3.284</v>
       </c>
       <c r="J36" t="n">
-        <v>3.506</v>
+        <v>3.568</v>
       </c>
       <c r="K36" t="n">
-        <v>3.713</v>
+        <v>3.796</v>
       </c>
       <c r="L36" t="n">
-        <v>3.753</v>
+        <v>3.838</v>
       </c>
       <c r="M36" t="n">
-        <v>3.839</v>
+        <v>3.926</v>
       </c>
       <c r="N36" t="n">
-        <v>3.855</v>
+        <v>3.951</v>
       </c>
       <c r="O36" t="n">
-        <v>3.917</v>
+        <v>4.003</v>
       </c>
       <c r="P36" t="n">
-        <v>3.941</v>
+        <v>4.035</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.205</v>
+        <v>4.295</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.765</v>
+        <v>3.767</v>
       </c>
       <c r="G37" t="n">
-        <v>4.215</v>
+        <v>4.22</v>
       </c>
       <c r="H37" t="n">
-        <v>4.714</v>
+        <v>4.726</v>
       </c>
       <c r="I37" t="n">
-        <v>5.051</v>
+        <v>5.068</v>
       </c>
       <c r="J37" t="n">
-        <v>5.84</v>
+        <v>5.904</v>
       </c>
       <c r="K37" t="n">
-        <v>6.718</v>
+        <v>6.802</v>
       </c>
       <c r="L37" t="n">
-        <v>7.034</v>
+        <v>7.119</v>
       </c>
       <c r="M37" t="n">
-        <v>7.41</v>
+        <v>7.497</v>
       </c>
       <c r="N37" t="n">
-        <v>7.571</v>
+        <v>7.667</v>
       </c>
       <c r="O37" t="n">
-        <v>7.764</v>
+        <v>7.85</v>
       </c>
       <c r="P37" t="n">
-        <v>7.798</v>
+        <v>7.891</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.236000000000001</v>
+        <v>8.324</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.822</v>
+        <v>4.824</v>
       </c>
       <c r="G38" t="n">
-        <v>5.526</v>
+        <v>5.531</v>
       </c>
       <c r="H38" t="n">
-        <v>6.238</v>
+        <v>6.25</v>
       </c>
       <c r="I38" t="n">
-        <v>6.731</v>
+        <v>6.748</v>
       </c>
       <c r="J38" t="n">
-        <v>7.78</v>
+        <v>7.844</v>
       </c>
       <c r="K38" t="n">
-        <v>8.834</v>
+        <v>8.919</v>
       </c>
       <c r="L38" t="n">
-        <v>9.31</v>
+        <v>9.397</v>
       </c>
       <c r="M38" t="n">
-        <v>9.818</v>
+        <v>9.906000000000001</v>
       </c>
       <c r="N38" t="n">
-        <v>9.989000000000001</v>
+        <v>10.085</v>
       </c>
       <c r="O38" t="n">
-        <v>10.164</v>
+        <v>10.25</v>
       </c>
       <c r="P38" t="n">
-        <v>10.196</v>
+        <v>10.289</v>
       </c>
       <c r="Q38" t="n">
-        <v>10.687</v>
+        <v>10.775</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.143</v>
+        <v>4.145</v>
       </c>
       <c r="G39" t="n">
-        <v>4.724</v>
+        <v>4.729</v>
       </c>
       <c r="H39" t="n">
-        <v>5.303</v>
+        <v>5.315</v>
       </c>
       <c r="I39" t="n">
-        <v>5.735</v>
+        <v>5.752</v>
       </c>
       <c r="J39" t="n">
-        <v>6.653</v>
+        <v>6.717</v>
       </c>
       <c r="K39" t="n">
-        <v>7.667</v>
+        <v>7.752</v>
       </c>
       <c r="L39" t="n">
-        <v>8.068</v>
+        <v>8.154999999999999</v>
       </c>
       <c r="M39" t="n">
-        <v>8.456</v>
+        <v>8.542999999999999</v>
       </c>
       <c r="N39" t="n">
-        <v>8.617000000000001</v>
+        <v>8.712999999999999</v>
       </c>
       <c r="O39" t="n">
-        <v>8.814</v>
+        <v>8.9</v>
       </c>
       <c r="P39" t="n">
-        <v>8.85</v>
+        <v>8.943</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.332000000000001</v>
+        <v>9.42</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.288</v>
+        <v>3.29</v>
       </c>
       <c r="G40" t="n">
-        <v>3.398</v>
+        <v>3.404</v>
       </c>
       <c r="H40" t="n">
-        <v>3.586</v>
+        <v>3.598</v>
       </c>
       <c r="I40" t="n">
-        <v>3.827</v>
+        <v>3.849</v>
       </c>
       <c r="J40" t="n">
-        <v>4.152</v>
+        <v>4.216</v>
       </c>
       <c r="K40" t="n">
-        <v>4.452</v>
+        <v>4.534</v>
       </c>
       <c r="L40" t="n">
-        <v>4.547</v>
+        <v>4.631</v>
       </c>
       <c r="M40" t="n">
-        <v>4.748</v>
+        <v>4.833</v>
       </c>
       <c r="N40" t="n">
-        <v>4.92</v>
+        <v>5.016</v>
       </c>
       <c r="O40" t="n">
-        <v>5.231</v>
+        <v>5.316</v>
       </c>
       <c r="P40" t="n">
-        <v>5.432</v>
+        <v>5.525</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.222</v>
+        <v>6.312</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.671</v>
+        <v>3.673</v>
       </c>
       <c r="G41" t="n">
-        <v>3.823</v>
+        <v>3.828</v>
       </c>
       <c r="H41" t="n">
-        <v>4.068</v>
+        <v>4.08</v>
       </c>
       <c r="I41" t="n">
-        <v>4.329</v>
+        <v>4.351</v>
       </c>
       <c r="J41" t="n">
-        <v>4.706</v>
+        <v>4.77</v>
       </c>
       <c r="K41" t="n">
-        <v>5.051</v>
+        <v>5.134</v>
       </c>
       <c r="L41" t="n">
-        <v>5.225</v>
+        <v>5.309</v>
       </c>
       <c r="M41" t="n">
-        <v>5.55</v>
+        <v>5.635</v>
       </c>
       <c r="N41" t="n">
-        <v>5.849</v>
+        <v>5.945</v>
       </c>
       <c r="O41" t="n">
-        <v>6.343</v>
+        <v>6.428</v>
       </c>
       <c r="P41" t="n">
-        <v>6.491</v>
+        <v>6.584</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.269</v>
+        <v>7.359</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.408</v>
+        <v>3.41</v>
       </c>
       <c r="G42" t="n">
-        <v>3.546</v>
+        <v>3.552</v>
       </c>
       <c r="H42" t="n">
-        <v>3.76</v>
+        <v>3.772</v>
       </c>
       <c r="I42" t="n">
-        <v>4.016</v>
+        <v>4.038</v>
       </c>
       <c r="J42" t="n">
-        <v>4.355</v>
+        <v>4.419</v>
       </c>
       <c r="K42" t="n">
-        <v>4.673</v>
+        <v>4.755</v>
       </c>
       <c r="L42" t="n">
-        <v>4.783</v>
+        <v>4.868</v>
       </c>
       <c r="M42" t="n">
-        <v>5.055</v>
+        <v>5.141</v>
       </c>
       <c r="N42" t="n">
-        <v>5.334</v>
+        <v>5.43</v>
       </c>
       <c r="O42" t="n">
-        <v>5.722</v>
+        <v>5.807</v>
       </c>
       <c r="P42" t="n">
-        <v>5.933</v>
+        <v>6.026</v>
       </c>
       <c r="Q42" t="n">
-        <v>6.735</v>
+        <v>6.825</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.118</v>
+        <v>3.12</v>
       </c>
       <c r="G43" t="n">
-        <v>3.212</v>
+        <v>3.217</v>
       </c>
       <c r="H43" t="n">
-        <v>3.347</v>
+        <v>3.358</v>
       </c>
       <c r="I43" t="n">
-        <v>3.546</v>
+        <v>3.566</v>
       </c>
       <c r="J43" t="n">
-        <v>3.799</v>
+        <v>3.86</v>
       </c>
       <c r="K43" t="n">
-        <v>4.02</v>
+        <v>4.104</v>
       </c>
       <c r="L43" t="n">
-        <v>4.07</v>
+        <v>4.156</v>
       </c>
       <c r="M43" t="n">
-        <v>4.194</v>
+        <v>4.28</v>
       </c>
       <c r="N43" t="n">
-        <v>4.222</v>
+        <v>4.318</v>
       </c>
       <c r="O43" t="n">
-        <v>4.32</v>
+        <v>4.406</v>
       </c>
       <c r="P43" t="n">
-        <v>4.408</v>
+        <v>4.501</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.098</v>
+        <v>5.188</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46134</v>
+        <v>46135</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>2.99</v>
+        <v>2.992</v>
       </c>
       <c r="G44" t="n">
-        <v>3.08</v>
+        <v>3.084</v>
       </c>
       <c r="H44" t="n">
-        <v>3.198</v>
+        <v>3.207</v>
       </c>
       <c r="I44" t="n">
-        <v>3.392</v>
+        <v>3.412</v>
       </c>
       <c r="J44" t="n">
-        <v>3.647</v>
+        <v>3.71</v>
       </c>
       <c r="K44" t="n">
-        <v>3.863</v>
+        <v>3.947</v>
       </c>
       <c r="L44" t="n">
-        <v>3.913</v>
+        <v>3.998</v>
       </c>
       <c r="M44" t="n">
-        <v>4.008</v>
+        <v>4.095</v>
       </c>
       <c r="N44" t="n">
-        <v>4.037</v>
+        <v>4.133</v>
       </c>
       <c r="O44" t="n">
-        <v>4.117</v>
+        <v>4.202</v>
       </c>
       <c r="P44" t="n">
-        <v>4.171</v>
+        <v>4.265</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.469</v>
+        <v>4.559</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-04-24 ~ 2026-04-24
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.211</v>
+        <v>3.209</v>
       </c>
       <c r="G2" t="n">
-        <v>3.418</v>
+        <v>3.417</v>
       </c>
       <c r="H2" t="n">
         <v>3.584</v>
       </c>
       <c r="I2" t="n">
-        <v>3.787</v>
+        <v>3.785</v>
       </c>
       <c r="J2" t="n">
-        <v>4.084</v>
+        <v>4.108</v>
       </c>
       <c r="K2" t="n">
-        <v>4.482</v>
+        <v>4.516</v>
       </c>
       <c r="L2" t="n">
-        <v>4.653</v>
+        <v>4.7</v>
       </c>
       <c r="M2" t="n">
-        <v>4.958</v>
+        <v>4.993</v>
       </c>
       <c r="N2" t="n">
-        <v>5.225</v>
+        <v>5.259</v>
       </c>
       <c r="O2" t="n">
-        <v>5.454</v>
+        <v>5.483</v>
       </c>
       <c r="P2" t="n">
-        <v>5.627</v>
+        <v>5.657</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.257</v>
+        <v>6.285</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.234</v>
+        <v>4.232</v>
       </c>
       <c r="G3" t="n">
-        <v>4.623</v>
+        <v>4.621</v>
       </c>
       <c r="H3" t="n">
         <v>4.822</v>
       </c>
       <c r="I3" t="n">
-        <v>5.021</v>
+        <v>5.019</v>
       </c>
       <c r="J3" t="n">
-        <v>5.33</v>
+        <v>5.353</v>
       </c>
       <c r="K3" t="n">
-        <v>5.798</v>
+        <v>5.831</v>
       </c>
       <c r="L3" t="n">
-        <v>6.039</v>
+        <v>6.085</v>
       </c>
       <c r="M3" t="n">
-        <v>6.375</v>
+        <v>6.411</v>
       </c>
       <c r="N3" t="n">
-        <v>6.585</v>
+        <v>6.619</v>
       </c>
       <c r="O3" t="n">
-        <v>6.764</v>
+        <v>6.792</v>
       </c>
       <c r="P3" t="n">
-        <v>6.807</v>
+        <v>6.837</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.325</v>
+        <v>7.353</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.727</v>
+        <v>3.725</v>
       </c>
       <c r="G4" t="n">
-        <v>4.004</v>
+        <v>4.002</v>
       </c>
       <c r="H4" t="n">
         <v>4.232</v>
       </c>
       <c r="I4" t="n">
-        <v>4.464</v>
+        <v>4.462</v>
       </c>
       <c r="J4" t="n">
-        <v>4.778</v>
+        <v>4.801</v>
       </c>
       <c r="K4" t="n">
-        <v>5.238</v>
+        <v>5.271</v>
       </c>
       <c r="L4" t="n">
-        <v>5.409</v>
+        <v>5.455</v>
       </c>
       <c r="M4" t="n">
-        <v>5.733</v>
+        <v>5.768</v>
       </c>
       <c r="N4" t="n">
-        <v>5.913</v>
+        <v>5.947</v>
       </c>
       <c r="O4" t="n">
-        <v>6.116</v>
+        <v>6.145</v>
       </c>
       <c r="P4" t="n">
-        <v>6.157</v>
+        <v>6.187</v>
       </c>
       <c r="Q4" t="n">
-        <v>6.678</v>
+        <v>6.706</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.906</v>
+        <v>2.903</v>
       </c>
       <c r="G5" t="n">
-        <v>2.959</v>
+        <v>2.956</v>
       </c>
       <c r="H5" t="n">
-        <v>3.082</v>
+        <v>3.081</v>
       </c>
       <c r="I5" t="n">
-        <v>3.357</v>
+        <v>3.354</v>
       </c>
       <c r="J5" t="n">
-        <v>3.645</v>
+        <v>3.668</v>
       </c>
       <c r="K5" t="n">
-        <v>3.902</v>
+        <v>3.934</v>
       </c>
       <c r="L5" t="n">
-        <v>3.916</v>
+        <v>3.961</v>
       </c>
       <c r="M5" t="n">
-        <v>4.022</v>
+        <v>4.057</v>
       </c>
       <c r="N5" t="n">
-        <v>4.042</v>
+        <v>4.075</v>
       </c>
       <c r="O5" t="n">
-        <v>4.053</v>
+        <v>4.081</v>
       </c>
       <c r="P5" t="n">
-        <v>4.296</v>
+        <v>4.326</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.169</v>
+        <v>5.197</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2.945</v>
+        <v>2.943</v>
       </c>
       <c r="G6" t="n">
-        <v>3.012</v>
+        <v>3.01</v>
       </c>
       <c r="H6" t="n">
         <v>3.152</v>
       </c>
       <c r="I6" t="n">
-        <v>3.439</v>
+        <v>3.436</v>
       </c>
       <c r="J6" t="n">
-        <v>3.734</v>
+        <v>3.756</v>
       </c>
       <c r="K6" t="n">
-        <v>4.012</v>
+        <v>4.046</v>
       </c>
       <c r="L6" t="n">
-        <v>4.035</v>
+        <v>4.08</v>
       </c>
       <c r="M6" t="n">
-        <v>4.181</v>
+        <v>4.215</v>
       </c>
       <c r="N6" t="n">
-        <v>4.209</v>
+        <v>4.243</v>
       </c>
       <c r="O6" t="n">
-        <v>4.321</v>
+        <v>4.35</v>
       </c>
       <c r="P6" t="n">
-        <v>4.728</v>
+        <v>4.758</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.565</v>
+        <v>5.593</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2.926</v>
+        <v>2.924</v>
       </c>
       <c r="G7" t="n">
-        <v>2.976</v>
+        <v>2.974</v>
       </c>
       <c r="H7" t="n">
         <v>3.097</v>
       </c>
       <c r="I7" t="n">
-        <v>3.372</v>
+        <v>3.369</v>
       </c>
       <c r="J7" t="n">
-        <v>3.671</v>
+        <v>3.693</v>
       </c>
       <c r="K7" t="n">
-        <v>3.929</v>
+        <v>3.961</v>
       </c>
       <c r="L7" t="n">
-        <v>3.941</v>
+        <v>3.986</v>
       </c>
       <c r="M7" t="n">
-        <v>4.085</v>
+        <v>4.119</v>
       </c>
       <c r="N7" t="n">
-        <v>4.102</v>
+        <v>4.136</v>
       </c>
       <c r="O7" t="n">
-        <v>4.218</v>
+        <v>4.247</v>
       </c>
       <c r="P7" t="n">
-        <v>4.512</v>
+        <v>4.542</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.333</v>
+        <v>5.361</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,10 +990,10 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.343</v>
+        <v>5.342</v>
       </c>
       <c r="G8" t="n">
-        <v>5.921</v>
+        <v>5.919</v>
       </c>
       <c r="H8" t="n">
         <v>6.271</v>
@@ -1002,28 +1002,28 @@
         <v>6.546</v>
       </c>
       <c r="J8" t="n">
-        <v>6.919</v>
+        <v>6.944</v>
       </c>
       <c r="K8" t="n">
-        <v>7.666</v>
+        <v>7.702</v>
       </c>
       <c r="L8" t="n">
-        <v>7.996</v>
+        <v>8.042999999999999</v>
       </c>
       <c r="M8" t="n">
-        <v>8.363</v>
+        <v>8.398999999999999</v>
       </c>
       <c r="N8" t="n">
-        <v>8.507999999999999</v>
+        <v>8.542</v>
       </c>
       <c r="O8" t="n">
-        <v>8.773</v>
+        <v>8.801</v>
       </c>
       <c r="P8" t="n">
-        <v>8.917999999999999</v>
+        <v>8.948</v>
       </c>
       <c r="Q8" t="n">
-        <v>9.634</v>
+        <v>9.662000000000001</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1066,54 +1066,54 @@
         <v>2.623</v>
       </c>
       <c r="G9" t="n">
-        <v>2.694</v>
+        <v>2.703</v>
       </c>
       <c r="H9" t="n">
-        <v>2.801</v>
+        <v>2.809</v>
       </c>
       <c r="I9" t="n">
-        <v>2.963</v>
+        <v>2.985</v>
       </c>
       <c r="J9" t="n">
-        <v>3.194</v>
+        <v>3.227</v>
       </c>
       <c r="K9" t="n">
-        <v>3.331</v>
+        <v>3.383</v>
       </c>
       <c r="L9" t="n">
-        <v>3.365</v>
+        <v>3.418</v>
       </c>
       <c r="M9" t="n">
-        <v>3.453</v>
+        <v>3.495</v>
       </c>
       <c r="N9" t="n">
-        <v>3.615</v>
+        <v>3.652</v>
       </c>
       <c r="O9" t="n">
-        <v>3.65</v>
+        <v>3.681</v>
       </c>
       <c r="P9" t="n">
-        <v>3.718</v>
+        <v>3.748</v>
       </c>
       <c r="Q9" t="n">
-        <v>3.787</v>
+        <v>3.815</v>
       </c>
       <c r="R9" t="n">
-        <v>3.759</v>
+        <v>3.786</v>
       </c>
       <c r="S9" t="n">
-        <v>3.729</v>
+        <v>3.755</v>
       </c>
       <c r="T9" t="n">
-        <v>3.65</v>
+        <v>3.671</v>
       </c>
       <c r="U9" t="n">
-        <v>3.522</v>
+        <v>3.543</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1139,31 +1139,31 @@
         <v>2.636</v>
       </c>
       <c r="G10" t="n">
-        <v>2.728</v>
+        <v>2.738</v>
       </c>
       <c r="H10" t="n">
-        <v>2.816</v>
+        <v>2.825</v>
       </c>
       <c r="I10" t="n">
-        <v>2.976</v>
+        <v>2.996</v>
       </c>
       <c r="J10" t="n">
-        <v>3.219</v>
+        <v>3.253</v>
       </c>
       <c r="K10" t="n">
-        <v>3.364</v>
+        <v>3.417</v>
       </c>
       <c r="L10" t="n">
-        <v>3.415</v>
+        <v>3.47</v>
       </c>
       <c r="M10" t="n">
-        <v>3.55</v>
+        <v>3.591</v>
       </c>
       <c r="N10" t="n">
-        <v>3.628</v>
+        <v>3.668</v>
       </c>
       <c r="O10" t="n">
-        <v>3.864</v>
+        <v>3.908</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1212,37 +1212,37 @@
         <v>2.452</v>
       </c>
       <c r="G11" t="n">
-        <v>2.538</v>
+        <v>2.548</v>
       </c>
       <c r="H11" t="n">
-        <v>2.64</v>
+        <v>2.649</v>
       </c>
       <c r="I11" t="n">
-        <v>2.779</v>
+        <v>2.799</v>
       </c>
       <c r="J11" t="n">
-        <v>3.014</v>
+        <v>3.047</v>
       </c>
       <c r="K11" t="n">
-        <v>3.152</v>
+        <v>3.204</v>
       </c>
       <c r="L11" t="n">
-        <v>3.209</v>
+        <v>3.264</v>
       </c>
       <c r="M11" t="n">
-        <v>3.356</v>
+        <v>3.397</v>
       </c>
       <c r="N11" t="n">
-        <v>3.437</v>
+        <v>3.476</v>
       </c>
       <c r="O11" t="n">
-        <v>3.631</v>
+        <v>3.674</v>
       </c>
       <c r="P11" t="n">
-        <v>3.664</v>
+        <v>3.695</v>
       </c>
       <c r="Q11" t="n">
-        <v>3.988</v>
+        <v>4.016</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1285,43 +1285,43 @@
         <v>3.193</v>
       </c>
       <c r="G12" t="n">
-        <v>3.349</v>
+        <v>3.348</v>
       </c>
       <c r="H12" t="n">
-        <v>3.458</v>
+        <v>3.461</v>
       </c>
       <c r="I12" t="n">
-        <v>3.696</v>
+        <v>3.704</v>
       </c>
       <c r="J12" t="n">
-        <v>4.051</v>
+        <v>4.079</v>
       </c>
       <c r="K12" t="n">
-        <v>4.249</v>
+        <v>4.286</v>
       </c>
       <c r="L12" t="n">
-        <v>4.309</v>
+        <v>4.357</v>
       </c>
       <c r="M12" t="n">
-        <v>4.454</v>
+        <v>4.493</v>
       </c>
       <c r="N12" t="n">
-        <v>4.501</v>
+        <v>4.538</v>
       </c>
       <c r="O12" t="n">
-        <v>4.651</v>
+        <v>4.683</v>
       </c>
       <c r="P12" t="n">
-        <v>4.763</v>
+        <v>4.793</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.116</v>
+        <v>5.144</v>
       </c>
       <c r="R12" t="n">
-        <v>5.26</v>
+        <v>5.286</v>
       </c>
       <c r="S12" t="n">
-        <v>5.44</v>
+        <v>5.465</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1358,43 +1358,43 @@
         <v>2.947</v>
       </c>
       <c r="G13" t="n">
-        <v>3.039</v>
+        <v>3.038</v>
       </c>
       <c r="H13" t="n">
-        <v>3.126</v>
+        <v>3.129</v>
       </c>
       <c r="I13" t="n">
-        <v>3.344</v>
+        <v>3.352</v>
       </c>
       <c r="J13" t="n">
-        <v>3.688</v>
+        <v>3.716</v>
       </c>
       <c r="K13" t="n">
-        <v>3.882</v>
+        <v>3.919</v>
       </c>
       <c r="L13" t="n">
-        <v>3.949</v>
+        <v>3.997</v>
       </c>
       <c r="M13" t="n">
-        <v>4.081</v>
+        <v>4.12</v>
       </c>
       <c r="N13" t="n">
-        <v>4.13</v>
+        <v>4.166</v>
       </c>
       <c r="O13" t="n">
-        <v>4.279</v>
+        <v>4.311</v>
       </c>
       <c r="P13" t="n">
-        <v>4.354</v>
+        <v>4.385</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.636</v>
+        <v>4.664</v>
       </c>
       <c r="R13" t="n">
-        <v>4.808</v>
+        <v>4.834</v>
       </c>
       <c r="S13" t="n">
-        <v>5.003</v>
+        <v>5.028</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1434,40 +1434,40 @@
         <v>2.844</v>
       </c>
       <c r="H14" t="n">
-        <v>2.929</v>
+        <v>2.932</v>
       </c>
       <c r="I14" t="n">
-        <v>3.127</v>
+        <v>3.136</v>
       </c>
       <c r="J14" t="n">
-        <v>3.428</v>
+        <v>3.457</v>
       </c>
       <c r="K14" t="n">
-        <v>3.57</v>
+        <v>3.607</v>
       </c>
       <c r="L14" t="n">
-        <v>3.621</v>
+        <v>3.668</v>
       </c>
       <c r="M14" t="n">
-        <v>3.767</v>
+        <v>3.805</v>
       </c>
       <c r="N14" t="n">
-        <v>3.809</v>
+        <v>3.845</v>
       </c>
       <c r="O14" t="n">
-        <v>3.935</v>
+        <v>3.966</v>
       </c>
       <c r="P14" t="n">
-        <v>3.989</v>
+        <v>4.02</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.225</v>
+        <v>4.253</v>
       </c>
       <c r="R14" t="n">
-        <v>4.323</v>
+        <v>4.35</v>
       </c>
       <c r="S14" t="n">
-        <v>4.455</v>
+        <v>4.481</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1504,43 +1504,43 @@
         <v>2.744</v>
       </c>
       <c r="G15" t="n">
-        <v>2.819</v>
+        <v>2.818</v>
       </c>
       <c r="H15" t="n">
-        <v>2.898</v>
+        <v>2.901</v>
       </c>
       <c r="I15" t="n">
-        <v>3.08</v>
+        <v>3.088</v>
       </c>
       <c r="J15" t="n">
-        <v>3.367</v>
+        <v>3.396</v>
       </c>
       <c r="K15" t="n">
-        <v>3.523</v>
+        <v>3.56</v>
       </c>
       <c r="L15" t="n">
-        <v>3.556</v>
+        <v>3.604</v>
       </c>
       <c r="M15" t="n">
-        <v>3.68</v>
+        <v>3.719</v>
       </c>
       <c r="N15" t="n">
-        <v>3.713</v>
+        <v>3.749</v>
       </c>
       <c r="O15" t="n">
-        <v>3.864</v>
+        <v>3.905</v>
       </c>
       <c r="P15" t="n">
-        <v>3.888</v>
+        <v>3.92</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.13</v>
+        <v>4.158</v>
       </c>
       <c r="R15" t="n">
-        <v>4.219</v>
+        <v>4.246</v>
       </c>
       <c r="S15" t="n">
-        <v>4.351</v>
+        <v>4.376</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1577,43 +1577,43 @@
         <v>2.744</v>
       </c>
       <c r="G16" t="n">
-        <v>2.819</v>
+        <v>2.818</v>
       </c>
       <c r="H16" t="n">
-        <v>2.898</v>
+        <v>2.901</v>
       </c>
       <c r="I16" t="n">
-        <v>3.08</v>
+        <v>3.088</v>
       </c>
       <c r="J16" t="n">
-        <v>3.367</v>
+        <v>3.396</v>
       </c>
       <c r="K16" t="n">
-        <v>3.523</v>
+        <v>3.56</v>
       </c>
       <c r="L16" t="n">
-        <v>3.556</v>
+        <v>3.604</v>
       </c>
       <c r="M16" t="n">
-        <v>3.68</v>
+        <v>3.719</v>
       </c>
       <c r="N16" t="n">
-        <v>3.716</v>
+        <v>3.752</v>
       </c>
       <c r="O16" t="n">
-        <v>3.871</v>
+        <v>3.911</v>
       </c>
       <c r="P16" t="n">
-        <v>3.912</v>
+        <v>3.943</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.157</v>
+        <v>4.185</v>
       </c>
       <c r="R16" t="n">
-        <v>4.247</v>
+        <v>4.274</v>
       </c>
       <c r="S16" t="n">
-        <v>4.38</v>
+        <v>4.405</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1650,34 +1650,34 @@
         <v>2.699</v>
       </c>
       <c r="G17" t="n">
-        <v>2.817</v>
+        <v>2.828</v>
       </c>
       <c r="H17" t="n">
-        <v>2.91</v>
+        <v>2.918</v>
       </c>
       <c r="I17" t="n">
-        <v>3.058</v>
+        <v>3.078</v>
       </c>
       <c r="J17" t="n">
-        <v>3.29</v>
+        <v>3.324</v>
       </c>
       <c r="K17" t="n">
-        <v>3.439</v>
+        <v>3.493</v>
       </c>
       <c r="L17" t="n">
-        <v>3.493</v>
+        <v>3.549</v>
       </c>
       <c r="M17" t="n">
-        <v>3.67</v>
+        <v>3.711</v>
       </c>
       <c r="N17" t="n">
-        <v>3.729</v>
+        <v>3.769</v>
       </c>
       <c r="O17" t="n">
-        <v>3.892</v>
+        <v>3.935</v>
       </c>
       <c r="P17" t="n">
-        <v>3.936</v>
+        <v>3.969</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1723,31 +1723,31 @@
         <v>2.7</v>
       </c>
       <c r="G18" t="n">
-        <v>2.818</v>
+        <v>2.829</v>
       </c>
       <c r="H18" t="n">
-        <v>2.91</v>
+        <v>2.918</v>
       </c>
       <c r="I18" t="n">
-        <v>3.058</v>
+        <v>3.078</v>
       </c>
       <c r="J18" t="n">
-        <v>3.29</v>
+        <v>3.324</v>
       </c>
       <c r="K18" t="n">
-        <v>3.44</v>
+        <v>3.494</v>
       </c>
       <c r="L18" t="n">
-        <v>3.493</v>
+        <v>3.549</v>
       </c>
       <c r="M18" t="n">
-        <v>3.67</v>
+        <v>3.711</v>
       </c>
       <c r="N18" t="n">
-        <v>3.73</v>
+        <v>3.77</v>
       </c>
       <c r="O18" t="n">
-        <v>3.89</v>
+        <v>3.934</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1796,43 +1796,43 @@
         <v>2.757</v>
       </c>
       <c r="G19" t="n">
-        <v>2.836</v>
+        <v>2.835</v>
       </c>
       <c r="H19" t="n">
-        <v>2.919</v>
+        <v>2.921</v>
       </c>
       <c r="I19" t="n">
-        <v>3.114</v>
+        <v>3.123</v>
       </c>
       <c r="J19" t="n">
-        <v>3.412</v>
+        <v>3.44</v>
       </c>
       <c r="K19" t="n">
-        <v>3.567</v>
+        <v>3.604</v>
       </c>
       <c r="L19" t="n">
-        <v>3.618</v>
+        <v>3.665</v>
       </c>
       <c r="M19" t="n">
-        <v>3.758</v>
+        <v>3.797</v>
       </c>
       <c r="N19" t="n">
-        <v>3.796</v>
+        <v>3.833</v>
       </c>
       <c r="O19" t="n">
-        <v>3.915</v>
+        <v>3.95</v>
       </c>
       <c r="P19" t="n">
-        <v>3.95</v>
+        <v>3.98</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.173</v>
+        <v>4.2</v>
       </c>
       <c r="R19" t="n">
-        <v>4.271</v>
+        <v>4.297</v>
       </c>
       <c r="S19" t="n">
-        <v>4.394</v>
+        <v>4.419</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1878,16 +1878,16 @@
         <v>2.834</v>
       </c>
       <c r="J20" t="n">
-        <v>3.19</v>
+        <v>3.22</v>
       </c>
       <c r="K20" t="n">
-        <v>3.354</v>
+        <v>3.397</v>
       </c>
       <c r="L20" t="n">
-        <v>3.397</v>
+        <v>3.439</v>
       </c>
       <c r="M20" t="n">
-        <v>3.498</v>
+        <v>3.54</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1942,43 +1942,43 @@
         <v>2.866</v>
       </c>
       <c r="G21" t="n">
-        <v>2.943</v>
+        <v>2.942</v>
       </c>
       <c r="H21" t="n">
-        <v>3.065</v>
+        <v>3.071</v>
       </c>
       <c r="I21" t="n">
-        <v>3.237</v>
+        <v>3.245</v>
       </c>
       <c r="J21" t="n">
-        <v>3.547</v>
+        <v>3.578</v>
       </c>
       <c r="K21" t="n">
-        <v>3.807</v>
+        <v>3.841</v>
       </c>
       <c r="L21" t="n">
-        <v>3.864</v>
+        <v>3.907</v>
       </c>
       <c r="M21" t="n">
-        <v>4.003</v>
+        <v>4.036</v>
       </c>
       <c r="N21" t="n">
-        <v>4.058</v>
+        <v>4.088</v>
       </c>
       <c r="O21" t="n">
-        <v>4.138</v>
+        <v>4.166</v>
       </c>
       <c r="P21" t="n">
-        <v>4.215</v>
+        <v>4.246</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.338</v>
+        <v>4.366</v>
       </c>
       <c r="R21" t="n">
-        <v>4.321</v>
+        <v>4.349</v>
       </c>
       <c r="S21" t="n">
-        <v>4.354</v>
+        <v>4.38</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2015,43 +2015,43 @@
         <v>2.813</v>
       </c>
       <c r="G22" t="n">
-        <v>2.89</v>
+        <v>2.888</v>
       </c>
       <c r="H22" t="n">
-        <v>2.997</v>
+        <v>3.003</v>
       </c>
       <c r="I22" t="n">
-        <v>3.157</v>
+        <v>3.165</v>
       </c>
       <c r="J22" t="n">
-        <v>3.431</v>
+        <v>3.462</v>
       </c>
       <c r="K22" t="n">
-        <v>3.687</v>
+        <v>3.72</v>
       </c>
       <c r="L22" t="n">
-        <v>3.732</v>
+        <v>3.775</v>
       </c>
       <c r="M22" t="n">
-        <v>3.872</v>
+        <v>3.906</v>
       </c>
       <c r="N22" t="n">
-        <v>3.93</v>
+        <v>3.961</v>
       </c>
       <c r="O22" t="n">
-        <v>4.006</v>
+        <v>4.034</v>
       </c>
       <c r="P22" t="n">
-        <v>4.078</v>
+        <v>4.108</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.196</v>
+        <v>4.224</v>
       </c>
       <c r="R22" t="n">
-        <v>4.169</v>
+        <v>4.197</v>
       </c>
       <c r="S22" t="n">
-        <v>4.2</v>
+        <v>4.225</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2088,46 +2088,46 @@
         <v>2.766</v>
       </c>
       <c r="G23" t="n">
-        <v>2.844</v>
+        <v>2.843</v>
       </c>
       <c r="H23" t="n">
-        <v>2.937</v>
+        <v>2.942</v>
       </c>
       <c r="I23" t="n">
-        <v>3.11</v>
+        <v>3.118</v>
       </c>
       <c r="J23" t="n">
-        <v>3.376</v>
+        <v>3.407</v>
       </c>
       <c r="K23" t="n">
-        <v>3.6</v>
+        <v>3.633</v>
       </c>
       <c r="L23" t="n">
-        <v>3.643</v>
+        <v>3.686</v>
       </c>
       <c r="M23" t="n">
-        <v>3.776</v>
+        <v>3.81</v>
       </c>
       <c r="N23" t="n">
-        <v>3.827</v>
+        <v>3.857</v>
       </c>
       <c r="O23" t="n">
-        <v>3.881</v>
+        <v>3.91</v>
       </c>
       <c r="P23" t="n">
-        <v>3.939</v>
+        <v>3.969</v>
       </c>
       <c r="Q23" t="n">
-        <v>4.004</v>
+        <v>4.031</v>
       </c>
       <c r="R23" t="n">
-        <v>3.953</v>
+        <v>3.98</v>
       </c>
       <c r="S23" t="n">
-        <v>3.954</v>
+        <v>3.979</v>
       </c>
       <c r="T23" t="n">
-        <v>3.865</v>
+        <v>3.887</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2161,43 +2161,43 @@
         <v>2.701</v>
       </c>
       <c r="G24" t="n">
-        <v>2.759</v>
+        <v>2.757</v>
       </c>
       <c r="H24" t="n">
-        <v>2.838</v>
+        <v>2.843</v>
       </c>
       <c r="I24" t="n">
-        <v>3.02</v>
+        <v>3.028</v>
       </c>
       <c r="J24" t="n">
-        <v>3.275</v>
+        <v>3.306</v>
       </c>
       <c r="K24" t="n">
-        <v>3.484</v>
+        <v>3.517</v>
       </c>
       <c r="L24" t="n">
-        <v>3.517</v>
+        <v>3.56</v>
       </c>
       <c r="M24" t="n">
-        <v>3.636</v>
+        <v>3.669</v>
       </c>
       <c r="N24" t="n">
-        <v>3.7</v>
+        <v>3.734</v>
       </c>
       <c r="O24" t="n">
-        <v>3.859</v>
+        <v>3.902</v>
       </c>
       <c r="P24" t="n">
-        <v>3.88</v>
+        <v>3.913</v>
       </c>
       <c r="Q24" t="n">
-        <v>3.926</v>
+        <v>3.954</v>
       </c>
       <c r="R24" t="n">
-        <v>3.874</v>
+        <v>3.901</v>
       </c>
       <c r="S24" t="n">
-        <v>3.869</v>
+        <v>3.895</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2234,46 +2234,46 @@
         <v>2.759</v>
       </c>
       <c r="G25" t="n">
-        <v>2.844</v>
+        <v>2.842</v>
       </c>
       <c r="H25" t="n">
-        <v>2.94</v>
+        <v>2.945</v>
       </c>
       <c r="I25" t="n">
-        <v>3.118</v>
+        <v>3.126</v>
       </c>
       <c r="J25" t="n">
-        <v>3.392</v>
+        <v>3.422</v>
       </c>
       <c r="K25" t="n">
-        <v>3.633</v>
+        <v>3.665</v>
       </c>
       <c r="L25" t="n">
-        <v>3.672</v>
+        <v>3.716</v>
       </c>
       <c r="M25" t="n">
-        <v>3.807</v>
+        <v>3.84</v>
       </c>
       <c r="N25" t="n">
-        <v>3.854</v>
+        <v>3.884</v>
       </c>
       <c r="O25" t="n">
-        <v>3.91</v>
+        <v>3.939</v>
       </c>
       <c r="P25" t="n">
-        <v>3.961</v>
+        <v>3.991</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.037</v>
+        <v>4.064</v>
       </c>
       <c r="R25" t="n">
-        <v>3.976</v>
+        <v>4.004</v>
       </c>
       <c r="S25" t="n">
-        <v>3.977</v>
+        <v>4.003</v>
       </c>
       <c r="T25" t="n">
-        <v>3.884</v>
+        <v>3.905</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.064</v>
+        <v>3.062</v>
       </c>
       <c r="G26" t="n">
-        <v>3.195</v>
+        <v>3.194</v>
       </c>
       <c r="H26" t="n">
-        <v>3.405</v>
+        <v>3.41</v>
       </c>
       <c r="I26" t="n">
-        <v>3.647</v>
+        <v>3.65</v>
       </c>
       <c r="J26" t="n">
-        <v>4.055</v>
+        <v>4.083</v>
       </c>
       <c r="K26" t="n">
-        <v>4.438</v>
+        <v>4.476</v>
       </c>
       <c r="L26" t="n">
-        <v>4.539</v>
+        <v>4.588</v>
       </c>
       <c r="M26" t="n">
-        <v>4.731</v>
+        <v>4.77</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>4.987</v>
+        <v>5.018</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2380,31 +2380,31 @@
         <v>2.857</v>
       </c>
       <c r="G27" t="n">
-        <v>2.926</v>
+        <v>2.925</v>
       </c>
       <c r="H27" t="n">
-        <v>3.036</v>
+        <v>3.041</v>
       </c>
       <c r="I27" t="n">
-        <v>3.239</v>
+        <v>3.246</v>
       </c>
       <c r="J27" t="n">
-        <v>3.552</v>
+        <v>3.581</v>
       </c>
       <c r="K27" t="n">
-        <v>3.75</v>
+        <v>3.786</v>
       </c>
       <c r="L27" t="n">
-        <v>3.804</v>
+        <v>3.851</v>
       </c>
       <c r="M27" t="n">
-        <v>3.937</v>
+        <v>3.976</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.078</v>
+        <v>4.11</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2453,31 +2453,31 @@
         <v>2.96</v>
       </c>
       <c r="G28" t="n">
-        <v>3.037</v>
+        <v>3.036</v>
       </c>
       <c r="H28" t="n">
-        <v>3.162</v>
+        <v>3.167</v>
       </c>
       <c r="I28" t="n">
-        <v>3.377</v>
+        <v>3.384</v>
       </c>
       <c r="J28" t="n">
-        <v>3.725</v>
+        <v>3.754</v>
       </c>
       <c r="K28" t="n">
-        <v>3.942</v>
+        <v>3.979</v>
       </c>
       <c r="L28" t="n">
-        <v>4.008</v>
+        <v>4.055</v>
       </c>
       <c r="M28" t="n">
-        <v>4.149</v>
+        <v>4.188</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.372</v>
+        <v>4.404</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2526,31 +2526,31 @@
         <v>2.813</v>
       </c>
       <c r="G29" t="n">
-        <v>2.883</v>
+        <v>2.882</v>
       </c>
       <c r="H29" t="n">
-        <v>2.98</v>
+        <v>2.982</v>
       </c>
       <c r="I29" t="n">
-        <v>3.173</v>
+        <v>3.18</v>
       </c>
       <c r="J29" t="n">
-        <v>3.464</v>
+        <v>3.493</v>
       </c>
       <c r="K29" t="n">
-        <v>3.646</v>
+        <v>3.682</v>
       </c>
       <c r="L29" t="n">
-        <v>3.689</v>
+        <v>3.736</v>
       </c>
       <c r="M29" t="n">
-        <v>3.799</v>
+        <v>3.838</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>3.941</v>
+        <v>3.976</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2602,34 +2602,34 @@
         <v>3.165</v>
       </c>
       <c r="H30" t="n">
-        <v>3.338</v>
+        <v>3.348</v>
       </c>
       <c r="I30" t="n">
-        <v>3.574</v>
+        <v>3.58</v>
       </c>
       <c r="J30" t="n">
-        <v>3.923</v>
+        <v>3.953</v>
       </c>
       <c r="K30" t="n">
-        <v>4.229</v>
+        <v>4.269</v>
       </c>
       <c r="L30" t="n">
-        <v>4.307</v>
+        <v>4.357</v>
       </c>
       <c r="M30" t="n">
-        <v>4.492</v>
+        <v>4.532</v>
       </c>
       <c r="N30" t="n">
-        <v>4.658</v>
+        <v>4.696</v>
       </c>
       <c r="O30" t="n">
-        <v>4.938</v>
+        <v>4.969</v>
       </c>
       <c r="P30" t="n">
-        <v>5.104</v>
+        <v>5.133</v>
       </c>
       <c r="Q30" t="n">
-        <v>5.861</v>
+        <v>5.889</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2675,34 +2675,34 @@
         <v>3.525</v>
       </c>
       <c r="H31" t="n">
-        <v>3.75</v>
+        <v>3.759</v>
       </c>
       <c r="I31" t="n">
-        <v>4.002</v>
+        <v>4.008</v>
       </c>
       <c r="J31" t="n">
-        <v>4.413</v>
+        <v>4.443</v>
       </c>
       <c r="K31" t="n">
-        <v>4.762</v>
+        <v>4.801</v>
       </c>
       <c r="L31" t="n">
-        <v>4.919</v>
+        <v>4.968</v>
       </c>
       <c r="M31" t="n">
-        <v>5.222</v>
+        <v>5.262</v>
       </c>
       <c r="N31" t="n">
-        <v>5.515</v>
+        <v>5.553</v>
       </c>
       <c r="O31" t="n">
-        <v>5.971</v>
+        <v>6.003</v>
       </c>
       <c r="P31" t="n">
-        <v>6.091</v>
+        <v>6.12</v>
       </c>
       <c r="Q31" t="n">
-        <v>6.834</v>
+        <v>6.863</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2748,34 +2748,34 @@
         <v>3.281</v>
       </c>
       <c r="H32" t="n">
-        <v>3.48</v>
+        <v>3.49</v>
       </c>
       <c r="I32" t="n">
-        <v>3.733</v>
+        <v>3.739</v>
       </c>
       <c r="J32" t="n">
-        <v>4.102</v>
+        <v>4.132</v>
       </c>
       <c r="K32" t="n">
-        <v>4.415</v>
+        <v>4.454</v>
       </c>
       <c r="L32" t="n">
-        <v>4.512</v>
+        <v>4.561</v>
       </c>
       <c r="M32" t="n">
-        <v>4.765</v>
+        <v>4.805</v>
       </c>
       <c r="N32" t="n">
-        <v>5.019</v>
+        <v>5.056</v>
       </c>
       <c r="O32" t="n">
-        <v>5.382</v>
+        <v>5.414</v>
       </c>
       <c r="P32" t="n">
-        <v>5.563</v>
+        <v>5.592</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.322</v>
+        <v>6.35</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2821,34 +2821,34 @@
         <v>3.034</v>
       </c>
       <c r="H33" t="n">
-        <v>3.158</v>
+        <v>3.166</v>
       </c>
       <c r="I33" t="n">
-        <v>3.357</v>
+        <v>3.362</v>
       </c>
       <c r="J33" t="n">
-        <v>3.632</v>
+        <v>3.661</v>
       </c>
       <c r="K33" t="n">
-        <v>3.873</v>
+        <v>3.911</v>
       </c>
       <c r="L33" t="n">
-        <v>3.914</v>
+        <v>3.964</v>
       </c>
       <c r="M33" t="n">
-        <v>4.027</v>
+        <v>4.066</v>
       </c>
       <c r="N33" t="n">
-        <v>4.049</v>
+        <v>4.087</v>
       </c>
       <c r="O33" t="n">
-        <v>4.093</v>
+        <v>4.125</v>
       </c>
       <c r="P33" t="n">
-        <v>4.136</v>
+        <v>4.165</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.578</v>
+        <v>4.606</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2894,34 +2894,34 @@
         <v>3.088</v>
       </c>
       <c r="H34" t="n">
-        <v>3.218</v>
+        <v>3.227</v>
       </c>
       <c r="I34" t="n">
-        <v>3.425</v>
+        <v>3.43</v>
       </c>
       <c r="J34" t="n">
-        <v>3.704</v>
+        <v>3.733</v>
       </c>
       <c r="K34" t="n">
-        <v>3.95</v>
+        <v>3.988</v>
       </c>
       <c r="L34" t="n">
-        <v>3.994</v>
+        <v>4.043</v>
       </c>
       <c r="M34" t="n">
-        <v>4.117</v>
+        <v>4.157</v>
       </c>
       <c r="N34" t="n">
-        <v>4.154</v>
+        <v>4.192</v>
       </c>
       <c r="O34" t="n">
-        <v>4.261</v>
+        <v>4.294</v>
       </c>
       <c r="P34" t="n">
-        <v>4.43</v>
+        <v>4.46</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.279</v>
+        <v>5.307</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2967,34 +2967,34 @@
         <v>3.061</v>
       </c>
       <c r="H35" t="n">
-        <v>3.186</v>
+        <v>3.195</v>
       </c>
       <c r="I35" t="n">
-        <v>3.391</v>
+        <v>3.396</v>
       </c>
       <c r="J35" t="n">
-        <v>3.672</v>
+        <v>3.701</v>
       </c>
       <c r="K35" t="n">
-        <v>3.904</v>
+        <v>3.942</v>
       </c>
       <c r="L35" t="n">
-        <v>3.948</v>
+        <v>3.998</v>
       </c>
       <c r="M35" t="n">
-        <v>4.064</v>
+        <v>4.104</v>
       </c>
       <c r="N35" t="n">
-        <v>4.09</v>
+        <v>4.128</v>
       </c>
       <c r="O35" t="n">
-        <v>4.159</v>
+        <v>4.192</v>
       </c>
       <c r="P35" t="n">
-        <v>4.233</v>
+        <v>4.262</v>
       </c>
       <c r="Q35" t="n">
-        <v>4.915</v>
+        <v>4.943</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3040,34 +3040,34 @@
         <v>2.974</v>
       </c>
       <c r="H36" t="n">
-        <v>3.083</v>
+        <v>3.088</v>
       </c>
       <c r="I36" t="n">
-        <v>3.284</v>
+        <v>3.289</v>
       </c>
       <c r="J36" t="n">
-        <v>3.568</v>
+        <v>3.597</v>
       </c>
       <c r="K36" t="n">
-        <v>3.796</v>
+        <v>3.834</v>
       </c>
       <c r="L36" t="n">
-        <v>3.838</v>
+        <v>3.887</v>
       </c>
       <c r="M36" t="n">
-        <v>3.926</v>
+        <v>3.965</v>
       </c>
       <c r="N36" t="n">
-        <v>3.951</v>
+        <v>3.989</v>
       </c>
       <c r="O36" t="n">
-        <v>4.003</v>
+        <v>4.035</v>
       </c>
       <c r="P36" t="n">
-        <v>4.035</v>
+        <v>4.064</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.295</v>
+        <v>4.323</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3113,34 +3113,34 @@
         <v>4.22</v>
       </c>
       <c r="H37" t="n">
-        <v>4.726</v>
+        <v>4.734</v>
       </c>
       <c r="I37" t="n">
-        <v>5.068</v>
+        <v>5.073</v>
       </c>
       <c r="J37" t="n">
-        <v>5.904</v>
+        <v>5.934</v>
       </c>
       <c r="K37" t="n">
-        <v>6.802</v>
+        <v>6.841</v>
       </c>
       <c r="L37" t="n">
-        <v>7.119</v>
+        <v>7.168</v>
       </c>
       <c r="M37" t="n">
-        <v>7.497</v>
+        <v>7.535</v>
       </c>
       <c r="N37" t="n">
-        <v>7.667</v>
+        <v>7.703</v>
       </c>
       <c r="O37" t="n">
-        <v>7.85</v>
+        <v>7.882</v>
       </c>
       <c r="P37" t="n">
-        <v>7.891</v>
+        <v>7.92</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.324</v>
+        <v>8.352</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3186,34 +3186,34 @@
         <v>5.531</v>
       </c>
       <c r="H38" t="n">
-        <v>6.25</v>
+        <v>6.258</v>
       </c>
       <c r="I38" t="n">
-        <v>6.748</v>
+        <v>6.753</v>
       </c>
       <c r="J38" t="n">
-        <v>7.844</v>
+        <v>7.874</v>
       </c>
       <c r="K38" t="n">
-        <v>8.919</v>
+        <v>8.959</v>
       </c>
       <c r="L38" t="n">
-        <v>9.397</v>
+        <v>9.446999999999999</v>
       </c>
       <c r="M38" t="n">
-        <v>9.906000000000001</v>
+        <v>9.945</v>
       </c>
       <c r="N38" t="n">
-        <v>10.085</v>
+        <v>10.121</v>
       </c>
       <c r="O38" t="n">
-        <v>10.25</v>
+        <v>10.281</v>
       </c>
       <c r="P38" t="n">
-        <v>10.289</v>
+        <v>10.318</v>
       </c>
       <c r="Q38" t="n">
-        <v>10.775</v>
+        <v>10.803</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3259,34 +3259,34 @@
         <v>4.729</v>
       </c>
       <c r="H39" t="n">
-        <v>5.315</v>
+        <v>5.323</v>
       </c>
       <c r="I39" t="n">
-        <v>5.752</v>
+        <v>5.757</v>
       </c>
       <c r="J39" t="n">
-        <v>6.717</v>
+        <v>6.747</v>
       </c>
       <c r="K39" t="n">
-        <v>7.752</v>
+        <v>7.792</v>
       </c>
       <c r="L39" t="n">
-        <v>8.154999999999999</v>
+        <v>8.204000000000001</v>
       </c>
       <c r="M39" t="n">
-        <v>8.542999999999999</v>
+        <v>8.581</v>
       </c>
       <c r="N39" t="n">
-        <v>8.712999999999999</v>
+        <v>8.747999999999999</v>
       </c>
       <c r="O39" t="n">
-        <v>8.9</v>
+        <v>8.930999999999999</v>
       </c>
       <c r="P39" t="n">
-        <v>8.943</v>
+        <v>8.972</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.42</v>
+        <v>9.448</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3332,34 +3332,34 @@
         <v>3.404</v>
       </c>
       <c r="H40" t="n">
-        <v>3.598</v>
+        <v>3.607</v>
       </c>
       <c r="I40" t="n">
-        <v>3.849</v>
+        <v>3.855</v>
       </c>
       <c r="J40" t="n">
-        <v>4.216</v>
+        <v>4.246</v>
       </c>
       <c r="K40" t="n">
-        <v>4.534</v>
+        <v>4.574</v>
       </c>
       <c r="L40" t="n">
-        <v>4.631</v>
+        <v>4.681</v>
       </c>
       <c r="M40" t="n">
-        <v>4.833</v>
+        <v>4.874</v>
       </c>
       <c r="N40" t="n">
-        <v>5.016</v>
+        <v>5.053</v>
       </c>
       <c r="O40" t="n">
-        <v>5.316</v>
+        <v>5.348</v>
       </c>
       <c r="P40" t="n">
-        <v>5.525</v>
+        <v>5.554</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.312</v>
+        <v>6.34</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3405,34 +3405,34 @@
         <v>3.828</v>
       </c>
       <c r="H41" t="n">
-        <v>4.08</v>
+        <v>4.089</v>
       </c>
       <c r="I41" t="n">
-        <v>4.351</v>
+        <v>4.357</v>
       </c>
       <c r="J41" t="n">
-        <v>4.77</v>
+        <v>4.8</v>
       </c>
       <c r="K41" t="n">
-        <v>5.134</v>
+        <v>5.174</v>
       </c>
       <c r="L41" t="n">
-        <v>5.309</v>
+        <v>5.358</v>
       </c>
       <c r="M41" t="n">
-        <v>5.635</v>
+        <v>5.675</v>
       </c>
       <c r="N41" t="n">
-        <v>5.945</v>
+        <v>5.982</v>
       </c>
       <c r="O41" t="n">
-        <v>6.428</v>
+        <v>6.46</v>
       </c>
       <c r="P41" t="n">
-        <v>6.584</v>
+        <v>6.613</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.359</v>
+        <v>7.387</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3478,34 +3478,34 @@
         <v>3.552</v>
       </c>
       <c r="H42" t="n">
-        <v>3.772</v>
+        <v>3.782</v>
       </c>
       <c r="I42" t="n">
-        <v>4.038</v>
+        <v>4.043</v>
       </c>
       <c r="J42" t="n">
-        <v>4.419</v>
+        <v>4.449</v>
       </c>
       <c r="K42" t="n">
-        <v>4.755</v>
+        <v>4.795</v>
       </c>
       <c r="L42" t="n">
-        <v>4.868</v>
+        <v>4.917</v>
       </c>
       <c r="M42" t="n">
-        <v>5.141</v>
+        <v>5.181</v>
       </c>
       <c r="N42" t="n">
-        <v>5.43</v>
+        <v>5.468</v>
       </c>
       <c r="O42" t="n">
-        <v>5.807</v>
+        <v>5.838</v>
       </c>
       <c r="P42" t="n">
-        <v>6.026</v>
+        <v>6.055</v>
       </c>
       <c r="Q42" t="n">
-        <v>6.825</v>
+        <v>6.853</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3551,34 +3551,34 @@
         <v>3.217</v>
       </c>
       <c r="H43" t="n">
-        <v>3.358</v>
+        <v>3.367</v>
       </c>
       <c r="I43" t="n">
-        <v>3.566</v>
+        <v>3.571</v>
       </c>
       <c r="J43" t="n">
-        <v>3.86</v>
+        <v>3.889</v>
       </c>
       <c r="K43" t="n">
-        <v>4.104</v>
+        <v>4.142</v>
       </c>
       <c r="L43" t="n">
-        <v>4.156</v>
+        <v>4.205</v>
       </c>
       <c r="M43" t="n">
-        <v>4.28</v>
+        <v>4.32</v>
       </c>
       <c r="N43" t="n">
-        <v>4.318</v>
+        <v>4.356</v>
       </c>
       <c r="O43" t="n">
-        <v>4.406</v>
+        <v>4.438</v>
       </c>
       <c r="P43" t="n">
-        <v>4.501</v>
+        <v>4.531</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.188</v>
+        <v>5.216</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46135</v>
+        <v>46136</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3624,34 +3624,34 @@
         <v>3.084</v>
       </c>
       <c r="H44" t="n">
-        <v>3.207</v>
+        <v>3.212</v>
       </c>
       <c r="I44" t="n">
-        <v>3.412</v>
+        <v>3.417</v>
       </c>
       <c r="J44" t="n">
-        <v>3.71</v>
+        <v>3.739</v>
       </c>
       <c r="K44" t="n">
-        <v>3.947</v>
+        <v>3.985</v>
       </c>
       <c r="L44" t="n">
-        <v>3.998</v>
+        <v>4.048</v>
       </c>
       <c r="M44" t="n">
-        <v>4.095</v>
+        <v>4.134</v>
       </c>
       <c r="N44" t="n">
-        <v>4.133</v>
+        <v>4.171</v>
       </c>
       <c r="O44" t="n">
-        <v>4.202</v>
+        <v>4.234</v>
       </c>
       <c r="P44" t="n">
-        <v>4.265</v>
+        <v>4.295</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.559</v>
+        <v>4.587</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-04-28 ~ 2026-04-28
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.201</v>
+        <v>3.198</v>
       </c>
       <c r="G2" t="n">
-        <v>3.411</v>
+        <v>3.408</v>
       </c>
       <c r="H2" t="n">
-        <v>3.581</v>
+        <v>3.586</v>
       </c>
       <c r="I2" t="n">
-        <v>3.779</v>
+        <v>3.781</v>
       </c>
       <c r="J2" t="n">
-        <v>4.098</v>
+        <v>4.115</v>
       </c>
       <c r="K2" t="n">
-        <v>4.509</v>
+        <v>4.539</v>
       </c>
       <c r="L2" t="n">
-        <v>4.697</v>
+        <v>4.73</v>
       </c>
       <c r="M2" t="n">
-        <v>4.991</v>
+        <v>5.022</v>
       </c>
       <c r="N2" t="n">
-        <v>5.256</v>
+        <v>5.292</v>
       </c>
       <c r="O2" t="n">
-        <v>5.478</v>
+        <v>5.516</v>
       </c>
       <c r="P2" t="n">
-        <v>5.661</v>
+        <v>5.704</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.29</v>
+        <v>6.335</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.224</v>
+        <v>4.221</v>
       </c>
       <c r="G3" t="n">
-        <v>4.615</v>
+        <v>4.612</v>
       </c>
       <c r="H3" t="n">
-        <v>4.819</v>
+        <v>4.824</v>
       </c>
       <c r="I3" t="n">
-        <v>5.012</v>
+        <v>5.015</v>
       </c>
       <c r="J3" t="n">
-        <v>5.344</v>
+        <v>5.36</v>
       </c>
       <c r="K3" t="n">
-        <v>5.824</v>
+        <v>5.854</v>
       </c>
       <c r="L3" t="n">
-        <v>6.082</v>
+        <v>6.115</v>
       </c>
       <c r="M3" t="n">
-        <v>6.409</v>
+        <v>6.44</v>
       </c>
       <c r="N3" t="n">
-        <v>6.616</v>
+        <v>6.651</v>
       </c>
       <c r="O3" t="n">
-        <v>6.788</v>
+        <v>6.826</v>
       </c>
       <c r="P3" t="n">
-        <v>6.841</v>
+        <v>6.884</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.358</v>
+        <v>7.403</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.717</v>
+        <v>3.714</v>
       </c>
       <c r="G4" t="n">
-        <v>3.996</v>
+        <v>3.993</v>
       </c>
       <c r="H4" t="n">
-        <v>4.229</v>
+        <v>4.234</v>
       </c>
       <c r="I4" t="n">
-        <v>4.455</v>
+        <v>4.458</v>
       </c>
       <c r="J4" t="n">
-        <v>4.79</v>
+        <v>4.806</v>
       </c>
       <c r="K4" t="n">
-        <v>5.263</v>
+        <v>5.293</v>
       </c>
       <c r="L4" t="n">
-        <v>5.451</v>
+        <v>5.484</v>
       </c>
       <c r="M4" t="n">
-        <v>5.766</v>
+        <v>5.797</v>
       </c>
       <c r="N4" t="n">
-        <v>5.944</v>
+        <v>5.979</v>
       </c>
       <c r="O4" t="n">
-        <v>6.14</v>
+        <v>6.177</v>
       </c>
       <c r="P4" t="n">
-        <v>6.191</v>
+        <v>6.234</v>
       </c>
       <c r="Q4" t="n">
-        <v>6.711</v>
+        <v>6.756</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.898</v>
+        <v>2.896</v>
       </c>
       <c r="G5" t="n">
-        <v>2.953</v>
+        <v>2.951</v>
       </c>
       <c r="H5" t="n">
-        <v>3.081</v>
+        <v>3.087</v>
       </c>
       <c r="I5" t="n">
-        <v>3.349</v>
+        <v>3.352</v>
       </c>
       <c r="J5" t="n">
-        <v>3.66</v>
+        <v>3.678</v>
       </c>
       <c r="K5" t="n">
-        <v>3.928</v>
+        <v>3.96</v>
       </c>
       <c r="L5" t="n">
-        <v>3.958</v>
+        <v>3.993</v>
       </c>
       <c r="M5" t="n">
-        <v>4.054</v>
+        <v>4.087</v>
       </c>
       <c r="N5" t="n">
-        <v>4.072</v>
+        <v>4.108</v>
       </c>
       <c r="O5" t="n">
-        <v>4.077</v>
+        <v>4.115</v>
       </c>
       <c r="P5" t="n">
-        <v>4.329</v>
+        <v>4.372</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.202</v>
+        <v>5.247</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2.938</v>
+        <v>2.935</v>
       </c>
       <c r="G6" t="n">
-        <v>3.007</v>
+        <v>3.004</v>
       </c>
       <c r="H6" t="n">
-        <v>3.152</v>
+        <v>3.156</v>
       </c>
       <c r="I6" t="n">
-        <v>3.431</v>
+        <v>3.432</v>
       </c>
       <c r="J6" t="n">
-        <v>3.749</v>
+        <v>3.765</v>
       </c>
       <c r="K6" t="n">
-        <v>4.04</v>
+        <v>4.069</v>
       </c>
       <c r="L6" t="n">
-        <v>4.077</v>
+        <v>4.109</v>
       </c>
       <c r="M6" t="n">
-        <v>4.213</v>
+        <v>4.243</v>
       </c>
       <c r="N6" t="n">
-        <v>4.24</v>
+        <v>4.275</v>
       </c>
       <c r="O6" t="n">
-        <v>4.345</v>
+        <v>4.382</v>
       </c>
       <c r="P6" t="n">
-        <v>4.762</v>
+        <v>4.805</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.598</v>
+        <v>5.643</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2.919</v>
+        <v>2.916</v>
       </c>
       <c r="G7" t="n">
-        <v>2.971</v>
+        <v>2.968</v>
       </c>
       <c r="H7" t="n">
-        <v>3.097</v>
+        <v>3.102</v>
       </c>
       <c r="I7" t="n">
-        <v>3.364</v>
+        <v>3.366</v>
       </c>
       <c r="J7" t="n">
-        <v>3.686</v>
+        <v>3.703</v>
       </c>
       <c r="K7" t="n">
-        <v>3.955</v>
+        <v>3.986</v>
       </c>
       <c r="L7" t="n">
-        <v>3.983</v>
+        <v>4.017</v>
       </c>
       <c r="M7" t="n">
-        <v>4.117</v>
+        <v>4.148</v>
       </c>
       <c r="N7" t="n">
-        <v>4.132</v>
+        <v>4.168</v>
       </c>
       <c r="O7" t="n">
-        <v>4.242</v>
+        <v>4.279</v>
       </c>
       <c r="P7" t="n">
-        <v>4.545</v>
+        <v>4.588</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.366</v>
+        <v>5.411</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.334</v>
+        <v>5.331</v>
       </c>
       <c r="G8" t="n">
-        <v>5.913</v>
+        <v>5.91</v>
       </c>
       <c r="H8" t="n">
-        <v>6.268</v>
+        <v>6.273</v>
       </c>
       <c r="I8" t="n">
-        <v>6.539</v>
+        <v>6.542</v>
       </c>
       <c r="J8" t="n">
-        <v>6.935</v>
+        <v>6.951</v>
       </c>
       <c r="K8" t="n">
-        <v>7.695</v>
+        <v>7.725</v>
       </c>
       <c r="L8" t="n">
-        <v>8.041</v>
+        <v>8.074</v>
       </c>
       <c r="M8" t="n">
-        <v>8.397</v>
+        <v>8.428000000000001</v>
       </c>
       <c r="N8" t="n">
-        <v>8.539</v>
+        <v>8.574999999999999</v>
       </c>
       <c r="O8" t="n">
-        <v>8.797000000000001</v>
+        <v>8.834</v>
       </c>
       <c r="P8" t="n">
-        <v>8.952</v>
+        <v>8.994999999999999</v>
       </c>
       <c r="Q8" t="n">
-        <v>9.667</v>
+        <v>9.712999999999999</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1069,51 +1069,51 @@
         <v>2.699</v>
       </c>
       <c r="H9" t="n">
-        <v>2.797</v>
+        <v>2.8</v>
       </c>
       <c r="I9" t="n">
-        <v>2.987</v>
+        <v>2.99</v>
       </c>
       <c r="J9" t="n">
-        <v>3.223</v>
+        <v>3.232</v>
       </c>
       <c r="K9" t="n">
-        <v>3.38</v>
+        <v>3.41</v>
       </c>
       <c r="L9" t="n">
-        <v>3.42</v>
+        <v>3.454</v>
       </c>
       <c r="M9" t="n">
-        <v>3.497</v>
+        <v>3.53</v>
       </c>
       <c r="N9" t="n">
-        <v>3.652</v>
+        <v>3.689</v>
       </c>
       <c r="O9" t="n">
-        <v>3.677</v>
+        <v>3.715</v>
       </c>
       <c r="P9" t="n">
-        <v>3.752</v>
+        <v>3.795</v>
       </c>
       <c r="Q9" t="n">
-        <v>3.819</v>
+        <v>3.865</v>
       </c>
       <c r="R9" t="n">
-        <v>3.791</v>
+        <v>3.832</v>
       </c>
       <c r="S9" t="n">
-        <v>3.759</v>
+        <v>3.795</v>
       </c>
       <c r="T9" t="n">
-        <v>3.677</v>
+        <v>3.712</v>
       </c>
       <c r="U9" t="n">
-        <v>3.548</v>
+        <v>3.584</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1142,28 +1142,28 @@
         <v>2.732</v>
       </c>
       <c r="H10" t="n">
-        <v>2.812</v>
+        <v>2.814</v>
       </c>
       <c r="I10" t="n">
-        <v>2.997</v>
+        <v>3.001</v>
       </c>
       <c r="J10" t="n">
-        <v>3.249</v>
+        <v>3.258</v>
       </c>
       <c r="K10" t="n">
-        <v>3.413</v>
+        <v>3.443</v>
       </c>
       <c r="L10" t="n">
-        <v>3.471</v>
+        <v>3.506</v>
       </c>
       <c r="M10" t="n">
-        <v>3.594</v>
+        <v>3.627</v>
       </c>
       <c r="N10" t="n">
-        <v>3.668</v>
+        <v>3.704</v>
       </c>
       <c r="O10" t="n">
-        <v>3.899</v>
+        <v>3.938</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1215,34 +1215,34 @@
         <v>2.542</v>
       </c>
       <c r="H11" t="n">
-        <v>2.636</v>
+        <v>2.638</v>
       </c>
       <c r="I11" t="n">
-        <v>2.8</v>
+        <v>2.804</v>
       </c>
       <c r="J11" t="n">
-        <v>3.043</v>
+        <v>3.052</v>
       </c>
       <c r="K11" t="n">
-        <v>3.2</v>
+        <v>3.231</v>
       </c>
       <c r="L11" t="n">
-        <v>3.265</v>
+        <v>3.3</v>
       </c>
       <c r="M11" t="n">
-        <v>3.399</v>
+        <v>3.432</v>
       </c>
       <c r="N11" t="n">
-        <v>3.476</v>
+        <v>3.513</v>
       </c>
       <c r="O11" t="n">
-        <v>3.665</v>
+        <v>3.705</v>
       </c>
       <c r="P11" t="n">
-        <v>3.698</v>
+        <v>3.741</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.021</v>
+        <v>4.066</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.185</v>
+        <v>3.184</v>
       </c>
       <c r="G12" t="n">
         <v>3.34</v>
       </c>
       <c r="H12" t="n">
-        <v>3.458</v>
+        <v>3.461</v>
       </c>
       <c r="I12" t="n">
-        <v>3.696</v>
+        <v>3.704</v>
       </c>
       <c r="J12" t="n">
-        <v>4.072</v>
+        <v>4.088</v>
       </c>
       <c r="K12" t="n">
-        <v>4.282</v>
+        <v>4.309</v>
       </c>
       <c r="L12" t="n">
-        <v>4.354</v>
+        <v>4.383</v>
       </c>
       <c r="M12" t="n">
-        <v>4.492</v>
+        <v>4.52</v>
       </c>
       <c r="N12" t="n">
-        <v>4.538</v>
+        <v>4.574</v>
       </c>
       <c r="O12" t="n">
-        <v>4.678</v>
+        <v>4.716</v>
       </c>
       <c r="P12" t="n">
-        <v>4.797</v>
+        <v>4.84</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.149</v>
+        <v>5.194</v>
       </c>
       <c r="R12" t="n">
-        <v>5.291</v>
+        <v>5.333</v>
       </c>
       <c r="S12" t="n">
-        <v>5.471</v>
+        <v>5.506</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2.939</v>
+        <v>2.937</v>
       </c>
       <c r="G13" t="n">
         <v>3.03</v>
       </c>
       <c r="H13" t="n">
-        <v>3.126</v>
+        <v>3.128</v>
       </c>
       <c r="I13" t="n">
-        <v>3.344</v>
+        <v>3.352</v>
       </c>
       <c r="J13" t="n">
-        <v>3.709</v>
+        <v>3.725</v>
       </c>
       <c r="K13" t="n">
-        <v>3.916</v>
+        <v>3.943</v>
       </c>
       <c r="L13" t="n">
-        <v>3.994</v>
+        <v>4.023</v>
       </c>
       <c r="M13" t="n">
-        <v>4.119</v>
+        <v>4.147</v>
       </c>
       <c r="N13" t="n">
-        <v>4.166</v>
+        <v>4.202</v>
       </c>
       <c r="O13" t="n">
-        <v>4.307</v>
+        <v>4.344</v>
       </c>
       <c r="P13" t="n">
-        <v>4.388</v>
+        <v>4.431</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.669</v>
+        <v>4.714</v>
       </c>
       <c r="R13" t="n">
-        <v>4.84</v>
+        <v>4.881</v>
       </c>
       <c r="S13" t="n">
-        <v>5.033</v>
+        <v>5.068</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.758</v>
+        <v>2.757</v>
       </c>
       <c r="G14" t="n">
         <v>2.836</v>
       </c>
       <c r="H14" t="n">
-        <v>2.929</v>
+        <v>2.931</v>
       </c>
       <c r="I14" t="n">
-        <v>3.128</v>
+        <v>3.136</v>
       </c>
       <c r="J14" t="n">
-        <v>3.449</v>
+        <v>3.465</v>
       </c>
       <c r="K14" t="n">
-        <v>3.604</v>
+        <v>3.631</v>
       </c>
       <c r="L14" t="n">
-        <v>3.666</v>
+        <v>3.695</v>
       </c>
       <c r="M14" t="n">
-        <v>3.804</v>
+        <v>3.833</v>
       </c>
       <c r="N14" t="n">
-        <v>3.845</v>
+        <v>3.881</v>
       </c>
       <c r="O14" t="n">
-        <v>3.961</v>
+        <v>3.999</v>
       </c>
       <c r="P14" t="n">
-        <v>4.023</v>
+        <v>4.066</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.258</v>
+        <v>4.303</v>
       </c>
       <c r="R14" t="n">
-        <v>4.354</v>
+        <v>4.396</v>
       </c>
       <c r="S14" t="n">
-        <v>4.486</v>
+        <v>4.521</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.736</v>
+        <v>2.735</v>
       </c>
       <c r="G15" t="n">
         <v>2.81</v>
       </c>
       <c r="H15" t="n">
-        <v>2.9</v>
+        <v>2.902</v>
       </c>
       <c r="I15" t="n">
-        <v>3.079</v>
+        <v>3.087</v>
       </c>
       <c r="J15" t="n">
-        <v>3.388</v>
+        <v>3.404</v>
       </c>
       <c r="K15" t="n">
-        <v>3.557</v>
+        <v>3.583</v>
       </c>
       <c r="L15" t="n">
-        <v>3.601</v>
+        <v>3.63</v>
       </c>
       <c r="M15" t="n">
-        <v>3.718</v>
+        <v>3.746</v>
       </c>
       <c r="N15" t="n">
-        <v>3.749</v>
+        <v>3.785</v>
       </c>
       <c r="O15" t="n">
-        <v>3.901</v>
+        <v>3.941</v>
       </c>
       <c r="P15" t="n">
-        <v>3.923</v>
+        <v>3.966</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.163</v>
+        <v>4.208</v>
       </c>
       <c r="R15" t="n">
-        <v>4.251</v>
+        <v>4.292</v>
       </c>
       <c r="S15" t="n">
-        <v>4.381</v>
+        <v>4.416</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.736</v>
+        <v>2.735</v>
       </c>
       <c r="G16" t="n">
         <v>2.81</v>
       </c>
       <c r="H16" t="n">
-        <v>2.9</v>
+        <v>2.902</v>
       </c>
       <c r="I16" t="n">
-        <v>3.079</v>
+        <v>3.087</v>
       </c>
       <c r="J16" t="n">
-        <v>3.388</v>
+        <v>3.404</v>
       </c>
       <c r="K16" t="n">
-        <v>3.557</v>
+        <v>3.583</v>
       </c>
       <c r="L16" t="n">
-        <v>3.601</v>
+        <v>3.63</v>
       </c>
       <c r="M16" t="n">
-        <v>3.718</v>
+        <v>3.746</v>
       </c>
       <c r="N16" t="n">
-        <v>3.752</v>
+        <v>3.788</v>
       </c>
       <c r="O16" t="n">
-        <v>3.908</v>
+        <v>3.947</v>
       </c>
       <c r="P16" t="n">
-        <v>3.947</v>
+        <v>3.989</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.19</v>
+        <v>4.235</v>
       </c>
       <c r="R16" t="n">
-        <v>4.279</v>
+        <v>4.32</v>
       </c>
       <c r="S16" t="n">
-        <v>4.41</v>
+        <v>4.445</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1650,34 +1650,34 @@
         <v>2.693</v>
       </c>
       <c r="G17" t="n">
-        <v>2.823</v>
+        <v>2.822</v>
       </c>
       <c r="H17" t="n">
-        <v>2.905</v>
+        <v>2.907</v>
       </c>
       <c r="I17" t="n">
-        <v>3.079</v>
+        <v>3.082</v>
       </c>
       <c r="J17" t="n">
-        <v>3.319</v>
+        <v>3.328</v>
       </c>
       <c r="K17" t="n">
-        <v>3.488</v>
+        <v>3.519</v>
       </c>
       <c r="L17" t="n">
-        <v>3.551</v>
+        <v>3.586</v>
       </c>
       <c r="M17" t="n">
-        <v>3.713</v>
+        <v>3.746</v>
       </c>
       <c r="N17" t="n">
-        <v>3.771</v>
+        <v>3.807</v>
       </c>
       <c r="O17" t="n">
-        <v>3.925</v>
+        <v>3.966</v>
       </c>
       <c r="P17" t="n">
-        <v>3.974</v>
+        <v>4.017</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1723,31 +1723,31 @@
         <v>2.694</v>
       </c>
       <c r="G18" t="n">
-        <v>2.824</v>
+        <v>2.823</v>
       </c>
       <c r="H18" t="n">
-        <v>2.905</v>
+        <v>2.907</v>
       </c>
       <c r="I18" t="n">
-        <v>3.079</v>
+        <v>3.083</v>
       </c>
       <c r="J18" t="n">
-        <v>3.319</v>
+        <v>3.328</v>
       </c>
       <c r="K18" t="n">
-        <v>3.489</v>
+        <v>3.52</v>
       </c>
       <c r="L18" t="n">
-        <v>3.551</v>
+        <v>3.586</v>
       </c>
       <c r="M18" t="n">
-        <v>3.713</v>
+        <v>3.746</v>
       </c>
       <c r="N18" t="n">
-        <v>3.772</v>
+        <v>3.808</v>
       </c>
       <c r="O18" t="n">
-        <v>3.925</v>
+        <v>3.965</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.749</v>
+        <v>2.748</v>
       </c>
       <c r="G19" t="n">
         <v>2.827</v>
       </c>
       <c r="H19" t="n">
-        <v>2.918</v>
+        <v>2.921</v>
       </c>
       <c r="I19" t="n">
-        <v>3.115</v>
+        <v>3.123</v>
       </c>
       <c r="J19" t="n">
-        <v>3.432</v>
+        <v>3.449</v>
       </c>
       <c r="K19" t="n">
-        <v>3.6</v>
+        <v>3.627</v>
       </c>
       <c r="L19" t="n">
-        <v>3.663</v>
+        <v>3.692</v>
       </c>
       <c r="M19" t="n">
-        <v>3.796</v>
+        <v>3.824</v>
       </c>
       <c r="N19" t="n">
-        <v>3.833</v>
+        <v>3.868</v>
       </c>
       <c r="O19" t="n">
-        <v>3.945</v>
+        <v>3.982</v>
       </c>
       <c r="P19" t="n">
-        <v>3.983</v>
+        <v>4.026</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.205</v>
+        <v>4.25</v>
       </c>
       <c r="R19" t="n">
-        <v>4.301</v>
+        <v>4.343</v>
       </c>
       <c r="S19" t="n">
-        <v>4.424</v>
+        <v>4.459</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2.574</v>
+        <v>2.573</v>
       </c>
       <c r="G20" t="n">
-        <v>2.645</v>
+        <v>2.644</v>
       </c>
       <c r="H20" t="n">
-        <v>2.69</v>
+        <v>2.691</v>
       </c>
       <c r="I20" t="n">
-        <v>2.828</v>
+        <v>2.83</v>
       </c>
       <c r="J20" t="n">
-        <v>3.215</v>
+        <v>3.233</v>
       </c>
       <c r="K20" t="n">
-        <v>3.397</v>
+        <v>3.43</v>
       </c>
       <c r="L20" t="n">
-        <v>3.435</v>
+        <v>3.465</v>
       </c>
       <c r="M20" t="n">
-        <v>3.53</v>
+        <v>3.56</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2.861</v>
+        <v>2.859</v>
       </c>
       <c r="G21" t="n">
-        <v>2.937</v>
+        <v>2.935</v>
       </c>
       <c r="H21" t="n">
-        <v>3.067</v>
+        <v>3.07</v>
       </c>
       <c r="I21" t="n">
-        <v>3.238</v>
+        <v>3.245</v>
       </c>
       <c r="J21" t="n">
-        <v>3.57</v>
+        <v>3.588</v>
       </c>
       <c r="K21" t="n">
-        <v>3.835</v>
+        <v>3.865</v>
       </c>
       <c r="L21" t="n">
-        <v>3.908</v>
+        <v>3.939</v>
       </c>
       <c r="M21" t="n">
-        <v>4.036</v>
+        <v>4.065</v>
       </c>
       <c r="N21" t="n">
-        <v>4.088</v>
+        <v>4.123</v>
       </c>
       <c r="O21" t="n">
-        <v>4.161</v>
+        <v>4.199</v>
       </c>
       <c r="P21" t="n">
-        <v>4.25</v>
+        <v>4.293</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.368</v>
+        <v>4.412</v>
       </c>
       <c r="R21" t="n">
-        <v>4.354</v>
+        <v>4.394</v>
       </c>
       <c r="S21" t="n">
-        <v>4.385</v>
+        <v>4.42</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.808</v>
+        <v>2.806</v>
       </c>
       <c r="G22" t="n">
-        <v>2.883</v>
+        <v>2.882</v>
       </c>
       <c r="H22" t="n">
-        <v>2.999</v>
+        <v>3.002</v>
       </c>
       <c r="I22" t="n">
-        <v>3.158</v>
+        <v>3.163</v>
       </c>
       <c r="J22" t="n">
-        <v>3.453</v>
+        <v>3.471</v>
       </c>
       <c r="K22" t="n">
-        <v>3.714</v>
+        <v>3.745</v>
       </c>
       <c r="L22" t="n">
-        <v>3.776</v>
+        <v>3.807</v>
       </c>
       <c r="M22" t="n">
-        <v>3.906</v>
+        <v>3.934</v>
       </c>
       <c r="N22" t="n">
-        <v>3.96</v>
+        <v>3.995</v>
       </c>
       <c r="O22" t="n">
-        <v>4.029</v>
+        <v>4.067</v>
       </c>
       <c r="P22" t="n">
-        <v>4.112</v>
+        <v>4.155</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.227</v>
+        <v>4.271</v>
       </c>
       <c r="R22" t="n">
-        <v>4.202</v>
+        <v>4.243</v>
       </c>
       <c r="S22" t="n">
-        <v>4.23</v>
+        <v>4.265</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.761</v>
+        <v>2.759</v>
       </c>
       <c r="G23" t="n">
-        <v>2.838</v>
+        <v>2.836</v>
       </c>
       <c r="H23" t="n">
-        <v>2.938</v>
+        <v>2.941</v>
       </c>
       <c r="I23" t="n">
-        <v>3.111</v>
+        <v>3.118</v>
       </c>
       <c r="J23" t="n">
-        <v>3.399</v>
+        <v>3.416</v>
       </c>
       <c r="K23" t="n">
-        <v>3.625</v>
+        <v>3.654</v>
       </c>
       <c r="L23" t="n">
-        <v>3.685</v>
+        <v>3.715</v>
       </c>
       <c r="M23" t="n">
-        <v>3.808</v>
+        <v>3.835</v>
       </c>
       <c r="N23" t="n">
-        <v>3.857</v>
+        <v>3.891</v>
       </c>
       <c r="O23" t="n">
-        <v>3.905</v>
+        <v>3.943</v>
       </c>
       <c r="P23" t="n">
-        <v>3.973</v>
+        <v>4.017</v>
       </c>
       <c r="Q23" t="n">
-        <v>4.034</v>
+        <v>4.077</v>
       </c>
       <c r="R23" t="n">
-        <v>3.985</v>
+        <v>4.026</v>
       </c>
       <c r="S23" t="n">
-        <v>3.985</v>
+        <v>4.02</v>
       </c>
       <c r="T23" t="n">
-        <v>3.892</v>
+        <v>3.927</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.696</v>
+        <v>2.694</v>
       </c>
       <c r="G24" t="n">
-        <v>2.752</v>
+        <v>2.75</v>
       </c>
       <c r="H24" t="n">
-        <v>2.839</v>
+        <v>2.842</v>
       </c>
       <c r="I24" t="n">
-        <v>3.021</v>
+        <v>3.028</v>
       </c>
       <c r="J24" t="n">
-        <v>3.297</v>
+        <v>3.315</v>
       </c>
       <c r="K24" t="n">
-        <v>3.511</v>
+        <v>3.538</v>
       </c>
       <c r="L24" t="n">
-        <v>3.559</v>
+        <v>3.589</v>
       </c>
       <c r="M24" t="n">
-        <v>3.667</v>
+        <v>3.695</v>
       </c>
       <c r="N24" t="n">
-        <v>3.734</v>
+        <v>3.768</v>
       </c>
       <c r="O24" t="n">
-        <v>3.899</v>
+        <v>3.938</v>
       </c>
       <c r="P24" t="n">
-        <v>3.917</v>
+        <v>3.959</v>
       </c>
       <c r="Q24" t="n">
-        <v>3.957</v>
+        <v>4</v>
       </c>
       <c r="R24" t="n">
-        <v>3.906</v>
+        <v>3.947</v>
       </c>
       <c r="S24" t="n">
-        <v>3.9</v>
+        <v>3.935</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.754</v>
+        <v>2.752</v>
       </c>
       <c r="G25" t="n">
-        <v>2.837</v>
+        <v>2.835</v>
       </c>
       <c r="H25" t="n">
-        <v>2.941</v>
+        <v>2.944</v>
       </c>
       <c r="I25" t="n">
-        <v>3.119</v>
+        <v>3.126</v>
       </c>
       <c r="J25" t="n">
-        <v>3.414</v>
+        <v>3.432</v>
       </c>
       <c r="K25" t="n">
-        <v>3.657</v>
+        <v>3.687</v>
       </c>
       <c r="L25" t="n">
-        <v>3.714</v>
+        <v>3.744</v>
       </c>
       <c r="M25" t="n">
-        <v>3.838</v>
+        <v>3.865</v>
       </c>
       <c r="N25" t="n">
-        <v>3.884</v>
+        <v>3.918</v>
       </c>
       <c r="O25" t="n">
-        <v>3.935</v>
+        <v>3.972</v>
       </c>
       <c r="P25" t="n">
-        <v>3.995</v>
+        <v>4.038</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.066</v>
+        <v>4.11</v>
       </c>
       <c r="R25" t="n">
-        <v>4.009</v>
+        <v>4.049</v>
       </c>
       <c r="S25" t="n">
-        <v>4.008</v>
+        <v>4.043</v>
       </c>
       <c r="T25" t="n">
-        <v>3.91</v>
+        <v>3.945</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.054</v>
+        <v>3.05</v>
       </c>
       <c r="G26" t="n">
-        <v>3.189</v>
+        <v>3.186</v>
       </c>
       <c r="H26" t="n">
-        <v>3.408</v>
+        <v>3.41</v>
       </c>
       <c r="I26" t="n">
-        <v>3.643</v>
+        <v>3.645</v>
       </c>
       <c r="J26" t="n">
-        <v>4.074</v>
+        <v>4.092</v>
       </c>
       <c r="K26" t="n">
-        <v>4.47</v>
+        <v>4.5</v>
       </c>
       <c r="L26" t="n">
-        <v>4.586</v>
+        <v>4.618</v>
       </c>
       <c r="M26" t="n">
-        <v>4.769</v>
+        <v>4.799</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.014</v>
+        <v>5.052</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.848</v>
+        <v>2.847</v>
       </c>
       <c r="G27" t="n">
         <v>2.918</v>
       </c>
       <c r="H27" t="n">
-        <v>3.038</v>
+        <v>3.041</v>
       </c>
       <c r="I27" t="n">
-        <v>3.238</v>
+        <v>3.245</v>
       </c>
       <c r="J27" t="n">
-        <v>3.572</v>
+        <v>3.588</v>
       </c>
       <c r="K27" t="n">
-        <v>3.783</v>
+        <v>3.811</v>
       </c>
       <c r="L27" t="n">
-        <v>3.849</v>
+        <v>3.878</v>
       </c>
       <c r="M27" t="n">
-        <v>3.976</v>
+        <v>4.003</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.105</v>
+        <v>4.143</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2.951</v>
+        <v>2.95</v>
       </c>
       <c r="G28" t="n">
         <v>3.029</v>
       </c>
       <c r="H28" t="n">
-        <v>3.164</v>
+        <v>3.166</v>
       </c>
       <c r="I28" t="n">
-        <v>3.376</v>
+        <v>3.383</v>
       </c>
       <c r="J28" t="n">
-        <v>3.745</v>
+        <v>3.761</v>
       </c>
       <c r="K28" t="n">
-        <v>3.976</v>
+        <v>4.003</v>
       </c>
       <c r="L28" t="n">
-        <v>4.053</v>
+        <v>4.081</v>
       </c>
       <c r="M28" t="n">
-        <v>4.188</v>
+        <v>4.215</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.399</v>
+        <v>4.437</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.804</v>
+        <v>2.802</v>
       </c>
       <c r="G29" t="n">
         <v>2.874</v>
       </c>
       <c r="H29" t="n">
-        <v>2.979</v>
+        <v>2.981</v>
       </c>
       <c r="I29" t="n">
-        <v>3.171</v>
+        <v>3.177</v>
       </c>
       <c r="J29" t="n">
-        <v>3.484</v>
+        <v>3.501</v>
       </c>
       <c r="K29" t="n">
-        <v>3.679</v>
+        <v>3.707</v>
       </c>
       <c r="L29" t="n">
-        <v>3.734</v>
+        <v>3.763</v>
       </c>
       <c r="M29" t="n">
-        <v>3.838</v>
+        <v>3.866</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>3.972</v>
+        <v>4.011</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.089</v>
+        <v>3.085</v>
       </c>
       <c r="G30" t="n">
-        <v>3.161</v>
+        <v>3.158</v>
       </c>
       <c r="H30" t="n">
-        <v>3.345</v>
+        <v>3.346</v>
       </c>
       <c r="I30" t="n">
-        <v>3.573</v>
+        <v>3.575</v>
       </c>
       <c r="J30" t="n">
-        <v>3.944</v>
+        <v>3.961</v>
       </c>
       <c r="K30" t="n">
-        <v>4.265</v>
+        <v>4.295</v>
       </c>
       <c r="L30" t="n">
-        <v>4.356</v>
+        <v>4.387</v>
       </c>
       <c r="M30" t="n">
-        <v>4.532</v>
+        <v>4.562</v>
       </c>
       <c r="N30" t="n">
-        <v>4.695</v>
+        <v>4.73</v>
       </c>
       <c r="O30" t="n">
-        <v>4.965</v>
+        <v>5.003</v>
       </c>
       <c r="P30" t="n">
-        <v>5.137</v>
+        <v>5.18</v>
       </c>
       <c r="Q30" t="n">
-        <v>5.894</v>
+        <v>5.939</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.415</v>
+        <v>3.411</v>
       </c>
       <c r="G31" t="n">
-        <v>3.521</v>
+        <v>3.518</v>
       </c>
       <c r="H31" t="n">
-        <v>3.756</v>
+        <v>3.758</v>
       </c>
       <c r="I31" t="n">
-        <v>4</v>
+        <v>4.003</v>
       </c>
       <c r="J31" t="n">
-        <v>4.434</v>
+        <v>4.451</v>
       </c>
       <c r="K31" t="n">
-        <v>4.797</v>
+        <v>4.827</v>
       </c>
       <c r="L31" t="n">
-        <v>4.967</v>
+        <v>4.999</v>
       </c>
       <c r="M31" t="n">
-        <v>5.262</v>
+        <v>5.292</v>
       </c>
       <c r="N31" t="n">
-        <v>5.552</v>
+        <v>5.587</v>
       </c>
       <c r="O31" t="n">
-        <v>5.998</v>
+        <v>6.036</v>
       </c>
       <c r="P31" t="n">
-        <v>6.124</v>
+        <v>6.167</v>
       </c>
       <c r="Q31" t="n">
-        <v>6.868</v>
+        <v>6.912</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.187</v>
+        <v>3.183</v>
       </c>
       <c r="G32" t="n">
-        <v>3.277</v>
+        <v>3.274</v>
       </c>
       <c r="H32" t="n">
-        <v>3.487</v>
+        <v>3.489</v>
       </c>
       <c r="I32" t="n">
-        <v>3.732</v>
+        <v>3.734</v>
       </c>
       <c r="J32" t="n">
-        <v>4.123</v>
+        <v>4.14</v>
       </c>
       <c r="K32" t="n">
-        <v>4.45</v>
+        <v>4.48</v>
       </c>
       <c r="L32" t="n">
-        <v>4.56</v>
+        <v>4.591</v>
       </c>
       <c r="M32" t="n">
-        <v>4.805</v>
+        <v>4.835</v>
       </c>
       <c r="N32" t="n">
-        <v>5.056</v>
+        <v>5.09</v>
       </c>
       <c r="O32" t="n">
-        <v>5.409</v>
+        <v>5.447</v>
       </c>
       <c r="P32" t="n">
-        <v>5.596</v>
+        <v>5.639</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.355</v>
+        <v>6.4</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2.962</v>
+        <v>2.956</v>
       </c>
       <c r="G33" t="n">
-        <v>3.03</v>
+        <v>3.026</v>
       </c>
       <c r="H33" t="n">
-        <v>3.163</v>
+        <v>3.164</v>
       </c>
       <c r="I33" t="n">
-        <v>3.354</v>
+        <v>3.356</v>
       </c>
       <c r="J33" t="n">
-        <v>3.651</v>
+        <v>3.667</v>
       </c>
       <c r="K33" t="n">
-        <v>3.906</v>
+        <v>3.935</v>
       </c>
       <c r="L33" t="n">
-        <v>3.962</v>
+        <v>3.993</v>
       </c>
       <c r="M33" t="n">
-        <v>4.066</v>
+        <v>4.095</v>
       </c>
       <c r="N33" t="n">
-        <v>4.086</v>
+        <v>4.122</v>
       </c>
       <c r="O33" t="n">
-        <v>4.121</v>
+        <v>4.16</v>
       </c>
       <c r="P33" t="n">
-        <v>4.169</v>
+        <v>4.212</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.611</v>
+        <v>4.656</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.021</v>
+        <v>3.015</v>
       </c>
       <c r="G34" t="n">
-        <v>3.084</v>
+        <v>3.08</v>
       </c>
       <c r="H34" t="n">
-        <v>3.224</v>
+        <v>3.226</v>
       </c>
       <c r="I34" t="n">
-        <v>3.422</v>
+        <v>3.424</v>
       </c>
       <c r="J34" t="n">
-        <v>3.723</v>
+        <v>3.739</v>
       </c>
       <c r="K34" t="n">
-        <v>3.982</v>
+        <v>4.011</v>
       </c>
       <c r="L34" t="n">
-        <v>4.041</v>
+        <v>4.072</v>
       </c>
       <c r="M34" t="n">
-        <v>4.156</v>
+        <v>4.185</v>
       </c>
       <c r="N34" t="n">
-        <v>4.191</v>
+        <v>4.227</v>
       </c>
       <c r="O34" t="n">
-        <v>4.289</v>
+        <v>4.328</v>
       </c>
       <c r="P34" t="n">
-        <v>4.463</v>
+        <v>4.506</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.312</v>
+        <v>5.357</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>2.996</v>
+        <v>2.99</v>
       </c>
       <c r="G35" t="n">
-        <v>3.057</v>
+        <v>3.053</v>
       </c>
       <c r="H35" t="n">
-        <v>3.192</v>
+        <v>3.194</v>
       </c>
       <c r="I35" t="n">
-        <v>3.389</v>
+        <v>3.39</v>
       </c>
       <c r="J35" t="n">
-        <v>3.691</v>
+        <v>3.707</v>
       </c>
       <c r="K35" t="n">
-        <v>3.937</v>
+        <v>3.966</v>
       </c>
       <c r="L35" t="n">
-        <v>3.996</v>
+        <v>4.027</v>
       </c>
       <c r="M35" t="n">
-        <v>4.103</v>
+        <v>4.132</v>
       </c>
       <c r="N35" t="n">
-        <v>4.128</v>
+        <v>4.163</v>
       </c>
       <c r="O35" t="n">
-        <v>4.187</v>
+        <v>4.226</v>
       </c>
       <c r="P35" t="n">
-        <v>4.266</v>
+        <v>4.309</v>
       </c>
       <c r="Q35" t="n">
-        <v>4.947</v>
+        <v>4.993</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.904</v>
+        <v>2.898</v>
       </c>
       <c r="G36" t="n">
-        <v>2.968</v>
+        <v>2.963</v>
       </c>
       <c r="H36" t="n">
-        <v>3.084</v>
+        <v>3.085</v>
       </c>
       <c r="I36" t="n">
-        <v>3.281</v>
+        <v>3.282</v>
       </c>
       <c r="J36" t="n">
-        <v>3.587</v>
+        <v>3.603</v>
       </c>
       <c r="K36" t="n">
-        <v>3.829</v>
+        <v>3.858</v>
       </c>
       <c r="L36" t="n">
-        <v>3.886</v>
+        <v>3.917</v>
       </c>
       <c r="M36" t="n">
-        <v>3.965</v>
+        <v>3.994</v>
       </c>
       <c r="N36" t="n">
-        <v>3.989</v>
+        <v>4.024</v>
       </c>
       <c r="O36" t="n">
-        <v>4.031</v>
+        <v>4.068</v>
       </c>
       <c r="P36" t="n">
-        <v>4.068</v>
+        <v>4.111</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.328</v>
+        <v>4.373</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.759</v>
+        <v>3.754</v>
       </c>
       <c r="G37" t="n">
-        <v>4.216</v>
+        <v>4.212</v>
       </c>
       <c r="H37" t="n">
-        <v>4.731</v>
+        <v>4.733</v>
       </c>
       <c r="I37" t="n">
-        <v>5.066</v>
+        <v>5.068</v>
       </c>
       <c r="J37" t="n">
-        <v>5.925</v>
+        <v>5.942</v>
       </c>
       <c r="K37" t="n">
-        <v>6.837</v>
+        <v>6.867</v>
       </c>
       <c r="L37" t="n">
-        <v>7.168</v>
+        <v>7.199</v>
       </c>
       <c r="M37" t="n">
-        <v>7.534</v>
+        <v>7.565</v>
       </c>
       <c r="N37" t="n">
-        <v>7.702</v>
+        <v>7.737</v>
       </c>
       <c r="O37" t="n">
-        <v>7.877</v>
+        <v>7.915</v>
       </c>
       <c r="P37" t="n">
-        <v>7.923</v>
+        <v>7.967</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.356</v>
+        <v>8.401</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.818</v>
+        <v>4.813</v>
       </c>
       <c r="G38" t="n">
-        <v>5.528</v>
+        <v>5.524</v>
       </c>
       <c r="H38" t="n">
-        <v>6.255</v>
+        <v>6.257</v>
       </c>
       <c r="I38" t="n">
-        <v>6.747</v>
+        <v>6.749</v>
       </c>
       <c r="J38" t="n">
-        <v>7.867</v>
+        <v>7.884</v>
       </c>
       <c r="K38" t="n">
-        <v>8.956</v>
+        <v>8.984999999999999</v>
       </c>
       <c r="L38" t="n">
-        <v>9.446</v>
+        <v>9.477</v>
       </c>
       <c r="M38" t="n">
-        <v>9.944000000000001</v>
+        <v>9.974</v>
       </c>
       <c r="N38" t="n">
-        <v>10.12</v>
+        <v>10.155</v>
       </c>
       <c r="O38" t="n">
-        <v>10.277</v>
+        <v>10.315</v>
       </c>
       <c r="P38" t="n">
-        <v>10.321</v>
+        <v>10.364</v>
       </c>
       <c r="Q38" t="n">
-        <v>10.806</v>
+        <v>10.852</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.139</v>
+        <v>4.134</v>
       </c>
       <c r="G39" t="n">
-        <v>4.726</v>
+        <v>4.722</v>
       </c>
       <c r="H39" t="n">
-        <v>5.32</v>
+        <v>5.322</v>
       </c>
       <c r="I39" t="n">
-        <v>5.75</v>
+        <v>5.753</v>
       </c>
       <c r="J39" t="n">
-        <v>6.739</v>
+        <v>6.756</v>
       </c>
       <c r="K39" t="n">
-        <v>7.789</v>
+        <v>7.818</v>
       </c>
       <c r="L39" t="n">
-        <v>8.202999999999999</v>
+        <v>8.234999999999999</v>
       </c>
       <c r="M39" t="n">
-        <v>8.581</v>
+        <v>8.611000000000001</v>
       </c>
       <c r="N39" t="n">
-        <v>8.747999999999999</v>
+        <v>8.782999999999999</v>
       </c>
       <c r="O39" t="n">
-        <v>8.927</v>
+        <v>8.965</v>
       </c>
       <c r="P39" t="n">
-        <v>8.976000000000001</v>
+        <v>9.019</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.452</v>
+        <v>9.497</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.282</v>
+        <v>3.278</v>
       </c>
       <c r="G40" t="n">
-        <v>3.4</v>
+        <v>3.397</v>
       </c>
       <c r="H40" t="n">
-        <v>3.604</v>
+        <v>3.606</v>
       </c>
       <c r="I40" t="n">
-        <v>3.848</v>
+        <v>3.85</v>
       </c>
       <c r="J40" t="n">
-        <v>4.236</v>
+        <v>4.254</v>
       </c>
       <c r="K40" t="n">
-        <v>4.57</v>
+        <v>4.599</v>
       </c>
       <c r="L40" t="n">
-        <v>4.68</v>
+        <v>4.711</v>
       </c>
       <c r="M40" t="n">
-        <v>4.873</v>
+        <v>4.903</v>
       </c>
       <c r="N40" t="n">
-        <v>5.053</v>
+        <v>5.087</v>
       </c>
       <c r="O40" t="n">
-        <v>5.343</v>
+        <v>5.381</v>
       </c>
       <c r="P40" t="n">
-        <v>5.558</v>
+        <v>5.601</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.345</v>
+        <v>6.39</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.665</v>
+        <v>3.661</v>
       </c>
       <c r="G41" t="n">
-        <v>3.824</v>
+        <v>3.821</v>
       </c>
       <c r="H41" t="n">
-        <v>4.086</v>
+        <v>4.088</v>
       </c>
       <c r="I41" t="n">
-        <v>4.349</v>
+        <v>4.352</v>
       </c>
       <c r="J41" t="n">
-        <v>4.79</v>
+        <v>4.807</v>
       </c>
       <c r="K41" t="n">
-        <v>5.17</v>
+        <v>5.199</v>
       </c>
       <c r="L41" t="n">
-        <v>5.357</v>
+        <v>5.389</v>
       </c>
       <c r="M41" t="n">
-        <v>5.675</v>
+        <v>5.705</v>
       </c>
       <c r="N41" t="n">
-        <v>5.982</v>
+        <v>6.016</v>
       </c>
       <c r="O41" t="n">
-        <v>6.456</v>
+        <v>6.494</v>
       </c>
       <c r="P41" t="n">
-        <v>6.616</v>
+        <v>6.659</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.392</v>
+        <v>7.437</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.402</v>
+        <v>3.398</v>
       </c>
       <c r="G42" t="n">
-        <v>3.548</v>
+        <v>3.545</v>
       </c>
       <c r="H42" t="n">
-        <v>3.779</v>
+        <v>3.781</v>
       </c>
       <c r="I42" t="n">
-        <v>4.036</v>
+        <v>4.038</v>
       </c>
       <c r="J42" t="n">
-        <v>4.439</v>
+        <v>4.457</v>
       </c>
       <c r="K42" t="n">
-        <v>4.791</v>
+        <v>4.82</v>
       </c>
       <c r="L42" t="n">
-        <v>4.916</v>
+        <v>4.947</v>
       </c>
       <c r="M42" t="n">
-        <v>5.18</v>
+        <v>5.21</v>
       </c>
       <c r="N42" t="n">
-        <v>5.467</v>
+        <v>5.502</v>
       </c>
       <c r="O42" t="n">
-        <v>5.834</v>
+        <v>5.872</v>
       </c>
       <c r="P42" t="n">
-        <v>6.059</v>
+        <v>6.102</v>
       </c>
       <c r="Q42" t="n">
-        <v>6.858</v>
+        <v>6.903</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.11</v>
+        <v>3.104</v>
       </c>
       <c r="G43" t="n">
-        <v>3.213</v>
+        <v>3.209</v>
       </c>
       <c r="H43" t="n">
-        <v>3.364</v>
+        <v>3.365</v>
       </c>
       <c r="I43" t="n">
-        <v>3.564</v>
+        <v>3.565</v>
       </c>
       <c r="J43" t="n">
-        <v>3.879</v>
+        <v>3.895</v>
       </c>
       <c r="K43" t="n">
-        <v>4.137</v>
+        <v>4.166</v>
       </c>
       <c r="L43" t="n">
-        <v>4.203</v>
+        <v>4.234</v>
       </c>
       <c r="M43" t="n">
-        <v>4.319</v>
+        <v>4.349</v>
       </c>
       <c r="N43" t="n">
-        <v>4.356</v>
+        <v>4.392</v>
       </c>
       <c r="O43" t="n">
-        <v>4.433</v>
+        <v>4.472</v>
       </c>
       <c r="P43" t="n">
-        <v>4.535</v>
+        <v>4.578</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.221</v>
+        <v>5.266</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46139</v>
+        <v>46140</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>2.982</v>
+        <v>2.976</v>
       </c>
       <c r="G44" t="n">
-        <v>3.078</v>
+        <v>3.073</v>
       </c>
       <c r="H44" t="n">
-        <v>3.208</v>
+        <v>3.209</v>
       </c>
       <c r="I44" t="n">
-        <v>3.409</v>
+        <v>3.41</v>
       </c>
       <c r="J44" t="n">
-        <v>3.728</v>
+        <v>3.744</v>
       </c>
       <c r="K44" t="n">
-        <v>3.98</v>
+        <v>4.009</v>
       </c>
       <c r="L44" t="n">
-        <v>4.046</v>
+        <v>4.077</v>
       </c>
       <c r="M44" t="n">
-        <v>4.134</v>
+        <v>4.163</v>
       </c>
       <c r="N44" t="n">
-        <v>4.171</v>
+        <v>4.205</v>
       </c>
       <c r="O44" t="n">
-        <v>4.23</v>
+        <v>4.267</v>
       </c>
       <c r="P44" t="n">
-        <v>4.298</v>
+        <v>4.341</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.592</v>
+        <v>4.637</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-04-29 ~ 2026-04-29
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.198</v>
+        <v>3.191</v>
       </c>
       <c r="G2" t="n">
-        <v>3.408</v>
+        <v>3.403</v>
       </c>
       <c r="H2" t="n">
-        <v>3.586</v>
+        <v>3.594</v>
       </c>
       <c r="I2" t="n">
-        <v>3.781</v>
+        <v>3.793</v>
       </c>
       <c r="J2" t="n">
-        <v>4.115</v>
+        <v>4.118</v>
       </c>
       <c r="K2" t="n">
-        <v>4.539</v>
+        <v>4.531</v>
       </c>
       <c r="L2" t="n">
-        <v>4.73</v>
+        <v>4.722</v>
       </c>
       <c r="M2" t="n">
-        <v>5.022</v>
+        <v>5.016</v>
       </c>
       <c r="N2" t="n">
-        <v>5.292</v>
+        <v>5.284</v>
       </c>
       <c r="O2" t="n">
-        <v>5.516</v>
+        <v>5.503</v>
       </c>
       <c r="P2" t="n">
-        <v>5.704</v>
+        <v>5.689</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.335</v>
+        <v>6.312</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.221</v>
+        <v>4.214</v>
       </c>
       <c r="G3" t="n">
-        <v>4.612</v>
+        <v>4.607</v>
       </c>
       <c r="H3" t="n">
-        <v>4.824</v>
+        <v>4.832</v>
       </c>
       <c r="I3" t="n">
-        <v>5.015</v>
+        <v>5.026</v>
       </c>
       <c r="J3" t="n">
-        <v>5.36</v>
+        <v>5.363</v>
       </c>
       <c r="K3" t="n">
-        <v>5.854</v>
+        <v>5.846</v>
       </c>
       <c r="L3" t="n">
-        <v>6.115</v>
+        <v>6.108</v>
       </c>
       <c r="M3" t="n">
-        <v>6.44</v>
+        <v>6.433</v>
       </c>
       <c r="N3" t="n">
-        <v>6.651</v>
+        <v>6.644</v>
       </c>
       <c r="O3" t="n">
-        <v>6.826</v>
+        <v>6.813</v>
       </c>
       <c r="P3" t="n">
-        <v>6.884</v>
+        <v>6.869</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.403</v>
+        <v>7.38</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.714</v>
+        <v>3.707</v>
       </c>
       <c r="G4" t="n">
-        <v>3.993</v>
+        <v>3.988</v>
       </c>
       <c r="H4" t="n">
-        <v>4.234</v>
+        <v>4.242</v>
       </c>
       <c r="I4" t="n">
-        <v>4.458</v>
+        <v>4.469</v>
       </c>
       <c r="J4" t="n">
-        <v>4.806</v>
+        <v>4.809</v>
       </c>
       <c r="K4" t="n">
-        <v>5.293</v>
+        <v>5.285</v>
       </c>
       <c r="L4" t="n">
-        <v>5.484</v>
+        <v>5.477</v>
       </c>
       <c r="M4" t="n">
-        <v>5.797</v>
+        <v>5.791</v>
       </c>
       <c r="N4" t="n">
-        <v>5.979</v>
+        <v>5.972</v>
       </c>
       <c r="O4" t="n">
-        <v>6.177</v>
+        <v>6.164</v>
       </c>
       <c r="P4" t="n">
-        <v>6.234</v>
+        <v>6.219</v>
       </c>
       <c r="Q4" t="n">
-        <v>6.756</v>
+        <v>6.733</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.896</v>
+        <v>2.889</v>
       </c>
       <c r="G5" t="n">
-        <v>2.951</v>
+        <v>2.946</v>
       </c>
       <c r="H5" t="n">
-        <v>3.087</v>
+        <v>3.094</v>
       </c>
       <c r="I5" t="n">
-        <v>3.352</v>
+        <v>3.364</v>
       </c>
       <c r="J5" t="n">
-        <v>3.678</v>
+        <v>3.681</v>
       </c>
       <c r="K5" t="n">
-        <v>3.96</v>
+        <v>3.951</v>
       </c>
       <c r="L5" t="n">
-        <v>3.993</v>
+        <v>3.984</v>
       </c>
       <c r="M5" t="n">
-        <v>4.087</v>
+        <v>4.08</v>
       </c>
       <c r="N5" t="n">
-        <v>4.108</v>
+        <v>4.101</v>
       </c>
       <c r="O5" t="n">
-        <v>4.115</v>
+        <v>4.102</v>
       </c>
       <c r="P5" t="n">
-        <v>4.372</v>
+        <v>4.357</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.247</v>
+        <v>5.224</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2.935</v>
+        <v>2.928</v>
       </c>
       <c r="G6" t="n">
-        <v>3.004</v>
+        <v>2.999</v>
       </c>
       <c r="H6" t="n">
-        <v>3.156</v>
+        <v>3.164</v>
       </c>
       <c r="I6" t="n">
-        <v>3.432</v>
+        <v>3.444</v>
       </c>
       <c r="J6" t="n">
-        <v>3.765</v>
+        <v>3.768</v>
       </c>
       <c r="K6" t="n">
-        <v>4.069</v>
+        <v>4.061</v>
       </c>
       <c r="L6" t="n">
-        <v>4.109</v>
+        <v>4.101</v>
       </c>
       <c r="M6" t="n">
-        <v>4.243</v>
+        <v>4.236</v>
       </c>
       <c r="N6" t="n">
-        <v>4.275</v>
+        <v>4.268</v>
       </c>
       <c r="O6" t="n">
-        <v>4.382</v>
+        <v>4.369</v>
       </c>
       <c r="P6" t="n">
-        <v>4.805</v>
+        <v>4.79</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.643</v>
+        <v>5.62</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2.916</v>
+        <v>2.909</v>
       </c>
       <c r="G7" t="n">
-        <v>2.968</v>
+        <v>2.963</v>
       </c>
       <c r="H7" t="n">
-        <v>3.102</v>
+        <v>3.11</v>
       </c>
       <c r="I7" t="n">
-        <v>3.366</v>
+        <v>3.378</v>
       </c>
       <c r="J7" t="n">
-        <v>3.703</v>
+        <v>3.706</v>
       </c>
       <c r="K7" t="n">
-        <v>3.986</v>
+        <v>3.978</v>
       </c>
       <c r="L7" t="n">
-        <v>4.017</v>
+        <v>4.008</v>
       </c>
       <c r="M7" t="n">
-        <v>4.148</v>
+        <v>4.142</v>
       </c>
       <c r="N7" t="n">
-        <v>4.168</v>
+        <v>4.16</v>
       </c>
       <c r="O7" t="n">
-        <v>4.279</v>
+        <v>4.266</v>
       </c>
       <c r="P7" t="n">
-        <v>4.588</v>
+        <v>4.573</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.411</v>
+        <v>5.388</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.331</v>
+        <v>5.324</v>
       </c>
       <c r="G8" t="n">
-        <v>5.91</v>
+        <v>5.905</v>
       </c>
       <c r="H8" t="n">
-        <v>6.273</v>
+        <v>6.281</v>
       </c>
       <c r="I8" t="n">
-        <v>6.542</v>
+        <v>6.553</v>
       </c>
       <c r="J8" t="n">
-        <v>6.951</v>
+        <v>6.954</v>
       </c>
       <c r="K8" t="n">
-        <v>7.725</v>
+        <v>7.717</v>
       </c>
       <c r="L8" t="n">
-        <v>8.074</v>
+        <v>8.066000000000001</v>
       </c>
       <c r="M8" t="n">
-        <v>8.428000000000001</v>
+        <v>8.420999999999999</v>
       </c>
       <c r="N8" t="n">
-        <v>8.574999999999999</v>
+        <v>8.567</v>
       </c>
       <c r="O8" t="n">
-        <v>8.834</v>
+        <v>8.821999999999999</v>
       </c>
       <c r="P8" t="n">
-        <v>8.994999999999999</v>
+        <v>8.98</v>
       </c>
       <c r="Q8" t="n">
-        <v>9.712999999999999</v>
+        <v>9.69</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,57 +1063,57 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.618</v>
+        <v>2.62</v>
       </c>
       <c r="G9" t="n">
         <v>2.699</v>
       </c>
       <c r="H9" t="n">
-        <v>2.8</v>
+        <v>2.805</v>
       </c>
       <c r="I9" t="n">
         <v>2.99</v>
       </c>
       <c r="J9" t="n">
-        <v>3.232</v>
+        <v>3.229</v>
       </c>
       <c r="K9" t="n">
-        <v>3.41</v>
+        <v>3.405</v>
       </c>
       <c r="L9" t="n">
-        <v>3.454</v>
+        <v>3.45</v>
       </c>
       <c r="M9" t="n">
-        <v>3.53</v>
+        <v>3.525</v>
       </c>
       <c r="N9" t="n">
-        <v>3.689</v>
+        <v>3.682</v>
       </c>
       <c r="O9" t="n">
-        <v>3.715</v>
+        <v>3.701</v>
       </c>
       <c r="P9" t="n">
-        <v>3.795</v>
+        <v>3.78</v>
       </c>
       <c r="Q9" t="n">
-        <v>3.865</v>
+        <v>3.842</v>
       </c>
       <c r="R9" t="n">
-        <v>3.832</v>
+        <v>3.807</v>
       </c>
       <c r="S9" t="n">
-        <v>3.795</v>
+        <v>3.777</v>
       </c>
       <c r="T9" t="n">
-        <v>3.712</v>
+        <v>3.69</v>
       </c>
       <c r="U9" t="n">
-        <v>3.584</v>
+        <v>3.561</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.632</v>
+        <v>2.634</v>
       </c>
       <c r="G10" t="n">
         <v>2.732</v>
       </c>
       <c r="H10" t="n">
-        <v>2.814</v>
+        <v>2.819</v>
       </c>
       <c r="I10" t="n">
-        <v>3.001</v>
+        <v>3.002</v>
       </c>
       <c r="J10" t="n">
-        <v>3.258</v>
+        <v>3.255</v>
       </c>
       <c r="K10" t="n">
-        <v>3.443</v>
+        <v>3.438</v>
       </c>
       <c r="L10" t="n">
-        <v>3.506</v>
+        <v>3.5</v>
       </c>
       <c r="M10" t="n">
-        <v>3.627</v>
+        <v>3.622</v>
       </c>
       <c r="N10" t="n">
-        <v>3.704</v>
+        <v>3.699</v>
       </c>
       <c r="O10" t="n">
-        <v>3.938</v>
+        <v>3.925</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.447</v>
+        <v>2.449</v>
       </c>
       <c r="G11" t="n">
         <v>2.542</v>
       </c>
       <c r="H11" t="n">
-        <v>2.638</v>
+        <v>2.643</v>
       </c>
       <c r="I11" t="n">
-        <v>2.804</v>
+        <v>2.805</v>
       </c>
       <c r="J11" t="n">
-        <v>3.052</v>
+        <v>3.049</v>
       </c>
       <c r="K11" t="n">
-        <v>3.231</v>
+        <v>3.226</v>
       </c>
       <c r="L11" t="n">
-        <v>3.3</v>
+        <v>3.294</v>
       </c>
       <c r="M11" t="n">
-        <v>3.432</v>
+        <v>3.427</v>
       </c>
       <c r="N11" t="n">
-        <v>3.513</v>
+        <v>3.508</v>
       </c>
       <c r="O11" t="n">
-        <v>3.705</v>
+        <v>3.692</v>
       </c>
       <c r="P11" t="n">
-        <v>3.741</v>
+        <v>3.726</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.066</v>
+        <v>4.043</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.184</v>
+        <v>3.181</v>
       </c>
       <c r="G12" t="n">
-        <v>3.34</v>
+        <v>3.338</v>
       </c>
       <c r="H12" t="n">
-        <v>3.461</v>
+        <v>3.464</v>
       </c>
       <c r="I12" t="n">
-        <v>3.704</v>
+        <v>3.713</v>
       </c>
       <c r="J12" t="n">
-        <v>4.088</v>
+        <v>4.092</v>
       </c>
       <c r="K12" t="n">
-        <v>4.309</v>
+        <v>4.304</v>
       </c>
       <c r="L12" t="n">
-        <v>4.383</v>
+        <v>4.378</v>
       </c>
       <c r="M12" t="n">
-        <v>4.52</v>
+        <v>4.515</v>
       </c>
       <c r="N12" t="n">
-        <v>4.574</v>
+        <v>4.565</v>
       </c>
       <c r="O12" t="n">
-        <v>4.716</v>
+        <v>4.702</v>
       </c>
       <c r="P12" t="n">
-        <v>4.84</v>
+        <v>4.825</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.194</v>
+        <v>5.17</v>
       </c>
       <c r="R12" t="n">
-        <v>5.333</v>
+        <v>5.307</v>
       </c>
       <c r="S12" t="n">
-        <v>5.506</v>
+        <v>5.487</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2.937</v>
+        <v>2.934</v>
       </c>
       <c r="G13" t="n">
-        <v>3.03</v>
+        <v>3.028</v>
       </c>
       <c r="H13" t="n">
-        <v>3.128</v>
+        <v>3.132</v>
       </c>
       <c r="I13" t="n">
-        <v>3.352</v>
+        <v>3.361</v>
       </c>
       <c r="J13" t="n">
-        <v>3.725</v>
+        <v>3.729</v>
       </c>
       <c r="K13" t="n">
-        <v>3.943</v>
+        <v>3.938</v>
       </c>
       <c r="L13" t="n">
-        <v>4.023</v>
+        <v>4.018</v>
       </c>
       <c r="M13" t="n">
-        <v>4.147</v>
+        <v>4.143</v>
       </c>
       <c r="N13" t="n">
-        <v>4.202</v>
+        <v>4.194</v>
       </c>
       <c r="O13" t="n">
-        <v>4.344</v>
+        <v>4.33</v>
       </c>
       <c r="P13" t="n">
-        <v>4.431</v>
+        <v>4.416</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.714</v>
+        <v>4.69</v>
       </c>
       <c r="R13" t="n">
-        <v>4.881</v>
+        <v>4.856</v>
       </c>
       <c r="S13" t="n">
-        <v>5.068</v>
+        <v>5.049</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.757</v>
+        <v>2.753</v>
       </c>
       <c r="G14" t="n">
-        <v>2.836</v>
+        <v>2.834</v>
       </c>
       <c r="H14" t="n">
-        <v>2.931</v>
+        <v>2.935</v>
       </c>
       <c r="I14" t="n">
-        <v>3.136</v>
+        <v>3.144</v>
       </c>
       <c r="J14" t="n">
-        <v>3.465</v>
+        <v>3.47</v>
       </c>
       <c r="K14" t="n">
-        <v>3.631</v>
+        <v>3.626</v>
       </c>
       <c r="L14" t="n">
-        <v>3.695</v>
+        <v>3.69</v>
       </c>
       <c r="M14" t="n">
-        <v>3.833</v>
+        <v>3.828</v>
       </c>
       <c r="N14" t="n">
-        <v>3.881</v>
+        <v>3.873</v>
       </c>
       <c r="O14" t="n">
-        <v>3.999</v>
+        <v>3.986</v>
       </c>
       <c r="P14" t="n">
-        <v>4.066</v>
+        <v>4.051</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.303</v>
+        <v>4.279</v>
       </c>
       <c r="R14" t="n">
-        <v>4.396</v>
+        <v>4.371</v>
       </c>
       <c r="S14" t="n">
-        <v>4.521</v>
+        <v>4.502</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.735</v>
+        <v>2.731</v>
       </c>
       <c r="G15" t="n">
-        <v>2.81</v>
+        <v>2.808</v>
       </c>
       <c r="H15" t="n">
-        <v>2.902</v>
+        <v>2.905</v>
       </c>
       <c r="I15" t="n">
-        <v>3.087</v>
+        <v>3.096</v>
       </c>
       <c r="J15" t="n">
-        <v>3.404</v>
+        <v>3.409</v>
       </c>
       <c r="K15" t="n">
-        <v>3.583</v>
+        <v>3.578</v>
       </c>
       <c r="L15" t="n">
-        <v>3.63</v>
+        <v>3.625</v>
       </c>
       <c r="M15" t="n">
-        <v>3.746</v>
+        <v>3.741</v>
       </c>
       <c r="N15" t="n">
-        <v>3.785</v>
+        <v>3.776</v>
       </c>
       <c r="O15" t="n">
-        <v>3.941</v>
+        <v>3.928</v>
       </c>
       <c r="P15" t="n">
-        <v>3.966</v>
+        <v>3.951</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.208</v>
+        <v>4.184</v>
       </c>
       <c r="R15" t="n">
-        <v>4.292</v>
+        <v>4.267</v>
       </c>
       <c r="S15" t="n">
-        <v>4.416</v>
+        <v>4.397</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.735</v>
+        <v>2.731</v>
       </c>
       <c r="G16" t="n">
-        <v>2.81</v>
+        <v>2.808</v>
       </c>
       <c r="H16" t="n">
-        <v>2.902</v>
+        <v>2.905</v>
       </c>
       <c r="I16" t="n">
-        <v>3.087</v>
+        <v>3.096</v>
       </c>
       <c r="J16" t="n">
-        <v>3.404</v>
+        <v>3.409</v>
       </c>
       <c r="K16" t="n">
-        <v>3.583</v>
+        <v>3.578</v>
       </c>
       <c r="L16" t="n">
-        <v>3.63</v>
+        <v>3.625</v>
       </c>
       <c r="M16" t="n">
-        <v>3.746</v>
+        <v>3.741</v>
       </c>
       <c r="N16" t="n">
-        <v>3.788</v>
+        <v>3.78</v>
       </c>
       <c r="O16" t="n">
-        <v>3.947</v>
+        <v>3.934</v>
       </c>
       <c r="P16" t="n">
-        <v>3.989</v>
+        <v>3.975</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.235</v>
+        <v>4.211</v>
       </c>
       <c r="R16" t="n">
-        <v>4.32</v>
+        <v>4.295</v>
       </c>
       <c r="S16" t="n">
-        <v>4.445</v>
+        <v>4.426</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.693</v>
+        <v>2.695</v>
       </c>
       <c r="G17" t="n">
-        <v>2.822</v>
+        <v>2.823</v>
       </c>
       <c r="H17" t="n">
-        <v>2.907</v>
+        <v>2.913</v>
       </c>
       <c r="I17" t="n">
-        <v>3.082</v>
+        <v>3.083</v>
       </c>
       <c r="J17" t="n">
-        <v>3.328</v>
+        <v>3.325</v>
       </c>
       <c r="K17" t="n">
-        <v>3.519</v>
+        <v>3.514</v>
       </c>
       <c r="L17" t="n">
-        <v>3.586</v>
+        <v>3.579</v>
       </c>
       <c r="M17" t="n">
-        <v>3.746</v>
+        <v>3.741</v>
       </c>
       <c r="N17" t="n">
-        <v>3.807</v>
+        <v>3.802</v>
       </c>
       <c r="O17" t="n">
-        <v>3.966</v>
+        <v>3.954</v>
       </c>
       <c r="P17" t="n">
-        <v>4.017</v>
+        <v>4.002</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.694</v>
+        <v>2.696</v>
       </c>
       <c r="G18" t="n">
-        <v>2.823</v>
+        <v>2.824</v>
       </c>
       <c r="H18" t="n">
-        <v>2.907</v>
+        <v>2.913</v>
       </c>
       <c r="I18" t="n">
-        <v>3.083</v>
+        <v>3.084</v>
       </c>
       <c r="J18" t="n">
-        <v>3.328</v>
+        <v>3.325</v>
       </c>
       <c r="K18" t="n">
-        <v>3.52</v>
+        <v>3.515</v>
       </c>
       <c r="L18" t="n">
-        <v>3.586</v>
+        <v>3.579</v>
       </c>
       <c r="M18" t="n">
-        <v>3.746</v>
+        <v>3.741</v>
       </c>
       <c r="N18" t="n">
-        <v>3.808</v>
+        <v>3.802</v>
       </c>
       <c r="O18" t="n">
-        <v>3.965</v>
+        <v>3.953</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.748</v>
+        <v>2.745</v>
       </c>
       <c r="G19" t="n">
-        <v>2.827</v>
+        <v>2.825</v>
       </c>
       <c r="H19" t="n">
-        <v>2.921</v>
+        <v>2.924</v>
       </c>
       <c r="I19" t="n">
-        <v>3.123</v>
+        <v>3.132</v>
       </c>
       <c r="J19" t="n">
-        <v>3.449</v>
+        <v>3.453</v>
       </c>
       <c r="K19" t="n">
-        <v>3.627</v>
+        <v>3.622</v>
       </c>
       <c r="L19" t="n">
-        <v>3.692</v>
+        <v>3.687</v>
       </c>
       <c r="M19" t="n">
-        <v>3.824</v>
+        <v>3.819</v>
       </c>
       <c r="N19" t="n">
-        <v>3.868</v>
+        <v>3.862</v>
       </c>
       <c r="O19" t="n">
-        <v>3.982</v>
+        <v>3.97</v>
       </c>
       <c r="P19" t="n">
-        <v>4.026</v>
+        <v>4.01</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.25</v>
+        <v>4.225</v>
       </c>
       <c r="R19" t="n">
-        <v>4.343</v>
+        <v>4.317</v>
       </c>
       <c r="S19" t="n">
-        <v>4.459</v>
+        <v>4.439</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2.573</v>
+        <v>2.572</v>
       </c>
       <c r="G20" t="n">
-        <v>2.644</v>
+        <v>2.643</v>
       </c>
       <c r="H20" t="n">
-        <v>2.691</v>
+        <v>2.694</v>
       </c>
       <c r="I20" t="n">
-        <v>2.83</v>
+        <v>2.836</v>
       </c>
       <c r="J20" t="n">
-        <v>3.233</v>
+        <v>3.234</v>
       </c>
       <c r="K20" t="n">
-        <v>3.43</v>
+        <v>3.425</v>
       </c>
       <c r="L20" t="n">
-        <v>3.465</v>
+        <v>3.46</v>
       </c>
       <c r="M20" t="n">
-        <v>3.56</v>
+        <v>3.555</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2.859</v>
+        <v>2.858</v>
       </c>
       <c r="G21" t="n">
         <v>2.935</v>
       </c>
       <c r="H21" t="n">
-        <v>3.07</v>
+        <v>3.074</v>
       </c>
       <c r="I21" t="n">
-        <v>3.245</v>
+        <v>3.251</v>
       </c>
       <c r="J21" t="n">
-        <v>3.588</v>
+        <v>3.59</v>
       </c>
       <c r="K21" t="n">
-        <v>3.865</v>
+        <v>3.857</v>
       </c>
       <c r="L21" t="n">
-        <v>3.939</v>
+        <v>3.932</v>
       </c>
       <c r="M21" t="n">
-        <v>4.065</v>
+        <v>4.056</v>
       </c>
       <c r="N21" t="n">
-        <v>4.123</v>
+        <v>4.115</v>
       </c>
       <c r="O21" t="n">
-        <v>4.199</v>
+        <v>4.187</v>
       </c>
       <c r="P21" t="n">
-        <v>4.293</v>
+        <v>4.278</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.412</v>
+        <v>4.388</v>
       </c>
       <c r="R21" t="n">
-        <v>4.394</v>
+        <v>4.37</v>
       </c>
       <c r="S21" t="n">
-        <v>4.42</v>
+        <v>4.402</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.806</v>
+        <v>2.805</v>
       </c>
       <c r="G22" t="n">
         <v>2.882</v>
       </c>
       <c r="H22" t="n">
-        <v>3.002</v>
+        <v>3.006</v>
       </c>
       <c r="I22" t="n">
-        <v>3.163</v>
+        <v>3.169</v>
       </c>
       <c r="J22" t="n">
-        <v>3.471</v>
+        <v>3.473</v>
       </c>
       <c r="K22" t="n">
-        <v>3.745</v>
+        <v>3.737</v>
       </c>
       <c r="L22" t="n">
-        <v>3.807</v>
+        <v>3.8</v>
       </c>
       <c r="M22" t="n">
-        <v>3.934</v>
+        <v>3.925</v>
       </c>
       <c r="N22" t="n">
-        <v>3.995</v>
+        <v>3.988</v>
       </c>
       <c r="O22" t="n">
-        <v>4.067</v>
+        <v>4.055</v>
       </c>
       <c r="P22" t="n">
-        <v>4.155</v>
+        <v>4.14</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.271</v>
+        <v>4.246</v>
       </c>
       <c r="R22" t="n">
-        <v>4.243</v>
+        <v>4.219</v>
       </c>
       <c r="S22" t="n">
-        <v>4.265</v>
+        <v>4.247</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.759</v>
+        <v>2.758</v>
       </c>
       <c r="G23" t="n">
         <v>2.836</v>
       </c>
       <c r="H23" t="n">
-        <v>2.941</v>
+        <v>2.945</v>
       </c>
       <c r="I23" t="n">
-        <v>3.118</v>
+        <v>3.125</v>
       </c>
       <c r="J23" t="n">
-        <v>3.416</v>
+        <v>3.418</v>
       </c>
       <c r="K23" t="n">
-        <v>3.654</v>
+        <v>3.646</v>
       </c>
       <c r="L23" t="n">
-        <v>3.715</v>
+        <v>3.708</v>
       </c>
       <c r="M23" t="n">
-        <v>3.835</v>
+        <v>3.825</v>
       </c>
       <c r="N23" t="n">
-        <v>3.891</v>
+        <v>3.883</v>
       </c>
       <c r="O23" t="n">
-        <v>3.943</v>
+        <v>3.931</v>
       </c>
       <c r="P23" t="n">
-        <v>4.017</v>
+        <v>4.002</v>
       </c>
       <c r="Q23" t="n">
-        <v>4.077</v>
+        <v>4.052</v>
       </c>
       <c r="R23" t="n">
-        <v>4.026</v>
+        <v>4.002</v>
       </c>
       <c r="S23" t="n">
-        <v>4.02</v>
+        <v>4.002</v>
       </c>
       <c r="T23" t="n">
-        <v>3.927</v>
+        <v>3.905</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.694</v>
+        <v>2.693</v>
       </c>
       <c r="G24" t="n">
         <v>2.75</v>
       </c>
       <c r="H24" t="n">
-        <v>2.842</v>
+        <v>2.846</v>
       </c>
       <c r="I24" t="n">
-        <v>3.028</v>
+        <v>3.035</v>
       </c>
       <c r="J24" t="n">
-        <v>3.315</v>
+        <v>3.317</v>
       </c>
       <c r="K24" t="n">
-        <v>3.538</v>
+        <v>3.53</v>
       </c>
       <c r="L24" t="n">
-        <v>3.589</v>
+        <v>3.582</v>
       </c>
       <c r="M24" t="n">
-        <v>3.695</v>
+        <v>3.686</v>
       </c>
       <c r="N24" t="n">
-        <v>3.768</v>
+        <v>3.761</v>
       </c>
       <c r="O24" t="n">
-        <v>3.938</v>
+        <v>3.926</v>
       </c>
       <c r="P24" t="n">
-        <v>3.959</v>
+        <v>3.943</v>
       </c>
       <c r="Q24" t="n">
-        <v>4</v>
+        <v>3.977</v>
       </c>
       <c r="R24" t="n">
-        <v>3.947</v>
+        <v>3.923</v>
       </c>
       <c r="S24" t="n">
-        <v>3.935</v>
+        <v>3.917</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.752</v>
+        <v>2.751</v>
       </c>
       <c r="G25" t="n">
         <v>2.835</v>
       </c>
       <c r="H25" t="n">
-        <v>2.944</v>
+        <v>2.948</v>
       </c>
       <c r="I25" t="n">
-        <v>3.126</v>
+        <v>3.133</v>
       </c>
       <c r="J25" t="n">
-        <v>3.432</v>
+        <v>3.434</v>
       </c>
       <c r="K25" t="n">
-        <v>3.687</v>
+        <v>3.679</v>
       </c>
       <c r="L25" t="n">
-        <v>3.744</v>
+        <v>3.737</v>
       </c>
       <c r="M25" t="n">
-        <v>3.865</v>
+        <v>3.855</v>
       </c>
       <c r="N25" t="n">
-        <v>3.918</v>
+        <v>3.91</v>
       </c>
       <c r="O25" t="n">
-        <v>3.972</v>
+        <v>3.96</v>
       </c>
       <c r="P25" t="n">
-        <v>4.038</v>
+        <v>4.023</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.11</v>
+        <v>4.086</v>
       </c>
       <c r="R25" t="n">
-        <v>4.049</v>
+        <v>4.025</v>
       </c>
       <c r="S25" t="n">
-        <v>4.043</v>
+        <v>4.025</v>
       </c>
       <c r="T25" t="n">
-        <v>3.945</v>
+        <v>3.923</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.05</v>
+        <v>3.045</v>
       </c>
       <c r="G26" t="n">
-        <v>3.186</v>
+        <v>3.182</v>
       </c>
       <c r="H26" t="n">
-        <v>3.41</v>
+        <v>3.413</v>
       </c>
       <c r="I26" t="n">
-        <v>3.645</v>
+        <v>3.652</v>
       </c>
       <c r="J26" t="n">
-        <v>4.092</v>
+        <v>4.093</v>
       </c>
       <c r="K26" t="n">
-        <v>4.5</v>
+        <v>4.494</v>
       </c>
       <c r="L26" t="n">
-        <v>4.618</v>
+        <v>4.612</v>
       </c>
       <c r="M26" t="n">
-        <v>4.799</v>
+        <v>4.794</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.052</v>
+        <v>5.039</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.847</v>
+        <v>2.843</v>
       </c>
       <c r="G27" t="n">
-        <v>2.918</v>
+        <v>2.916</v>
       </c>
       <c r="H27" t="n">
-        <v>3.041</v>
+        <v>3.043</v>
       </c>
       <c r="I27" t="n">
-        <v>3.245</v>
+        <v>3.252</v>
       </c>
       <c r="J27" t="n">
-        <v>3.588</v>
+        <v>3.591</v>
       </c>
       <c r="K27" t="n">
-        <v>3.811</v>
+        <v>3.806</v>
       </c>
       <c r="L27" t="n">
-        <v>3.878</v>
+        <v>3.873</v>
       </c>
       <c r="M27" t="n">
-        <v>4.003</v>
+        <v>3.999</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.143</v>
+        <v>4.13</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2.95</v>
+        <v>2.946</v>
       </c>
       <c r="G28" t="n">
-        <v>3.029</v>
+        <v>3.027</v>
       </c>
       <c r="H28" t="n">
-        <v>3.166</v>
+        <v>3.168</v>
       </c>
       <c r="I28" t="n">
-        <v>3.383</v>
+        <v>3.39</v>
       </c>
       <c r="J28" t="n">
-        <v>3.761</v>
+        <v>3.764</v>
       </c>
       <c r="K28" t="n">
-        <v>4.003</v>
+        <v>3.998</v>
       </c>
       <c r="L28" t="n">
-        <v>4.081</v>
+        <v>4.076</v>
       </c>
       <c r="M28" t="n">
-        <v>4.215</v>
+        <v>4.211</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.437</v>
+        <v>4.423</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.802</v>
+        <v>2.799</v>
       </c>
       <c r="G29" t="n">
-        <v>2.874</v>
+        <v>2.871</v>
       </c>
       <c r="H29" t="n">
-        <v>2.981</v>
+        <v>2.984</v>
       </c>
       <c r="I29" t="n">
-        <v>3.177</v>
+        <v>3.185</v>
       </c>
       <c r="J29" t="n">
-        <v>3.501</v>
+        <v>3.504</v>
       </c>
       <c r="K29" t="n">
-        <v>3.707</v>
+        <v>3.702</v>
       </c>
       <c r="L29" t="n">
-        <v>3.763</v>
+        <v>3.759</v>
       </c>
       <c r="M29" t="n">
-        <v>3.866</v>
+        <v>3.862</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>4.011</v>
+        <v>3.999</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.085</v>
+        <v>3.081</v>
       </c>
       <c r="G30" t="n">
-        <v>3.158</v>
+        <v>3.155</v>
       </c>
       <c r="H30" t="n">
-        <v>3.346</v>
+        <v>3.345</v>
       </c>
       <c r="I30" t="n">
-        <v>3.575</v>
+        <v>3.581</v>
       </c>
       <c r="J30" t="n">
-        <v>3.961</v>
+        <v>3.962</v>
       </c>
       <c r="K30" t="n">
-        <v>4.295</v>
+        <v>4.289</v>
       </c>
       <c r="L30" t="n">
-        <v>4.387</v>
+        <v>4.381</v>
       </c>
       <c r="M30" t="n">
-        <v>4.562</v>
+        <v>4.557</v>
       </c>
       <c r="N30" t="n">
-        <v>4.73</v>
+        <v>4.722</v>
       </c>
       <c r="O30" t="n">
-        <v>5.003</v>
+        <v>4.989</v>
       </c>
       <c r="P30" t="n">
-        <v>5.18</v>
+        <v>5.165</v>
       </c>
       <c r="Q30" t="n">
-        <v>5.939</v>
+        <v>5.916</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.411</v>
+        <v>3.408</v>
       </c>
       <c r="G31" t="n">
-        <v>3.518</v>
+        <v>3.516</v>
       </c>
       <c r="H31" t="n">
-        <v>3.758</v>
+        <v>3.76</v>
       </c>
       <c r="I31" t="n">
-        <v>4.003</v>
+        <v>4.009</v>
       </c>
       <c r="J31" t="n">
-        <v>4.451</v>
+        <v>4.452</v>
       </c>
       <c r="K31" t="n">
-        <v>4.827</v>
+        <v>4.821</v>
       </c>
       <c r="L31" t="n">
-        <v>4.999</v>
+        <v>4.993</v>
       </c>
       <c r="M31" t="n">
-        <v>5.292</v>
+        <v>5.286</v>
       </c>
       <c r="N31" t="n">
-        <v>5.587</v>
+        <v>5.579</v>
       </c>
       <c r="O31" t="n">
-        <v>6.036</v>
+        <v>6.023</v>
       </c>
       <c r="P31" t="n">
-        <v>6.167</v>
+        <v>6.152</v>
       </c>
       <c r="Q31" t="n">
-        <v>6.912</v>
+        <v>6.89</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.183</v>
+        <v>3.18</v>
       </c>
       <c r="G32" t="n">
-        <v>3.274</v>
+        <v>3.272</v>
       </c>
       <c r="H32" t="n">
         <v>3.489</v>
       </c>
       <c r="I32" t="n">
-        <v>3.734</v>
+        <v>3.739</v>
       </c>
       <c r="J32" t="n">
-        <v>4.14</v>
+        <v>4.141</v>
       </c>
       <c r="K32" t="n">
-        <v>4.48</v>
+        <v>4.474</v>
       </c>
       <c r="L32" t="n">
-        <v>4.591</v>
+        <v>4.585</v>
       </c>
       <c r="M32" t="n">
-        <v>4.835</v>
+        <v>4.829</v>
       </c>
       <c r="N32" t="n">
-        <v>5.09</v>
+        <v>5.083</v>
       </c>
       <c r="O32" t="n">
-        <v>5.447</v>
+        <v>5.434</v>
       </c>
       <c r="P32" t="n">
-        <v>5.639</v>
+        <v>5.624</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.4</v>
+        <v>6.377</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2.956</v>
+        <v>2.951</v>
       </c>
       <c r="G33" t="n">
-        <v>3.026</v>
+        <v>3.022</v>
       </c>
       <c r="H33" t="n">
-        <v>3.164</v>
+        <v>3.163</v>
       </c>
       <c r="I33" t="n">
-        <v>3.356</v>
+        <v>3.361</v>
       </c>
       <c r="J33" t="n">
-        <v>3.667</v>
+        <v>3.669</v>
       </c>
       <c r="K33" t="n">
-        <v>3.935</v>
+        <v>3.93</v>
       </c>
       <c r="L33" t="n">
-        <v>3.993</v>
+        <v>3.988</v>
       </c>
       <c r="M33" t="n">
-        <v>4.095</v>
+        <v>4.09</v>
       </c>
       <c r="N33" t="n">
-        <v>4.122</v>
+        <v>4.115</v>
       </c>
       <c r="O33" t="n">
-        <v>4.16</v>
+        <v>4.147</v>
       </c>
       <c r="P33" t="n">
-        <v>4.212</v>
+        <v>4.197</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.656</v>
+        <v>4.633</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.015</v>
+        <v>3.01</v>
       </c>
       <c r="G34" t="n">
-        <v>3.08</v>
+        <v>3.076</v>
       </c>
       <c r="H34" t="n">
-        <v>3.226</v>
+        <v>3.225</v>
       </c>
       <c r="I34" t="n">
-        <v>3.424</v>
+        <v>3.429</v>
       </c>
       <c r="J34" t="n">
-        <v>3.739</v>
+        <v>3.741</v>
       </c>
       <c r="K34" t="n">
-        <v>4.011</v>
+        <v>4.006</v>
       </c>
       <c r="L34" t="n">
-        <v>4.072</v>
+        <v>4.067</v>
       </c>
       <c r="M34" t="n">
-        <v>4.185</v>
+        <v>4.181</v>
       </c>
       <c r="N34" t="n">
-        <v>4.227</v>
+        <v>4.22</v>
       </c>
       <c r="O34" t="n">
-        <v>4.328</v>
+        <v>4.316</v>
       </c>
       <c r="P34" t="n">
-        <v>4.506</v>
+        <v>4.491</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.357</v>
+        <v>5.334</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>2.99</v>
+        <v>2.985</v>
       </c>
       <c r="G35" t="n">
-        <v>3.053</v>
+        <v>3.049</v>
       </c>
       <c r="H35" t="n">
-        <v>3.194</v>
+        <v>3.193</v>
       </c>
       <c r="I35" t="n">
-        <v>3.39</v>
+        <v>3.396</v>
       </c>
       <c r="J35" t="n">
-        <v>3.707</v>
+        <v>3.709</v>
       </c>
       <c r="K35" t="n">
-        <v>3.966</v>
+        <v>3.961</v>
       </c>
       <c r="L35" t="n">
-        <v>4.027</v>
+        <v>4.022</v>
       </c>
       <c r="M35" t="n">
-        <v>4.132</v>
+        <v>4.128</v>
       </c>
       <c r="N35" t="n">
-        <v>4.163</v>
+        <v>4.156</v>
       </c>
       <c r="O35" t="n">
-        <v>4.226</v>
+        <v>4.214</v>
       </c>
       <c r="P35" t="n">
-        <v>4.309</v>
+        <v>4.294</v>
       </c>
       <c r="Q35" t="n">
-        <v>4.993</v>
+        <v>4.97</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.898</v>
+        <v>2.893</v>
       </c>
       <c r="G36" t="n">
-        <v>2.963</v>
+        <v>2.959</v>
       </c>
       <c r="H36" t="n">
-        <v>3.085</v>
+        <v>3.084</v>
       </c>
       <c r="I36" t="n">
-        <v>3.282</v>
+        <v>3.288</v>
       </c>
       <c r="J36" t="n">
-        <v>3.603</v>
+        <v>3.605</v>
       </c>
       <c r="K36" t="n">
-        <v>3.858</v>
+        <v>3.853</v>
       </c>
       <c r="L36" t="n">
-        <v>3.917</v>
+        <v>3.913</v>
       </c>
       <c r="M36" t="n">
-        <v>3.994</v>
+        <v>3.99</v>
       </c>
       <c r="N36" t="n">
-        <v>4.024</v>
+        <v>4.018</v>
       </c>
       <c r="O36" t="n">
-        <v>4.068</v>
+        <v>4.057</v>
       </c>
       <c r="P36" t="n">
-        <v>4.111</v>
+        <v>4.096</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.373</v>
+        <v>4.35</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.754</v>
+        <v>3.751</v>
       </c>
       <c r="G37" t="n">
-        <v>4.212</v>
+        <v>4.21</v>
       </c>
       <c r="H37" t="n">
-        <v>4.733</v>
+        <v>4.736</v>
       </c>
       <c r="I37" t="n">
-        <v>5.068</v>
+        <v>5.074</v>
       </c>
       <c r="J37" t="n">
-        <v>5.942</v>
+        <v>5.943</v>
       </c>
       <c r="K37" t="n">
-        <v>6.867</v>
+        <v>6.861</v>
       </c>
       <c r="L37" t="n">
-        <v>7.199</v>
+        <v>7.193</v>
       </c>
       <c r="M37" t="n">
-        <v>7.565</v>
+        <v>7.559</v>
       </c>
       <c r="N37" t="n">
-        <v>7.737</v>
+        <v>7.729</v>
       </c>
       <c r="O37" t="n">
-        <v>7.915</v>
+        <v>7.902</v>
       </c>
       <c r="P37" t="n">
-        <v>7.967</v>
+        <v>7.952</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.401</v>
+        <v>8.378</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.813</v>
+        <v>4.81</v>
       </c>
       <c r="G38" t="n">
-        <v>5.524</v>
+        <v>5.522</v>
       </c>
       <c r="H38" t="n">
-        <v>6.257</v>
+        <v>6.26</v>
       </c>
       <c r="I38" t="n">
-        <v>6.749</v>
+        <v>6.755</v>
       </c>
       <c r="J38" t="n">
-        <v>7.884</v>
+        <v>7.885</v>
       </c>
       <c r="K38" t="n">
-        <v>8.984999999999999</v>
+        <v>8.978999999999999</v>
       </c>
       <c r="L38" t="n">
-        <v>9.477</v>
+        <v>9.471</v>
       </c>
       <c r="M38" t="n">
-        <v>9.974</v>
+        <v>9.968999999999999</v>
       </c>
       <c r="N38" t="n">
-        <v>10.155</v>
+        <v>10.147</v>
       </c>
       <c r="O38" t="n">
-        <v>10.315</v>
+        <v>10.301</v>
       </c>
       <c r="P38" t="n">
-        <v>10.364</v>
+        <v>10.349</v>
       </c>
       <c r="Q38" t="n">
-        <v>10.852</v>
+        <v>10.828</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.134</v>
+        <v>4.131</v>
       </c>
       <c r="G39" t="n">
-        <v>4.722</v>
+        <v>4.72</v>
       </c>
       <c r="H39" t="n">
-        <v>5.322</v>
+        <v>5.325</v>
       </c>
       <c r="I39" t="n">
-        <v>5.753</v>
+        <v>5.758</v>
       </c>
       <c r="J39" t="n">
-        <v>6.756</v>
+        <v>6.757</v>
       </c>
       <c r="K39" t="n">
-        <v>7.818</v>
+        <v>7.812</v>
       </c>
       <c r="L39" t="n">
-        <v>8.234999999999999</v>
+        <v>8.228999999999999</v>
       </c>
       <c r="M39" t="n">
-        <v>8.611000000000001</v>
+        <v>8.605</v>
       </c>
       <c r="N39" t="n">
-        <v>8.782999999999999</v>
+        <v>8.775</v>
       </c>
       <c r="O39" t="n">
-        <v>8.965</v>
+        <v>8.952</v>
       </c>
       <c r="P39" t="n">
-        <v>9.019</v>
+        <v>9.004</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.497</v>
+        <v>9.474</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.278</v>
+        <v>3.274</v>
       </c>
       <c r="G40" t="n">
-        <v>3.397</v>
+        <v>3.393</v>
       </c>
       <c r="H40" t="n">
-        <v>3.606</v>
+        <v>3.605</v>
       </c>
       <c r="I40" t="n">
-        <v>3.85</v>
+        <v>3.855</v>
       </c>
       <c r="J40" t="n">
-        <v>4.254</v>
+        <v>4.255</v>
       </c>
       <c r="K40" t="n">
-        <v>4.599</v>
+        <v>4.593</v>
       </c>
       <c r="L40" t="n">
-        <v>4.711</v>
+        <v>4.705</v>
       </c>
       <c r="M40" t="n">
-        <v>4.903</v>
+        <v>4.898</v>
       </c>
       <c r="N40" t="n">
-        <v>5.087</v>
+        <v>5.08</v>
       </c>
       <c r="O40" t="n">
-        <v>5.381</v>
+        <v>5.368</v>
       </c>
       <c r="P40" t="n">
-        <v>5.601</v>
+        <v>5.586</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.39</v>
+        <v>6.367</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.661</v>
+        <v>3.658</v>
       </c>
       <c r="G41" t="n">
-        <v>3.821</v>
+        <v>3.819</v>
       </c>
       <c r="H41" t="n">
-        <v>4.088</v>
+        <v>4.09</v>
       </c>
       <c r="I41" t="n">
-        <v>4.352</v>
+        <v>4.358</v>
       </c>
       <c r="J41" t="n">
-        <v>4.807</v>
+        <v>4.808</v>
       </c>
       <c r="K41" t="n">
-        <v>5.199</v>
+        <v>5.193</v>
       </c>
       <c r="L41" t="n">
-        <v>5.389</v>
+        <v>5.383</v>
       </c>
       <c r="M41" t="n">
-        <v>5.705</v>
+        <v>5.699</v>
       </c>
       <c r="N41" t="n">
-        <v>6.016</v>
+        <v>6.009</v>
       </c>
       <c r="O41" t="n">
-        <v>6.494</v>
+        <v>6.48</v>
       </c>
       <c r="P41" t="n">
-        <v>6.659</v>
+        <v>6.644</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.437</v>
+        <v>7.414</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.398</v>
+        <v>3.395</v>
       </c>
       <c r="G42" t="n">
-        <v>3.545</v>
+        <v>3.543</v>
       </c>
       <c r="H42" t="n">
         <v>3.781</v>
       </c>
       <c r="I42" t="n">
-        <v>4.038</v>
+        <v>4.044</v>
       </c>
       <c r="J42" t="n">
-        <v>4.457</v>
+        <v>4.458</v>
       </c>
       <c r="K42" t="n">
-        <v>4.82</v>
+        <v>4.814</v>
       </c>
       <c r="L42" t="n">
-        <v>4.947</v>
+        <v>4.941</v>
       </c>
       <c r="M42" t="n">
-        <v>5.21</v>
+        <v>5.205</v>
       </c>
       <c r="N42" t="n">
-        <v>5.502</v>
+        <v>5.494</v>
       </c>
       <c r="O42" t="n">
-        <v>5.872</v>
+        <v>5.858</v>
       </c>
       <c r="P42" t="n">
-        <v>6.102</v>
+        <v>6.087</v>
       </c>
       <c r="Q42" t="n">
-        <v>6.903</v>
+        <v>6.88</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.104</v>
+        <v>3.099</v>
       </c>
       <c r="G43" t="n">
-        <v>3.209</v>
+        <v>3.205</v>
       </c>
       <c r="H43" t="n">
-        <v>3.365</v>
+        <v>3.364</v>
       </c>
       <c r="I43" t="n">
-        <v>3.565</v>
+        <v>3.571</v>
       </c>
       <c r="J43" t="n">
-        <v>3.895</v>
+        <v>3.897</v>
       </c>
       <c r="K43" t="n">
-        <v>4.166</v>
+        <v>4.161</v>
       </c>
       <c r="L43" t="n">
-        <v>4.234</v>
+        <v>4.229</v>
       </c>
       <c r="M43" t="n">
-        <v>4.349</v>
+        <v>4.344</v>
       </c>
       <c r="N43" t="n">
-        <v>4.392</v>
+        <v>4.385</v>
       </c>
       <c r="O43" t="n">
-        <v>4.472</v>
+        <v>4.46</v>
       </c>
       <c r="P43" t="n">
-        <v>4.578</v>
+        <v>4.563</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.266</v>
+        <v>5.243</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46140</v>
+        <v>46141</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>2.976</v>
+        <v>2.971</v>
       </c>
       <c r="G44" t="n">
-        <v>3.073</v>
+        <v>3.069</v>
       </c>
       <c r="H44" t="n">
-        <v>3.209</v>
+        <v>3.208</v>
       </c>
       <c r="I44" t="n">
-        <v>3.41</v>
+        <v>3.416</v>
       </c>
       <c r="J44" t="n">
-        <v>3.744</v>
+        <v>3.746</v>
       </c>
       <c r="K44" t="n">
-        <v>4.009</v>
+        <v>4.004</v>
       </c>
       <c r="L44" t="n">
-        <v>4.077</v>
+        <v>4.073</v>
       </c>
       <c r="M44" t="n">
-        <v>4.163</v>
+        <v>4.159</v>
       </c>
       <c r="N44" t="n">
-        <v>4.205</v>
+        <v>4.2</v>
       </c>
       <c r="O44" t="n">
-        <v>4.267</v>
+        <v>4.256</v>
       </c>
       <c r="P44" t="n">
-        <v>4.341</v>
+        <v>4.326</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.637</v>
+        <v>4.614</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-04-30 ~ 2026-04-30
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.191</v>
+        <v>3.194</v>
       </c>
       <c r="G2" t="n">
-        <v>3.403</v>
+        <v>3.409</v>
       </c>
       <c r="H2" t="n">
-        <v>3.594</v>
+        <v>3.615</v>
       </c>
       <c r="I2" t="n">
-        <v>3.793</v>
+        <v>3.814</v>
       </c>
       <c r="J2" t="n">
-        <v>4.118</v>
+        <v>4.152</v>
       </c>
       <c r="K2" t="n">
-        <v>4.531</v>
+        <v>4.591</v>
       </c>
       <c r="L2" t="n">
-        <v>4.722</v>
+        <v>4.797</v>
       </c>
       <c r="M2" t="n">
-        <v>5.016</v>
+        <v>5.08</v>
       </c>
       <c r="N2" t="n">
-        <v>5.284</v>
+        <v>5.352</v>
       </c>
       <c r="O2" t="n">
-        <v>5.503</v>
+        <v>5.576</v>
       </c>
       <c r="P2" t="n">
-        <v>5.689</v>
+        <v>5.76</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.312</v>
+        <v>6.385</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.214</v>
+        <v>4.217</v>
       </c>
       <c r="G3" t="n">
-        <v>4.607</v>
+        <v>4.613</v>
       </c>
       <c r="H3" t="n">
-        <v>4.832</v>
+        <v>4.853</v>
       </c>
       <c r="I3" t="n">
-        <v>5.026</v>
+        <v>5.047</v>
       </c>
       <c r="J3" t="n">
-        <v>5.363</v>
+        <v>5.397</v>
       </c>
       <c r="K3" t="n">
-        <v>5.846</v>
+        <v>5.907</v>
       </c>
       <c r="L3" t="n">
-        <v>6.108</v>
+        <v>6.183</v>
       </c>
       <c r="M3" t="n">
-        <v>6.433</v>
+        <v>6.498</v>
       </c>
       <c r="N3" t="n">
-        <v>6.644</v>
+        <v>6.711</v>
       </c>
       <c r="O3" t="n">
-        <v>6.813</v>
+        <v>6.886</v>
       </c>
       <c r="P3" t="n">
-        <v>6.869</v>
+        <v>6.94</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.38</v>
+        <v>7.453</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>3.707</v>
+        <v>3.71</v>
       </c>
       <c r="G4" t="n">
-        <v>3.988</v>
+        <v>3.994</v>
       </c>
       <c r="H4" t="n">
-        <v>4.242</v>
+        <v>4.263</v>
       </c>
       <c r="I4" t="n">
-        <v>4.469</v>
+        <v>4.49</v>
       </c>
       <c r="J4" t="n">
-        <v>4.809</v>
+        <v>4.843</v>
       </c>
       <c r="K4" t="n">
-        <v>5.285</v>
+        <v>5.346</v>
       </c>
       <c r="L4" t="n">
-        <v>5.477</v>
+        <v>5.552</v>
       </c>
       <c r="M4" t="n">
-        <v>5.791</v>
+        <v>5.855</v>
       </c>
       <c r="N4" t="n">
-        <v>5.972</v>
+        <v>6.039</v>
       </c>
       <c r="O4" t="n">
-        <v>6.164</v>
+        <v>6.237</v>
       </c>
       <c r="P4" t="n">
-        <v>6.219</v>
+        <v>6.29</v>
       </c>
       <c r="Q4" t="n">
-        <v>6.733</v>
+        <v>6.806</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -774,37 +774,37 @@
         <v>2.889</v>
       </c>
       <c r="G5" t="n">
-        <v>2.946</v>
+        <v>2.952</v>
       </c>
       <c r="H5" t="n">
-        <v>3.094</v>
+        <v>3.116</v>
       </c>
       <c r="I5" t="n">
-        <v>3.364</v>
+        <v>3.385</v>
       </c>
       <c r="J5" t="n">
-        <v>3.681</v>
+        <v>3.715</v>
       </c>
       <c r="K5" t="n">
-        <v>3.951</v>
+        <v>4.011</v>
       </c>
       <c r="L5" t="n">
-        <v>3.984</v>
+        <v>4.056</v>
       </c>
       <c r="M5" t="n">
-        <v>4.08</v>
+        <v>4.143</v>
       </c>
       <c r="N5" t="n">
-        <v>4.101</v>
+        <v>4.166</v>
       </c>
       <c r="O5" t="n">
-        <v>4.102</v>
+        <v>4.175</v>
       </c>
       <c r="P5" t="n">
-        <v>4.357</v>
+        <v>4.429</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.224</v>
+        <v>5.297</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -847,37 +847,37 @@
         <v>2.928</v>
       </c>
       <c r="G6" t="n">
-        <v>2.999</v>
+        <v>3.005</v>
       </c>
       <c r="H6" t="n">
-        <v>3.164</v>
+        <v>3.185</v>
       </c>
       <c r="I6" t="n">
-        <v>3.444</v>
+        <v>3.465</v>
       </c>
       <c r="J6" t="n">
-        <v>3.768</v>
+        <v>3.802</v>
       </c>
       <c r="K6" t="n">
-        <v>4.061</v>
+        <v>4.12</v>
       </c>
       <c r="L6" t="n">
-        <v>4.101</v>
+        <v>4.173</v>
       </c>
       <c r="M6" t="n">
-        <v>4.236</v>
+        <v>4.299</v>
       </c>
       <c r="N6" t="n">
-        <v>4.268</v>
+        <v>4.333</v>
       </c>
       <c r="O6" t="n">
-        <v>4.369</v>
+        <v>4.442</v>
       </c>
       <c r="P6" t="n">
-        <v>4.79</v>
+        <v>4.861</v>
       </c>
       <c r="Q6" t="n">
-        <v>5.62</v>
+        <v>5.693</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -920,37 +920,37 @@
         <v>2.909</v>
       </c>
       <c r="G7" t="n">
-        <v>2.963</v>
+        <v>2.969</v>
       </c>
       <c r="H7" t="n">
-        <v>3.11</v>
+        <v>3.131</v>
       </c>
       <c r="I7" t="n">
-        <v>3.378</v>
+        <v>3.399</v>
       </c>
       <c r="J7" t="n">
-        <v>3.706</v>
+        <v>3.74</v>
       </c>
       <c r="K7" t="n">
-        <v>3.978</v>
+        <v>4.037</v>
       </c>
       <c r="L7" t="n">
-        <v>4.008</v>
+        <v>4.08</v>
       </c>
       <c r="M7" t="n">
-        <v>4.142</v>
+        <v>4.204</v>
       </c>
       <c r="N7" t="n">
-        <v>4.16</v>
+        <v>4.225</v>
       </c>
       <c r="O7" t="n">
-        <v>4.266</v>
+        <v>4.34</v>
       </c>
       <c r="P7" t="n">
-        <v>4.573</v>
+        <v>4.645</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.388</v>
+        <v>5.461</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.324</v>
+        <v>5.327</v>
       </c>
       <c r="G8" t="n">
-        <v>5.905</v>
+        <v>5.911</v>
       </c>
       <c r="H8" t="n">
-        <v>6.281</v>
+        <v>6.302</v>
       </c>
       <c r="I8" t="n">
-        <v>6.553</v>
+        <v>6.574</v>
       </c>
       <c r="J8" t="n">
-        <v>6.954</v>
+        <v>6.989</v>
       </c>
       <c r="K8" t="n">
-        <v>7.717</v>
+        <v>7.779</v>
       </c>
       <c r="L8" t="n">
-        <v>8.066000000000001</v>
+        <v>8.141999999999999</v>
       </c>
       <c r="M8" t="n">
-        <v>8.420999999999999</v>
+        <v>8.487</v>
       </c>
       <c r="N8" t="n">
-        <v>8.567</v>
+        <v>8.635</v>
       </c>
       <c r="O8" t="n">
-        <v>8.821999999999999</v>
+        <v>8.895</v>
       </c>
       <c r="P8" t="n">
-        <v>8.98</v>
+        <v>9.051</v>
       </c>
       <c r="Q8" t="n">
-        <v>9.69</v>
+        <v>9.763</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,57 +1063,57 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2.62</v>
+        <v>2.622</v>
       </c>
       <c r="G9" t="n">
-        <v>2.699</v>
+        <v>2.702</v>
       </c>
       <c r="H9" t="n">
-        <v>2.805</v>
+        <v>2.81</v>
       </c>
       <c r="I9" t="n">
-        <v>2.99</v>
+        <v>3.02</v>
       </c>
       <c r="J9" t="n">
-        <v>3.229</v>
+        <v>3.268</v>
       </c>
       <c r="K9" t="n">
-        <v>3.405</v>
+        <v>3.485</v>
       </c>
       <c r="L9" t="n">
-        <v>3.45</v>
+        <v>3.53</v>
       </c>
       <c r="M9" t="n">
-        <v>3.525</v>
+        <v>3.592</v>
       </c>
       <c r="N9" t="n">
-        <v>3.682</v>
+        <v>3.75</v>
       </c>
       <c r="O9" t="n">
-        <v>3.701</v>
+        <v>3.775</v>
       </c>
       <c r="P9" t="n">
-        <v>3.78</v>
+        <v>3.851</v>
       </c>
       <c r="Q9" t="n">
-        <v>3.842</v>
+        <v>3.915</v>
       </c>
       <c r="R9" t="n">
-        <v>3.807</v>
+        <v>3.889</v>
       </c>
       <c r="S9" t="n">
-        <v>3.777</v>
+        <v>3.865</v>
       </c>
       <c r="T9" t="n">
-        <v>3.69</v>
+        <v>3.785</v>
       </c>
       <c r="U9" t="n">
-        <v>3.561</v>
+        <v>3.656</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2.634</v>
+        <v>2.636</v>
       </c>
       <c r="G10" t="n">
-        <v>2.732</v>
+        <v>2.735</v>
       </c>
       <c r="H10" t="n">
-        <v>2.819</v>
+        <v>2.824</v>
       </c>
       <c r="I10" t="n">
-        <v>3.002</v>
+        <v>3.032</v>
       </c>
       <c r="J10" t="n">
-        <v>3.255</v>
+        <v>3.293</v>
       </c>
       <c r="K10" t="n">
-        <v>3.438</v>
+        <v>3.518</v>
       </c>
       <c r="L10" t="n">
-        <v>3.5</v>
+        <v>3.581</v>
       </c>
       <c r="M10" t="n">
-        <v>3.622</v>
+        <v>3.69</v>
       </c>
       <c r="N10" t="n">
-        <v>3.699</v>
+        <v>3.767</v>
       </c>
       <c r="O10" t="n">
-        <v>3.925</v>
+        <v>3.991</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.449</v>
+        <v>2.451</v>
       </c>
       <c r="G11" t="n">
-        <v>2.542</v>
+        <v>2.545</v>
       </c>
       <c r="H11" t="n">
-        <v>2.643</v>
+        <v>2.648</v>
       </c>
       <c r="I11" t="n">
-        <v>2.805</v>
+        <v>2.835</v>
       </c>
       <c r="J11" t="n">
-        <v>3.049</v>
+        <v>3.088</v>
       </c>
       <c r="K11" t="n">
-        <v>3.226</v>
+        <v>3.306</v>
       </c>
       <c r="L11" t="n">
-        <v>3.294</v>
+        <v>3.374</v>
       </c>
       <c r="M11" t="n">
-        <v>3.427</v>
+        <v>3.495</v>
       </c>
       <c r="N11" t="n">
-        <v>3.508</v>
+        <v>3.575</v>
       </c>
       <c r="O11" t="n">
-        <v>3.692</v>
+        <v>3.757</v>
       </c>
       <c r="P11" t="n">
-        <v>3.726</v>
+        <v>3.798</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.043</v>
+        <v>4.116</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.181</v>
+        <v>3.185</v>
       </c>
       <c r="G12" t="n">
-        <v>3.338</v>
+        <v>3.347</v>
       </c>
       <c r="H12" t="n">
-        <v>3.464</v>
+        <v>3.491</v>
       </c>
       <c r="I12" t="n">
-        <v>3.713</v>
+        <v>3.745</v>
       </c>
       <c r="J12" t="n">
-        <v>4.092</v>
+        <v>4.128</v>
       </c>
       <c r="K12" t="n">
-        <v>4.304</v>
+        <v>4.361</v>
       </c>
       <c r="L12" t="n">
-        <v>4.378</v>
+        <v>4.452</v>
       </c>
       <c r="M12" t="n">
-        <v>4.515</v>
+        <v>4.581</v>
       </c>
       <c r="N12" t="n">
-        <v>4.565</v>
+        <v>4.631</v>
       </c>
       <c r="O12" t="n">
-        <v>4.702</v>
+        <v>4.775</v>
       </c>
       <c r="P12" t="n">
-        <v>4.825</v>
+        <v>4.896</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.17</v>
+        <v>5.243</v>
       </c>
       <c r="R12" t="n">
-        <v>5.307</v>
+        <v>5.389</v>
       </c>
       <c r="S12" t="n">
-        <v>5.487</v>
+        <v>5.575</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2.934</v>
+        <v>2.938</v>
       </c>
       <c r="G13" t="n">
-        <v>3.028</v>
+        <v>3.037</v>
       </c>
       <c r="H13" t="n">
-        <v>3.132</v>
+        <v>3.158</v>
       </c>
       <c r="I13" t="n">
-        <v>3.361</v>
+        <v>3.392</v>
       </c>
       <c r="J13" t="n">
-        <v>3.729</v>
+        <v>3.765</v>
       </c>
       <c r="K13" t="n">
-        <v>3.938</v>
+        <v>3.994</v>
       </c>
       <c r="L13" t="n">
-        <v>4.018</v>
+        <v>4.092</v>
       </c>
       <c r="M13" t="n">
-        <v>4.143</v>
+        <v>4.208</v>
       </c>
       <c r="N13" t="n">
-        <v>4.194</v>
+        <v>4.26</v>
       </c>
       <c r="O13" t="n">
-        <v>4.33</v>
+        <v>4.404</v>
       </c>
       <c r="P13" t="n">
-        <v>4.416</v>
+        <v>4.488</v>
       </c>
       <c r="Q13" t="n">
-        <v>4.69</v>
+        <v>4.763</v>
       </c>
       <c r="R13" t="n">
-        <v>4.856</v>
+        <v>4.937</v>
       </c>
       <c r="S13" t="n">
-        <v>5.049</v>
+        <v>5.137</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2.753</v>
+        <v>2.757</v>
       </c>
       <c r="G14" t="n">
-        <v>2.834</v>
+        <v>2.842</v>
       </c>
       <c r="H14" t="n">
-        <v>2.935</v>
+        <v>2.961</v>
       </c>
       <c r="I14" t="n">
-        <v>3.144</v>
+        <v>3.176</v>
       </c>
       <c r="J14" t="n">
-        <v>3.47</v>
+        <v>3.505</v>
       </c>
       <c r="K14" t="n">
-        <v>3.626</v>
+        <v>3.682</v>
       </c>
       <c r="L14" t="n">
-        <v>3.69</v>
+        <v>3.764</v>
       </c>
       <c r="M14" t="n">
-        <v>3.828</v>
+        <v>3.894</v>
       </c>
       <c r="N14" t="n">
-        <v>3.873</v>
+        <v>3.939</v>
       </c>
       <c r="O14" t="n">
-        <v>3.986</v>
+        <v>4.059</v>
       </c>
       <c r="P14" t="n">
-        <v>4.051</v>
+        <v>4.122</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.279</v>
+        <v>4.352</v>
       </c>
       <c r="R14" t="n">
-        <v>4.371</v>
+        <v>4.453</v>
       </c>
       <c r="S14" t="n">
-        <v>4.502</v>
+        <v>4.59</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>2.731</v>
+        <v>2.735</v>
       </c>
       <c r="G15" t="n">
-        <v>2.808</v>
+        <v>2.816</v>
       </c>
       <c r="H15" t="n">
-        <v>2.905</v>
+        <v>2.932</v>
       </c>
       <c r="I15" t="n">
-        <v>3.096</v>
+        <v>3.127</v>
       </c>
       <c r="J15" t="n">
-        <v>3.409</v>
+        <v>3.444</v>
       </c>
       <c r="K15" t="n">
-        <v>3.578</v>
+        <v>3.635</v>
       </c>
       <c r="L15" t="n">
-        <v>3.625</v>
+        <v>3.699</v>
       </c>
       <c r="M15" t="n">
-        <v>3.741</v>
+        <v>3.807</v>
       </c>
       <c r="N15" t="n">
-        <v>3.776</v>
+        <v>3.843</v>
       </c>
       <c r="O15" t="n">
-        <v>3.928</v>
+        <v>4.001</v>
       </c>
       <c r="P15" t="n">
-        <v>3.951</v>
+        <v>4.023</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.184</v>
+        <v>4.257</v>
       </c>
       <c r="R15" t="n">
-        <v>4.267</v>
+        <v>4.349</v>
       </c>
       <c r="S15" t="n">
-        <v>4.397</v>
+        <v>4.485</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2.731</v>
+        <v>2.735</v>
       </c>
       <c r="G16" t="n">
-        <v>2.808</v>
+        <v>2.816</v>
       </c>
       <c r="H16" t="n">
-        <v>2.905</v>
+        <v>2.932</v>
       </c>
       <c r="I16" t="n">
-        <v>3.096</v>
+        <v>3.127</v>
       </c>
       <c r="J16" t="n">
-        <v>3.409</v>
+        <v>3.444</v>
       </c>
       <c r="K16" t="n">
-        <v>3.578</v>
+        <v>3.635</v>
       </c>
       <c r="L16" t="n">
-        <v>3.625</v>
+        <v>3.699</v>
       </c>
       <c r="M16" t="n">
-        <v>3.741</v>
+        <v>3.807</v>
       </c>
       <c r="N16" t="n">
-        <v>3.78</v>
+        <v>3.846</v>
       </c>
       <c r="O16" t="n">
-        <v>3.934</v>
+        <v>4.007</v>
       </c>
       <c r="P16" t="n">
-        <v>3.975</v>
+        <v>4.046</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.211</v>
+        <v>4.284</v>
       </c>
       <c r="R16" t="n">
-        <v>4.295</v>
+        <v>4.377</v>
       </c>
       <c r="S16" t="n">
-        <v>4.426</v>
+        <v>4.514</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2.695</v>
+        <v>2.697</v>
       </c>
       <c r="G17" t="n">
-        <v>2.823</v>
+        <v>2.825</v>
       </c>
       <c r="H17" t="n">
-        <v>2.913</v>
+        <v>2.918</v>
       </c>
       <c r="I17" t="n">
-        <v>3.083</v>
+        <v>3.114</v>
       </c>
       <c r="J17" t="n">
-        <v>3.325</v>
+        <v>3.365</v>
       </c>
       <c r="K17" t="n">
-        <v>3.514</v>
+        <v>3.594</v>
       </c>
       <c r="L17" t="n">
-        <v>3.579</v>
+        <v>3.66</v>
       </c>
       <c r="M17" t="n">
-        <v>3.741</v>
+        <v>3.809</v>
       </c>
       <c r="N17" t="n">
-        <v>3.802</v>
+        <v>3.869</v>
       </c>
       <c r="O17" t="n">
-        <v>3.954</v>
+        <v>4.019</v>
       </c>
       <c r="P17" t="n">
-        <v>4.002</v>
+        <v>4.074</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2.696</v>
+        <v>2.698</v>
       </c>
       <c r="G18" t="n">
-        <v>2.824</v>
+        <v>2.826</v>
       </c>
       <c r="H18" t="n">
-        <v>2.913</v>
+        <v>2.919</v>
       </c>
       <c r="I18" t="n">
-        <v>3.084</v>
+        <v>3.114</v>
       </c>
       <c r="J18" t="n">
-        <v>3.325</v>
+        <v>3.365</v>
       </c>
       <c r="K18" t="n">
-        <v>3.515</v>
+        <v>3.595</v>
       </c>
       <c r="L18" t="n">
-        <v>3.579</v>
+        <v>3.66</v>
       </c>
       <c r="M18" t="n">
-        <v>3.741</v>
+        <v>3.809</v>
       </c>
       <c r="N18" t="n">
-        <v>3.802</v>
+        <v>3.87</v>
       </c>
       <c r="O18" t="n">
-        <v>3.953</v>
+        <v>4.018</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2.745</v>
+        <v>2.748</v>
       </c>
       <c r="G19" t="n">
-        <v>2.825</v>
+        <v>2.834</v>
       </c>
       <c r="H19" t="n">
-        <v>2.924</v>
+        <v>2.951</v>
       </c>
       <c r="I19" t="n">
-        <v>3.132</v>
+        <v>3.163</v>
       </c>
       <c r="J19" t="n">
-        <v>3.453</v>
+        <v>3.489</v>
       </c>
       <c r="K19" t="n">
-        <v>3.622</v>
+        <v>3.678</v>
       </c>
       <c r="L19" t="n">
-        <v>3.687</v>
+        <v>3.761</v>
       </c>
       <c r="M19" t="n">
-        <v>3.819</v>
+        <v>3.884</v>
       </c>
       <c r="N19" t="n">
-        <v>3.862</v>
+        <v>3.928</v>
       </c>
       <c r="O19" t="n">
-        <v>3.97</v>
+        <v>4.043</v>
       </c>
       <c r="P19" t="n">
-        <v>4.01</v>
+        <v>4.082</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.225</v>
+        <v>4.297</v>
       </c>
       <c r="R19" t="n">
-        <v>4.317</v>
+        <v>4.398</v>
       </c>
       <c r="S19" t="n">
-        <v>4.439</v>
+        <v>4.526</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2.572</v>
+        <v>2.577</v>
       </c>
       <c r="G20" t="n">
-        <v>2.643</v>
+        <v>2.652</v>
       </c>
       <c r="H20" t="n">
-        <v>2.694</v>
+        <v>2.708</v>
       </c>
       <c r="I20" t="n">
-        <v>2.836</v>
+        <v>2.857</v>
       </c>
       <c r="J20" t="n">
-        <v>3.234</v>
+        <v>3.27</v>
       </c>
       <c r="K20" t="n">
-        <v>3.425</v>
+        <v>3.49</v>
       </c>
       <c r="L20" t="n">
-        <v>3.46</v>
+        <v>3.535</v>
       </c>
       <c r="M20" t="n">
-        <v>3.555</v>
+        <v>3.632</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>2.858</v>
+        <v>2.861</v>
       </c>
       <c r="G21" t="n">
-        <v>2.935</v>
+        <v>2.94</v>
       </c>
       <c r="H21" t="n">
-        <v>3.074</v>
+        <v>3.093</v>
       </c>
       <c r="I21" t="n">
-        <v>3.251</v>
+        <v>3.279</v>
       </c>
       <c r="J21" t="n">
-        <v>3.59</v>
+        <v>3.626</v>
       </c>
       <c r="K21" t="n">
-        <v>3.857</v>
+        <v>3.913</v>
       </c>
       <c r="L21" t="n">
-        <v>3.932</v>
+        <v>4.003</v>
       </c>
       <c r="M21" t="n">
-        <v>4.056</v>
+        <v>4.119</v>
       </c>
       <c r="N21" t="n">
-        <v>4.115</v>
+        <v>4.181</v>
       </c>
       <c r="O21" t="n">
-        <v>4.187</v>
+        <v>4.26</v>
       </c>
       <c r="P21" t="n">
-        <v>4.278</v>
+        <v>4.349</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.388</v>
+        <v>4.46</v>
       </c>
       <c r="R21" t="n">
-        <v>4.37</v>
+        <v>4.453</v>
       </c>
       <c r="S21" t="n">
-        <v>4.402</v>
+        <v>4.49</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2.805</v>
+        <v>2.808</v>
       </c>
       <c r="G22" t="n">
-        <v>2.882</v>
+        <v>2.886</v>
       </c>
       <c r="H22" t="n">
-        <v>3.006</v>
+        <v>3.025</v>
       </c>
       <c r="I22" t="n">
-        <v>3.169</v>
+        <v>3.197</v>
       </c>
       <c r="J22" t="n">
-        <v>3.473</v>
+        <v>3.51</v>
       </c>
       <c r="K22" t="n">
-        <v>3.737</v>
+        <v>3.793</v>
       </c>
       <c r="L22" t="n">
-        <v>3.8</v>
+        <v>3.871</v>
       </c>
       <c r="M22" t="n">
-        <v>3.925</v>
+        <v>3.988</v>
       </c>
       <c r="N22" t="n">
-        <v>3.988</v>
+        <v>4.054</v>
       </c>
       <c r="O22" t="n">
-        <v>4.055</v>
+        <v>4.129</v>
       </c>
       <c r="P22" t="n">
-        <v>4.14</v>
+        <v>4.211</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.246</v>
+        <v>4.319</v>
       </c>
       <c r="R22" t="n">
-        <v>4.219</v>
+        <v>4.301</v>
       </c>
       <c r="S22" t="n">
-        <v>4.247</v>
+        <v>4.335</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2.758</v>
+        <v>2.761</v>
       </c>
       <c r="G23" t="n">
-        <v>2.836</v>
+        <v>2.841</v>
       </c>
       <c r="H23" t="n">
-        <v>2.945</v>
+        <v>2.964</v>
       </c>
       <c r="I23" t="n">
-        <v>3.125</v>
+        <v>3.153</v>
       </c>
       <c r="J23" t="n">
-        <v>3.418</v>
+        <v>3.455</v>
       </c>
       <c r="K23" t="n">
-        <v>3.646</v>
+        <v>3.7</v>
       </c>
       <c r="L23" t="n">
-        <v>3.708</v>
+        <v>3.777</v>
       </c>
       <c r="M23" t="n">
-        <v>3.825</v>
+        <v>3.887</v>
       </c>
       <c r="N23" t="n">
-        <v>3.883</v>
+        <v>3.949</v>
       </c>
       <c r="O23" t="n">
-        <v>3.931</v>
+        <v>4.007</v>
       </c>
       <c r="P23" t="n">
-        <v>4.002</v>
+        <v>4.075</v>
       </c>
       <c r="Q23" t="n">
-        <v>4.052</v>
+        <v>4.124</v>
       </c>
       <c r="R23" t="n">
-        <v>4.002</v>
+        <v>4.084</v>
       </c>
       <c r="S23" t="n">
-        <v>4.002</v>
+        <v>4.09</v>
       </c>
       <c r="T23" t="n">
-        <v>3.905</v>
+        <v>4</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2.693</v>
+        <v>2.696</v>
       </c>
       <c r="G24" t="n">
-        <v>2.75</v>
+        <v>2.756</v>
       </c>
       <c r="H24" t="n">
-        <v>2.846</v>
+        <v>2.866</v>
       </c>
       <c r="I24" t="n">
-        <v>3.035</v>
+        <v>3.064</v>
       </c>
       <c r="J24" t="n">
-        <v>3.317</v>
+        <v>3.354</v>
       </c>
       <c r="K24" t="n">
-        <v>3.53</v>
+        <v>3.586</v>
       </c>
       <c r="L24" t="n">
-        <v>3.582</v>
+        <v>3.653</v>
       </c>
       <c r="M24" t="n">
-        <v>3.686</v>
+        <v>3.749</v>
       </c>
       <c r="N24" t="n">
-        <v>3.761</v>
+        <v>3.826</v>
       </c>
       <c r="O24" t="n">
-        <v>3.926</v>
+        <v>4</v>
       </c>
       <c r="P24" t="n">
-        <v>3.943</v>
+        <v>4.015</v>
       </c>
       <c r="Q24" t="n">
-        <v>3.977</v>
+        <v>4.05</v>
       </c>
       <c r="R24" t="n">
-        <v>3.923</v>
+        <v>4.005</v>
       </c>
       <c r="S24" t="n">
-        <v>3.917</v>
+        <v>4.005</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2.751</v>
+        <v>2.754</v>
       </c>
       <c r="G25" t="n">
-        <v>2.835</v>
+        <v>2.84</v>
       </c>
       <c r="H25" t="n">
-        <v>2.948</v>
+        <v>2.967</v>
       </c>
       <c r="I25" t="n">
-        <v>3.133</v>
+        <v>3.161</v>
       </c>
       <c r="J25" t="n">
-        <v>3.434</v>
+        <v>3.471</v>
       </c>
       <c r="K25" t="n">
-        <v>3.679</v>
+        <v>3.733</v>
       </c>
       <c r="L25" t="n">
-        <v>3.737</v>
+        <v>3.806</v>
       </c>
       <c r="M25" t="n">
-        <v>3.855</v>
+        <v>3.917</v>
       </c>
       <c r="N25" t="n">
-        <v>3.91</v>
+        <v>3.976</v>
       </c>
       <c r="O25" t="n">
-        <v>3.96</v>
+        <v>4.036</v>
       </c>
       <c r="P25" t="n">
-        <v>4.023</v>
+        <v>4.097</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.086</v>
+        <v>4.158</v>
       </c>
       <c r="R25" t="n">
-        <v>4.025</v>
+        <v>4.108</v>
       </c>
       <c r="S25" t="n">
-        <v>4.025</v>
+        <v>4.113</v>
       </c>
       <c r="T25" t="n">
-        <v>3.923</v>
+        <v>4.018</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.045</v>
+        <v>3.046</v>
       </c>
       <c r="G26" t="n">
-        <v>3.182</v>
+        <v>3.188</v>
       </c>
       <c r="H26" t="n">
-        <v>3.413</v>
+        <v>3.431</v>
       </c>
       <c r="I26" t="n">
-        <v>3.652</v>
+        <v>3.673</v>
       </c>
       <c r="J26" t="n">
-        <v>4.093</v>
+        <v>4.128</v>
       </c>
       <c r="K26" t="n">
-        <v>4.494</v>
+        <v>4.557</v>
       </c>
       <c r="L26" t="n">
-        <v>4.612</v>
+        <v>4.69</v>
       </c>
       <c r="M26" t="n">
-        <v>4.794</v>
+        <v>4.861</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.039</v>
+        <v>5.113</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2.843</v>
+        <v>2.848</v>
       </c>
       <c r="G27" t="n">
-        <v>2.916</v>
+        <v>2.924</v>
       </c>
       <c r="H27" t="n">
-        <v>3.043</v>
+        <v>3.065</v>
       </c>
       <c r="I27" t="n">
-        <v>3.252</v>
+        <v>3.281</v>
       </c>
       <c r="J27" t="n">
-        <v>3.591</v>
+        <v>3.626</v>
       </c>
       <c r="K27" t="n">
-        <v>3.806</v>
+        <v>3.865</v>
       </c>
       <c r="L27" t="n">
-        <v>3.873</v>
+        <v>3.95</v>
       </c>
       <c r="M27" t="n">
-        <v>3.999</v>
+        <v>4.065</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.13</v>
+        <v>4.203</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2.946</v>
+        <v>2.95</v>
       </c>
       <c r="G28" t="n">
-        <v>3.027</v>
+        <v>3.035</v>
       </c>
       <c r="H28" t="n">
-        <v>3.168</v>
+        <v>3.191</v>
       </c>
       <c r="I28" t="n">
-        <v>3.39</v>
+        <v>3.418</v>
       </c>
       <c r="J28" t="n">
-        <v>3.764</v>
+        <v>3.799</v>
       </c>
       <c r="K28" t="n">
-        <v>3.998</v>
+        <v>4.057</v>
       </c>
       <c r="L28" t="n">
-        <v>4.076</v>
+        <v>4.153</v>
       </c>
       <c r="M28" t="n">
-        <v>4.211</v>
+        <v>4.278</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.423</v>
+        <v>4.496</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2.799</v>
+        <v>2.803</v>
       </c>
       <c r="G29" t="n">
-        <v>2.871</v>
+        <v>2.879</v>
       </c>
       <c r="H29" t="n">
-        <v>2.984</v>
+        <v>3.006</v>
       </c>
       <c r="I29" t="n">
-        <v>3.185</v>
+        <v>3.213</v>
       </c>
       <c r="J29" t="n">
-        <v>3.504</v>
+        <v>3.539</v>
       </c>
       <c r="K29" t="n">
-        <v>3.702</v>
+        <v>3.761</v>
       </c>
       <c r="L29" t="n">
-        <v>3.759</v>
+        <v>3.835</v>
       </c>
       <c r="M29" t="n">
-        <v>3.862</v>
+        <v>3.929</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>3.999</v>
+        <v>4.072</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.081</v>
+        <v>3.084</v>
       </c>
       <c r="G30" t="n">
-        <v>3.155</v>
+        <v>3.162</v>
       </c>
       <c r="H30" t="n">
-        <v>3.345</v>
+        <v>3.361</v>
       </c>
       <c r="I30" t="n">
-        <v>3.581</v>
+        <v>3.603</v>
       </c>
       <c r="J30" t="n">
-        <v>3.962</v>
+        <v>3.996</v>
       </c>
       <c r="K30" t="n">
-        <v>4.289</v>
+        <v>4.352</v>
       </c>
       <c r="L30" t="n">
-        <v>4.381</v>
+        <v>4.461</v>
       </c>
       <c r="M30" t="n">
-        <v>4.557</v>
+        <v>4.623</v>
       </c>
       <c r="N30" t="n">
-        <v>4.722</v>
+        <v>4.79</v>
       </c>
       <c r="O30" t="n">
-        <v>4.989</v>
+        <v>5.062</v>
       </c>
       <c r="P30" t="n">
-        <v>5.165</v>
+        <v>5.236</v>
       </c>
       <c r="Q30" t="n">
-        <v>5.916</v>
+        <v>5.989</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.408</v>
+        <v>3.411</v>
       </c>
       <c r="G31" t="n">
-        <v>3.516</v>
+        <v>3.524</v>
       </c>
       <c r="H31" t="n">
-        <v>3.76</v>
+        <v>3.776</v>
       </c>
       <c r="I31" t="n">
-        <v>4.009</v>
+        <v>4.031</v>
       </c>
       <c r="J31" t="n">
-        <v>4.452</v>
+        <v>4.486</v>
       </c>
       <c r="K31" t="n">
-        <v>4.821</v>
+        <v>4.884</v>
       </c>
       <c r="L31" t="n">
-        <v>4.993</v>
+        <v>5.073</v>
       </c>
       <c r="M31" t="n">
-        <v>5.286</v>
+        <v>5.353</v>
       </c>
       <c r="N31" t="n">
-        <v>5.579</v>
+        <v>5.647</v>
       </c>
       <c r="O31" t="n">
-        <v>6.023</v>
+        <v>6.096</v>
       </c>
       <c r="P31" t="n">
-        <v>6.152</v>
+        <v>6.223</v>
       </c>
       <c r="Q31" t="n">
-        <v>6.89</v>
+        <v>6.962</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.18</v>
+        <v>3.183</v>
       </c>
       <c r="G32" t="n">
-        <v>3.272</v>
+        <v>3.279</v>
       </c>
       <c r="H32" t="n">
-        <v>3.489</v>
+        <v>3.505</v>
       </c>
       <c r="I32" t="n">
-        <v>3.739</v>
+        <v>3.761</v>
       </c>
       <c r="J32" t="n">
-        <v>4.141</v>
+        <v>4.175</v>
       </c>
       <c r="K32" t="n">
-        <v>4.474</v>
+        <v>4.537</v>
       </c>
       <c r="L32" t="n">
-        <v>4.585</v>
+        <v>4.665</v>
       </c>
       <c r="M32" t="n">
-        <v>4.829</v>
+        <v>4.896</v>
       </c>
       <c r="N32" t="n">
-        <v>5.083</v>
+        <v>5.151</v>
       </c>
       <c r="O32" t="n">
-        <v>5.434</v>
+        <v>5.508</v>
       </c>
       <c r="P32" t="n">
-        <v>5.624</v>
+        <v>5.695</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.377</v>
+        <v>6.45</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2.951</v>
+        <v>2.954</v>
       </c>
       <c r="G33" t="n">
-        <v>3.022</v>
+        <v>3.028</v>
       </c>
       <c r="H33" t="n">
-        <v>3.163</v>
+        <v>3.179</v>
       </c>
       <c r="I33" t="n">
-        <v>3.361</v>
+        <v>3.382</v>
       </c>
       <c r="J33" t="n">
-        <v>3.669</v>
+        <v>3.705</v>
       </c>
       <c r="K33" t="n">
-        <v>3.93</v>
+        <v>3.995</v>
       </c>
       <c r="L33" t="n">
-        <v>3.988</v>
+        <v>4.068</v>
       </c>
       <c r="M33" t="n">
-        <v>4.09</v>
+        <v>4.159</v>
       </c>
       <c r="N33" t="n">
-        <v>4.115</v>
+        <v>4.184</v>
       </c>
       <c r="O33" t="n">
-        <v>4.147</v>
+        <v>4.221</v>
       </c>
       <c r="P33" t="n">
-        <v>4.197</v>
+        <v>4.268</v>
       </c>
       <c r="Q33" t="n">
-        <v>4.633</v>
+        <v>4.706</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.01</v>
+        <v>3.013</v>
       </c>
       <c r="G34" t="n">
-        <v>3.076</v>
+        <v>3.082</v>
       </c>
       <c r="H34" t="n">
-        <v>3.225</v>
+        <v>3.241</v>
       </c>
       <c r="I34" t="n">
-        <v>3.429</v>
+        <v>3.45</v>
       </c>
       <c r="J34" t="n">
-        <v>3.741</v>
+        <v>3.776</v>
       </c>
       <c r="K34" t="n">
-        <v>4.006</v>
+        <v>4.072</v>
       </c>
       <c r="L34" t="n">
-        <v>4.067</v>
+        <v>4.148</v>
       </c>
       <c r="M34" t="n">
-        <v>4.181</v>
+        <v>4.249</v>
       </c>
       <c r="N34" t="n">
-        <v>4.22</v>
+        <v>4.289</v>
       </c>
       <c r="O34" t="n">
-        <v>4.316</v>
+        <v>4.389</v>
       </c>
       <c r="P34" t="n">
-        <v>4.491</v>
+        <v>4.563</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.334</v>
+        <v>5.407</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>2.985</v>
+        <v>2.988</v>
       </c>
       <c r="G35" t="n">
-        <v>3.049</v>
+        <v>3.055</v>
       </c>
       <c r="H35" t="n">
-        <v>3.193</v>
+        <v>3.209</v>
       </c>
       <c r="I35" t="n">
-        <v>3.396</v>
+        <v>3.417</v>
       </c>
       <c r="J35" t="n">
-        <v>3.709</v>
+        <v>3.745</v>
       </c>
       <c r="K35" t="n">
-        <v>3.961</v>
+        <v>4.026</v>
       </c>
       <c r="L35" t="n">
-        <v>4.022</v>
+        <v>4.102</v>
       </c>
       <c r="M35" t="n">
-        <v>4.128</v>
+        <v>4.196</v>
       </c>
       <c r="N35" t="n">
-        <v>4.156</v>
+        <v>4.225</v>
       </c>
       <c r="O35" t="n">
-        <v>4.214</v>
+        <v>4.287</v>
       </c>
       <c r="P35" t="n">
-        <v>4.294</v>
+        <v>4.365</v>
       </c>
       <c r="Q35" t="n">
-        <v>4.97</v>
+        <v>5.043</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>2.893</v>
+        <v>2.895</v>
       </c>
       <c r="G36" t="n">
-        <v>2.959</v>
+        <v>2.964</v>
       </c>
       <c r="H36" t="n">
-        <v>3.084</v>
+        <v>3.1</v>
       </c>
       <c r="I36" t="n">
-        <v>3.288</v>
+        <v>3.31</v>
       </c>
       <c r="J36" t="n">
-        <v>3.605</v>
+        <v>3.639</v>
       </c>
       <c r="K36" t="n">
-        <v>3.853</v>
+        <v>3.917</v>
       </c>
       <c r="L36" t="n">
-        <v>3.913</v>
+        <v>3.992</v>
       </c>
       <c r="M36" t="n">
-        <v>3.99</v>
+        <v>4.059</v>
       </c>
       <c r="N36" t="n">
-        <v>4.018</v>
+        <v>4.086</v>
       </c>
       <c r="O36" t="n">
-        <v>4.057</v>
+        <v>4.13</v>
       </c>
       <c r="P36" t="n">
-        <v>4.096</v>
+        <v>4.168</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.35</v>
+        <v>4.423</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3.751</v>
+        <v>3.754</v>
       </c>
       <c r="G37" t="n">
-        <v>4.21</v>
+        <v>4.217</v>
       </c>
       <c r="H37" t="n">
-        <v>4.736</v>
+        <v>4.752</v>
       </c>
       <c r="I37" t="n">
-        <v>5.074</v>
+        <v>5.095</v>
       </c>
       <c r="J37" t="n">
-        <v>5.943</v>
+        <v>5.978</v>
       </c>
       <c r="K37" t="n">
-        <v>6.861</v>
+        <v>6.925</v>
       </c>
       <c r="L37" t="n">
-        <v>7.193</v>
+        <v>7.273</v>
       </c>
       <c r="M37" t="n">
-        <v>7.559</v>
+        <v>7.625</v>
       </c>
       <c r="N37" t="n">
-        <v>7.729</v>
+        <v>7.797</v>
       </c>
       <c r="O37" t="n">
-        <v>7.902</v>
+        <v>7.976</v>
       </c>
       <c r="P37" t="n">
-        <v>7.952</v>
+        <v>8.023</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.378</v>
+        <v>8.451000000000001</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4.81</v>
+        <v>4.813</v>
       </c>
       <c r="G38" t="n">
-        <v>5.522</v>
+        <v>5.53</v>
       </c>
       <c r="H38" t="n">
-        <v>6.26</v>
+        <v>6.276</v>
       </c>
       <c r="I38" t="n">
-        <v>6.755</v>
+        <v>6.776</v>
       </c>
       <c r="J38" t="n">
-        <v>7.885</v>
+        <v>7.92</v>
       </c>
       <c r="K38" t="n">
-        <v>8.978999999999999</v>
+        <v>9.042999999999999</v>
       </c>
       <c r="L38" t="n">
-        <v>9.471</v>
+        <v>9.551</v>
       </c>
       <c r="M38" t="n">
-        <v>9.968999999999999</v>
+        <v>10.035</v>
       </c>
       <c r="N38" t="n">
-        <v>10.147</v>
+        <v>10.215</v>
       </c>
       <c r="O38" t="n">
-        <v>10.301</v>
+        <v>10.375</v>
       </c>
       <c r="P38" t="n">
-        <v>10.349</v>
+        <v>10.421</v>
       </c>
       <c r="Q38" t="n">
-        <v>10.828</v>
+        <v>10.902</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.131</v>
+        <v>4.134</v>
       </c>
       <c r="G39" t="n">
-        <v>4.72</v>
+        <v>4.728</v>
       </c>
       <c r="H39" t="n">
-        <v>5.325</v>
+        <v>5.341</v>
       </c>
       <c r="I39" t="n">
-        <v>5.758</v>
+        <v>5.78</v>
       </c>
       <c r="J39" t="n">
-        <v>6.757</v>
+        <v>6.792</v>
       </c>
       <c r="K39" t="n">
-        <v>7.812</v>
+        <v>7.876</v>
       </c>
       <c r="L39" t="n">
-        <v>8.228999999999999</v>
+        <v>8.308999999999999</v>
       </c>
       <c r="M39" t="n">
-        <v>8.605</v>
+        <v>8.672000000000001</v>
       </c>
       <c r="N39" t="n">
-        <v>8.775</v>
+        <v>8.843</v>
       </c>
       <c r="O39" t="n">
-        <v>8.952</v>
+        <v>9.025</v>
       </c>
       <c r="P39" t="n">
-        <v>9.004</v>
+        <v>9.074999999999999</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.474</v>
+        <v>9.547000000000001</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.274</v>
+        <v>3.276</v>
       </c>
       <c r="G40" t="n">
-        <v>3.393</v>
+        <v>3.401</v>
       </c>
       <c r="H40" t="n">
-        <v>3.605</v>
+        <v>3.621</v>
       </c>
       <c r="I40" t="n">
-        <v>3.855</v>
+        <v>3.877</v>
       </c>
       <c r="J40" t="n">
-        <v>4.255</v>
+        <v>4.288</v>
       </c>
       <c r="K40" t="n">
-        <v>4.593</v>
+        <v>4.656</v>
       </c>
       <c r="L40" t="n">
-        <v>4.705</v>
+        <v>4.785</v>
       </c>
       <c r="M40" t="n">
-        <v>4.898</v>
+        <v>4.964</v>
       </c>
       <c r="N40" t="n">
-        <v>5.08</v>
+        <v>5.148</v>
       </c>
       <c r="O40" t="n">
-        <v>5.368</v>
+        <v>5.44</v>
       </c>
       <c r="P40" t="n">
-        <v>5.586</v>
+        <v>5.657</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.367</v>
+        <v>6.44</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>3.658</v>
+        <v>3.661</v>
       </c>
       <c r="G41" t="n">
-        <v>3.819</v>
+        <v>3.827</v>
       </c>
       <c r="H41" t="n">
-        <v>4.09</v>
+        <v>4.106</v>
       </c>
       <c r="I41" t="n">
-        <v>4.358</v>
+        <v>4.38</v>
       </c>
       <c r="J41" t="n">
-        <v>4.808</v>
+        <v>4.842</v>
       </c>
       <c r="K41" t="n">
-        <v>5.193</v>
+        <v>5.256</v>
       </c>
       <c r="L41" t="n">
-        <v>5.383</v>
+        <v>5.463</v>
       </c>
       <c r="M41" t="n">
-        <v>5.699</v>
+        <v>5.766</v>
       </c>
       <c r="N41" t="n">
-        <v>6.009</v>
+        <v>6.077</v>
       </c>
       <c r="O41" t="n">
-        <v>6.48</v>
+        <v>6.554</v>
       </c>
       <c r="P41" t="n">
-        <v>6.644</v>
+        <v>6.716</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.414</v>
+        <v>7.487</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.395</v>
+        <v>3.398</v>
       </c>
       <c r="G42" t="n">
-        <v>3.543</v>
+        <v>3.55</v>
       </c>
       <c r="H42" t="n">
-        <v>3.781</v>
+        <v>3.797</v>
       </c>
       <c r="I42" t="n">
-        <v>4.044</v>
+        <v>4.066</v>
       </c>
       <c r="J42" t="n">
-        <v>4.458</v>
+        <v>4.492</v>
       </c>
       <c r="K42" t="n">
-        <v>4.814</v>
+        <v>4.877</v>
       </c>
       <c r="L42" t="n">
-        <v>4.941</v>
+        <v>5.021</v>
       </c>
       <c r="M42" t="n">
-        <v>5.205</v>
+        <v>5.271</v>
       </c>
       <c r="N42" t="n">
-        <v>5.494</v>
+        <v>5.562</v>
       </c>
       <c r="O42" t="n">
-        <v>5.858</v>
+        <v>5.932</v>
       </c>
       <c r="P42" t="n">
-        <v>6.087</v>
+        <v>6.158</v>
       </c>
       <c r="Q42" t="n">
-        <v>6.88</v>
+        <v>6.953</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.099</v>
+        <v>3.102</v>
       </c>
       <c r="G43" t="n">
-        <v>3.205</v>
+        <v>3.211</v>
       </c>
       <c r="H43" t="n">
-        <v>3.364</v>
+        <v>3.381</v>
       </c>
       <c r="I43" t="n">
-        <v>3.571</v>
+        <v>3.592</v>
       </c>
       <c r="J43" t="n">
-        <v>3.897</v>
+        <v>3.933</v>
       </c>
       <c r="K43" t="n">
-        <v>4.161</v>
+        <v>4.226</v>
       </c>
       <c r="L43" t="n">
-        <v>4.229</v>
+        <v>4.31</v>
       </c>
       <c r="M43" t="n">
-        <v>4.344</v>
+        <v>4.412</v>
       </c>
       <c r="N43" t="n">
-        <v>4.385</v>
+        <v>4.454</v>
       </c>
       <c r="O43" t="n">
-        <v>4.46</v>
+        <v>4.534</v>
       </c>
       <c r="P43" t="n">
-        <v>4.563</v>
+        <v>4.634</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.243</v>
+        <v>5.316</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46141</v>
+        <v>46142</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>2.971</v>
+        <v>2.973</v>
       </c>
       <c r="G44" t="n">
-        <v>3.069</v>
+        <v>3.074</v>
       </c>
       <c r="H44" t="n">
-        <v>3.208</v>
+        <v>3.224</v>
       </c>
       <c r="I44" t="n">
-        <v>3.416</v>
+        <v>3.438</v>
       </c>
       <c r="J44" t="n">
-        <v>3.746</v>
+        <v>3.781</v>
       </c>
       <c r="K44" t="n">
-        <v>4.004</v>
+        <v>4.068</v>
       </c>
       <c r="L44" t="n">
-        <v>4.073</v>
+        <v>4.152</v>
       </c>
       <c r="M44" t="n">
-        <v>4.159</v>
+        <v>4.227</v>
       </c>
       <c r="N44" t="n">
-        <v>4.2</v>
+        <v>4.268</v>
       </c>
       <c r="O44" t="n">
-        <v>4.256</v>
+        <v>4.33</v>
       </c>
       <c r="P44" t="n">
-        <v>4.326</v>
+        <v>4.398</v>
       </c>
       <c r="Q44" t="n">
-        <v>4.614</v>
+        <v>4.687</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-09-07 ~ 2026-09-07
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.646</v>
+        <v>3.655</v>
       </c>
       <c r="G2" t="n">
-        <v>4.129</v>
+        <v>4.135</v>
       </c>
       <c r="H2" t="n">
-        <v>4.388</v>
+        <v>4.395</v>
       </c>
       <c r="I2" t="n">
-        <v>4.387</v>
+        <v>4.394</v>
       </c>
       <c r="J2" t="n">
-        <v>4.591</v>
+        <v>4.596</v>
       </c>
       <c r="K2" t="n">
-        <v>4.9</v>
+        <v>4.917</v>
       </c>
       <c r="L2" t="n">
-        <v>5.121</v>
+        <v>5.136</v>
       </c>
       <c r="M2" t="n">
-        <v>5.383</v>
+        <v>5.393</v>
       </c>
       <c r="N2" t="n">
-        <v>5.64</v>
+        <v>5.662</v>
       </c>
       <c r="O2" t="n">
-        <v>5.915</v>
+        <v>5.945</v>
       </c>
       <c r="P2" t="n">
-        <v>6.124</v>
+        <v>6.156</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.807</v>
+        <v>6.847</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.665</v>
+        <v>4.673</v>
       </c>
       <c r="G3" t="n">
-        <v>5.328</v>
+        <v>5.335</v>
       </c>
       <c r="H3" t="n">
-        <v>5.621</v>
+        <v>5.627</v>
       </c>
       <c r="I3" t="n">
-        <v>5.616</v>
+        <v>5.622</v>
       </c>
       <c r="J3" t="n">
-        <v>5.835</v>
+        <v>5.84</v>
       </c>
       <c r="K3" t="n">
-        <v>6.216</v>
+        <v>6.233</v>
       </c>
       <c r="L3" t="n">
-        <v>6.507</v>
+        <v>6.522</v>
       </c>
       <c r="M3" t="n">
-        <v>6.798</v>
+        <v>6.808</v>
       </c>
       <c r="N3" t="n">
-        <v>7</v>
+        <v>7.022</v>
       </c>
       <c r="O3" t="n">
-        <v>7.225</v>
+        <v>7.255</v>
       </c>
       <c r="P3" t="n">
-        <v>7.301</v>
+        <v>7.334</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.873</v>
+        <v>7.913</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>4.157</v>
+        <v>4.165</v>
       </c>
       <c r="G4" t="n">
-        <v>4.71</v>
+        <v>4.714</v>
       </c>
       <c r="H4" t="n">
-        <v>5.029</v>
+        <v>5.034</v>
       </c>
       <c r="I4" t="n">
-        <v>5.058</v>
+        <v>5.063</v>
       </c>
       <c r="J4" t="n">
-        <v>5.278</v>
+        <v>5.282</v>
       </c>
       <c r="K4" t="n">
-        <v>5.654</v>
+        <v>5.669</v>
       </c>
       <c r="L4" t="n">
-        <v>5.875</v>
+        <v>5.888</v>
       </c>
       <c r="M4" t="n">
-        <v>6.156</v>
+        <v>6.166</v>
       </c>
       <c r="N4" t="n">
-        <v>6.328</v>
+        <v>6.349</v>
       </c>
       <c r="O4" t="n">
-        <v>6.577</v>
+        <v>6.606</v>
       </c>
       <c r="P4" t="n">
-        <v>6.653</v>
+        <v>6.686</v>
       </c>
       <c r="Q4" t="n">
-        <v>7.228</v>
+        <v>7.268</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>3.339</v>
+        <v>3.35</v>
       </c>
       <c r="G5" t="n">
-        <v>3.685</v>
+        <v>3.694</v>
       </c>
       <c r="H5" t="n">
-        <v>3.918</v>
+        <v>3.926</v>
       </c>
       <c r="I5" t="n">
-        <v>3.949</v>
+        <v>3.955</v>
       </c>
       <c r="J5" t="n">
-        <v>4.165</v>
+        <v>4.17</v>
       </c>
       <c r="K5" t="n">
-        <v>4.301</v>
+        <v>4.316</v>
       </c>
       <c r="L5" t="n">
-        <v>4.365</v>
+        <v>4.38</v>
       </c>
       <c r="M5" t="n">
-        <v>4.447</v>
+        <v>4.457</v>
       </c>
       <c r="N5" t="n">
-        <v>4.46</v>
+        <v>4.482</v>
       </c>
       <c r="O5" t="n">
-        <v>4.515</v>
+        <v>4.545</v>
       </c>
       <c r="P5" t="n">
-        <v>4.791</v>
+        <v>4.824</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.713</v>
+        <v>5.753</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>3.379</v>
+        <v>3.388</v>
       </c>
       <c r="G6" t="n">
-        <v>3.739</v>
+        <v>3.747</v>
       </c>
       <c r="H6" t="n">
-        <v>3.987</v>
+        <v>3.995</v>
       </c>
       <c r="I6" t="n">
-        <v>4.029</v>
+        <v>4.035</v>
       </c>
       <c r="J6" t="n">
-        <v>4.257</v>
+        <v>4.262</v>
       </c>
       <c r="K6" t="n">
-        <v>4.418</v>
+        <v>4.433</v>
       </c>
       <c r="L6" t="n">
-        <v>4.486</v>
+        <v>4.502</v>
       </c>
       <c r="M6" t="n">
-        <v>4.599</v>
+        <v>4.609</v>
       </c>
       <c r="N6" t="n">
-        <v>4.625</v>
+        <v>4.647</v>
       </c>
       <c r="O6" t="n">
-        <v>4.782</v>
+        <v>4.812</v>
       </c>
       <c r="P6" t="n">
-        <v>5.225</v>
+        <v>5.257</v>
       </c>
       <c r="Q6" t="n">
-        <v>6.111</v>
+        <v>6.151</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>3.359</v>
+        <v>3.369</v>
       </c>
       <c r="G7" t="n">
-        <v>3.7</v>
+        <v>3.71</v>
       </c>
       <c r="H7" t="n">
-        <v>3.934</v>
+        <v>3.942</v>
       </c>
       <c r="I7" t="n">
-        <v>3.967</v>
+        <v>3.973</v>
       </c>
       <c r="J7" t="n">
-        <v>4.189</v>
+        <v>4.195</v>
       </c>
       <c r="K7" t="n">
-        <v>4.329</v>
+        <v>4.344</v>
       </c>
       <c r="L7" t="n">
-        <v>4.392</v>
+        <v>4.407</v>
       </c>
       <c r="M7" t="n">
-        <v>4.505</v>
+        <v>4.515</v>
       </c>
       <c r="N7" t="n">
-        <v>4.522</v>
+        <v>4.544</v>
       </c>
       <c r="O7" t="n">
-        <v>4.681</v>
+        <v>4.711</v>
       </c>
       <c r="P7" t="n">
-        <v>5.009</v>
+        <v>5.041</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.879</v>
+        <v>5.919</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.778</v>
+        <v>5.787</v>
       </c>
       <c r="G8" t="n">
-        <v>6.63</v>
+        <v>6.637</v>
       </c>
       <c r="H8" t="n">
-        <v>7.076</v>
+        <v>7.082</v>
       </c>
       <c r="I8" t="n">
-        <v>7.142</v>
+        <v>7.149</v>
       </c>
       <c r="J8" t="n">
-        <v>7.433</v>
+        <v>7.438</v>
       </c>
       <c r="K8" t="n">
-        <v>8.090999999999999</v>
+        <v>8.106999999999999</v>
       </c>
       <c r="L8" t="n">
-        <v>8.464</v>
+        <v>8.478999999999999</v>
       </c>
       <c r="M8" t="n">
-        <v>8.789</v>
+        <v>8.798999999999999</v>
       </c>
       <c r="N8" t="n">
-        <v>8.923999999999999</v>
+        <v>8.945</v>
       </c>
       <c r="O8" t="n">
-        <v>9.234999999999999</v>
+        <v>9.265000000000001</v>
       </c>
       <c r="P8" t="n">
-        <v>9.416</v>
+        <v>9.448</v>
       </c>
       <c r="Q8" t="n">
-        <v>10.19</v>
+        <v>10.23</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,57 +1063,57 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>3.016</v>
+        <v>3.022</v>
       </c>
       <c r="G9" t="n">
-        <v>3.138</v>
+        <v>3.145</v>
       </c>
       <c r="H9" t="n">
-        <v>3.364</v>
+        <v>3.375</v>
       </c>
       <c r="I9" t="n">
-        <v>3.475</v>
+        <v>3.485</v>
       </c>
       <c r="J9" t="n">
-        <v>3.606</v>
+        <v>3.623</v>
       </c>
       <c r="K9" t="n">
-        <v>3.705</v>
+        <v>3.722</v>
       </c>
       <c r="L9" t="n">
-        <v>3.79</v>
+        <v>3.808</v>
       </c>
       <c r="M9" t="n">
-        <v>3.884</v>
+        <v>3.897</v>
       </c>
       <c r="N9" t="n">
-        <v>3.971</v>
+        <v>3.993</v>
       </c>
       <c r="O9" t="n">
-        <v>4.094</v>
+        <v>4.125</v>
       </c>
       <c r="P9" t="n">
-        <v>4.232</v>
+        <v>4.264</v>
       </c>
       <c r="Q9" t="n">
-        <v>4.35</v>
+        <v>4.39</v>
       </c>
       <c r="R9" t="n">
-        <v>4.477</v>
+        <v>4.499</v>
       </c>
       <c r="S9" t="n">
-        <v>4.57</v>
+        <v>4.577</v>
       </c>
       <c r="T9" t="n">
-        <v>4.637</v>
+        <v>4.638</v>
       </c>
       <c r="U9" t="n">
-        <v>4.597</v>
+        <v>4.598</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>3.086</v>
+        <v>3.101</v>
       </c>
       <c r="G10" t="n">
-        <v>3.22</v>
+        <v>3.235</v>
       </c>
       <c r="H10" t="n">
-        <v>3.424</v>
+        <v>3.44</v>
       </c>
       <c r="I10" t="n">
-        <v>3.527</v>
+        <v>3.545</v>
       </c>
       <c r="J10" t="n">
-        <v>3.663</v>
+        <v>3.687</v>
       </c>
       <c r="K10" t="n">
-        <v>3.749</v>
+        <v>3.77</v>
       </c>
       <c r="L10" t="n">
-        <v>3.831</v>
+        <v>3.852</v>
       </c>
       <c r="M10" t="n">
-        <v>3.944</v>
+        <v>3.957</v>
       </c>
       <c r="N10" t="n">
-        <v>4.013</v>
+        <v>4.036</v>
       </c>
       <c r="O10" t="n">
-        <v>4.332</v>
+        <v>4.364</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.897</v>
+        <v>2.911</v>
       </c>
       <c r="G11" t="n">
-        <v>3.017</v>
+        <v>3.032</v>
       </c>
       <c r="H11" t="n">
-        <v>3.229</v>
+        <v>3.245</v>
       </c>
       <c r="I11" t="n">
-        <v>3.317</v>
+        <v>3.333</v>
       </c>
       <c r="J11" t="n">
-        <v>3.453</v>
+        <v>3.476</v>
       </c>
       <c r="K11" t="n">
-        <v>3.531</v>
+        <v>3.552</v>
       </c>
       <c r="L11" t="n">
-        <v>3.618</v>
+        <v>3.64</v>
       </c>
       <c r="M11" t="n">
-        <v>3.754</v>
+        <v>3.766</v>
       </c>
       <c r="N11" t="n">
-        <v>3.809</v>
+        <v>3.833</v>
       </c>
       <c r="O11" t="n">
-        <v>4.104</v>
+        <v>4.137</v>
       </c>
       <c r="P11" t="n">
-        <v>4.178</v>
+        <v>4.21</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.548</v>
+        <v>4.588</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.66</v>
+        <v>3.672</v>
       </c>
       <c r="G12" t="n">
-        <v>4.014</v>
+        <v>4.031</v>
       </c>
       <c r="H12" t="n">
-        <v>4.307</v>
+        <v>4.316</v>
       </c>
       <c r="I12" t="n">
-        <v>4.379</v>
+        <v>4.39</v>
       </c>
       <c r="J12" t="n">
-        <v>4.598</v>
+        <v>4.606</v>
       </c>
       <c r="K12" t="n">
-        <v>4.699</v>
+        <v>4.719</v>
       </c>
       <c r="L12" t="n">
-        <v>4.784</v>
+        <v>4.802</v>
       </c>
       <c r="M12" t="n">
-        <v>4.904</v>
+        <v>4.916</v>
       </c>
       <c r="N12" t="n">
-        <v>4.959</v>
+        <v>4.981</v>
       </c>
       <c r="O12" t="n">
-        <v>5.139</v>
+        <v>5.169</v>
       </c>
       <c r="P12" t="n">
-        <v>5.284</v>
+        <v>5.317</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.664</v>
+        <v>5.704</v>
       </c>
       <c r="R12" t="n">
-        <v>5.969</v>
+        <v>5.991</v>
       </c>
       <c r="S12" t="n">
-        <v>6.27</v>
+        <v>6.276</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>3.413</v>
+        <v>3.426</v>
       </c>
       <c r="G13" t="n">
-        <v>3.706</v>
+        <v>3.722</v>
       </c>
       <c r="H13" t="n">
-        <v>3.975</v>
+        <v>3.983</v>
       </c>
       <c r="I13" t="n">
-        <v>4.026</v>
+        <v>4.038</v>
       </c>
       <c r="J13" t="n">
-        <v>4.235</v>
+        <v>4.244</v>
       </c>
       <c r="K13" t="n">
-        <v>4.333</v>
+        <v>4.353</v>
       </c>
       <c r="L13" t="n">
-        <v>4.424</v>
+        <v>4.442</v>
       </c>
       <c r="M13" t="n">
-        <v>4.532</v>
+        <v>4.544</v>
       </c>
       <c r="N13" t="n">
-        <v>4.587</v>
+        <v>4.609</v>
       </c>
       <c r="O13" t="n">
-        <v>4.766</v>
+        <v>4.796</v>
       </c>
       <c r="P13" t="n">
-        <v>4.875</v>
+        <v>4.908</v>
       </c>
       <c r="Q13" t="n">
-        <v>5.187</v>
+        <v>5.227</v>
       </c>
       <c r="R13" t="n">
-        <v>5.52</v>
+        <v>5.541</v>
       </c>
       <c r="S13" t="n">
-        <v>5.838</v>
+        <v>5.844</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>3.23</v>
+        <v>3.243</v>
       </c>
       <c r="G14" t="n">
-        <v>3.504</v>
+        <v>3.52</v>
       </c>
       <c r="H14" t="n">
-        <v>3.773</v>
+        <v>3.782</v>
       </c>
       <c r="I14" t="n">
-        <v>3.811</v>
+        <v>3.822</v>
       </c>
       <c r="J14" t="n">
-        <v>3.978</v>
+        <v>3.986</v>
       </c>
       <c r="K14" t="n">
-        <v>4.022</v>
+        <v>4.042</v>
       </c>
       <c r="L14" t="n">
-        <v>4.096</v>
+        <v>4.115</v>
       </c>
       <c r="M14" t="n">
-        <v>4.218</v>
+        <v>4.231</v>
       </c>
       <c r="N14" t="n">
-        <v>4.267</v>
+        <v>4.288</v>
       </c>
       <c r="O14" t="n">
-        <v>4.424</v>
+        <v>4.454</v>
       </c>
       <c r="P14" t="n">
-        <v>4.515</v>
+        <v>4.547</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.776</v>
+        <v>4.816</v>
       </c>
       <c r="R14" t="n">
-        <v>5.034</v>
+        <v>5.055</v>
       </c>
       <c r="S14" t="n">
-        <v>5.29</v>
+        <v>5.297</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>3.203</v>
+        <v>3.215</v>
       </c>
       <c r="G15" t="n">
-        <v>3.475</v>
+        <v>3.49</v>
       </c>
       <c r="H15" t="n">
-        <v>3.739</v>
+        <v>3.746</v>
       </c>
       <c r="I15" t="n">
-        <v>3.747</v>
+        <v>3.757</v>
       </c>
       <c r="J15" t="n">
-        <v>3.913</v>
+        <v>3.921</v>
       </c>
       <c r="K15" t="n">
-        <v>3.969</v>
+        <v>3.989</v>
       </c>
       <c r="L15" t="n">
-        <v>4.026</v>
+        <v>4.045</v>
       </c>
       <c r="M15" t="n">
-        <v>4.127</v>
+        <v>4.139</v>
       </c>
       <c r="N15" t="n">
-        <v>4.17</v>
+        <v>4.192</v>
       </c>
       <c r="O15" t="n">
-        <v>4.372</v>
+        <v>4.402</v>
       </c>
       <c r="P15" t="n">
-        <v>4.415</v>
+        <v>4.448</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.677</v>
+        <v>4.717</v>
       </c>
       <c r="R15" t="n">
-        <v>4.928</v>
+        <v>4.949</v>
       </c>
       <c r="S15" t="n">
-        <v>5.18</v>
+        <v>5.187</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>3.203</v>
+        <v>3.215</v>
       </c>
       <c r="G16" t="n">
-        <v>3.475</v>
+        <v>3.49</v>
       </c>
       <c r="H16" t="n">
-        <v>3.739</v>
+        <v>3.746</v>
       </c>
       <c r="I16" t="n">
-        <v>3.747</v>
+        <v>3.757</v>
       </c>
       <c r="J16" t="n">
-        <v>3.913</v>
+        <v>3.921</v>
       </c>
       <c r="K16" t="n">
-        <v>3.969</v>
+        <v>3.989</v>
       </c>
       <c r="L16" t="n">
-        <v>4.026</v>
+        <v>4.045</v>
       </c>
       <c r="M16" t="n">
-        <v>4.127</v>
+        <v>4.139</v>
       </c>
       <c r="N16" t="n">
-        <v>4.173</v>
+        <v>4.195</v>
       </c>
       <c r="O16" t="n">
-        <v>4.377</v>
+        <v>4.407</v>
       </c>
       <c r="P16" t="n">
-        <v>4.439</v>
+        <v>4.471</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.704</v>
+        <v>4.744</v>
       </c>
       <c r="R16" t="n">
-        <v>4.956</v>
+        <v>4.977</v>
       </c>
       <c r="S16" t="n">
-        <v>5.211</v>
+        <v>5.218</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>3.133</v>
+        <v>3.148</v>
       </c>
       <c r="G17" t="n">
-        <v>3.283</v>
+        <v>3.298</v>
       </c>
       <c r="H17" t="n">
-        <v>3.46</v>
+        <v>3.477</v>
       </c>
       <c r="I17" t="n">
-        <v>3.574</v>
+        <v>3.591</v>
       </c>
       <c r="J17" t="n">
-        <v>3.735</v>
+        <v>3.758</v>
       </c>
       <c r="K17" t="n">
-        <v>3.845</v>
+        <v>3.864</v>
       </c>
       <c r="L17" t="n">
-        <v>3.919</v>
+        <v>3.942</v>
       </c>
       <c r="M17" t="n">
-        <v>4.082</v>
+        <v>4.094</v>
       </c>
       <c r="N17" t="n">
-        <v>4.128</v>
+        <v>4.154</v>
       </c>
       <c r="O17" t="n">
-        <v>4.358</v>
+        <v>4.389</v>
       </c>
       <c r="P17" t="n">
-        <v>4.458</v>
+        <v>4.491</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>3.133</v>
+        <v>3.148</v>
       </c>
       <c r="G18" t="n">
-        <v>3.283</v>
+        <v>3.298</v>
       </c>
       <c r="H18" t="n">
-        <v>3.46</v>
+        <v>3.477</v>
       </c>
       <c r="I18" t="n">
-        <v>3.574</v>
+        <v>3.59</v>
       </c>
       <c r="J18" t="n">
-        <v>3.735</v>
+        <v>3.758</v>
       </c>
       <c r="K18" t="n">
-        <v>3.845</v>
+        <v>3.864</v>
       </c>
       <c r="L18" t="n">
-        <v>3.919</v>
+        <v>3.942</v>
       </c>
       <c r="M18" t="n">
-        <v>4.081</v>
+        <v>4.093</v>
       </c>
       <c r="N18" t="n">
-        <v>4.128</v>
+        <v>4.154</v>
       </c>
       <c r="O18" t="n">
-        <v>4.357</v>
+        <v>4.389</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>3.22</v>
+        <v>3.232</v>
       </c>
       <c r="G19" t="n">
-        <v>3.5</v>
+        <v>3.514</v>
       </c>
       <c r="H19" t="n">
-        <v>3.763</v>
+        <v>3.77</v>
       </c>
       <c r="I19" t="n">
-        <v>3.798</v>
+        <v>3.807</v>
       </c>
       <c r="J19" t="n">
-        <v>3.976</v>
+        <v>3.985</v>
       </c>
       <c r="K19" t="n">
-        <v>4.032</v>
+        <v>4.052</v>
       </c>
       <c r="L19" t="n">
-        <v>4.103</v>
+        <v>4.122</v>
       </c>
       <c r="M19" t="n">
-        <v>4.217</v>
+        <v>4.229</v>
       </c>
       <c r="N19" t="n">
-        <v>4.258</v>
+        <v>4.281</v>
       </c>
       <c r="O19" t="n">
-        <v>4.413</v>
+        <v>4.443</v>
       </c>
       <c r="P19" t="n">
-        <v>4.474</v>
+        <v>4.506</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.715</v>
+        <v>4.755</v>
       </c>
       <c r="R19" t="n">
-        <v>4.975</v>
+        <v>4.996</v>
       </c>
       <c r="S19" t="n">
-        <v>5.224</v>
+        <v>5.231</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>3.017</v>
+        <v>3.024</v>
       </c>
       <c r="G20" t="n">
-        <v>3.045</v>
+        <v>3.051</v>
       </c>
       <c r="H20" t="n">
-        <v>3.16</v>
+        <v>3.166</v>
       </c>
       <c r="I20" t="n">
-        <v>3.284</v>
+        <v>3.29</v>
       </c>
       <c r="J20" t="n">
-        <v>3.671</v>
+        <v>3.678</v>
       </c>
       <c r="K20" t="n">
-        <v>3.764</v>
+        <v>3.785</v>
       </c>
       <c r="L20" t="n">
-        <v>3.779</v>
+        <v>3.794</v>
       </c>
       <c r="M20" t="n">
-        <v>3.879</v>
+        <v>3.893</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>3.297</v>
+        <v>3.306</v>
       </c>
       <c r="G21" t="n">
-        <v>3.598</v>
+        <v>3.607</v>
       </c>
       <c r="H21" t="n">
-        <v>3.883</v>
+        <v>3.891</v>
       </c>
       <c r="I21" t="n">
-        <v>3.934</v>
+        <v>3.944</v>
       </c>
       <c r="J21" t="n">
-        <v>4.141</v>
+        <v>4.153</v>
       </c>
       <c r="K21" t="n">
-        <v>4.25</v>
+        <v>4.27</v>
       </c>
       <c r="L21" t="n">
-        <v>4.33</v>
+        <v>4.35</v>
       </c>
       <c r="M21" t="n">
-        <v>4.445</v>
+        <v>4.457</v>
       </c>
       <c r="N21" t="n">
-        <v>4.503</v>
+        <v>4.524</v>
       </c>
       <c r="O21" t="n">
-        <v>4.643</v>
+        <v>4.672</v>
       </c>
       <c r="P21" t="n">
-        <v>4.717</v>
+        <v>4.75</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.867</v>
+        <v>4.907</v>
       </c>
       <c r="R21" t="n">
-        <v>5.026</v>
+        <v>5.047</v>
       </c>
       <c r="S21" t="n">
-        <v>5.178</v>
+        <v>5.184</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>3.241</v>
+        <v>3.25</v>
       </c>
       <c r="G22" t="n">
-        <v>3.543</v>
+        <v>3.553</v>
       </c>
       <c r="H22" t="n">
-        <v>3.815</v>
+        <v>3.823</v>
       </c>
       <c r="I22" t="n">
-        <v>3.851</v>
+        <v>3.861</v>
       </c>
       <c r="J22" t="n">
-        <v>4.029</v>
+        <v>4.04</v>
       </c>
       <c r="K22" t="n">
-        <v>4.129</v>
+        <v>4.149</v>
       </c>
       <c r="L22" t="n">
-        <v>4.203</v>
+        <v>4.223</v>
       </c>
       <c r="M22" t="n">
-        <v>4.317</v>
+        <v>4.329</v>
       </c>
       <c r="N22" t="n">
-        <v>4.379</v>
+        <v>4.4</v>
       </c>
       <c r="O22" t="n">
-        <v>4.513</v>
+        <v>4.542</v>
       </c>
       <c r="P22" t="n">
-        <v>4.581</v>
+        <v>4.614</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.725</v>
+        <v>4.765</v>
       </c>
       <c r="R22" t="n">
-        <v>4.875</v>
+        <v>4.896</v>
       </c>
       <c r="S22" t="n">
-        <v>5.023</v>
+        <v>5.03</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>3.191</v>
+        <v>3.201</v>
       </c>
       <c r="G23" t="n">
-        <v>3.494</v>
+        <v>3.504</v>
       </c>
       <c r="H23" t="n">
-        <v>3.754</v>
+        <v>3.762</v>
       </c>
       <c r="I23" t="n">
-        <v>3.787</v>
+        <v>3.797</v>
       </c>
       <c r="J23" t="n">
-        <v>3.946</v>
+        <v>3.958</v>
       </c>
       <c r="K23" t="n">
-        <v>4.021</v>
+        <v>4.04</v>
       </c>
       <c r="L23" t="n">
-        <v>4.096</v>
+        <v>4.116</v>
       </c>
       <c r="M23" t="n">
-        <v>4.207</v>
+        <v>4.219</v>
       </c>
       <c r="N23" t="n">
-        <v>4.266</v>
+        <v>4.287</v>
       </c>
       <c r="O23" t="n">
-        <v>4.388</v>
+        <v>4.417</v>
       </c>
       <c r="P23" t="n">
-        <v>4.443</v>
+        <v>4.475</v>
       </c>
       <c r="Q23" t="n">
-        <v>4.528</v>
+        <v>4.568</v>
       </c>
       <c r="R23" t="n">
-        <v>4.66</v>
+        <v>4.681</v>
       </c>
       <c r="S23" t="n">
-        <v>4.779</v>
+        <v>4.786</v>
       </c>
       <c r="T23" t="n">
-        <v>4.852</v>
+        <v>4.854</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>3.142</v>
+        <v>3.151</v>
       </c>
       <c r="G24" t="n">
-        <v>3.408</v>
+        <v>3.418</v>
       </c>
       <c r="H24" t="n">
-        <v>3.641</v>
+        <v>3.649</v>
       </c>
       <c r="I24" t="n">
-        <v>3.697</v>
+        <v>3.707</v>
       </c>
       <c r="J24" t="n">
-        <v>3.84</v>
+        <v>3.852</v>
       </c>
       <c r="K24" t="n">
-        <v>3.913</v>
+        <v>3.934</v>
       </c>
       <c r="L24" t="n">
-        <v>3.979</v>
+        <v>3.999</v>
       </c>
       <c r="M24" t="n">
-        <v>4.065</v>
+        <v>4.077</v>
       </c>
       <c r="N24" t="n">
-        <v>4.136</v>
+        <v>4.157</v>
       </c>
       <c r="O24" t="n">
-        <v>4.345</v>
+        <v>4.372</v>
       </c>
       <c r="P24" t="n">
-        <v>4.384</v>
+        <v>4.417</v>
       </c>
       <c r="Q24" t="n">
-        <v>4.457</v>
+        <v>4.497</v>
       </c>
       <c r="R24" t="n">
-        <v>4.582</v>
+        <v>4.604</v>
       </c>
       <c r="S24" t="n">
-        <v>4.694</v>
+        <v>4.701</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>3.185</v>
+        <v>3.194</v>
       </c>
       <c r="G25" t="n">
-        <v>3.495</v>
+        <v>3.505</v>
       </c>
       <c r="H25" t="n">
-        <v>3.758</v>
+        <v>3.765</v>
       </c>
       <c r="I25" t="n">
-        <v>3.798</v>
+        <v>3.808</v>
       </c>
       <c r="J25" t="n">
-        <v>3.968</v>
+        <v>3.98</v>
       </c>
       <c r="K25" t="n">
-        <v>4.058</v>
+        <v>4.078</v>
       </c>
       <c r="L25" t="n">
-        <v>4.128</v>
+        <v>4.148</v>
       </c>
       <c r="M25" t="n">
-        <v>4.239</v>
+        <v>4.251</v>
       </c>
       <c r="N25" t="n">
-        <v>4.293</v>
+        <v>4.314</v>
       </c>
       <c r="O25" t="n">
-        <v>4.418</v>
+        <v>4.447</v>
       </c>
       <c r="P25" t="n">
-        <v>4.465</v>
+        <v>4.498</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.56</v>
+        <v>4.6</v>
       </c>
       <c r="R25" t="n">
-        <v>4.684</v>
+        <v>4.705</v>
       </c>
       <c r="S25" t="n">
-        <v>4.803</v>
+        <v>4.809</v>
       </c>
       <c r="T25" t="n">
-        <v>4.869</v>
+        <v>4.871</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.441</v>
+        <v>3.45</v>
       </c>
       <c r="G26" t="n">
-        <v>3.912</v>
+        <v>3.923</v>
       </c>
       <c r="H26" t="n">
-        <v>4.204</v>
+        <v>4.211</v>
       </c>
       <c r="I26" t="n">
-        <v>4.247</v>
+        <v>4.253</v>
       </c>
       <c r="J26" t="n">
-        <v>4.592</v>
+        <v>4.598</v>
       </c>
       <c r="K26" t="n">
-        <v>4.89</v>
+        <v>4.907</v>
       </c>
       <c r="L26" t="n">
-        <v>5.007</v>
+        <v>5.024</v>
       </c>
       <c r="M26" t="n">
-        <v>5.172</v>
+        <v>5.183</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.457</v>
+        <v>5.487</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>3.285</v>
+        <v>3.297</v>
       </c>
       <c r="G27" t="n">
-        <v>3.614</v>
+        <v>3.627</v>
       </c>
       <c r="H27" t="n">
-        <v>3.861</v>
+        <v>3.868</v>
       </c>
       <c r="I27" t="n">
-        <v>3.9</v>
+        <v>3.908</v>
       </c>
       <c r="J27" t="n">
-        <v>4.096</v>
+        <v>4.103</v>
       </c>
       <c r="K27" t="n">
-        <v>4.202</v>
+        <v>4.221</v>
       </c>
       <c r="L27" t="n">
-        <v>4.276</v>
+        <v>4.294</v>
       </c>
       <c r="M27" t="n">
-        <v>4.384</v>
+        <v>4.396</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.556</v>
+        <v>4.586</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>3.393</v>
+        <v>3.406</v>
       </c>
       <c r="G28" t="n">
-        <v>3.736</v>
+        <v>3.749</v>
       </c>
       <c r="H28" t="n">
-        <v>3.995</v>
+        <v>4.002</v>
       </c>
       <c r="I28" t="n">
-        <v>4.039</v>
+        <v>4.047</v>
       </c>
       <c r="J28" t="n">
-        <v>4.269</v>
+        <v>4.276</v>
       </c>
       <c r="K28" t="n">
-        <v>4.394</v>
+        <v>4.413</v>
       </c>
       <c r="L28" t="n">
-        <v>4.479</v>
+        <v>4.498</v>
       </c>
       <c r="M28" t="n">
-        <v>4.596</v>
+        <v>4.608</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.848</v>
+        <v>4.878</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>3.232</v>
+        <v>3.243</v>
       </c>
       <c r="G29" t="n">
-        <v>3.555</v>
+        <v>3.568</v>
       </c>
       <c r="H29" t="n">
-        <v>3.794</v>
+        <v>3.8</v>
       </c>
       <c r="I29" t="n">
-        <v>3.816</v>
+        <v>3.824</v>
       </c>
       <c r="J29" t="n">
-        <v>4.004</v>
+        <v>4.012</v>
       </c>
       <c r="K29" t="n">
-        <v>4.096</v>
+        <v>4.115</v>
       </c>
       <c r="L29" t="n">
-        <v>4.157</v>
+        <v>4.175</v>
       </c>
       <c r="M29" t="n">
-        <v>4.246</v>
+        <v>4.258</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>4.429</v>
+        <v>4.459</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.487</v>
+        <v>3.495</v>
       </c>
       <c r="G30" t="n">
-        <v>3.917</v>
+        <v>3.926</v>
       </c>
       <c r="H30" t="n">
-        <v>4.148</v>
+        <v>4.156</v>
       </c>
       <c r="I30" t="n">
-        <v>4.187</v>
+        <v>4.194</v>
       </c>
       <c r="J30" t="n">
-        <v>4.468</v>
+        <v>4.475</v>
       </c>
       <c r="K30" t="n">
-        <v>4.692</v>
+        <v>4.709</v>
       </c>
       <c r="L30" t="n">
-        <v>4.788</v>
+        <v>4.805</v>
       </c>
       <c r="M30" t="n">
-        <v>4.942</v>
+        <v>4.954</v>
       </c>
       <c r="N30" t="n">
-        <v>5.092</v>
+        <v>5.114</v>
       </c>
       <c r="O30" t="n">
-        <v>5.398</v>
+        <v>5.428</v>
       </c>
       <c r="P30" t="n">
-        <v>5.619</v>
+        <v>5.651</v>
       </c>
       <c r="Q30" t="n">
-        <v>6.41</v>
+        <v>6.45</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.816</v>
+        <v>3.824</v>
       </c>
       <c r="G31" t="n">
-        <v>4.281</v>
+        <v>4.29</v>
       </c>
       <c r="H31" t="n">
-        <v>4.563</v>
+        <v>4.57</v>
       </c>
       <c r="I31" t="n">
-        <v>4.615</v>
+        <v>4.622</v>
       </c>
       <c r="J31" t="n">
-        <v>4.961</v>
+        <v>4.968</v>
       </c>
       <c r="K31" t="n">
-        <v>5.233</v>
+        <v>5.25</v>
       </c>
       <c r="L31" t="n">
-        <v>5.4</v>
+        <v>5.417</v>
       </c>
       <c r="M31" t="n">
-        <v>5.67</v>
+        <v>5.682</v>
       </c>
       <c r="N31" t="n">
-        <v>5.951</v>
+        <v>5.973</v>
       </c>
       <c r="O31" t="n">
-        <v>6.434</v>
+        <v>6.464</v>
       </c>
       <c r="P31" t="n">
-        <v>6.607</v>
+        <v>6.64</v>
       </c>
       <c r="Q31" t="n">
-        <v>7.383</v>
+        <v>7.423</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.585</v>
+        <v>3.593</v>
       </c>
       <c r="G32" t="n">
-        <v>4.033</v>
+        <v>4.042</v>
       </c>
       <c r="H32" t="n">
-        <v>4.291</v>
+        <v>4.298</v>
       </c>
       <c r="I32" t="n">
-        <v>4.345</v>
+        <v>4.352</v>
       </c>
       <c r="J32" t="n">
-        <v>4.649</v>
+        <v>4.656</v>
       </c>
       <c r="K32" t="n">
-        <v>4.879</v>
+        <v>4.896</v>
       </c>
       <c r="L32" t="n">
-        <v>4.993</v>
+        <v>5.009</v>
       </c>
       <c r="M32" t="n">
-        <v>5.214</v>
+        <v>5.226</v>
       </c>
       <c r="N32" t="n">
-        <v>5.454</v>
+        <v>5.475</v>
       </c>
       <c r="O32" t="n">
-        <v>5.843</v>
+        <v>5.874</v>
       </c>
       <c r="P32" t="n">
-        <v>6.079</v>
+        <v>6.111</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.871</v>
+        <v>6.911</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>3.341</v>
+        <v>3.35</v>
       </c>
       <c r="G33" t="n">
-        <v>3.76</v>
+        <v>3.769</v>
       </c>
       <c r="H33" t="n">
-        <v>3.951</v>
+        <v>3.958</v>
       </c>
       <c r="I33" t="n">
-        <v>3.974</v>
+        <v>3.981</v>
       </c>
       <c r="J33" t="n">
-        <v>4.168</v>
+        <v>4.175</v>
       </c>
       <c r="K33" t="n">
-        <v>4.332</v>
+        <v>4.349</v>
       </c>
       <c r="L33" t="n">
-        <v>4.388</v>
+        <v>4.405</v>
       </c>
       <c r="M33" t="n">
-        <v>4.466</v>
+        <v>4.478</v>
       </c>
       <c r="N33" t="n">
-        <v>4.486</v>
+        <v>4.508</v>
       </c>
       <c r="O33" t="n">
-        <v>4.563</v>
+        <v>4.593</v>
       </c>
       <c r="P33" t="n">
-        <v>4.655</v>
+        <v>4.688</v>
       </c>
       <c r="Q33" t="n">
-        <v>5.126</v>
+        <v>5.166</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.404</v>
+        <v>3.413</v>
       </c>
       <c r="G34" t="n">
-        <v>3.822</v>
+        <v>3.831</v>
       </c>
       <c r="H34" t="n">
-        <v>4.018</v>
+        <v>4.025</v>
       </c>
       <c r="I34" t="n">
-        <v>4.046</v>
+        <v>4.053</v>
       </c>
       <c r="J34" t="n">
-        <v>4.242</v>
+        <v>4.249</v>
       </c>
       <c r="K34" t="n">
-        <v>4.412</v>
+        <v>4.429</v>
       </c>
       <c r="L34" t="n">
-        <v>4.468</v>
+        <v>4.485</v>
       </c>
       <c r="M34" t="n">
-        <v>4.558</v>
+        <v>4.57</v>
       </c>
       <c r="N34" t="n">
-        <v>4.591</v>
+        <v>4.613</v>
       </c>
       <c r="O34" t="n">
-        <v>4.732</v>
+        <v>4.762</v>
       </c>
       <c r="P34" t="n">
-        <v>4.95</v>
+        <v>4.982</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.827</v>
+        <v>5.867</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.375</v>
+        <v>3.384</v>
       </c>
       <c r="G35" t="n">
-        <v>3.791</v>
+        <v>3.8</v>
       </c>
       <c r="H35" t="n">
-        <v>3.986</v>
+        <v>3.993</v>
       </c>
       <c r="I35" t="n">
-        <v>4.01</v>
+        <v>4.017</v>
       </c>
       <c r="J35" t="n">
-        <v>4.208</v>
+        <v>4.215</v>
       </c>
       <c r="K35" t="n">
-        <v>4.363</v>
+        <v>4.38</v>
       </c>
       <c r="L35" t="n">
-        <v>4.422</v>
+        <v>4.439</v>
       </c>
       <c r="M35" t="n">
-        <v>4.504</v>
+        <v>4.516</v>
       </c>
       <c r="N35" t="n">
-        <v>4.527</v>
+        <v>4.549</v>
       </c>
       <c r="O35" t="n">
-        <v>4.629</v>
+        <v>4.659</v>
       </c>
       <c r="P35" t="n">
-        <v>4.752</v>
+        <v>4.785</v>
       </c>
       <c r="Q35" t="n">
-        <v>5.463</v>
+        <v>5.503</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>3.256</v>
+        <v>3.264</v>
       </c>
       <c r="G36" t="n">
-        <v>3.66</v>
+        <v>3.668</v>
       </c>
       <c r="H36" t="n">
-        <v>3.852</v>
+        <v>3.859</v>
       </c>
       <c r="I36" t="n">
-        <v>3.879</v>
+        <v>3.886</v>
       </c>
       <c r="J36" t="n">
-        <v>4.101</v>
+        <v>4.108</v>
       </c>
       <c r="K36" t="n">
-        <v>4.257</v>
+        <v>4.274</v>
       </c>
       <c r="L36" t="n">
-        <v>4.309</v>
+        <v>4.326</v>
       </c>
       <c r="M36" t="n">
-        <v>4.368</v>
+        <v>4.38</v>
       </c>
       <c r="N36" t="n">
-        <v>4.387</v>
+        <v>4.409</v>
       </c>
       <c r="O36" t="n">
-        <v>4.471</v>
+        <v>4.501</v>
       </c>
       <c r="P36" t="n">
-        <v>4.554</v>
+        <v>4.586</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.841</v>
+        <v>4.881</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>4.162</v>
+        <v>4.17</v>
       </c>
       <c r="G37" t="n">
-        <v>4.971</v>
+        <v>4.981</v>
       </c>
       <c r="H37" t="n">
-        <v>5.536</v>
+        <v>5.543</v>
       </c>
       <c r="I37" t="n">
-        <v>5.676</v>
+        <v>5.683</v>
       </c>
       <c r="J37" t="n">
-        <v>6.453</v>
+        <v>6.46</v>
       </c>
       <c r="K37" t="n">
-        <v>7.273</v>
+        <v>7.29</v>
       </c>
       <c r="L37" t="n">
-        <v>7.595</v>
+        <v>7.612</v>
       </c>
       <c r="M37" t="n">
-        <v>7.938</v>
+        <v>7.95</v>
       </c>
       <c r="N37" t="n">
-        <v>8.108000000000001</v>
+        <v>8.130000000000001</v>
       </c>
       <c r="O37" t="n">
-        <v>8.314</v>
+        <v>8.343999999999999</v>
       </c>
       <c r="P37" t="n">
-        <v>8.409000000000001</v>
+        <v>8.441000000000001</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.875999999999999</v>
+        <v>8.916</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>5.224</v>
+        <v>5.232</v>
       </c>
       <c r="G38" t="n">
-        <v>6.288</v>
+        <v>6.297</v>
       </c>
       <c r="H38" t="n">
-        <v>7.063</v>
+        <v>7.07</v>
       </c>
       <c r="I38" t="n">
-        <v>7.361</v>
+        <v>7.368</v>
       </c>
       <c r="J38" t="n">
-        <v>8.398999999999999</v>
+        <v>8.406000000000001</v>
       </c>
       <c r="K38" t="n">
-        <v>9.4</v>
+        <v>9.417</v>
       </c>
       <c r="L38" t="n">
-        <v>9.885</v>
+        <v>9.901999999999999</v>
       </c>
       <c r="M38" t="n">
-        <v>10.351</v>
+        <v>10.363</v>
       </c>
       <c r="N38" t="n">
-        <v>10.527</v>
+        <v>10.549</v>
       </c>
       <c r="O38" t="n">
-        <v>10.714</v>
+        <v>10.744</v>
       </c>
       <c r="P38" t="n">
-        <v>10.806</v>
+        <v>10.839</v>
       </c>
       <c r="Q38" t="n">
-        <v>11.326</v>
+        <v>11.366</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.544</v>
+        <v>4.552</v>
       </c>
       <c r="G39" t="n">
-        <v>5.487</v>
+        <v>5.496</v>
       </c>
       <c r="H39" t="n">
-        <v>6.129</v>
+        <v>6.136</v>
       </c>
       <c r="I39" t="n">
-        <v>6.364</v>
+        <v>6.371</v>
       </c>
       <c r="J39" t="n">
-        <v>7.271</v>
+        <v>7.278</v>
       </c>
       <c r="K39" t="n">
-        <v>8.231</v>
+        <v>8.247999999999999</v>
       </c>
       <c r="L39" t="n">
-        <v>8.638</v>
+        <v>8.654999999999999</v>
       </c>
       <c r="M39" t="n">
-        <v>8.987</v>
+        <v>8.999000000000001</v>
       </c>
       <c r="N39" t="n">
-        <v>9.154999999999999</v>
+        <v>9.177</v>
       </c>
       <c r="O39" t="n">
-        <v>9.364000000000001</v>
+        <v>9.394</v>
       </c>
       <c r="P39" t="n">
-        <v>9.461</v>
+        <v>9.494</v>
       </c>
       <c r="Q39" t="n">
-        <v>9.972</v>
+        <v>10.012</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.678</v>
+        <v>3.686</v>
       </c>
       <c r="G40" t="n">
-        <v>4.155</v>
+        <v>4.164</v>
       </c>
       <c r="H40" t="n">
-        <v>4.407</v>
+        <v>4.415</v>
       </c>
       <c r="I40" t="n">
-        <v>4.463</v>
+        <v>4.47</v>
       </c>
       <c r="J40" t="n">
-        <v>4.759</v>
+        <v>4.766</v>
       </c>
       <c r="K40" t="n">
-        <v>4.997</v>
+        <v>5.014</v>
       </c>
       <c r="L40" t="n">
-        <v>5.116</v>
+        <v>5.133</v>
       </c>
       <c r="M40" t="n">
-        <v>5.284</v>
+        <v>5.296</v>
       </c>
       <c r="N40" t="n">
-        <v>5.452</v>
+        <v>5.473</v>
       </c>
       <c r="O40" t="n">
-        <v>5.779</v>
+        <v>5.809</v>
       </c>
       <c r="P40" t="n">
-        <v>6.04</v>
+        <v>6.072</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.861</v>
+        <v>6.901</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>4.065</v>
+        <v>4.073</v>
       </c>
       <c r="G41" t="n">
-        <v>4.583</v>
+        <v>4.592</v>
       </c>
       <c r="H41" t="n">
-        <v>4.892</v>
+        <v>4.899</v>
       </c>
       <c r="I41" t="n">
-        <v>4.965</v>
+        <v>4.972</v>
       </c>
       <c r="J41" t="n">
-        <v>5.316</v>
+        <v>5.323</v>
       </c>
       <c r="K41" t="n">
-        <v>5.607</v>
+        <v>5.624</v>
       </c>
       <c r="L41" t="n">
-        <v>5.791</v>
+        <v>5.808</v>
       </c>
       <c r="M41" t="n">
-        <v>6.085</v>
+        <v>6.097</v>
       </c>
       <c r="N41" t="n">
-        <v>6.38</v>
+        <v>6.402</v>
       </c>
       <c r="O41" t="n">
-        <v>6.892</v>
+        <v>6.922</v>
       </c>
       <c r="P41" t="n">
-        <v>7.1</v>
+        <v>7.132</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.908</v>
+        <v>7.948</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.8</v>
+        <v>3.808</v>
       </c>
       <c r="G42" t="n">
-        <v>4.303</v>
+        <v>4.312</v>
       </c>
       <c r="H42" t="n">
-        <v>4.582</v>
+        <v>4.589</v>
       </c>
       <c r="I42" t="n">
-        <v>4.65</v>
+        <v>4.657</v>
       </c>
       <c r="J42" t="n">
-        <v>4.964</v>
+        <v>4.971</v>
       </c>
       <c r="K42" t="n">
-        <v>5.22</v>
+        <v>5.237</v>
       </c>
       <c r="L42" t="n">
-        <v>5.351</v>
+        <v>5.368</v>
       </c>
       <c r="M42" t="n">
-        <v>5.592</v>
+        <v>5.604</v>
       </c>
       <c r="N42" t="n">
-        <v>5.865</v>
+        <v>5.887</v>
       </c>
       <c r="O42" t="n">
-        <v>6.269</v>
+        <v>6.299</v>
       </c>
       <c r="P42" t="n">
-        <v>6.542</v>
+        <v>6.575</v>
       </c>
       <c r="Q42" t="n">
-        <v>7.374</v>
+        <v>7.414</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.491</v>
+        <v>3.5</v>
       </c>
       <c r="G43" t="n">
-        <v>3.947</v>
+        <v>3.956</v>
       </c>
       <c r="H43" t="n">
-        <v>4.156</v>
+        <v>4.163</v>
       </c>
       <c r="I43" t="n">
-        <v>4.187</v>
+        <v>4.194</v>
       </c>
       <c r="J43" t="n">
-        <v>4.395</v>
+        <v>4.402</v>
       </c>
       <c r="K43" t="n">
-        <v>4.564</v>
+        <v>4.582</v>
       </c>
       <c r="L43" t="n">
-        <v>4.631</v>
+        <v>4.648</v>
       </c>
       <c r="M43" t="n">
-        <v>4.722</v>
+        <v>4.734</v>
       </c>
       <c r="N43" t="n">
-        <v>4.756</v>
+        <v>4.777</v>
       </c>
       <c r="O43" t="n">
-        <v>4.877</v>
+        <v>4.907</v>
       </c>
       <c r="P43" t="n">
-        <v>5.021</v>
+        <v>5.053</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.736</v>
+        <v>5.776</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46269</v>
+        <v>46272</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>3.336</v>
+        <v>3.344</v>
       </c>
       <c r="G44" t="n">
-        <v>3.77</v>
+        <v>3.779</v>
       </c>
       <c r="H44" t="n">
-        <v>3.974</v>
+        <v>3.981</v>
       </c>
       <c r="I44" t="n">
-        <v>4.01</v>
+        <v>4.017</v>
       </c>
       <c r="J44" t="n">
-        <v>4.242</v>
+        <v>4.249</v>
       </c>
       <c r="K44" t="n">
-        <v>4.408</v>
+        <v>4.425</v>
       </c>
       <c r="L44" t="n">
-        <v>4.471</v>
+        <v>4.488</v>
       </c>
       <c r="M44" t="n">
-        <v>4.539</v>
+        <v>4.55</v>
       </c>
       <c r="N44" t="n">
-        <v>4.569</v>
+        <v>4.59</v>
       </c>
       <c r="O44" t="n">
-        <v>4.671</v>
+        <v>4.701</v>
       </c>
       <c r="P44" t="n">
-        <v>4.784</v>
+        <v>4.816</v>
       </c>
       <c r="Q44" t="n">
-        <v>5.105</v>
+        <v>5.145</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-09-08 ~ 2026-09-08
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,40 +552,40 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.655</v>
+        <v>3.661</v>
       </c>
       <c r="G2" t="n">
-        <v>4.135</v>
+        <v>4.143</v>
       </c>
       <c r="H2" t="n">
-        <v>4.395</v>
+        <v>4.404</v>
       </c>
       <c r="I2" t="n">
-        <v>4.394</v>
+        <v>4.41</v>
       </c>
       <c r="J2" t="n">
         <v>4.596</v>
       </c>
       <c r="K2" t="n">
-        <v>4.917</v>
+        <v>4.927</v>
       </c>
       <c r="L2" t="n">
-        <v>5.136</v>
+        <v>5.131</v>
       </c>
       <c r="M2" t="n">
-        <v>5.393</v>
+        <v>5.389</v>
       </c>
       <c r="N2" t="n">
-        <v>5.662</v>
+        <v>5.671</v>
       </c>
       <c r="O2" t="n">
-        <v>5.945</v>
+        <v>5.947</v>
       </c>
       <c r="P2" t="n">
-        <v>6.156</v>
+        <v>6.161</v>
       </c>
       <c r="Q2" t="n">
-        <v>6.847</v>
+        <v>6.857</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,40 +625,40 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.673</v>
+        <v>4.679</v>
       </c>
       <c r="G3" t="n">
-        <v>5.335</v>
+        <v>5.343</v>
       </c>
       <c r="H3" t="n">
-        <v>5.627</v>
+        <v>5.637</v>
       </c>
       <c r="I3" t="n">
-        <v>5.622</v>
+        <v>5.638</v>
       </c>
       <c r="J3" t="n">
         <v>5.84</v>
       </c>
       <c r="K3" t="n">
-        <v>6.233</v>
+        <v>6.243</v>
       </c>
       <c r="L3" t="n">
-        <v>6.522</v>
+        <v>6.518</v>
       </c>
       <c r="M3" t="n">
-        <v>6.808</v>
+        <v>6.804</v>
       </c>
       <c r="N3" t="n">
-        <v>7.022</v>
+        <v>7.031</v>
       </c>
       <c r="O3" t="n">
-        <v>7.255</v>
+        <v>7.257</v>
       </c>
       <c r="P3" t="n">
-        <v>7.334</v>
+        <v>7.338</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.913</v>
+        <v>7.923</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,40 +698,40 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>4.165</v>
+        <v>4.171</v>
       </c>
       <c r="G4" t="n">
-        <v>4.714</v>
+        <v>4.722</v>
       </c>
       <c r="H4" t="n">
-        <v>5.034</v>
+        <v>5.044</v>
       </c>
       <c r="I4" t="n">
-        <v>5.063</v>
+        <v>5.079</v>
       </c>
       <c r="J4" t="n">
-        <v>5.282</v>
+        <v>5.281</v>
       </c>
       <c r="K4" t="n">
-        <v>5.669</v>
+        <v>5.679</v>
       </c>
       <c r="L4" t="n">
-        <v>5.888</v>
+        <v>5.884</v>
       </c>
       <c r="M4" t="n">
-        <v>6.166</v>
+        <v>6.162</v>
       </c>
       <c r="N4" t="n">
-        <v>6.349</v>
+        <v>6.358</v>
       </c>
       <c r="O4" t="n">
-        <v>6.606</v>
+        <v>6.609</v>
       </c>
       <c r="P4" t="n">
-        <v>6.686</v>
+        <v>6.69</v>
       </c>
       <c r="Q4" t="n">
-        <v>7.268</v>
+        <v>7.278</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,40 +771,40 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>3.35</v>
+        <v>3.354</v>
       </c>
       <c r="G5" t="n">
-        <v>3.694</v>
+        <v>3.701</v>
       </c>
       <c r="H5" t="n">
-        <v>3.926</v>
+        <v>3.935</v>
       </c>
       <c r="I5" t="n">
-        <v>3.955</v>
+        <v>3.97</v>
       </c>
       <c r="J5" t="n">
         <v>4.17</v>
       </c>
       <c r="K5" t="n">
-        <v>4.316</v>
+        <v>4.326</v>
       </c>
       <c r="L5" t="n">
-        <v>4.38</v>
+        <v>4.375</v>
       </c>
       <c r="M5" t="n">
-        <v>4.457</v>
+        <v>4.453</v>
       </c>
       <c r="N5" t="n">
-        <v>4.482</v>
+        <v>4.491</v>
       </c>
       <c r="O5" t="n">
-        <v>4.545</v>
+        <v>4.547</v>
       </c>
       <c r="P5" t="n">
-        <v>4.824</v>
+        <v>4.828</v>
       </c>
       <c r="Q5" t="n">
-        <v>5.753</v>
+        <v>5.763</v>
       </c>
       <c r="R5" t="n">
         <v>0</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,40 +844,40 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>3.388</v>
+        <v>3.394</v>
       </c>
       <c r="G6" t="n">
-        <v>3.747</v>
+        <v>3.754</v>
       </c>
       <c r="H6" t="n">
-        <v>3.995</v>
+        <v>4.005</v>
       </c>
       <c r="I6" t="n">
-        <v>4.035</v>
+        <v>4.051</v>
       </c>
       <c r="J6" t="n">
         <v>4.262</v>
       </c>
       <c r="K6" t="n">
-        <v>4.433</v>
+        <v>4.443</v>
       </c>
       <c r="L6" t="n">
-        <v>4.502</v>
+        <v>4.497</v>
       </c>
       <c r="M6" t="n">
-        <v>4.609</v>
+        <v>4.604</v>
       </c>
       <c r="N6" t="n">
-        <v>4.647</v>
+        <v>4.656</v>
       </c>
       <c r="O6" t="n">
-        <v>4.812</v>
+        <v>4.814</v>
       </c>
       <c r="P6" t="n">
-        <v>5.257</v>
+        <v>5.262</v>
       </c>
       <c r="Q6" t="n">
-        <v>6.151</v>
+        <v>6.161</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,40 +917,40 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>3.369</v>
+        <v>3.373</v>
       </c>
       <c r="G7" t="n">
-        <v>3.71</v>
+        <v>3.717</v>
       </c>
       <c r="H7" t="n">
-        <v>3.942</v>
+        <v>3.951</v>
       </c>
       <c r="I7" t="n">
-        <v>3.973</v>
+        <v>3.988</v>
       </c>
       <c r="J7" t="n">
         <v>4.195</v>
       </c>
       <c r="K7" t="n">
-        <v>4.344</v>
+        <v>4.354</v>
       </c>
       <c r="L7" t="n">
-        <v>4.407</v>
+        <v>4.402</v>
       </c>
       <c r="M7" t="n">
-        <v>4.515</v>
+        <v>4.511</v>
       </c>
       <c r="N7" t="n">
-        <v>4.544</v>
+        <v>4.553</v>
       </c>
       <c r="O7" t="n">
-        <v>4.711</v>
+        <v>4.713</v>
       </c>
       <c r="P7" t="n">
-        <v>5.041</v>
+        <v>5.046</v>
       </c>
       <c r="Q7" t="n">
-        <v>5.919</v>
+        <v>5.929</v>
       </c>
       <c r="R7" t="n">
         <v>0</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,40 +990,40 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.787</v>
+        <v>5.793</v>
       </c>
       <c r="G8" t="n">
-        <v>6.637</v>
+        <v>6.644</v>
       </c>
       <c r="H8" t="n">
-        <v>7.082</v>
+        <v>7.092</v>
       </c>
       <c r="I8" t="n">
-        <v>7.149</v>
+        <v>7.165</v>
       </c>
       <c r="J8" t="n">
         <v>7.438</v>
       </c>
       <c r="K8" t="n">
-        <v>8.106999999999999</v>
+        <v>8.118</v>
       </c>
       <c r="L8" t="n">
-        <v>8.478999999999999</v>
+        <v>8.475</v>
       </c>
       <c r="M8" t="n">
-        <v>8.798999999999999</v>
+        <v>8.795</v>
       </c>
       <c r="N8" t="n">
-        <v>8.945</v>
+        <v>8.954000000000001</v>
       </c>
       <c r="O8" t="n">
-        <v>9.265000000000001</v>
+        <v>9.266999999999999</v>
       </c>
       <c r="P8" t="n">
-        <v>9.448</v>
+        <v>9.452999999999999</v>
       </c>
       <c r="Q8" t="n">
-        <v>10.23</v>
+        <v>10.24</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,22 +1063,22 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>3.022</v>
+        <v>3.029</v>
       </c>
       <c r="G9" t="n">
-        <v>3.145</v>
+        <v>3.16</v>
       </c>
       <c r="H9" t="n">
-        <v>3.375</v>
+        <v>3.384</v>
       </c>
       <c r="I9" t="n">
-        <v>3.485</v>
+        <v>3.496</v>
       </c>
       <c r="J9" t="n">
-        <v>3.623</v>
+        <v>3.627</v>
       </c>
       <c r="K9" t="n">
-        <v>3.722</v>
+        <v>3.715</v>
       </c>
       <c r="L9" t="n">
         <v>3.808</v>
@@ -1087,33 +1087,33 @@
         <v>3.897</v>
       </c>
       <c r="N9" t="n">
-        <v>3.993</v>
+        <v>4.002</v>
       </c>
       <c r="O9" t="n">
-        <v>4.125</v>
+        <v>4.127</v>
       </c>
       <c r="P9" t="n">
-        <v>4.264</v>
+        <v>4.269</v>
       </c>
       <c r="Q9" t="n">
-        <v>4.39</v>
+        <v>4.4</v>
       </c>
       <c r="R9" t="n">
-        <v>4.499</v>
+        <v>4.494</v>
       </c>
       <c r="S9" t="n">
-        <v>4.577</v>
+        <v>4.561</v>
       </c>
       <c r="T9" t="n">
-        <v>4.638</v>
+        <v>4.64</v>
       </c>
       <c r="U9" t="n">
-        <v>4.598</v>
+        <v>4.6</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>3.101</v>
+        <v>3.118</v>
       </c>
       <c r="G10" t="n">
-        <v>3.235</v>
+        <v>3.26</v>
       </c>
       <c r="H10" t="n">
-        <v>3.44</v>
+        <v>3.455</v>
       </c>
       <c r="I10" t="n">
-        <v>3.545</v>
+        <v>3.562</v>
       </c>
       <c r="J10" t="n">
-        <v>3.687</v>
+        <v>3.696</v>
       </c>
       <c r="K10" t="n">
-        <v>3.77</v>
+        <v>3.768</v>
       </c>
       <c r="L10" t="n">
-        <v>3.852</v>
+        <v>3.856</v>
       </c>
       <c r="M10" t="n">
-        <v>3.957</v>
+        <v>3.958</v>
       </c>
       <c r="N10" t="n">
-        <v>4.036</v>
+        <v>4.048</v>
       </c>
       <c r="O10" t="n">
-        <v>4.364</v>
+        <v>4.385</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,40 +1209,40 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.911</v>
+        <v>2.928</v>
       </c>
       <c r="G11" t="n">
-        <v>3.032</v>
+        <v>3.056</v>
       </c>
       <c r="H11" t="n">
-        <v>3.245</v>
+        <v>3.26</v>
       </c>
       <c r="I11" t="n">
-        <v>3.333</v>
+        <v>3.35</v>
       </c>
       <c r="J11" t="n">
-        <v>3.476</v>
+        <v>3.485</v>
       </c>
       <c r="K11" t="n">
-        <v>3.552</v>
+        <v>3.55</v>
       </c>
       <c r="L11" t="n">
-        <v>3.64</v>
+        <v>3.644</v>
       </c>
       <c r="M11" t="n">
-        <v>3.766</v>
+        <v>3.767</v>
       </c>
       <c r="N11" t="n">
-        <v>3.833</v>
+        <v>3.845</v>
       </c>
       <c r="O11" t="n">
-        <v>4.137</v>
+        <v>4.157</v>
       </c>
       <c r="P11" t="n">
-        <v>4.21</v>
+        <v>4.215</v>
       </c>
       <c r="Q11" t="n">
-        <v>4.588</v>
+        <v>4.598</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.672</v>
+        <v>3.682</v>
       </c>
       <c r="G12" t="n">
-        <v>4.031</v>
+        <v>4.041</v>
       </c>
       <c r="H12" t="n">
-        <v>4.316</v>
+        <v>4.327</v>
       </c>
       <c r="I12" t="n">
-        <v>4.39</v>
+        <v>4.406</v>
       </c>
       <c r="J12" t="n">
-        <v>4.606</v>
+        <v>4.61</v>
       </c>
       <c r="K12" t="n">
-        <v>4.719</v>
+        <v>4.732</v>
       </c>
       <c r="L12" t="n">
-        <v>4.802</v>
+        <v>4.803</v>
       </c>
       <c r="M12" t="n">
         <v>4.916</v>
       </c>
       <c r="N12" t="n">
-        <v>4.981</v>
+        <v>4.99</v>
       </c>
       <c r="O12" t="n">
-        <v>5.169</v>
+        <v>5.171</v>
       </c>
       <c r="P12" t="n">
-        <v>5.317</v>
+        <v>5.321</v>
       </c>
       <c r="Q12" t="n">
-        <v>5.704</v>
+        <v>5.714</v>
       </c>
       <c r="R12" t="n">
-        <v>5.991</v>
+        <v>5.986</v>
       </c>
       <c r="S12" t="n">
-        <v>6.276</v>
+        <v>6.261</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>3.426</v>
+        <v>3.435</v>
       </c>
       <c r="G13" t="n">
-        <v>3.722</v>
+        <v>3.732</v>
       </c>
       <c r="H13" t="n">
-        <v>3.983</v>
+        <v>3.994</v>
       </c>
       <c r="I13" t="n">
-        <v>4.038</v>
+        <v>4.054</v>
       </c>
       <c r="J13" t="n">
-        <v>4.244</v>
+        <v>4.248</v>
       </c>
       <c r="K13" t="n">
-        <v>4.353</v>
+        <v>4.365</v>
       </c>
       <c r="L13" t="n">
-        <v>4.442</v>
+        <v>4.443</v>
       </c>
       <c r="M13" t="n">
-        <v>4.544</v>
+        <v>4.545</v>
       </c>
       <c r="N13" t="n">
-        <v>4.609</v>
+        <v>4.618</v>
       </c>
       <c r="O13" t="n">
-        <v>4.796</v>
+        <v>4.798</v>
       </c>
       <c r="P13" t="n">
-        <v>4.908</v>
+        <v>4.913</v>
       </c>
       <c r="Q13" t="n">
-        <v>5.227</v>
+        <v>5.237</v>
       </c>
       <c r="R13" t="n">
-        <v>5.541</v>
+        <v>5.536</v>
       </c>
       <c r="S13" t="n">
-        <v>5.844</v>
+        <v>5.829</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>3.243</v>
+        <v>3.252</v>
       </c>
       <c r="G14" t="n">
-        <v>3.52</v>
+        <v>3.531</v>
       </c>
       <c r="H14" t="n">
-        <v>3.782</v>
+        <v>3.793</v>
       </c>
       <c r="I14" t="n">
-        <v>3.822</v>
+        <v>3.839</v>
       </c>
       <c r="J14" t="n">
-        <v>3.986</v>
+        <v>3.99</v>
       </c>
       <c r="K14" t="n">
-        <v>4.042</v>
+        <v>4.054</v>
       </c>
       <c r="L14" t="n">
-        <v>4.115</v>
+        <v>4.116</v>
       </c>
       <c r="M14" t="n">
         <v>4.231</v>
       </c>
       <c r="N14" t="n">
-        <v>4.288</v>
+        <v>4.297</v>
       </c>
       <c r="O14" t="n">
-        <v>4.454</v>
+        <v>4.456</v>
       </c>
       <c r="P14" t="n">
-        <v>4.547</v>
+        <v>4.552</v>
       </c>
       <c r="Q14" t="n">
-        <v>4.816</v>
+        <v>4.826</v>
       </c>
       <c r="R14" t="n">
-        <v>5.055</v>
+        <v>5.051</v>
       </c>
       <c r="S14" t="n">
-        <v>5.297</v>
+        <v>5.281</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>3.215</v>
+        <v>3.225</v>
       </c>
       <c r="G15" t="n">
-        <v>3.49</v>
+        <v>3.501</v>
       </c>
       <c r="H15" t="n">
-        <v>3.746</v>
+        <v>3.757</v>
       </c>
       <c r="I15" t="n">
-        <v>3.757</v>
+        <v>3.772</v>
       </c>
       <c r="J15" t="n">
-        <v>3.921</v>
+        <v>3.926</v>
       </c>
       <c r="K15" t="n">
-        <v>3.989</v>
+        <v>4.001</v>
       </c>
       <c r="L15" t="n">
         <v>4.045</v>
       </c>
       <c r="M15" t="n">
-        <v>4.139</v>
+        <v>4.141</v>
       </c>
       <c r="N15" t="n">
-        <v>4.192</v>
+        <v>4.201</v>
       </c>
       <c r="O15" t="n">
-        <v>4.402</v>
+        <v>4.404</v>
       </c>
       <c r="P15" t="n">
-        <v>4.448</v>
+        <v>4.453</v>
       </c>
       <c r="Q15" t="n">
-        <v>4.717</v>
+        <v>4.727</v>
       </c>
       <c r="R15" t="n">
-        <v>4.949</v>
+        <v>4.944</v>
       </c>
       <c r="S15" t="n">
-        <v>5.187</v>
+        <v>5.171</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>3.215</v>
+        <v>3.225</v>
       </c>
       <c r="G16" t="n">
-        <v>3.49</v>
+        <v>3.501</v>
       </c>
       <c r="H16" t="n">
-        <v>3.746</v>
+        <v>3.757</v>
       </c>
       <c r="I16" t="n">
-        <v>3.757</v>
+        <v>3.772</v>
       </c>
       <c r="J16" t="n">
-        <v>3.921</v>
+        <v>3.926</v>
       </c>
       <c r="K16" t="n">
-        <v>3.989</v>
+        <v>4.001</v>
       </c>
       <c r="L16" t="n">
         <v>4.045</v>
       </c>
       <c r="M16" t="n">
-        <v>4.139</v>
+        <v>4.141</v>
       </c>
       <c r="N16" t="n">
-        <v>4.195</v>
+        <v>4.204</v>
       </c>
       <c r="O16" t="n">
-        <v>4.407</v>
+        <v>4.409</v>
       </c>
       <c r="P16" t="n">
-        <v>4.471</v>
+        <v>4.476</v>
       </c>
       <c r="Q16" t="n">
-        <v>4.744</v>
+        <v>4.754</v>
       </c>
       <c r="R16" t="n">
-        <v>4.977</v>
+        <v>4.972</v>
       </c>
       <c r="S16" t="n">
-        <v>5.218</v>
+        <v>5.202</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>3.148</v>
+        <v>3.164</v>
       </c>
       <c r="G17" t="n">
-        <v>3.298</v>
+        <v>3.322</v>
       </c>
       <c r="H17" t="n">
-        <v>3.477</v>
+        <v>3.493</v>
       </c>
       <c r="I17" t="n">
-        <v>3.591</v>
+        <v>3.607</v>
       </c>
       <c r="J17" t="n">
-        <v>3.758</v>
+        <v>3.767</v>
       </c>
       <c r="K17" t="n">
-        <v>3.864</v>
+        <v>3.863</v>
       </c>
       <c r="L17" t="n">
-        <v>3.942</v>
+        <v>3.946</v>
       </c>
       <c r="M17" t="n">
         <v>4.094</v>
       </c>
       <c r="N17" t="n">
-        <v>4.154</v>
+        <v>4.167</v>
       </c>
       <c r="O17" t="n">
-        <v>4.389</v>
+        <v>4.41</v>
       </c>
       <c r="P17" t="n">
-        <v>4.491</v>
+        <v>4.495</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>3.148</v>
+        <v>3.164</v>
       </c>
       <c r="G18" t="n">
-        <v>3.298</v>
+        <v>3.322</v>
       </c>
       <c r="H18" t="n">
-        <v>3.477</v>
+        <v>3.493</v>
       </c>
       <c r="I18" t="n">
-        <v>3.59</v>
+        <v>3.607</v>
       </c>
       <c r="J18" t="n">
-        <v>3.758</v>
+        <v>3.767</v>
       </c>
       <c r="K18" t="n">
         <v>3.864</v>
       </c>
       <c r="L18" t="n">
-        <v>3.942</v>
+        <v>3.946</v>
       </c>
       <c r="M18" t="n">
-        <v>4.093</v>
+        <v>4.094</v>
       </c>
       <c r="N18" t="n">
-        <v>4.154</v>
+        <v>4.167</v>
       </c>
       <c r="O18" t="n">
-        <v>4.389</v>
+        <v>4.41</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,22 +1793,22 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>3.232</v>
+        <v>3.241</v>
       </c>
       <c r="G19" t="n">
-        <v>3.514</v>
+        <v>3.525</v>
       </c>
       <c r="H19" t="n">
-        <v>3.77</v>
+        <v>3.781</v>
       </c>
       <c r="I19" t="n">
-        <v>3.807</v>
+        <v>3.823</v>
       </c>
       <c r="J19" t="n">
-        <v>3.985</v>
+        <v>3.989</v>
       </c>
       <c r="K19" t="n">
-        <v>4.052</v>
+        <v>4.064</v>
       </c>
       <c r="L19" t="n">
         <v>4.122</v>
@@ -1817,22 +1817,22 @@
         <v>4.229</v>
       </c>
       <c r="N19" t="n">
-        <v>4.281</v>
+        <v>4.29</v>
       </c>
       <c r="O19" t="n">
-        <v>4.443</v>
+        <v>4.445</v>
       </c>
       <c r="P19" t="n">
-        <v>4.506</v>
+        <v>4.511</v>
       </c>
       <c r="Q19" t="n">
-        <v>4.755</v>
+        <v>4.765</v>
       </c>
       <c r="R19" t="n">
-        <v>4.996</v>
+        <v>4.991</v>
       </c>
       <c r="S19" t="n">
-        <v>5.231</v>
+        <v>5.215</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>3.024</v>
+        <v>3.03</v>
       </c>
       <c r="G20" t="n">
-        <v>3.051</v>
+        <v>3.059</v>
       </c>
       <c r="H20" t="n">
-        <v>3.166</v>
+        <v>3.175</v>
       </c>
       <c r="I20" t="n">
-        <v>3.29</v>
+        <v>3.303</v>
       </c>
       <c r="J20" t="n">
-        <v>3.678</v>
+        <v>3.682</v>
       </c>
       <c r="K20" t="n">
-        <v>3.785</v>
+        <v>3.8</v>
       </c>
       <c r="L20" t="n">
-        <v>3.794</v>
+        <v>3.802</v>
       </c>
       <c r="M20" t="n">
-        <v>3.893</v>
+        <v>3.894</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>3.306</v>
+        <v>3.316</v>
       </c>
       <c r="G21" t="n">
-        <v>3.607</v>
+        <v>3.621</v>
       </c>
       <c r="H21" t="n">
-        <v>3.891</v>
+        <v>3.901</v>
       </c>
       <c r="I21" t="n">
-        <v>3.944</v>
+        <v>3.961</v>
       </c>
       <c r="J21" t="n">
-        <v>4.153</v>
+        <v>4.158</v>
       </c>
       <c r="K21" t="n">
-        <v>4.27</v>
+        <v>4.284</v>
       </c>
       <c r="L21" t="n">
-        <v>4.35</v>
+        <v>4.353</v>
       </c>
       <c r="M21" t="n">
-        <v>4.457</v>
+        <v>4.458</v>
       </c>
       <c r="N21" t="n">
-        <v>4.524</v>
+        <v>4.533</v>
       </c>
       <c r="O21" t="n">
-        <v>4.672</v>
+        <v>4.681</v>
       </c>
       <c r="P21" t="n">
-        <v>4.75</v>
+        <v>4.755</v>
       </c>
       <c r="Q21" t="n">
-        <v>4.907</v>
+        <v>4.917</v>
       </c>
       <c r="R21" t="n">
-        <v>5.047</v>
+        <v>5.042</v>
       </c>
       <c r="S21" t="n">
-        <v>5.184</v>
+        <v>5.169</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>3.25</v>
+        <v>3.26</v>
       </c>
       <c r="G22" t="n">
-        <v>3.553</v>
+        <v>3.567</v>
       </c>
       <c r="H22" t="n">
-        <v>3.823</v>
+        <v>3.833</v>
       </c>
       <c r="I22" t="n">
-        <v>3.861</v>
+        <v>3.878</v>
       </c>
       <c r="J22" t="n">
-        <v>4.04</v>
+        <v>4.046</v>
       </c>
       <c r="K22" t="n">
-        <v>4.149</v>
+        <v>4.163</v>
       </c>
       <c r="L22" t="n">
-        <v>4.223</v>
+        <v>4.225</v>
       </c>
       <c r="M22" t="n">
-        <v>4.329</v>
+        <v>4.33</v>
       </c>
       <c r="N22" t="n">
-        <v>4.4</v>
+        <v>4.409</v>
       </c>
       <c r="O22" t="n">
-        <v>4.542</v>
+        <v>4.551</v>
       </c>
       <c r="P22" t="n">
-        <v>4.614</v>
+        <v>4.618</v>
       </c>
       <c r="Q22" t="n">
-        <v>4.765</v>
+        <v>4.775</v>
       </c>
       <c r="R22" t="n">
-        <v>4.896</v>
+        <v>4.89</v>
       </c>
       <c r="S22" t="n">
-        <v>5.03</v>
+        <v>5.014</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>3.201</v>
+        <v>3.21</v>
       </c>
       <c r="G23" t="n">
-        <v>3.504</v>
+        <v>3.517</v>
       </c>
       <c r="H23" t="n">
-        <v>3.762</v>
+        <v>3.772</v>
       </c>
       <c r="I23" t="n">
-        <v>3.797</v>
+        <v>3.813</v>
       </c>
       <c r="J23" t="n">
-        <v>3.958</v>
+        <v>3.963</v>
       </c>
       <c r="K23" t="n">
-        <v>4.04</v>
+        <v>4.054</v>
       </c>
       <c r="L23" t="n">
-        <v>4.116</v>
+        <v>4.118</v>
       </c>
       <c r="M23" t="n">
-        <v>4.219</v>
+        <v>4.22</v>
       </c>
       <c r="N23" t="n">
-        <v>4.287</v>
+        <v>4.296</v>
       </c>
       <c r="O23" t="n">
-        <v>4.417</v>
+        <v>4.426</v>
       </c>
       <c r="P23" t="n">
-        <v>4.475</v>
+        <v>4.48</v>
       </c>
       <c r="Q23" t="n">
-        <v>4.568</v>
+        <v>4.578</v>
       </c>
       <c r="R23" t="n">
-        <v>4.681</v>
+        <v>4.676</v>
       </c>
       <c r="S23" t="n">
-        <v>4.786</v>
+        <v>4.77</v>
       </c>
       <c r="T23" t="n">
-        <v>4.854</v>
+        <v>4.855</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>3.151</v>
+        <v>3.161</v>
       </c>
       <c r="G24" t="n">
-        <v>3.418</v>
+        <v>3.431</v>
       </c>
       <c r="H24" t="n">
-        <v>3.649</v>
+        <v>3.659</v>
       </c>
       <c r="I24" t="n">
-        <v>3.707</v>
+        <v>3.723</v>
       </c>
       <c r="J24" t="n">
-        <v>3.852</v>
+        <v>3.857</v>
       </c>
       <c r="K24" t="n">
-        <v>3.934</v>
+        <v>3.948</v>
       </c>
       <c r="L24" t="n">
-        <v>3.999</v>
+        <v>4.001</v>
       </c>
       <c r="M24" t="n">
         <v>4.077</v>
       </c>
       <c r="N24" t="n">
-        <v>4.157</v>
+        <v>4.165</v>
       </c>
       <c r="O24" t="n">
-        <v>4.372</v>
+        <v>4.383</v>
       </c>
       <c r="P24" t="n">
-        <v>4.417</v>
+        <v>4.421</v>
       </c>
       <c r="Q24" t="n">
-        <v>4.497</v>
+        <v>4.507</v>
       </c>
       <c r="R24" t="n">
-        <v>4.604</v>
+        <v>4.598</v>
       </c>
       <c r="S24" t="n">
-        <v>4.701</v>
+        <v>4.685</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>3.194</v>
+        <v>3.203</v>
       </c>
       <c r="G25" t="n">
-        <v>3.505</v>
+        <v>3.518</v>
       </c>
       <c r="H25" t="n">
-        <v>3.765</v>
+        <v>3.776</v>
       </c>
       <c r="I25" t="n">
-        <v>3.808</v>
+        <v>3.824</v>
       </c>
       <c r="J25" t="n">
-        <v>3.98</v>
+        <v>3.985</v>
       </c>
       <c r="K25" t="n">
-        <v>4.078</v>
+        <v>4.091</v>
       </c>
       <c r="L25" t="n">
-        <v>4.148</v>
+        <v>4.15</v>
       </c>
       <c r="M25" t="n">
-        <v>4.251</v>
+        <v>4.252</v>
       </c>
       <c r="N25" t="n">
-        <v>4.314</v>
+        <v>4.323</v>
       </c>
       <c r="O25" t="n">
-        <v>4.447</v>
+        <v>4.456</v>
       </c>
       <c r="P25" t="n">
-        <v>4.498</v>
+        <v>4.502</v>
       </c>
       <c r="Q25" t="n">
-        <v>4.6</v>
+        <v>4.61</v>
       </c>
       <c r="R25" t="n">
-        <v>4.705</v>
+        <v>4.7</v>
       </c>
       <c r="S25" t="n">
-        <v>4.809</v>
+        <v>4.794</v>
       </c>
       <c r="T25" t="n">
-        <v>4.871</v>
+        <v>4.872</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.45</v>
+        <v>3.455</v>
       </c>
       <c r="G26" t="n">
-        <v>3.923</v>
+        <v>3.931</v>
       </c>
       <c r="H26" t="n">
-        <v>4.211</v>
+        <v>4.222</v>
       </c>
       <c r="I26" t="n">
-        <v>4.253</v>
+        <v>4.267</v>
       </c>
       <c r="J26" t="n">
-        <v>4.598</v>
+        <v>4.596</v>
       </c>
       <c r="K26" t="n">
-        <v>4.907</v>
+        <v>4.917</v>
       </c>
       <c r="L26" t="n">
-        <v>5.024</v>
+        <v>5.019</v>
       </c>
       <c r="M26" t="n">
-        <v>5.183</v>
+        <v>5.18</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.487</v>
+        <v>5.49</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>3.297</v>
+        <v>3.304</v>
       </c>
       <c r="G27" t="n">
-        <v>3.627</v>
+        <v>3.635</v>
       </c>
       <c r="H27" t="n">
-        <v>3.868</v>
+        <v>3.88</v>
       </c>
       <c r="I27" t="n">
-        <v>3.908</v>
+        <v>3.923</v>
       </c>
       <c r="J27" t="n">
-        <v>4.103</v>
+        <v>4.104</v>
       </c>
       <c r="K27" t="n">
-        <v>4.221</v>
+        <v>4.233</v>
       </c>
       <c r="L27" t="n">
-        <v>4.294</v>
+        <v>4.293</v>
       </c>
       <c r="M27" t="n">
-        <v>4.396</v>
+        <v>4.394</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.586</v>
+        <v>4.588</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>3.406</v>
+        <v>3.413</v>
       </c>
       <c r="G28" t="n">
-        <v>3.749</v>
+        <v>3.758</v>
       </c>
       <c r="H28" t="n">
-        <v>4.002</v>
+        <v>4.014</v>
       </c>
       <c r="I28" t="n">
-        <v>4.047</v>
+        <v>4.063</v>
       </c>
       <c r="J28" t="n">
-        <v>4.276</v>
+        <v>4.278</v>
       </c>
       <c r="K28" t="n">
-        <v>4.413</v>
+        <v>4.426</v>
       </c>
       <c r="L28" t="n">
-        <v>4.498</v>
+        <v>4.497</v>
       </c>
       <c r="M28" t="n">
-        <v>4.608</v>
+        <v>4.606</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.878</v>
+        <v>4.88</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>3.243</v>
+        <v>3.25</v>
       </c>
       <c r="G29" t="n">
-        <v>3.568</v>
+        <v>3.576</v>
       </c>
       <c r="H29" t="n">
-        <v>3.8</v>
+        <v>3.813</v>
       </c>
       <c r="I29" t="n">
-        <v>3.824</v>
+        <v>3.839</v>
       </c>
       <c r="J29" t="n">
-        <v>4.012</v>
+        <v>4.013</v>
       </c>
       <c r="K29" t="n">
-        <v>4.115</v>
+        <v>4.126</v>
       </c>
       <c r="L29" t="n">
-        <v>4.175</v>
+        <v>4.174</v>
       </c>
       <c r="M29" t="n">
-        <v>4.258</v>
+        <v>4.256</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>4.459</v>
+        <v>4.461</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,40 +2596,40 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.495</v>
+        <v>3.501</v>
       </c>
       <c r="G30" t="n">
-        <v>3.926</v>
+        <v>3.935</v>
       </c>
       <c r="H30" t="n">
-        <v>4.156</v>
+        <v>4.168</v>
       </c>
       <c r="I30" t="n">
-        <v>4.194</v>
+        <v>4.207</v>
       </c>
       <c r="J30" t="n">
         <v>4.475</v>
       </c>
       <c r="K30" t="n">
-        <v>4.709</v>
+        <v>4.721</v>
       </c>
       <c r="L30" t="n">
-        <v>4.805</v>
+        <v>4.802</v>
       </c>
       <c r="M30" t="n">
-        <v>4.954</v>
+        <v>4.951</v>
       </c>
       <c r="N30" t="n">
-        <v>5.114</v>
+        <v>5.123</v>
       </c>
       <c r="O30" t="n">
-        <v>5.428</v>
+        <v>5.43</v>
       </c>
       <c r="P30" t="n">
-        <v>5.651</v>
+        <v>5.656</v>
       </c>
       <c r="Q30" t="n">
-        <v>6.45</v>
+        <v>6.46</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,40 +2669,40 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.824</v>
+        <v>3.83</v>
       </c>
       <c r="G31" t="n">
-        <v>4.29</v>
+        <v>4.299</v>
       </c>
       <c r="H31" t="n">
-        <v>4.57</v>
+        <v>4.582</v>
       </c>
       <c r="I31" t="n">
-        <v>4.622</v>
+        <v>4.635</v>
       </c>
       <c r="J31" t="n">
         <v>4.968</v>
       </c>
       <c r="K31" t="n">
-        <v>5.25</v>
+        <v>5.262</v>
       </c>
       <c r="L31" t="n">
-        <v>5.417</v>
+        <v>5.414</v>
       </c>
       <c r="M31" t="n">
-        <v>5.682</v>
+        <v>5.68</v>
       </c>
       <c r="N31" t="n">
-        <v>5.973</v>
+        <v>5.982</v>
       </c>
       <c r="O31" t="n">
-        <v>6.464</v>
+        <v>6.466</v>
       </c>
       <c r="P31" t="n">
-        <v>6.64</v>
+        <v>6.644</v>
       </c>
       <c r="Q31" t="n">
-        <v>7.423</v>
+        <v>7.433</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,40 +2742,40 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.593</v>
+        <v>3.599</v>
       </c>
       <c r="G32" t="n">
-        <v>4.042</v>
+        <v>4.051</v>
       </c>
       <c r="H32" t="n">
-        <v>4.298</v>
+        <v>4.31</v>
       </c>
       <c r="I32" t="n">
-        <v>4.352</v>
+        <v>4.365</v>
       </c>
       <c r="J32" t="n">
         <v>4.656</v>
       </c>
       <c r="K32" t="n">
-        <v>4.896</v>
+        <v>4.907</v>
       </c>
       <c r="L32" t="n">
-        <v>5.009</v>
+        <v>5.006</v>
       </c>
       <c r="M32" t="n">
-        <v>5.226</v>
+        <v>5.224</v>
       </c>
       <c r="N32" t="n">
-        <v>5.475</v>
+        <v>5.484</v>
       </c>
       <c r="O32" t="n">
-        <v>5.874</v>
+        <v>5.875</v>
       </c>
       <c r="P32" t="n">
-        <v>6.111</v>
+        <v>6.116</v>
       </c>
       <c r="Q32" t="n">
-        <v>6.911</v>
+        <v>6.921</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,40 +2815,40 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>3.35</v>
+        <v>3.355</v>
       </c>
       <c r="G33" t="n">
-        <v>3.769</v>
+        <v>3.777</v>
       </c>
       <c r="H33" t="n">
-        <v>3.958</v>
+        <v>3.971</v>
       </c>
       <c r="I33" t="n">
-        <v>3.981</v>
+        <v>3.995</v>
       </c>
       <c r="J33" t="n">
-        <v>4.175</v>
+        <v>4.173</v>
       </c>
       <c r="K33" t="n">
-        <v>4.349</v>
+        <v>4.358</v>
       </c>
       <c r="L33" t="n">
-        <v>4.405</v>
+        <v>4.401</v>
       </c>
       <c r="M33" t="n">
-        <v>4.478</v>
+        <v>4.476</v>
       </c>
       <c r="N33" t="n">
-        <v>4.508</v>
+        <v>4.518</v>
       </c>
       <c r="O33" t="n">
-        <v>4.593</v>
+        <v>4.595</v>
       </c>
       <c r="P33" t="n">
-        <v>4.688</v>
+        <v>4.692</v>
       </c>
       <c r="Q33" t="n">
-        <v>5.166</v>
+        <v>5.176</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,40 +2888,40 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.413</v>
+        <v>3.418</v>
       </c>
       <c r="G34" t="n">
-        <v>3.831</v>
+        <v>3.839</v>
       </c>
       <c r="H34" t="n">
-        <v>4.025</v>
+        <v>4.038</v>
       </c>
       <c r="I34" t="n">
-        <v>4.053</v>
+        <v>4.066</v>
       </c>
       <c r="J34" t="n">
-        <v>4.249</v>
+        <v>4.247</v>
       </c>
       <c r="K34" t="n">
-        <v>4.429</v>
+        <v>4.438</v>
       </c>
       <c r="L34" t="n">
-        <v>4.485</v>
+        <v>4.481</v>
       </c>
       <c r="M34" t="n">
-        <v>4.57</v>
+        <v>4.568</v>
       </c>
       <c r="N34" t="n">
-        <v>4.613</v>
+        <v>4.623</v>
       </c>
       <c r="O34" t="n">
-        <v>4.762</v>
+        <v>4.764</v>
       </c>
       <c r="P34" t="n">
-        <v>4.982</v>
+        <v>4.987</v>
       </c>
       <c r="Q34" t="n">
-        <v>5.867</v>
+        <v>5.877</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,40 +2961,40 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.384</v>
+        <v>3.389</v>
       </c>
       <c r="G35" t="n">
-        <v>3.8</v>
+        <v>3.808</v>
       </c>
       <c r="H35" t="n">
-        <v>3.993</v>
+        <v>4.006</v>
       </c>
       <c r="I35" t="n">
-        <v>4.017</v>
+        <v>4.031</v>
       </c>
       <c r="J35" t="n">
-        <v>4.215</v>
+        <v>4.213</v>
       </c>
       <c r="K35" t="n">
-        <v>4.38</v>
+        <v>4.389</v>
       </c>
       <c r="L35" t="n">
-        <v>4.439</v>
+        <v>4.435</v>
       </c>
       <c r="M35" t="n">
-        <v>4.516</v>
+        <v>4.515</v>
       </c>
       <c r="N35" t="n">
-        <v>4.549</v>
+        <v>4.559</v>
       </c>
       <c r="O35" t="n">
-        <v>4.659</v>
+        <v>4.661</v>
       </c>
       <c r="P35" t="n">
-        <v>4.785</v>
+        <v>4.789</v>
       </c>
       <c r="Q35" t="n">
-        <v>5.503</v>
+        <v>5.513</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,40 +3034,40 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>3.264</v>
+        <v>3.27</v>
       </c>
       <c r="G36" t="n">
-        <v>3.668</v>
+        <v>3.676</v>
       </c>
       <c r="H36" t="n">
-        <v>3.859</v>
+        <v>3.871</v>
       </c>
       <c r="I36" t="n">
-        <v>3.886</v>
+        <v>3.899</v>
       </c>
       <c r="J36" t="n">
-        <v>4.108</v>
+        <v>4.106</v>
       </c>
       <c r="K36" t="n">
-        <v>4.274</v>
+        <v>4.283</v>
       </c>
       <c r="L36" t="n">
-        <v>4.326</v>
+        <v>4.321</v>
       </c>
       <c r="M36" t="n">
-        <v>4.38</v>
+        <v>4.376</v>
       </c>
       <c r="N36" t="n">
-        <v>4.409</v>
+        <v>4.419</v>
       </c>
       <c r="O36" t="n">
-        <v>4.501</v>
+        <v>4.504</v>
       </c>
       <c r="P36" t="n">
-        <v>4.586</v>
+        <v>4.591</v>
       </c>
       <c r="Q36" t="n">
-        <v>4.881</v>
+        <v>4.891</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,40 +3107,40 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>4.17</v>
+        <v>4.176</v>
       </c>
       <c r="G37" t="n">
-        <v>4.981</v>
+        <v>4.99</v>
       </c>
       <c r="H37" t="n">
-        <v>5.543</v>
+        <v>5.555</v>
       </c>
       <c r="I37" t="n">
-        <v>5.683</v>
+        <v>5.696</v>
       </c>
       <c r="J37" t="n">
         <v>6.46</v>
       </c>
       <c r="K37" t="n">
-        <v>7.29</v>
+        <v>7.302</v>
       </c>
       <c r="L37" t="n">
-        <v>7.612</v>
+        <v>7.608</v>
       </c>
       <c r="M37" t="n">
-        <v>7.95</v>
+        <v>7.947</v>
       </c>
       <c r="N37" t="n">
-        <v>8.130000000000001</v>
+        <v>8.138999999999999</v>
       </c>
       <c r="O37" t="n">
-        <v>8.343999999999999</v>
+        <v>8.346</v>
       </c>
       <c r="P37" t="n">
-        <v>8.441000000000001</v>
+        <v>8.446</v>
       </c>
       <c r="Q37" t="n">
-        <v>8.916</v>
+        <v>8.926</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,40 +3180,40 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>5.232</v>
+        <v>5.238</v>
       </c>
       <c r="G38" t="n">
-        <v>6.297</v>
+        <v>6.306</v>
       </c>
       <c r="H38" t="n">
-        <v>7.07</v>
+        <v>7.082</v>
       </c>
       <c r="I38" t="n">
-        <v>7.368</v>
+        <v>7.381</v>
       </c>
       <c r="J38" t="n">
         <v>8.406000000000001</v>
       </c>
       <c r="K38" t="n">
-        <v>9.417</v>
+        <v>9.428000000000001</v>
       </c>
       <c r="L38" t="n">
-        <v>9.901999999999999</v>
+        <v>9.898999999999999</v>
       </c>
       <c r="M38" t="n">
-        <v>10.363</v>
+        <v>10.36</v>
       </c>
       <c r="N38" t="n">
-        <v>10.549</v>
+        <v>10.558</v>
       </c>
       <c r="O38" t="n">
-        <v>10.744</v>
+        <v>10.746</v>
       </c>
       <c r="P38" t="n">
-        <v>10.839</v>
+        <v>10.844</v>
       </c>
       <c r="Q38" t="n">
-        <v>11.366</v>
+        <v>11.376</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,40 +3253,40 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.552</v>
+        <v>4.558</v>
       </c>
       <c r="G39" t="n">
-        <v>5.496</v>
+        <v>5.505</v>
       </c>
       <c r="H39" t="n">
-        <v>6.136</v>
+        <v>6.148</v>
       </c>
       <c r="I39" t="n">
-        <v>6.371</v>
+        <v>6.384</v>
       </c>
       <c r="J39" t="n">
         <v>7.278</v>
       </c>
       <c r="K39" t="n">
-        <v>8.247999999999999</v>
+        <v>8.26</v>
       </c>
       <c r="L39" t="n">
-        <v>8.654999999999999</v>
+        <v>8.651</v>
       </c>
       <c r="M39" t="n">
-        <v>8.999000000000001</v>
+        <v>8.997</v>
       </c>
       <c r="N39" t="n">
-        <v>9.177</v>
+        <v>9.186</v>
       </c>
       <c r="O39" t="n">
-        <v>9.394</v>
+        <v>9.396000000000001</v>
       </c>
       <c r="P39" t="n">
-        <v>9.494</v>
+        <v>9.497999999999999</v>
       </c>
       <c r="Q39" t="n">
-        <v>10.012</v>
+        <v>10.022</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,40 +3326,40 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.686</v>
+        <v>3.692</v>
       </c>
       <c r="G40" t="n">
-        <v>4.164</v>
+        <v>4.173</v>
       </c>
       <c r="H40" t="n">
-        <v>4.415</v>
+        <v>4.427</v>
       </c>
       <c r="I40" t="n">
-        <v>4.47</v>
+        <v>4.483</v>
       </c>
       <c r="J40" t="n">
         <v>4.766</v>
       </c>
       <c r="K40" t="n">
-        <v>5.014</v>
+        <v>5.026</v>
       </c>
       <c r="L40" t="n">
-        <v>5.133</v>
+        <v>5.129</v>
       </c>
       <c r="M40" t="n">
-        <v>5.296</v>
+        <v>5.294</v>
       </c>
       <c r="N40" t="n">
-        <v>5.473</v>
+        <v>5.482</v>
       </c>
       <c r="O40" t="n">
-        <v>5.809</v>
+        <v>5.811</v>
       </c>
       <c r="P40" t="n">
-        <v>6.072</v>
+        <v>6.077</v>
       </c>
       <c r="Q40" t="n">
-        <v>6.901</v>
+        <v>6.911</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,40 +3399,40 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>4.073</v>
+        <v>4.079</v>
       </c>
       <c r="G41" t="n">
-        <v>4.592</v>
+        <v>4.601</v>
       </c>
       <c r="H41" t="n">
-        <v>4.899</v>
+        <v>4.911</v>
       </c>
       <c r="I41" t="n">
-        <v>4.972</v>
+        <v>4.985</v>
       </c>
       <c r="J41" t="n">
         <v>5.323</v>
       </c>
       <c r="K41" t="n">
-        <v>5.624</v>
+        <v>5.636</v>
       </c>
       <c r="L41" t="n">
-        <v>5.808</v>
+        <v>5.804</v>
       </c>
       <c r="M41" t="n">
-        <v>6.097</v>
+        <v>6.095</v>
       </c>
       <c r="N41" t="n">
-        <v>6.402</v>
+        <v>6.411</v>
       </c>
       <c r="O41" t="n">
-        <v>6.922</v>
+        <v>6.924</v>
       </c>
       <c r="P41" t="n">
-        <v>7.132</v>
+        <v>7.137</v>
       </c>
       <c r="Q41" t="n">
-        <v>7.948</v>
+        <v>7.958</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,40 +3472,40 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.808</v>
+        <v>3.814</v>
       </c>
       <c r="G42" t="n">
-        <v>4.312</v>
+        <v>4.321</v>
       </c>
       <c r="H42" t="n">
-        <v>4.589</v>
+        <v>4.601</v>
       </c>
       <c r="I42" t="n">
-        <v>4.657</v>
+        <v>4.671</v>
       </c>
       <c r="J42" t="n">
         <v>4.971</v>
       </c>
       <c r="K42" t="n">
-        <v>5.237</v>
+        <v>5.249</v>
       </c>
       <c r="L42" t="n">
-        <v>5.368</v>
+        <v>5.365</v>
       </c>
       <c r="M42" t="n">
-        <v>5.604</v>
+        <v>5.601</v>
       </c>
       <c r="N42" t="n">
-        <v>5.887</v>
+        <v>5.896</v>
       </c>
       <c r="O42" t="n">
-        <v>6.299</v>
+        <v>6.301</v>
       </c>
       <c r="P42" t="n">
-        <v>6.575</v>
+        <v>6.579</v>
       </c>
       <c r="Q42" t="n">
-        <v>7.414</v>
+        <v>7.423</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,40 +3545,40 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.5</v>
+        <v>3.505</v>
       </c>
       <c r="G43" t="n">
-        <v>3.956</v>
+        <v>3.964</v>
       </c>
       <c r="H43" t="n">
-        <v>4.163</v>
+        <v>4.176</v>
       </c>
       <c r="I43" t="n">
-        <v>4.194</v>
+        <v>4.208</v>
       </c>
       <c r="J43" t="n">
-        <v>4.402</v>
+        <v>4.4</v>
       </c>
       <c r="K43" t="n">
-        <v>4.582</v>
+        <v>4.591</v>
       </c>
       <c r="L43" t="n">
-        <v>4.648</v>
+        <v>4.644</v>
       </c>
       <c r="M43" t="n">
-        <v>4.734</v>
+        <v>4.733</v>
       </c>
       <c r="N43" t="n">
-        <v>4.777</v>
+        <v>4.787</v>
       </c>
       <c r="O43" t="n">
-        <v>4.907</v>
+        <v>4.909</v>
       </c>
       <c r="P43" t="n">
-        <v>5.053</v>
+        <v>5.058</v>
       </c>
       <c r="Q43" t="n">
-        <v>5.776</v>
+        <v>5.786</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,40 +3618,40 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>3.344</v>
+        <v>3.35</v>
       </c>
       <c r="G44" t="n">
-        <v>3.779</v>
+        <v>3.787</v>
       </c>
       <c r="H44" t="n">
-        <v>3.981</v>
+        <v>3.993</v>
       </c>
       <c r="I44" t="n">
-        <v>4.017</v>
+        <v>4.03</v>
       </c>
       <c r="J44" t="n">
-        <v>4.249</v>
+        <v>4.247</v>
       </c>
       <c r="K44" t="n">
-        <v>4.425</v>
+        <v>4.434</v>
       </c>
       <c r="L44" t="n">
-        <v>4.488</v>
+        <v>4.483</v>
       </c>
       <c r="M44" t="n">
-        <v>4.55</v>
+        <v>4.546</v>
       </c>
       <c r="N44" t="n">
-        <v>4.59</v>
+        <v>4.6</v>
       </c>
       <c r="O44" t="n">
-        <v>4.701</v>
+        <v>4.704</v>
       </c>
       <c r="P44" t="n">
-        <v>4.816</v>
+        <v>4.821</v>
       </c>
       <c r="Q44" t="n">
-        <v>5.145</v>
+        <v>5.155</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
update: 2026-09-09 ~ 2026-09-09
</commit_message>
<xml_diff>
--- a/crawler/kofia.xlsx
+++ b/crawler/kofia.xlsx
@@ -529,7 +529,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -552,37 +552,37 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>3.661</v>
+        <v>3.669</v>
       </c>
       <c r="G2" t="n">
-        <v>4.143</v>
+        <v>4.151</v>
       </c>
       <c r="H2" t="n">
-        <v>4.404</v>
+        <v>4.412</v>
       </c>
       <c r="I2" t="n">
-        <v>4.41</v>
+        <v>4.417</v>
       </c>
       <c r="J2" t="n">
-        <v>4.596</v>
+        <v>4.598</v>
       </c>
       <c r="K2" t="n">
         <v>4.927</v>
       </c>
       <c r="L2" t="n">
-        <v>5.131</v>
+        <v>5.148</v>
       </c>
       <c r="M2" t="n">
-        <v>5.389</v>
+        <v>5.398</v>
       </c>
       <c r="N2" t="n">
-        <v>5.671</v>
+        <v>5.687</v>
       </c>
       <c r="O2" t="n">
-        <v>5.947</v>
+        <v>5.954</v>
       </c>
       <c r="P2" t="n">
-        <v>6.161</v>
+        <v>6.162</v>
       </c>
       <c r="Q2" t="n">
         <v>6.857</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -625,37 +625,37 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>4.679</v>
+        <v>4.687</v>
       </c>
       <c r="G3" t="n">
-        <v>5.343</v>
+        <v>5.351</v>
       </c>
       <c r="H3" t="n">
-        <v>5.637</v>
+        <v>5.645</v>
       </c>
       <c r="I3" t="n">
-        <v>5.638</v>
+        <v>5.645</v>
       </c>
       <c r="J3" t="n">
-        <v>5.84</v>
+        <v>5.842</v>
       </c>
       <c r="K3" t="n">
-        <v>6.243</v>
+        <v>6.244</v>
       </c>
       <c r="L3" t="n">
-        <v>6.518</v>
+        <v>6.534</v>
       </c>
       <c r="M3" t="n">
-        <v>6.804</v>
+        <v>6.812</v>
       </c>
       <c r="N3" t="n">
-        <v>7.031</v>
+        <v>7.047</v>
       </c>
       <c r="O3" t="n">
-        <v>7.257</v>
+        <v>7.264</v>
       </c>
       <c r="P3" t="n">
-        <v>7.338</v>
+        <v>7.34</v>
       </c>
       <c r="Q3" t="n">
         <v>7.923</v>
@@ -675,7 +675,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -698,37 +698,37 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>4.171</v>
+        <v>4.179</v>
       </c>
       <c r="G4" t="n">
-        <v>4.722</v>
+        <v>4.73</v>
       </c>
       <c r="H4" t="n">
-        <v>5.044</v>
+        <v>5.052</v>
       </c>
       <c r="I4" t="n">
-        <v>5.079</v>
+        <v>5.087</v>
       </c>
       <c r="J4" t="n">
-        <v>5.281</v>
+        <v>5.283</v>
       </c>
       <c r="K4" t="n">
-        <v>5.679</v>
+        <v>5.68</v>
       </c>
       <c r="L4" t="n">
-        <v>5.884</v>
+        <v>5.9</v>
       </c>
       <c r="M4" t="n">
-        <v>6.162</v>
+        <v>6.17</v>
       </c>
       <c r="N4" t="n">
-        <v>6.358</v>
+        <v>6.375</v>
       </c>
       <c r="O4" t="n">
-        <v>6.609</v>
+        <v>6.615</v>
       </c>
       <c r="P4" t="n">
-        <v>6.69</v>
+        <v>6.692</v>
       </c>
       <c r="Q4" t="n">
         <v>7.278</v>
@@ -748,7 +748,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -771,37 +771,37 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>3.354</v>
+        <v>3.362</v>
       </c>
       <c r="G5" t="n">
-        <v>3.701</v>
+        <v>3.709</v>
       </c>
       <c r="H5" t="n">
-        <v>3.935</v>
+        <v>3.943</v>
       </c>
       <c r="I5" t="n">
-        <v>3.97</v>
+        <v>3.979</v>
       </c>
       <c r="J5" t="n">
-        <v>4.17</v>
+        <v>4.172</v>
       </c>
       <c r="K5" t="n">
-        <v>4.326</v>
+        <v>4.327</v>
       </c>
       <c r="L5" t="n">
-        <v>4.375</v>
+        <v>4.392</v>
       </c>
       <c r="M5" t="n">
-        <v>4.453</v>
+        <v>4.462</v>
       </c>
       <c r="N5" t="n">
-        <v>4.491</v>
+        <v>4.508</v>
       </c>
       <c r="O5" t="n">
-        <v>4.547</v>
+        <v>4.554</v>
       </c>
       <c r="P5" t="n">
-        <v>4.828</v>
+        <v>4.83</v>
       </c>
       <c r="Q5" t="n">
         <v>5.763</v>
@@ -821,7 +821,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -844,37 +844,37 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>3.394</v>
+        <v>3.402</v>
       </c>
       <c r="G6" t="n">
-        <v>3.754</v>
+        <v>3.762</v>
       </c>
       <c r="H6" t="n">
-        <v>4.005</v>
+        <v>4.013</v>
       </c>
       <c r="I6" t="n">
-        <v>4.051</v>
+        <v>4.06</v>
       </c>
       <c r="J6" t="n">
-        <v>4.262</v>
+        <v>4.264</v>
       </c>
       <c r="K6" t="n">
-        <v>4.443</v>
+        <v>4.444</v>
       </c>
       <c r="L6" t="n">
-        <v>4.497</v>
+        <v>4.514</v>
       </c>
       <c r="M6" t="n">
-        <v>4.604</v>
+        <v>4.613</v>
       </c>
       <c r="N6" t="n">
-        <v>4.656</v>
+        <v>4.673</v>
       </c>
       <c r="O6" t="n">
-        <v>4.814</v>
+        <v>4.821</v>
       </c>
       <c r="P6" t="n">
-        <v>5.262</v>
+        <v>5.264</v>
       </c>
       <c r="Q6" t="n">
         <v>6.161</v>
@@ -894,7 +894,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -917,37 +917,37 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>3.373</v>
+        <v>3.381</v>
       </c>
       <c r="G7" t="n">
-        <v>3.717</v>
+        <v>3.725</v>
       </c>
       <c r="H7" t="n">
-        <v>3.951</v>
+        <v>3.959</v>
       </c>
       <c r="I7" t="n">
-        <v>3.988</v>
+        <v>3.996</v>
       </c>
       <c r="J7" t="n">
-        <v>4.195</v>
+        <v>4.197</v>
       </c>
       <c r="K7" t="n">
         <v>4.354</v>
       </c>
       <c r="L7" t="n">
-        <v>4.402</v>
+        <v>4.418</v>
       </c>
       <c r="M7" t="n">
-        <v>4.511</v>
+        <v>4.52</v>
       </c>
       <c r="N7" t="n">
-        <v>4.553</v>
+        <v>4.57</v>
       </c>
       <c r="O7" t="n">
-        <v>4.713</v>
+        <v>4.72</v>
       </c>
       <c r="P7" t="n">
-        <v>5.046</v>
+        <v>5.047</v>
       </c>
       <c r="Q7" t="n">
         <v>5.929</v>
@@ -967,7 +967,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -990,37 +990,37 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>5.793</v>
+        <v>5.801</v>
       </c>
       <c r="G8" t="n">
-        <v>6.644</v>
+        <v>6.652</v>
       </c>
       <c r="H8" t="n">
-        <v>7.092</v>
+        <v>7.1</v>
       </c>
       <c r="I8" t="n">
-        <v>7.165</v>
+        <v>7.173</v>
       </c>
       <c r="J8" t="n">
-        <v>7.438</v>
+        <v>7.44</v>
       </c>
       <c r="K8" t="n">
         <v>8.118</v>
       </c>
       <c r="L8" t="n">
-        <v>8.475</v>
+        <v>8.491</v>
       </c>
       <c r="M8" t="n">
-        <v>8.795</v>
+        <v>8.803000000000001</v>
       </c>
       <c r="N8" t="n">
-        <v>8.954000000000001</v>
+        <v>8.971</v>
       </c>
       <c r="O8" t="n">
-        <v>9.266999999999999</v>
+        <v>9.273999999999999</v>
       </c>
       <c r="P8" t="n">
-        <v>9.452999999999999</v>
+        <v>9.455</v>
       </c>
       <c r="Q8" t="n">
         <v>10.24</v>
@@ -1040,7 +1040,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1063,57 +1063,57 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>3.029</v>
+        <v>3.042</v>
       </c>
       <c r="G9" t="n">
-        <v>3.16</v>
+        <v>3.182</v>
       </c>
       <c r="H9" t="n">
-        <v>3.384</v>
+        <v>3.4</v>
       </c>
       <c r="I9" t="n">
-        <v>3.496</v>
+        <v>3.51</v>
       </c>
       <c r="J9" t="n">
-        <v>3.627</v>
+        <v>3.645</v>
       </c>
       <c r="K9" t="n">
-        <v>3.715</v>
+        <v>3.726</v>
       </c>
       <c r="L9" t="n">
-        <v>3.808</v>
+        <v>3.829</v>
       </c>
       <c r="M9" t="n">
-        <v>3.897</v>
+        <v>3.91</v>
       </c>
       <c r="N9" t="n">
-        <v>4.002</v>
+        <v>4.019</v>
       </c>
       <c r="O9" t="n">
-        <v>4.127</v>
+        <v>4.133</v>
       </c>
       <c r="P9" t="n">
-        <v>4.269</v>
+        <v>4.27</v>
       </c>
       <c r="Q9" t="n">
         <v>4.4</v>
       </c>
       <c r="R9" t="n">
-        <v>4.494</v>
+        <v>4.484</v>
       </c>
       <c r="S9" t="n">
-        <v>4.561</v>
+        <v>4.552</v>
       </c>
       <c r="T9" t="n">
-        <v>4.64</v>
+        <v>4.642</v>
       </c>
       <c r="U9" t="n">
-        <v>4.6</v>
+        <v>4.602</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1136,34 +1136,34 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>3.118</v>
+        <v>3.13</v>
       </c>
       <c r="G10" t="n">
-        <v>3.26</v>
+        <v>3.28</v>
       </c>
       <c r="H10" t="n">
-        <v>3.455</v>
+        <v>3.471</v>
       </c>
       <c r="I10" t="n">
-        <v>3.562</v>
+        <v>3.576</v>
       </c>
       <c r="J10" t="n">
-        <v>3.696</v>
+        <v>3.712</v>
       </c>
       <c r="K10" t="n">
-        <v>3.768</v>
+        <v>3.789</v>
       </c>
       <c r="L10" t="n">
-        <v>3.856</v>
+        <v>3.882</v>
       </c>
       <c r="M10" t="n">
-        <v>3.958</v>
+        <v>3.969</v>
       </c>
       <c r="N10" t="n">
-        <v>4.048</v>
+        <v>4.07</v>
       </c>
       <c r="O10" t="n">
-        <v>4.385</v>
+        <v>4.398</v>
       </c>
       <c r="P10" t="n">
         <v>0</v>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1209,37 +1209,37 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2.928</v>
+        <v>2.944</v>
       </c>
       <c r="G11" t="n">
-        <v>3.056</v>
+        <v>3.076</v>
       </c>
       <c r="H11" t="n">
-        <v>3.26</v>
+        <v>3.278</v>
       </c>
       <c r="I11" t="n">
-        <v>3.35</v>
+        <v>3.364</v>
       </c>
       <c r="J11" t="n">
-        <v>3.485</v>
+        <v>3.501</v>
       </c>
       <c r="K11" t="n">
-        <v>3.55</v>
+        <v>3.574</v>
       </c>
       <c r="L11" t="n">
-        <v>3.644</v>
+        <v>3.67</v>
       </c>
       <c r="M11" t="n">
-        <v>3.767</v>
+        <v>3.779</v>
       </c>
       <c r="N11" t="n">
-        <v>3.845</v>
+        <v>3.866</v>
       </c>
       <c r="O11" t="n">
-        <v>4.157</v>
+        <v>4.17</v>
       </c>
       <c r="P11" t="n">
-        <v>4.215</v>
+        <v>4.217</v>
       </c>
       <c r="Q11" t="n">
         <v>4.598</v>
@@ -1259,7 +1259,7 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1282,46 +1282,46 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3.682</v>
+        <v>3.688</v>
       </c>
       <c r="G12" t="n">
-        <v>4.041</v>
+        <v>4.048</v>
       </c>
       <c r="H12" t="n">
-        <v>4.327</v>
+        <v>4.333</v>
       </c>
       <c r="I12" t="n">
-        <v>4.406</v>
+        <v>4.413</v>
       </c>
       <c r="J12" t="n">
-        <v>4.61</v>
+        <v>4.617</v>
       </c>
       <c r="K12" t="n">
-        <v>4.732</v>
+        <v>4.738</v>
       </c>
       <c r="L12" t="n">
-        <v>4.803</v>
+        <v>4.824</v>
       </c>
       <c r="M12" t="n">
-        <v>4.916</v>
+        <v>4.929</v>
       </c>
       <c r="N12" t="n">
-        <v>4.99</v>
+        <v>5.007</v>
       </c>
       <c r="O12" t="n">
-        <v>5.171</v>
+        <v>5.178</v>
       </c>
       <c r="P12" t="n">
-        <v>5.321</v>
+        <v>5.323</v>
       </c>
       <c r="Q12" t="n">
         <v>5.714</v>
       </c>
       <c r="R12" t="n">
-        <v>5.986</v>
+        <v>5.976</v>
       </c>
       <c r="S12" t="n">
-        <v>6.261</v>
+        <v>6.251</v>
       </c>
       <c r="T12" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1355,46 +1355,46 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>3.435</v>
+        <v>3.442</v>
       </c>
       <c r="G13" t="n">
-        <v>3.732</v>
+        <v>3.739</v>
       </c>
       <c r="H13" t="n">
-        <v>3.994</v>
+        <v>4</v>
       </c>
       <c r="I13" t="n">
-        <v>4.054</v>
+        <v>4.061</v>
       </c>
       <c r="J13" t="n">
-        <v>4.248</v>
+        <v>4.255</v>
       </c>
       <c r="K13" t="n">
-        <v>4.365</v>
+        <v>4.372</v>
       </c>
       <c r="L13" t="n">
-        <v>4.443</v>
+        <v>4.465</v>
       </c>
       <c r="M13" t="n">
-        <v>4.545</v>
+        <v>4.557</v>
       </c>
       <c r="N13" t="n">
-        <v>4.618</v>
+        <v>4.635</v>
       </c>
       <c r="O13" t="n">
-        <v>4.798</v>
+        <v>4.804</v>
       </c>
       <c r="P13" t="n">
-        <v>4.913</v>
+        <v>4.914</v>
       </c>
       <c r="Q13" t="n">
         <v>5.237</v>
       </c>
       <c r="R13" t="n">
-        <v>5.536</v>
+        <v>5.527</v>
       </c>
       <c r="S13" t="n">
-        <v>5.829</v>
+        <v>5.819</v>
       </c>
       <c r="T13" t="n">
         <v>0</v>
@@ -1405,7 +1405,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1428,46 +1428,46 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>3.252</v>
+        <v>3.259</v>
       </c>
       <c r="G14" t="n">
-        <v>3.531</v>
+        <v>3.538</v>
       </c>
       <c r="H14" t="n">
-        <v>3.793</v>
+        <v>3.799</v>
       </c>
       <c r="I14" t="n">
-        <v>3.839</v>
+        <v>3.845</v>
       </c>
       <c r="J14" t="n">
-        <v>3.99</v>
+        <v>3.997</v>
       </c>
       <c r="K14" t="n">
-        <v>4.054</v>
+        <v>4.061</v>
       </c>
       <c r="L14" t="n">
-        <v>4.116</v>
+        <v>4.137</v>
       </c>
       <c r="M14" t="n">
-        <v>4.231</v>
+        <v>4.244</v>
       </c>
       <c r="N14" t="n">
-        <v>4.297</v>
+        <v>4.314</v>
       </c>
       <c r="O14" t="n">
-        <v>4.456</v>
+        <v>4.463</v>
       </c>
       <c r="P14" t="n">
-        <v>4.552</v>
+        <v>4.554</v>
       </c>
       <c r="Q14" t="n">
         <v>4.826</v>
       </c>
       <c r="R14" t="n">
-        <v>5.051</v>
+        <v>5.041</v>
       </c>
       <c r="S14" t="n">
-        <v>5.281</v>
+        <v>5.272</v>
       </c>
       <c r="T14" t="n">
         <v>0</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1501,46 +1501,46 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>3.225</v>
+        <v>3.231</v>
       </c>
       <c r="G15" t="n">
-        <v>3.501</v>
+        <v>3.508</v>
       </c>
       <c r="H15" t="n">
-        <v>3.757</v>
+        <v>3.763</v>
       </c>
       <c r="I15" t="n">
-        <v>3.772</v>
+        <v>3.779</v>
       </c>
       <c r="J15" t="n">
-        <v>3.926</v>
+        <v>3.933</v>
       </c>
       <c r="K15" t="n">
-        <v>4.001</v>
+        <v>4.008</v>
       </c>
       <c r="L15" t="n">
-        <v>4.045</v>
+        <v>4.067</v>
       </c>
       <c r="M15" t="n">
-        <v>4.141</v>
+        <v>4.153</v>
       </c>
       <c r="N15" t="n">
-        <v>4.201</v>
+        <v>4.218</v>
       </c>
       <c r="O15" t="n">
-        <v>4.404</v>
+        <v>4.411</v>
       </c>
       <c r="P15" t="n">
-        <v>4.453</v>
+        <v>4.454</v>
       </c>
       <c r="Q15" t="n">
         <v>4.727</v>
       </c>
       <c r="R15" t="n">
-        <v>4.944</v>
+        <v>4.935</v>
       </c>
       <c r="S15" t="n">
-        <v>5.171</v>
+        <v>5.162</v>
       </c>
       <c r="T15" t="n">
         <v>0</v>
@@ -1551,7 +1551,7 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1574,46 +1574,46 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>3.225</v>
+        <v>3.231</v>
       </c>
       <c r="G16" t="n">
-        <v>3.501</v>
+        <v>3.508</v>
       </c>
       <c r="H16" t="n">
-        <v>3.757</v>
+        <v>3.763</v>
       </c>
       <c r="I16" t="n">
-        <v>3.772</v>
+        <v>3.779</v>
       </c>
       <c r="J16" t="n">
-        <v>3.926</v>
+        <v>3.933</v>
       </c>
       <c r="K16" t="n">
-        <v>4.001</v>
+        <v>4.008</v>
       </c>
       <c r="L16" t="n">
-        <v>4.045</v>
+        <v>4.067</v>
       </c>
       <c r="M16" t="n">
-        <v>4.141</v>
+        <v>4.153</v>
       </c>
       <c r="N16" t="n">
-        <v>4.204</v>
+        <v>4.221</v>
       </c>
       <c r="O16" t="n">
-        <v>4.409</v>
+        <v>4.416</v>
       </c>
       <c r="P16" t="n">
-        <v>4.476</v>
+        <v>4.478</v>
       </c>
       <c r="Q16" t="n">
         <v>4.754</v>
       </c>
       <c r="R16" t="n">
-        <v>4.972</v>
+        <v>4.963</v>
       </c>
       <c r="S16" t="n">
-        <v>5.202</v>
+        <v>5.193</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -1624,7 +1624,7 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1647,37 +1647,37 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>3.164</v>
+        <v>3.175</v>
       </c>
       <c r="G17" t="n">
-        <v>3.322</v>
+        <v>3.342</v>
       </c>
       <c r="H17" t="n">
-        <v>3.493</v>
+        <v>3.508</v>
       </c>
       <c r="I17" t="n">
-        <v>3.607</v>
+        <v>3.621</v>
       </c>
       <c r="J17" t="n">
-        <v>3.767</v>
+        <v>3.782</v>
       </c>
       <c r="K17" t="n">
-        <v>3.863</v>
+        <v>3.878</v>
       </c>
       <c r="L17" t="n">
-        <v>3.946</v>
+        <v>3.97</v>
       </c>
       <c r="M17" t="n">
-        <v>4.094</v>
+        <v>4.108</v>
       </c>
       <c r="N17" t="n">
-        <v>4.167</v>
+        <v>4.189</v>
       </c>
       <c r="O17" t="n">
-        <v>4.41</v>
+        <v>4.422</v>
       </c>
       <c r="P17" t="n">
-        <v>4.495</v>
+        <v>4.497</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1720,34 +1720,34 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>3.164</v>
+        <v>3.175</v>
       </c>
       <c r="G18" t="n">
-        <v>3.322</v>
+        <v>3.342</v>
       </c>
       <c r="H18" t="n">
-        <v>3.493</v>
+        <v>3.508</v>
       </c>
       <c r="I18" t="n">
-        <v>3.607</v>
+        <v>3.62</v>
       </c>
       <c r="J18" t="n">
-        <v>3.767</v>
+        <v>3.782</v>
       </c>
       <c r="K18" t="n">
-        <v>3.864</v>
+        <v>3.879</v>
       </c>
       <c r="L18" t="n">
-        <v>3.946</v>
+        <v>3.97</v>
       </c>
       <c r="M18" t="n">
-        <v>4.094</v>
+        <v>4.107</v>
       </c>
       <c r="N18" t="n">
-        <v>4.167</v>
+        <v>4.189</v>
       </c>
       <c r="O18" t="n">
-        <v>4.41</v>
+        <v>4.422</v>
       </c>
       <c r="P18" t="n">
         <v>0</v>
@@ -1770,7 +1770,7 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1793,46 +1793,46 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>3.241</v>
+        <v>3.248</v>
       </c>
       <c r="G19" t="n">
-        <v>3.525</v>
+        <v>3.532</v>
       </c>
       <c r="H19" t="n">
-        <v>3.781</v>
+        <v>3.787</v>
       </c>
       <c r="I19" t="n">
-        <v>3.823</v>
+        <v>3.83</v>
       </c>
       <c r="J19" t="n">
-        <v>3.989</v>
+        <v>3.996</v>
       </c>
       <c r="K19" t="n">
-        <v>4.064</v>
+        <v>4.071</v>
       </c>
       <c r="L19" t="n">
-        <v>4.122</v>
+        <v>4.144</v>
       </c>
       <c r="M19" t="n">
-        <v>4.229</v>
+        <v>4.242</v>
       </c>
       <c r="N19" t="n">
-        <v>4.29</v>
+        <v>4.307</v>
       </c>
       <c r="O19" t="n">
-        <v>4.445</v>
+        <v>4.453</v>
       </c>
       <c r="P19" t="n">
-        <v>4.511</v>
+        <v>4.513</v>
       </c>
       <c r="Q19" t="n">
         <v>4.765</v>
       </c>
       <c r="R19" t="n">
-        <v>4.991</v>
+        <v>4.982</v>
       </c>
       <c r="S19" t="n">
-        <v>5.215</v>
+        <v>5.206</v>
       </c>
       <c r="T19" t="n">
         <v>0</v>
@@ -1843,7 +1843,7 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1866,28 +1866,28 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>3.03</v>
+        <v>3.034</v>
       </c>
       <c r="G20" t="n">
-        <v>3.059</v>
+        <v>3.063</v>
       </c>
       <c r="H20" t="n">
-        <v>3.175</v>
+        <v>3.18</v>
       </c>
       <c r="I20" t="n">
-        <v>3.303</v>
+        <v>3.307</v>
       </c>
       <c r="J20" t="n">
-        <v>3.682</v>
+        <v>3.688</v>
       </c>
       <c r="K20" t="n">
-        <v>3.8</v>
+        <v>3.805</v>
       </c>
       <c r="L20" t="n">
-        <v>3.802</v>
+        <v>3.811</v>
       </c>
       <c r="M20" t="n">
-        <v>3.894</v>
+        <v>3.905</v>
       </c>
       <c r="N20" t="n">
         <v>0</v>
@@ -1916,7 +1916,7 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1939,46 +1939,46 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>3.316</v>
+        <v>3.323</v>
       </c>
       <c r="G21" t="n">
-        <v>3.621</v>
+        <v>3.626</v>
       </c>
       <c r="H21" t="n">
-        <v>3.901</v>
+        <v>3.907</v>
       </c>
       <c r="I21" t="n">
-        <v>3.961</v>
+        <v>3.969</v>
       </c>
       <c r="J21" t="n">
-        <v>4.158</v>
+        <v>4.165</v>
       </c>
       <c r="K21" t="n">
-        <v>4.284</v>
+        <v>4.291</v>
       </c>
       <c r="L21" t="n">
-        <v>4.353</v>
+        <v>4.375</v>
       </c>
       <c r="M21" t="n">
-        <v>4.458</v>
+        <v>4.47</v>
       </c>
       <c r="N21" t="n">
-        <v>4.533</v>
+        <v>4.548</v>
       </c>
       <c r="O21" t="n">
-        <v>4.681</v>
+        <v>4.692</v>
       </c>
       <c r="P21" t="n">
-        <v>4.755</v>
+        <v>4.757</v>
       </c>
       <c r="Q21" t="n">
         <v>4.917</v>
       </c>
       <c r="R21" t="n">
-        <v>5.042</v>
+        <v>5.032</v>
       </c>
       <c r="S21" t="n">
-        <v>5.169</v>
+        <v>5.159</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -1989,7 +1989,7 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -2012,46 +2012,46 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>3.26</v>
+        <v>3.267</v>
       </c>
       <c r="G22" t="n">
-        <v>3.567</v>
+        <v>3.572</v>
       </c>
       <c r="H22" t="n">
-        <v>3.833</v>
+        <v>3.839</v>
       </c>
       <c r="I22" t="n">
-        <v>3.878</v>
+        <v>3.886</v>
       </c>
       <c r="J22" t="n">
-        <v>4.046</v>
+        <v>4.054</v>
       </c>
       <c r="K22" t="n">
-        <v>4.163</v>
+        <v>4.17</v>
       </c>
       <c r="L22" t="n">
-        <v>4.225</v>
+        <v>4.247</v>
       </c>
       <c r="M22" t="n">
-        <v>4.33</v>
+        <v>4.342</v>
       </c>
       <c r="N22" t="n">
-        <v>4.409</v>
+        <v>4.425</v>
       </c>
       <c r="O22" t="n">
-        <v>4.551</v>
+        <v>4.562</v>
       </c>
       <c r="P22" t="n">
-        <v>4.618</v>
+        <v>4.62</v>
       </c>
       <c r="Q22" t="n">
         <v>4.775</v>
       </c>
       <c r="R22" t="n">
-        <v>4.89</v>
+        <v>4.881</v>
       </c>
       <c r="S22" t="n">
-        <v>5.014</v>
+        <v>5.005</v>
       </c>
       <c r="T22" t="n">
         <v>0</v>
@@ -2062,7 +2062,7 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -2085,49 +2085,49 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>3.21</v>
+        <v>3.217</v>
       </c>
       <c r="G23" t="n">
-        <v>3.517</v>
+        <v>3.523</v>
       </c>
       <c r="H23" t="n">
-        <v>3.772</v>
+        <v>3.778</v>
       </c>
       <c r="I23" t="n">
-        <v>3.813</v>
+        <v>3.821</v>
       </c>
       <c r="J23" t="n">
-        <v>3.963</v>
+        <v>3.97</v>
       </c>
       <c r="K23" t="n">
-        <v>4.054</v>
+        <v>4.061</v>
       </c>
       <c r="L23" t="n">
-        <v>4.118</v>
+        <v>4.14</v>
       </c>
       <c r="M23" t="n">
-        <v>4.22</v>
+        <v>4.232</v>
       </c>
       <c r="N23" t="n">
-        <v>4.296</v>
+        <v>4.311</v>
       </c>
       <c r="O23" t="n">
-        <v>4.426</v>
+        <v>4.437</v>
       </c>
       <c r="P23" t="n">
-        <v>4.48</v>
+        <v>4.482</v>
       </c>
       <c r="Q23" t="n">
         <v>4.578</v>
       </c>
       <c r="R23" t="n">
-        <v>4.676</v>
+        <v>4.666</v>
       </c>
       <c r="S23" t="n">
-        <v>4.77</v>
+        <v>4.761</v>
       </c>
       <c r="T23" t="n">
-        <v>4.855</v>
+        <v>4.857</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2135,7 +2135,7 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -2158,46 +2158,46 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>3.161</v>
+        <v>3.168</v>
       </c>
       <c r="G24" t="n">
-        <v>3.431</v>
+        <v>3.437</v>
       </c>
       <c r="H24" t="n">
-        <v>3.659</v>
+        <v>3.665</v>
       </c>
       <c r="I24" t="n">
-        <v>3.723</v>
+        <v>3.731</v>
       </c>
       <c r="J24" t="n">
-        <v>3.857</v>
+        <v>3.864</v>
       </c>
       <c r="K24" t="n">
-        <v>3.948</v>
+        <v>3.956</v>
       </c>
       <c r="L24" t="n">
-        <v>4.001</v>
+        <v>4.023</v>
       </c>
       <c r="M24" t="n">
-        <v>4.077</v>
+        <v>4.089</v>
       </c>
       <c r="N24" t="n">
-        <v>4.165</v>
+        <v>4.181</v>
       </c>
       <c r="O24" t="n">
-        <v>4.383</v>
+        <v>4.397</v>
       </c>
       <c r="P24" t="n">
-        <v>4.421</v>
+        <v>4.423</v>
       </c>
       <c r="Q24" t="n">
         <v>4.507</v>
       </c>
       <c r="R24" t="n">
-        <v>4.598</v>
+        <v>4.589</v>
       </c>
       <c r="S24" t="n">
-        <v>4.685</v>
+        <v>4.676</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -2208,7 +2208,7 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -2231,49 +2231,49 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>3.203</v>
+        <v>3.211</v>
       </c>
       <c r="G25" t="n">
-        <v>3.518</v>
+        <v>3.524</v>
       </c>
       <c r="H25" t="n">
-        <v>3.776</v>
+        <v>3.782</v>
       </c>
       <c r="I25" t="n">
-        <v>3.824</v>
+        <v>3.832</v>
       </c>
       <c r="J25" t="n">
-        <v>3.985</v>
+        <v>3.992</v>
       </c>
       <c r="K25" t="n">
-        <v>4.091</v>
+        <v>4.098</v>
       </c>
       <c r="L25" t="n">
-        <v>4.15</v>
+        <v>4.172</v>
       </c>
       <c r="M25" t="n">
-        <v>4.252</v>
+        <v>4.264</v>
       </c>
       <c r="N25" t="n">
-        <v>4.323</v>
+        <v>4.339</v>
       </c>
       <c r="O25" t="n">
-        <v>4.456</v>
+        <v>4.466</v>
       </c>
       <c r="P25" t="n">
-        <v>4.502</v>
+        <v>4.504</v>
       </c>
       <c r="Q25" t="n">
         <v>4.61</v>
       </c>
       <c r="R25" t="n">
-        <v>4.7</v>
+        <v>4.691</v>
       </c>
       <c r="S25" t="n">
-        <v>4.794</v>
+        <v>4.784</v>
       </c>
       <c r="T25" t="n">
-        <v>4.872</v>
+        <v>4.874</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2281,7 +2281,7 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -2304,34 +2304,34 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>3.455</v>
+        <v>3.465</v>
       </c>
       <c r="G26" t="n">
-        <v>3.931</v>
+        <v>3.94</v>
       </c>
       <c r="H26" t="n">
-        <v>4.222</v>
+        <v>4.23</v>
       </c>
       <c r="I26" t="n">
-        <v>4.267</v>
+        <v>4.277</v>
       </c>
       <c r="J26" t="n">
-        <v>4.596</v>
+        <v>4.599</v>
       </c>
       <c r="K26" t="n">
-        <v>4.917</v>
+        <v>4.921</v>
       </c>
       <c r="L26" t="n">
-        <v>5.019</v>
+        <v>5.039</v>
       </c>
       <c r="M26" t="n">
-        <v>5.18</v>
+        <v>5.191</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>5.49</v>
+        <v>5.497</v>
       </c>
       <c r="P26" t="n">
         <v>0</v>
@@ -2354,7 +2354,7 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -2377,34 +2377,34 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>3.304</v>
+        <v>3.313</v>
       </c>
       <c r="G27" t="n">
-        <v>3.635</v>
+        <v>3.644</v>
       </c>
       <c r="H27" t="n">
-        <v>3.88</v>
+        <v>3.887</v>
       </c>
       <c r="I27" t="n">
-        <v>3.923</v>
+        <v>3.932</v>
       </c>
       <c r="J27" t="n">
-        <v>4.104</v>
+        <v>4.11</v>
       </c>
       <c r="K27" t="n">
-        <v>4.233</v>
+        <v>4.238</v>
       </c>
       <c r="L27" t="n">
-        <v>4.293</v>
+        <v>4.313</v>
       </c>
       <c r="M27" t="n">
-        <v>4.394</v>
+        <v>4.407</v>
       </c>
       <c r="N27" t="n">
         <v>0</v>
       </c>
       <c r="O27" t="n">
-        <v>4.588</v>
+        <v>4.595</v>
       </c>
       <c r="P27" t="n">
         <v>0</v>
@@ -2427,7 +2427,7 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -2450,34 +2450,34 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>3.413</v>
+        <v>3.421</v>
       </c>
       <c r="G28" t="n">
-        <v>3.758</v>
+        <v>3.767</v>
       </c>
       <c r="H28" t="n">
-        <v>4.014</v>
+        <v>4.021</v>
       </c>
       <c r="I28" t="n">
-        <v>4.063</v>
+        <v>4.071</v>
       </c>
       <c r="J28" t="n">
-        <v>4.278</v>
+        <v>4.284</v>
       </c>
       <c r="K28" t="n">
-        <v>4.426</v>
+        <v>4.431</v>
       </c>
       <c r="L28" t="n">
-        <v>4.497</v>
+        <v>4.517</v>
       </c>
       <c r="M28" t="n">
-        <v>4.606</v>
+        <v>4.619</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
       </c>
       <c r="O28" t="n">
-        <v>4.88</v>
+        <v>4.887</v>
       </c>
       <c r="P28" t="n">
         <v>0</v>
@@ -2500,7 +2500,7 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -2523,34 +2523,34 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>3.25</v>
+        <v>3.259</v>
       </c>
       <c r="G29" t="n">
-        <v>3.576</v>
+        <v>3.585</v>
       </c>
       <c r="H29" t="n">
-        <v>3.813</v>
+        <v>3.82</v>
       </c>
       <c r="I29" t="n">
-        <v>3.839</v>
+        <v>3.847</v>
       </c>
       <c r="J29" t="n">
-        <v>4.013</v>
+        <v>4.018</v>
       </c>
       <c r="K29" t="n">
-        <v>4.126</v>
+        <v>4.131</v>
       </c>
       <c r="L29" t="n">
-        <v>4.174</v>
+        <v>4.194</v>
       </c>
       <c r="M29" t="n">
-        <v>4.256</v>
+        <v>4.268</v>
       </c>
       <c r="N29" t="n">
         <v>0</v>
       </c>
       <c r="O29" t="n">
-        <v>4.461</v>
+        <v>4.468</v>
       </c>
       <c r="P29" t="n">
         <v>0</v>
@@ -2573,7 +2573,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -2596,37 +2596,37 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>3.501</v>
+        <v>3.511</v>
       </c>
       <c r="G30" t="n">
-        <v>3.935</v>
+        <v>3.945</v>
       </c>
       <c r="H30" t="n">
-        <v>4.168</v>
+        <v>4.177</v>
       </c>
       <c r="I30" t="n">
-        <v>4.207</v>
+        <v>4.217</v>
       </c>
       <c r="J30" t="n">
-        <v>4.475</v>
+        <v>4.479</v>
       </c>
       <c r="K30" t="n">
-        <v>4.721</v>
+        <v>4.726</v>
       </c>
       <c r="L30" t="n">
-        <v>4.802</v>
+        <v>4.821</v>
       </c>
       <c r="M30" t="n">
-        <v>4.951</v>
+        <v>4.963</v>
       </c>
       <c r="N30" t="n">
-        <v>5.123</v>
+        <v>5.139</v>
       </c>
       <c r="O30" t="n">
-        <v>5.43</v>
+        <v>5.437</v>
       </c>
       <c r="P30" t="n">
-        <v>5.656</v>
+        <v>5.657</v>
       </c>
       <c r="Q30" t="n">
         <v>6.46</v>
@@ -2646,7 +2646,7 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -2669,37 +2669,37 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3.83</v>
+        <v>3.84</v>
       </c>
       <c r="G31" t="n">
-        <v>4.299</v>
+        <v>4.309</v>
       </c>
       <c r="H31" t="n">
-        <v>4.582</v>
+        <v>4.591</v>
       </c>
       <c r="I31" t="n">
-        <v>4.635</v>
+        <v>4.645</v>
       </c>
       <c r="J31" t="n">
-        <v>4.968</v>
+        <v>4.972</v>
       </c>
       <c r="K31" t="n">
-        <v>5.262</v>
+        <v>5.268</v>
       </c>
       <c r="L31" t="n">
-        <v>5.414</v>
+        <v>5.433</v>
       </c>
       <c r="M31" t="n">
-        <v>5.68</v>
+        <v>5.692</v>
       </c>
       <c r="N31" t="n">
-        <v>5.982</v>
+        <v>5.998</v>
       </c>
       <c r="O31" t="n">
-        <v>6.466</v>
+        <v>6.473</v>
       </c>
       <c r="P31" t="n">
-        <v>6.644</v>
+        <v>6.646</v>
       </c>
       <c r="Q31" t="n">
         <v>7.433</v>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -2742,37 +2742,37 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>3.599</v>
+        <v>3.609</v>
       </c>
       <c r="G32" t="n">
-        <v>4.051</v>
+        <v>4.061</v>
       </c>
       <c r="H32" t="n">
-        <v>4.31</v>
+        <v>4.319</v>
       </c>
       <c r="I32" t="n">
-        <v>4.365</v>
+        <v>4.375</v>
       </c>
       <c r="J32" t="n">
-        <v>4.656</v>
+        <v>4.66</v>
       </c>
       <c r="K32" t="n">
-        <v>4.907</v>
+        <v>4.913</v>
       </c>
       <c r="L32" t="n">
-        <v>5.006</v>
+        <v>5.026</v>
       </c>
       <c r="M32" t="n">
-        <v>5.224</v>
+        <v>5.236</v>
       </c>
       <c r="N32" t="n">
-        <v>5.484</v>
+        <v>5.501</v>
       </c>
       <c r="O32" t="n">
-        <v>5.875</v>
+        <v>5.882</v>
       </c>
       <c r="P32" t="n">
-        <v>6.116</v>
+        <v>6.117</v>
       </c>
       <c r="Q32" t="n">
         <v>6.921</v>
@@ -2792,7 +2792,7 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -2815,37 +2815,37 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>3.355</v>
+        <v>3.365</v>
       </c>
       <c r="G33" t="n">
-        <v>3.777</v>
+        <v>3.787</v>
       </c>
       <c r="H33" t="n">
-        <v>3.971</v>
+        <v>3.98</v>
       </c>
       <c r="I33" t="n">
-        <v>3.995</v>
+        <v>4.005</v>
       </c>
       <c r="J33" t="n">
-        <v>4.173</v>
+        <v>4.177</v>
       </c>
       <c r="K33" t="n">
-        <v>4.358</v>
+        <v>4.364</v>
       </c>
       <c r="L33" t="n">
-        <v>4.401</v>
+        <v>4.421</v>
       </c>
       <c r="M33" t="n">
-        <v>4.476</v>
+        <v>4.488</v>
       </c>
       <c r="N33" t="n">
-        <v>4.518</v>
+        <v>4.534</v>
       </c>
       <c r="O33" t="n">
-        <v>4.595</v>
+        <v>4.602</v>
       </c>
       <c r="P33" t="n">
-        <v>4.692</v>
+        <v>4.694</v>
       </c>
       <c r="Q33" t="n">
         <v>5.176</v>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -2888,37 +2888,37 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>3.418</v>
+        <v>3.428</v>
       </c>
       <c r="G34" t="n">
-        <v>3.839</v>
+        <v>3.849</v>
       </c>
       <c r="H34" t="n">
-        <v>4.038</v>
+        <v>4.047</v>
       </c>
       <c r="I34" t="n">
-        <v>4.066</v>
+        <v>4.076</v>
       </c>
       <c r="J34" t="n">
-        <v>4.247</v>
+        <v>4.251</v>
       </c>
       <c r="K34" t="n">
-        <v>4.438</v>
+        <v>4.445</v>
       </c>
       <c r="L34" t="n">
-        <v>4.481</v>
+        <v>4.501</v>
       </c>
       <c r="M34" t="n">
-        <v>4.568</v>
+        <v>4.58</v>
       </c>
       <c r="N34" t="n">
-        <v>4.623</v>
+        <v>4.639</v>
       </c>
       <c r="O34" t="n">
-        <v>4.764</v>
+        <v>4.771</v>
       </c>
       <c r="P34" t="n">
-        <v>4.987</v>
+        <v>4.988</v>
       </c>
       <c r="Q34" t="n">
         <v>5.877</v>
@@ -2938,7 +2938,7 @@
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -2961,37 +2961,37 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>3.389</v>
+        <v>3.399</v>
       </c>
       <c r="G35" t="n">
-        <v>3.808</v>
+        <v>3.818</v>
       </c>
       <c r="H35" t="n">
-        <v>4.006</v>
+        <v>4.015</v>
       </c>
       <c r="I35" t="n">
-        <v>4.031</v>
+        <v>4.041</v>
       </c>
       <c r="J35" t="n">
-        <v>4.213</v>
+        <v>4.217</v>
       </c>
       <c r="K35" t="n">
-        <v>4.389</v>
+        <v>4.395</v>
       </c>
       <c r="L35" t="n">
-        <v>4.435</v>
+        <v>4.455</v>
       </c>
       <c r="M35" t="n">
-        <v>4.515</v>
+        <v>4.526</v>
       </c>
       <c r="N35" t="n">
-        <v>4.559</v>
+        <v>4.575</v>
       </c>
       <c r="O35" t="n">
-        <v>4.661</v>
+        <v>4.668</v>
       </c>
       <c r="P35" t="n">
-        <v>4.789</v>
+        <v>4.791</v>
       </c>
       <c r="Q35" t="n">
         <v>5.513</v>
@@ -3011,7 +3011,7 @@
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -3034,37 +3034,37 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>3.27</v>
+        <v>3.28</v>
       </c>
       <c r="G36" t="n">
-        <v>3.676</v>
+        <v>3.687</v>
       </c>
       <c r="H36" t="n">
-        <v>3.871</v>
+        <v>3.88</v>
       </c>
       <c r="I36" t="n">
-        <v>3.899</v>
+        <v>3.909</v>
       </c>
       <c r="J36" t="n">
-        <v>4.106</v>
+        <v>4.109</v>
       </c>
       <c r="K36" t="n">
-        <v>4.283</v>
+        <v>4.287</v>
       </c>
       <c r="L36" t="n">
-        <v>4.321</v>
+        <v>4.34</v>
       </c>
       <c r="M36" t="n">
-        <v>4.376</v>
+        <v>4.386</v>
       </c>
       <c r="N36" t="n">
-        <v>4.419</v>
+        <v>4.434</v>
       </c>
       <c r="O36" t="n">
-        <v>4.504</v>
+        <v>4.511</v>
       </c>
       <c r="P36" t="n">
-        <v>4.591</v>
+        <v>4.592</v>
       </c>
       <c r="Q36" t="n">
         <v>4.891</v>
@@ -3084,7 +3084,7 @@
     </row>
     <row r="37">
       <c r="A37" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -3107,37 +3107,37 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>4.176</v>
+        <v>4.186</v>
       </c>
       <c r="G37" t="n">
-        <v>4.99</v>
+        <v>5</v>
       </c>
       <c r="H37" t="n">
-        <v>5.555</v>
+        <v>5.564</v>
       </c>
       <c r="I37" t="n">
-        <v>5.696</v>
+        <v>5.706</v>
       </c>
       <c r="J37" t="n">
-        <v>6.46</v>
+        <v>6.464</v>
       </c>
       <c r="K37" t="n">
-        <v>7.302</v>
+        <v>7.307</v>
       </c>
       <c r="L37" t="n">
-        <v>7.608</v>
+        <v>7.628</v>
       </c>
       <c r="M37" t="n">
-        <v>7.947</v>
+        <v>7.959</v>
       </c>
       <c r="N37" t="n">
-        <v>8.138999999999999</v>
+        <v>8.156000000000001</v>
       </c>
       <c r="O37" t="n">
-        <v>8.346</v>
+        <v>8.352</v>
       </c>
       <c r="P37" t="n">
-        <v>8.446</v>
+        <v>8.446999999999999</v>
       </c>
       <c r="Q37" t="n">
         <v>8.926</v>
@@ -3157,7 +3157,7 @@
     </row>
     <row r="38">
       <c r="A38" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -3180,37 +3180,37 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>5.238</v>
+        <v>5.248</v>
       </c>
       <c r="G38" t="n">
-        <v>6.306</v>
+        <v>6.316</v>
       </c>
       <c r="H38" t="n">
-        <v>7.082</v>
+        <v>7.091</v>
       </c>
       <c r="I38" t="n">
-        <v>7.381</v>
+        <v>7.392</v>
       </c>
       <c r="J38" t="n">
-        <v>8.406000000000001</v>
+        <v>8.41</v>
       </c>
       <c r="K38" t="n">
-        <v>9.428000000000001</v>
+        <v>9.433999999999999</v>
       </c>
       <c r="L38" t="n">
-        <v>9.898999999999999</v>
+        <v>9.917999999999999</v>
       </c>
       <c r="M38" t="n">
-        <v>10.36</v>
+        <v>10.372</v>
       </c>
       <c r="N38" t="n">
-        <v>10.558</v>
+        <v>10.575</v>
       </c>
       <c r="O38" t="n">
-        <v>10.746</v>
+        <v>10.753</v>
       </c>
       <c r="P38" t="n">
-        <v>10.844</v>
+        <v>10.845</v>
       </c>
       <c r="Q38" t="n">
         <v>11.376</v>
@@ -3230,7 +3230,7 @@
     </row>
     <row r="39">
       <c r="A39" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -3253,37 +3253,37 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4.558</v>
+        <v>4.568</v>
       </c>
       <c r="G39" t="n">
-        <v>5.505</v>
+        <v>5.515</v>
       </c>
       <c r="H39" t="n">
-        <v>6.148</v>
+        <v>6.157</v>
       </c>
       <c r="I39" t="n">
-        <v>6.384</v>
+        <v>6.395</v>
       </c>
       <c r="J39" t="n">
-        <v>7.278</v>
+        <v>7.282</v>
       </c>
       <c r="K39" t="n">
-        <v>8.26</v>
+        <v>8.266</v>
       </c>
       <c r="L39" t="n">
-        <v>8.651</v>
+        <v>8.670999999999999</v>
       </c>
       <c r="M39" t="n">
-        <v>8.997</v>
+        <v>9.009</v>
       </c>
       <c r="N39" t="n">
-        <v>9.186</v>
+        <v>9.202</v>
       </c>
       <c r="O39" t="n">
-        <v>9.396000000000001</v>
+        <v>9.403</v>
       </c>
       <c r="P39" t="n">
-        <v>9.497999999999999</v>
+        <v>9.5</v>
       </c>
       <c r="Q39" t="n">
         <v>10.022</v>
@@ -3303,7 +3303,7 @@
     </row>
     <row r="40">
       <c r="A40" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -3326,37 +3326,37 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>3.692</v>
+        <v>3.702</v>
       </c>
       <c r="G40" t="n">
-        <v>4.173</v>
+        <v>4.183</v>
       </c>
       <c r="H40" t="n">
-        <v>4.427</v>
+        <v>4.436</v>
       </c>
       <c r="I40" t="n">
-        <v>4.483</v>
+        <v>4.493</v>
       </c>
       <c r="J40" t="n">
-        <v>4.766</v>
+        <v>4.77</v>
       </c>
       <c r="K40" t="n">
-        <v>5.026</v>
+        <v>5.032</v>
       </c>
       <c r="L40" t="n">
-        <v>5.129</v>
+        <v>5.149</v>
       </c>
       <c r="M40" t="n">
-        <v>5.294</v>
+        <v>5.306</v>
       </c>
       <c r="N40" t="n">
-        <v>5.482</v>
+        <v>5.499</v>
       </c>
       <c r="O40" t="n">
-        <v>5.811</v>
+        <v>5.818</v>
       </c>
       <c r="P40" t="n">
-        <v>6.077</v>
+        <v>6.079</v>
       </c>
       <c r="Q40" t="n">
         <v>6.911</v>
@@ -3376,7 +3376,7 @@
     </row>
     <row r="41">
       <c r="A41" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -3399,37 +3399,37 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>4.079</v>
+        <v>4.089</v>
       </c>
       <c r="G41" t="n">
-        <v>4.601</v>
+        <v>4.611</v>
       </c>
       <c r="H41" t="n">
-        <v>4.911</v>
+        <v>4.92</v>
       </c>
       <c r="I41" t="n">
-        <v>4.985</v>
+        <v>4.995</v>
       </c>
       <c r="J41" t="n">
-        <v>5.323</v>
+        <v>5.327</v>
       </c>
       <c r="K41" t="n">
-        <v>5.636</v>
+        <v>5.641</v>
       </c>
       <c r="L41" t="n">
-        <v>5.804</v>
+        <v>5.824</v>
       </c>
       <c r="M41" t="n">
-        <v>6.095</v>
+        <v>6.107</v>
       </c>
       <c r="N41" t="n">
-        <v>6.411</v>
+        <v>6.428</v>
       </c>
       <c r="O41" t="n">
-        <v>6.924</v>
+        <v>6.931</v>
       </c>
       <c r="P41" t="n">
-        <v>7.137</v>
+        <v>7.138</v>
       </c>
       <c r="Q41" t="n">
         <v>7.958</v>
@@ -3449,7 +3449,7 @@
     </row>
     <row r="42">
       <c r="A42" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -3472,37 +3472,37 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>3.814</v>
+        <v>3.824</v>
       </c>
       <c r="G42" t="n">
-        <v>4.321</v>
+        <v>4.331</v>
       </c>
       <c r="H42" t="n">
-        <v>4.601</v>
+        <v>4.61</v>
       </c>
       <c r="I42" t="n">
-        <v>4.671</v>
+        <v>4.681</v>
       </c>
       <c r="J42" t="n">
-        <v>4.971</v>
+        <v>4.975</v>
       </c>
       <c r="K42" t="n">
-        <v>5.249</v>
+        <v>5.254</v>
       </c>
       <c r="L42" t="n">
-        <v>5.365</v>
+        <v>5.384</v>
       </c>
       <c r="M42" t="n">
-        <v>5.601</v>
+        <v>5.613</v>
       </c>
       <c r="N42" t="n">
-        <v>5.896</v>
+        <v>5.912</v>
       </c>
       <c r="O42" t="n">
-        <v>6.301</v>
+        <v>6.308</v>
       </c>
       <c r="P42" t="n">
-        <v>6.579</v>
+        <v>6.581</v>
       </c>
       <c r="Q42" t="n">
         <v>7.423</v>
@@ -3522,7 +3522,7 @@
     </row>
     <row r="43">
       <c r="A43" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -3545,37 +3545,37 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>3.505</v>
+        <v>3.515</v>
       </c>
       <c r="G43" t="n">
-        <v>3.964</v>
+        <v>3.974</v>
       </c>
       <c r="H43" t="n">
-        <v>4.176</v>
+        <v>4.185</v>
       </c>
       <c r="I43" t="n">
-        <v>4.208</v>
+        <v>4.218</v>
       </c>
       <c r="J43" t="n">
-        <v>4.4</v>
+        <v>4.404</v>
       </c>
       <c r="K43" t="n">
-        <v>4.591</v>
+        <v>4.597</v>
       </c>
       <c r="L43" t="n">
-        <v>4.644</v>
+        <v>4.664</v>
       </c>
       <c r="M43" t="n">
-        <v>4.733</v>
+        <v>4.744</v>
       </c>
       <c r="N43" t="n">
-        <v>4.787</v>
+        <v>4.804</v>
       </c>
       <c r="O43" t="n">
-        <v>4.909</v>
+        <v>4.915</v>
       </c>
       <c r="P43" t="n">
-        <v>5.058</v>
+        <v>5.059</v>
       </c>
       <c r="Q43" t="n">
         <v>5.786</v>
@@ -3595,7 +3595,7 @@
     </row>
     <row r="44">
       <c r="A44" s="1" t="n">
-        <v>46273</v>
+        <v>46274</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -3618,37 +3618,37 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>3.35</v>
+        <v>3.36</v>
       </c>
       <c r="G44" t="n">
-        <v>3.787</v>
+        <v>3.797</v>
       </c>
       <c r="H44" t="n">
-        <v>3.993</v>
+        <v>4.002</v>
       </c>
       <c r="I44" t="n">
-        <v>4.03</v>
+        <v>4.04</v>
       </c>
       <c r="J44" t="n">
-        <v>4.247</v>
+        <v>4.25</v>
       </c>
       <c r="K44" t="n">
-        <v>4.434</v>
+        <v>4.437</v>
       </c>
       <c r="L44" t="n">
-        <v>4.483</v>
+        <v>4.502</v>
       </c>
       <c r="M44" t="n">
-        <v>4.546</v>
+        <v>4.557</v>
       </c>
       <c r="N44" t="n">
-        <v>4.6</v>
+        <v>4.616</v>
       </c>
       <c r="O44" t="n">
-        <v>4.704</v>
+        <v>4.711</v>
       </c>
       <c r="P44" t="n">
-        <v>4.821</v>
+        <v>4.822</v>
       </c>
       <c r="Q44" t="n">
         <v>5.155</v>

</xml_diff>